<commit_message>
chore: sneaker release update [2026-03-19 10:52 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -178,10 +178,10 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -625,7 +625,7 @@
         <v>46100</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Nike GT Future “Unseen Hours”</t>
+          <t>Dylan Harper x Nike GT Cut 1 “Unseen Hours”</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
         <v>46100</v>
       </c>
       <c r="B5" s="10" t="n">
-        <v>200</v>
+        <v>135</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
@@ -662,7 +662,7 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Dylan Harper x Nike GT Cut 1 “Unseen Hours”</t>
+          <t>Nike Ja 3 “At Dawn”</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
         <v>46100</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “At Dawn”</t>
+          <t>Nike GT Future “Unseen Hours”</t>
         </is>
       </c>
     </row>
@@ -901,21 +901,21 @@
         <v>46102</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>215</v>
-      </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>300</v>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Black University Blue” 2026</t>
+          <t>Pharrell adidas Adistar Jellyfish “Triple Black”</t>
         </is>
       </c>
     </row>
@@ -924,21 +924,21 @@
         <v>46102</v>
       </c>
       <c r="B17" s="10" t="n">
-        <v>300</v>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Pharrell adidas Adistar Jellyfish “Triple Black”</t>
+          <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
         </is>
       </c>
     </row>
@@ -947,21 +947,21 @@
         <v>46102</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>250</v>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>1005</v>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
+          <t>Swarovski x Air Jordan 1 High OG</t>
         </is>
       </c>
     </row>
@@ -970,11 +970,11 @@
         <v>46102</v>
       </c>
       <c r="B19" s="10" t="n">
-        <v>1005</v>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
+        <v>215</v>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Swarovski x Air Jordan 1 High OG</t>
+          <t>Air Jordan 14 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       <c r="B21" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1041,7 +1041,7 @@
       <c r="B22" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1064,7 +1064,7 @@
       <c r="B23" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1087,7 +1087,7 @@
       <c r="B24" s="6" t="n">
         <v>130</v>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1110,7 +1110,7 @@
       <c r="B25" s="10" t="n">
         <v>200</v>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1133,7 +1133,7 @@
       <c r="B26" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1225,7 +1225,7 @@
       <c r="B30" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1248,7 +1248,7 @@
       <c r="B31" s="10" t="n">
         <v>150</v>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1271,7 +1271,7 @@
       <c r="B32" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="C32" s="13" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1317,7 +1317,7 @@
       <c r="B34" s="6" t="n">
         <v>240</v>
       </c>
-      <c r="C34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1340,7 +1340,7 @@
       <c r="B35" s="10" t="n">
         <v>240</v>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1361,11 +1361,11 @@
         <v>46109</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>230</v>
-      </c>
-      <c r="C36" s="13" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
+        <v>215</v>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -1384,21 +1384,21 @@
         <v>46109</v>
       </c>
       <c r="B37" s="10" t="n">
-        <v>215</v>
-      </c>
-      <c r="C37" s="14" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Nike GT Future “Swooshman”</t>
         </is>
       </c>
     </row>
@@ -1409,9 +1409,9 @@
       <c r="B38" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Nike GT Future “Swooshman”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
@@ -1429,10 +1429,8 @@
       <c r="A39" s="9" t="n">
         <v>46109</v>
       </c>
-      <c r="B39" s="10" t="n">
-        <v>190</v>
-      </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr"/>
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1444,7 +1442,7 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
@@ -1452,20 +1450,22 @@
       <c r="A40" s="5" t="n">
         <v>46109</v>
       </c>
-      <c r="B40" s="6" t="inlineStr"/>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B40" s="6" t="n">
+        <v>160</v>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>adidas BadBo 1.0 “Rise”</t>
         </is>
       </c>
     </row>
@@ -1474,21 +1474,21 @@
         <v>46109</v>
       </c>
       <c r="B41" s="10" t="n">
-        <v>160</v>
-      </c>
-      <c r="C41" s="16" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>230</v>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>adidas BadBo 1.0 “Rise”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       <c r="B42" s="6" t="n">
         <v>162</v>
       </c>
-      <c r="C42" s="13" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1568,7 +1568,7 @@
       <c r="B45" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="C45" s="14" t="inlineStr">
+      <c r="C45" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1683,7 +1683,7 @@
       <c r="B50" s="6" t="n">
         <v>235</v>
       </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1706,7 +1706,7 @@
       <c r="B51" s="10" t="n">
         <v>205</v>
       </c>
-      <c r="C51" s="14" t="inlineStr">
+      <c r="C51" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1796,21 +1796,21 @@
         <v>46123</v>
       </c>
       <c r="B55" s="10" t="n">
-        <v>170</v>
-      </c>
-      <c r="C55" s="11" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>185</v>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="E55" s="12" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -1819,21 +1819,21 @@
         <v>46123</v>
       </c>
       <c r="B56" s="6" t="n">
-        <v>185</v>
-      </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1865,7 @@
         <v>46125</v>
       </c>
       <c r="B58" s="6" t="inlineStr"/>
-      <c r="C58" s="13" t="inlineStr">
+      <c r="C58" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1888,7 +1888,7 @@
       <c r="B59" s="10" t="n">
         <v>220</v>
       </c>
-      <c r="C59" s="14" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1934,7 +1934,7 @@
       <c r="B61" s="10" t="n">
         <v>240</v>
       </c>
-      <c r="C61" s="14" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1980,7 +1980,7 @@
       <c r="B63" s="10" t="n">
         <v>240</v>
       </c>
-      <c r="C63" s="14" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2076,21 +2076,21 @@
         <v>46102</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>215</v>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
+        <v>250</v>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Black University Blue” 2026</t>
+          <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
         </is>
       </c>
     </row>
@@ -2099,21 +2099,21 @@
         <v>46102</v>
       </c>
       <c r="B5" s="10" t="n">
-        <v>250</v>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>1005</v>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
+          <t>Swarovski x Air Jordan 1 High OG</t>
         </is>
       </c>
     </row>
@@ -2122,11 +2122,11 @@
         <v>46102</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>1005</v>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
+        <v>215</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Swarovski x Air Jordan 1 High OG</t>
+          <t>Air Jordan 14 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       <c r="B7" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2170,7 +2170,7 @@
       <c r="B8" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2193,7 +2193,7 @@
       <c r="B9" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2216,7 +2216,7 @@
       <c r="B10" s="6" t="n">
         <v>130</v>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2239,7 +2239,7 @@
       <c r="B11" s="10" t="n">
         <v>200</v>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2262,7 +2262,7 @@
       <c r="B12" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2285,7 +2285,7 @@
       <c r="B13" s="10" t="n">
         <v>200</v>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2308,7 +2308,7 @@
       <c r="B14" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2331,7 +2331,7 @@
       <c r="B15" s="10" t="n">
         <v>190</v>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2354,7 +2354,7 @@
       <c r="B16" s="6" t="n">
         <v>240</v>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2377,7 +2377,7 @@
       <c r="B17" s="10" t="n">
         <v>240</v>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2398,11 +2398,11 @@
         <v>46109</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>230</v>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
+        <v>215</v>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -2421,21 +2421,21 @@
         <v>46109</v>
       </c>
       <c r="B19" s="10" t="n">
-        <v>215</v>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
@@ -2443,10 +2443,8 @@
       <c r="A20" s="5" t="n">
         <v>46109</v>
       </c>
-      <c r="B20" s="6" t="n">
-        <v>190</v>
-      </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr"/>
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2458,7 +2456,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
@@ -2466,20 +2464,22 @@
       <c r="A21" s="9" t="n">
         <v>46109</v>
       </c>
-      <c r="B21" s="10" t="inlineStr"/>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B21" s="10" t="n">
+        <v>230</v>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       <c r="B22" s="6" t="n">
         <v>162</v>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2513,7 +2513,7 @@
       <c r="B23" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2536,7 +2536,7 @@
       <c r="B24" s="6" t="n">
         <v>235</v>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2559,7 +2559,7 @@
       <c r="B25" s="10" t="n">
         <v>205</v>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2582,7 +2582,7 @@
       <c r="B26" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2603,7 +2603,7 @@
         <v>46125</v>
       </c>
       <c r="B27" s="10" t="inlineStr"/>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2626,7 +2626,7 @@
       <c r="B28" s="6" t="n">
         <v>220</v>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2649,7 +2649,7 @@
       <c r="B29" s="10" t="n">
         <v>240</v>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2672,7 +2672,7 @@
       <c r="B30" s="6" t="n">
         <v>240</v>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2721,7 +2721,7 @@
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-19 10:44 UTC</t>
+          <t>Generated: 2026-03-19 10:52 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-19 11:10 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$3:$E$63</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Hype Alerts'!$A$3:$E$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$3:$F$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Hype Alerts'!$A$3:$F$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -561,14 +561,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -581,6 +582,7 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -592,6 +594,7 @@
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -611,10 +614,15 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
+          <t>Sale Method</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Style</t>
         </is>
@@ -634,10 +642,15 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Dylan Harper x Nike GT Cut 1 “Unseen Hours”</t>
         </is>
@@ -657,10 +670,15 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Nike Ja 3 “At Dawn”</t>
         </is>
@@ -680,10 +698,15 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Nike GT Future “Unseen Hours”</t>
         </is>
@@ -703,10 +726,15 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Fragment x Nike Mind 001</t>
         </is>
@@ -726,10 +754,15 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Fragment x Nike Mind 002</t>
         </is>
@@ -749,10 +782,15 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Nike Ja 3 “Tri-State”</t>
         </is>
@@ -772,10 +810,15 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Nike GT Cut “Dylan Harper”</t>
         </is>
@@ -795,10 +838,15 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Nike Book 2 “Must Be The Denim”</t>
         </is>
@@ -818,10 +866,15 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Nike Zoom Hyperflight “Black”</t>
         </is>
@@ -841,10 +894,15 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>Nike KD 6 “Peanut Butter Jelly” 2026</t>
         </is>
@@ -864,10 +922,15 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Nike KD 6 “PBJ”</t>
         </is>
@@ -887,10 +950,15 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>Nike Zoom Hyperflight</t>
         </is>
@@ -910,10 +978,15 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Pharrell adidas Adistar Jellyfish “Triple Black”</t>
         </is>
@@ -933,10 +1006,15 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
         </is>
@@ -956,10 +1034,15 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Swarovski x Air Jordan 1 High OG</t>
         </is>
@@ -979,10 +1062,15 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>Air Jordan 14 “Black University Blue” 2026</t>
         </is>
@@ -1002,10 +1090,15 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Avirex x adidas Superstar 82</t>
         </is>
@@ -1025,10 +1118,15 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
         </is>
@@ -1048,10 +1146,15 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
         </is>
@@ -1071,10 +1174,15 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
         </is>
@@ -1094,10 +1202,15 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
         </is>
@@ -1117,10 +1230,15 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
         </is>
@@ -1140,10 +1258,15 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Masked Menace”</t>
         </is>
@@ -1163,10 +1286,15 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Thug Club x adidas Adifom IIInfinity Mule</t>
         </is>
@@ -1186,10 +1314,15 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>Thug Club x adidas Superstar Vintage</t>
         </is>
@@ -1209,10 +1342,15 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Thug Club x adidas AdiFom Megaride</t>
         </is>
@@ -1232,10 +1370,15 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
         <is>
           <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
@@ -1255,10 +1398,15 @@
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
         <is>
           <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
@@ -1278,10 +1426,15 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
         <is>
           <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
@@ -1301,10 +1454,15 @@
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
         <is>
           <t>Nike Air Liquid Max “Poison Dart Frog”</t>
         </is>
@@ -1324,10 +1482,15 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
@@ -1347,10 +1510,15 @@
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
@@ -1370,10 +1538,15 @@
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="F36" s="8" t="inlineStr">
         <is>
           <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
@@ -1393,10 +1566,15 @@
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
         <is>
           <t>Nike GT Future “Swooshman”</t>
         </is>
@@ -1416,10 +1594,15 @@
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
         <is>
           <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
@@ -1437,10 +1620,15 @@
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
         <is>
           <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
@@ -1460,10 +1648,15 @@
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="F40" s="8" t="inlineStr">
         <is>
           <t>adidas BadBo 1.0 “Rise”</t>
         </is>
@@ -1483,10 +1676,15 @@
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E41" s="12" t="inlineStr">
+      <c r="F41" s="12" t="inlineStr">
         <is>
           <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
@@ -1506,10 +1704,15 @@
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
@@ -1529,10 +1732,15 @@
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
         <is>
           <t>Nike GT Future “Galaxy Aura”</t>
         </is>
@@ -1552,10 +1760,15 @@
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr">
+      <c r="F44" s="8" t="inlineStr">
         <is>
           <t>Jordan Jumpman Pro “Black Concord”</t>
         </is>
@@ -1575,10 +1788,15 @@
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
         <is>
           <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
@@ -1598,10 +1816,15 @@
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
         <is>
           <t>Nike Sabrina 3 “What The”</t>
         </is>
@@ -1621,10 +1844,15 @@
       </c>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E47" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
         <is>
           <t>Nike Mind 001 “Geode Teal”</t>
         </is>
@@ -1644,10 +1872,15 @@
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
           <t>Converse</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="F48" s="8" t="inlineStr">
         <is>
           <t>Converse SHAI 001 “Camo”</t>
         </is>
@@ -1667,10 +1900,15 @@
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr">
         <is>
           <t>Fragment x Nike Air Liquid Max</t>
         </is>
@@ -1690,10 +1928,15 @@
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
@@ -1713,10 +1956,15 @@
       </c>
       <c r="D51" s="12" t="inlineStr">
         <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E51" s="12" t="inlineStr">
+      <c r="F51" s="12" t="inlineStr">
         <is>
           <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
@@ -1736,10 +1984,15 @@
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
         <is>
           <t>Nike Ja 3 “Jurassic Park”</t>
         </is>
@@ -1759,10 +2012,15 @@
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F53" s="12" t="inlineStr">
         <is>
           <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
@@ -1782,10 +2040,15 @@
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
         <is>
           <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
@@ -1805,10 +2068,15 @@
       </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E55" s="12" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E55" s="12" t="inlineStr">
+      <c r="F55" s="12" t="inlineStr">
         <is>
           <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
@@ -1828,10 +2096,15 @@
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
         <is>
           <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
@@ -1851,10 +2124,15 @@
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="inlineStr">
+        <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="E57" s="12" t="inlineStr">
+      <c r="F57" s="12" t="inlineStr">
         <is>
           <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
@@ -1872,10 +2150,15 @@
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="inlineStr">
         <is>
           <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
@@ -1895,10 +2178,15 @@
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F59" s="12" t="inlineStr">
         <is>
           <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
@@ -1918,10 +2206,15 @@
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
+      <c r="F60" s="8" t="inlineStr">
         <is>
           <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
@@ -1941,10 +2234,15 @@
       </c>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E61" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F61" s="12" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
@@ -1964,10 +2262,15 @@
       </c>
       <c r="D62" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
         <is>
           <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
@@ -1987,20 +2290,25 @@
       </c>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F63" s="12" t="inlineStr">
+        <is>
           <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E63"/>
+  <autoFilter ref="A3:F63"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2012,14 +2320,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2032,6 +2341,7 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -2043,6 +2353,7 @@
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -2062,10 +2373,15 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
+          <t>Sale Method</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Style</t>
         </is>
@@ -2085,10 +2401,15 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
         </is>
@@ -2108,10 +2429,15 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Swarovski x Air Jordan 1 High OG</t>
         </is>
@@ -2131,10 +2457,15 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Air Jordan 14 “Black University Blue” 2026</t>
         </is>
@@ -2154,10 +2485,15 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
         </is>
@@ -2177,10 +2513,15 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
         </is>
@@ -2200,10 +2541,15 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
         </is>
@@ -2223,10 +2569,15 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
         </is>
@@ -2246,10 +2597,15 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
         </is>
@@ -2269,10 +2625,15 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Masked Menace”</t>
         </is>
@@ -2292,10 +2653,15 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
@@ -2315,10 +2681,15 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
@@ -2338,10 +2709,15 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
@@ -2361,10 +2737,15 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
@@ -2384,10 +2765,15 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
@@ -2407,10 +2793,15 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
@@ -2430,10 +2821,15 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
@@ -2451,10 +2847,15 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
@@ -2474,10 +2875,15 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
@@ -2497,10 +2903,15 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
@@ -2520,10 +2931,15 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
@@ -2543,10 +2959,15 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
@@ -2566,10 +2987,15 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
@@ -2589,10 +3015,15 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
@@ -2610,10 +3041,15 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
@@ -2633,10 +3069,15 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
@@ -2656,10 +3097,15 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
@@ -2679,20 +3125,25 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
           <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E30"/>
+  <autoFilter ref="A3:F30"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2721,7 +3172,7 @@
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-19 10:59 UTC</t>
+          <t>Generated: 2026-03-19 11:10 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-21 04:49 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$3:$F$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$3:$F$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Hype Alerts'!$A$3:$F$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -60,7 +60,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFC000"/>
+      <color rgb="00FF0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FF6B35"/>
       <sz val="11"/>
     </font>
     <font>
@@ -72,19 +78,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FF0000"/>
+      <color rgb="00FFC000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FF9800"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FF6B35"/>
       <sz val="11"/>
     </font>
     <font>
@@ -196,28 +196,16 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -226,15 +214,27 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -669,42 +669,42 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="5" t="n">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>145</v>
+        <v>1005</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Must Be The Denim”</t>
+          <t>Swarovski x Air Jordan 1 High OG</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="10" t="n">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B5" s="11" t="n">
-        <v>170</v>
+        <v>215</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -714,58 +714,58 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Black”</t>
+          <t>Air Jordan 14 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="n">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>140</v>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
+        <v>300</v>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Peanut Butter Jelly” 2026</t>
+          <t>Pharrell adidas Adistar Jellyfish “Triple Black”</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="10" t="n">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B7" s="11" t="n">
-        <v>145</v>
+        <v>250</v>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -775,104 +775,104 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Nike KD 6 “PBJ”</t>
+          <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="5" t="n">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>170</v>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight</t>
+          <t>Avirex x adidas Superstar 82</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="10" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>1005</v>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>120</v>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Swarovski x Air Jordan 1 High OG</t>
+          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="5" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>215</v>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Black University Blue” 2026</t>
+          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="10" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B11" s="11" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -882,30 +882,30 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Pharrell adidas Adistar Jellyfish “Triple Black”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="5" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>250</v>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>130</v>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -915,20 +915,20 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
+          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="10" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B13" s="11" t="n">
-        <v>180</v>
-      </c>
-      <c r="C13" s="20" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
@@ -938,30 +938,30 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Avirex x adidas Superstar 82</t>
+          <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="5" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>120</v>
-      </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>210</v>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -971,107 +971,107 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
+          <t>Nike LeBron 23 “Masked Menace”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="10" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B15" s="11" t="n">
-        <v>200</v>
-      </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D15" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>80</v>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
+          <t>Thug Club x adidas Adifom IIInfinity Mule</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="5" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>120</v>
-      </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
+          <t>Thug Club x adidas Superstar Vintage</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="10" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B17" s="11" t="n">
-        <v>130</v>
-      </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D17" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>170</v>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
+          <t>Thug Club x adidas AdiFom Megaride</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="5" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B18" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -1083,25 +1083,25 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
+          <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="10" t="n">
-        <v>46105</v>
+        <v>46107</v>
       </c>
       <c r="B19" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D19" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
@@ -1111,48 +1111,48 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Masked Menace”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="5" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>80</v>
-      </c>
-      <c r="C20" s="22" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Thug Club x adidas Adifom IIInfinity Mule</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="10" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B21" s="11" t="n">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="C21" s="20" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -1162,58 +1162,58 @@
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Thug Club x adidas Superstar Vintage</t>
+          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="5" t="n">
-        <v>46106</v>
+        <v>46108</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>170</v>
-      </c>
-      <c r="C22" s="22" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
+        <v>240</v>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Thug Club x adidas AdiFom Megaride</t>
+          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="10" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B23" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D23" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
@@ -1223,25 +1223,25 @@
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Paisley Bandana”</t>
+          <t>Nike GT Cut “Dylan Harper”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="5" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>150</v>
-      </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>240</v>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -1251,18 +1251,18 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="10" t="n">
-        <v>46107</v>
+        <v>46109</v>
       </c>
       <c r="B25" s="11" t="n">
         <v>190</v>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1279,25 +1279,23 @@
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="5" t="n">
-        <v>46107</v>
-      </c>
-      <c r="B26" s="6" t="n">
-        <v>230</v>
-      </c>
+        <v>46109</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr"/>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -1307,91 +1305,91 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="10" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B27" s="11" t="n">
-        <v>240</v>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D27" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
+          <t>adidas BadBo 1.0 “Rise”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="5" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Nike GT Cut “Dylan Harper”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="10" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B29" s="11" t="n">
-        <v>240</v>
-      </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D29" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>215</v>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F29" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -1402,12 +1400,12 @@
       <c r="B30" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -1419,7 +1417,7 @@
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>Nike GT Future “Swooshman”</t>
         </is>
       </c>
     </row>
@@ -1427,15 +1425,17 @@
       <c r="A31" s="10" t="n">
         <v>46109</v>
       </c>
-      <c r="B31" s="11" t="inlineStr"/>
-      <c r="C31" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D31" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B31" s="11" t="n">
+        <v>162</v>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="14" t="inlineStr">
@@ -1445,53 +1445,53 @@
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="5" t="n">
-        <v>46109</v>
+        <v>46111</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>160</v>
-      </c>
-      <c r="C32" s="22" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>210</v>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>adidas BadBo 1.0 “Rise”</t>
+          <t>Nike GT Future “Galaxy Aura”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="10" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B33" s="11" t="n">
-        <v>230</v>
-      </c>
-      <c r="C33" s="15" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D33" s="16" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>145</v>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="14" t="inlineStr">
@@ -1501,46 +1501,46 @@
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Jordan Jumpman Pro “Black Concord”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="5" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>215</v>
-      </c>
-      <c r="C34" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D34" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="10" t="n">
-        <v>46109</v>
+        <v>46113</v>
       </c>
       <c r="B35" s="11" t="n">
-        <v>190</v>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1557,25 +1557,25 @@
       </c>
       <c r="F35" s="14" t="inlineStr">
         <is>
-          <t>Nike GT Future “Swooshman”</t>
+          <t>Nike Sabrina 3 “What The”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="5" t="n">
-        <v>46109</v>
+        <v>46114</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>162</v>
-      </c>
-      <c r="C36" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D36" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>95</v>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
@@ -1585,18 +1585,18 @@
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 (GS)</t>
+          <t>Nike Mind 001 “Sail”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="10" t="n">
-        <v>46111</v>
+        <v>46114</v>
       </c>
       <c r="B37" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1613,53 +1613,53 @@
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>Nike GT Future “Galaxy Aura”</t>
+          <t>Nike Mind 001 “Geode Teal”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="5" t="n">
-        <v>46112</v>
+        <v>46115</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>145</v>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
+        <v>130</v>
+      </c>
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Jordan Jumpman Pro “Black Concord”</t>
+          <t>Converse SHAI 001 “Camo”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="10" t="n">
-        <v>46112</v>
+        <v>46115</v>
       </c>
       <c r="B39" s="11" t="n">
-        <v>130</v>
-      </c>
-      <c r="C39" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D39" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>225</v>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E39" s="14" t="inlineStr">
@@ -1669,23 +1669,23 @@
       </c>
       <c r="F39" s="14" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="5" t="n">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B40" s="6" t="n">
-        <v>145</v>
+        <v>235</v>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1697,20 +1697,20 @@
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Nike Sabrina 3 “What The”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="10" t="n">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B41" s="11" t="n">
-        <v>95</v>
+        <v>205</v>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
@@ -1720,28 +1720,28 @@
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="14" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Sail”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="5" t="n">
-        <v>46114</v>
+        <v>46122</v>
       </c>
       <c r="B42" s="6" t="n">
-        <v>95</v>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr">
+      <c r="D42" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1753,20 +1753,20 @@
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Geode Teal”</t>
+          <t>Nike Ja 3 “Jurassic Park”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="10" t="n">
-        <v>46115</v>
+        <v>46122</v>
       </c>
       <c r="B43" s="11" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C43" s="20" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
@@ -1776,28 +1776,28 @@
       </c>
       <c r="E43" s="14" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="14" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 “Camo”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="5" t="n">
-        <v>46115</v>
+        <v>46122</v>
       </c>
       <c r="B44" s="6" t="n">
-        <v>225</v>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D44" s="8" t="inlineStr">
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1809,25 +1809,25 @@
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="10" t="n">
-        <v>46115</v>
+        <v>46123</v>
       </c>
       <c r="B45" s="11" t="n">
-        <v>235</v>
-      </c>
-      <c r="C45" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D45" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>170</v>
+      </c>
+      <c r="C45" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E45" s="14" t="inlineStr">
@@ -1837,25 +1837,25 @@
       </c>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="5" t="n">
-        <v>46116</v>
+        <v>46123</v>
       </c>
       <c r="B46" s="6" t="n">
-        <v>205</v>
-      </c>
-      <c r="C46" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D46" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>185</v>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
@@ -1865,20 +1865,20 @@
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="10" t="n">
-        <v>46122</v>
+        <v>46124</v>
       </c>
       <c r="B47" s="11" t="n">
-        <v>135</v>
-      </c>
-      <c r="C47" s="12" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
@@ -1888,30 +1888,28 @@
       </c>
       <c r="E47" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F47" s="14" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Jurassic Park”</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="5" t="n">
-        <v>46122</v>
-      </c>
-      <c r="B48" s="6" t="n">
-        <v>135</v>
-      </c>
+        <v>46125</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr"/>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -1921,20 +1919,20 @@
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="10" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B49" s="11" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
@@ -1949,23 +1947,23 @@
       </c>
       <c r="F49" s="14" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="5" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B50" s="6" t="n">
-        <v>170</v>
+        <v>220</v>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1977,79 +1975,81 @@
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="10" t="n">
-        <v>46123</v>
+        <v>46128</v>
       </c>
       <c r="B51" s="11" t="n">
-        <v>185</v>
-      </c>
-      <c r="C51" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D51" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E51" s="14" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F51" s="14" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="5" t="n">
-        <v>46124</v>
+        <v>46129</v>
       </c>
       <c r="B52" s="6" t="n">
-        <v>130</v>
-      </c>
-      <c r="C52" s="22" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
+        <v>240</v>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="10" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B53" s="11" t="inlineStr"/>
-      <c r="C53" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D53" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>46130</v>
+      </c>
+      <c r="B53" s="11" t="n">
+        <v>240</v>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E53" s="14" t="inlineStr">
@@ -2059,23 +2059,23 @@
       </c>
       <c r="F53" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="5" t="n">
-        <v>46125</v>
+        <v>46130</v>
       </c>
       <c r="B54" s="6" t="n">
-        <v>190</v>
-      </c>
-      <c r="C54" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D54" s="18" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -2087,152 +2087,12 @@
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="15" customHeight="1">
-      <c r="A55" s="10" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B55" s="11" t="n">
-        <v>220</v>
-      </c>
-      <c r="C55" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D55" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="E55" s="14" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F55" s="14" t="inlineStr">
-        <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="5" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B56" s="6" t="n">
-        <v>160</v>
-      </c>
-      <c r="C56" s="22" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t>Adidas</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="inlineStr">
-        <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="10" t="n">
-        <v>46129</v>
-      </c>
-      <c r="B57" s="11" t="n">
-        <v>240</v>
-      </c>
-      <c r="C57" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D57" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F57" s="14" t="inlineStr">
-        <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="15" customHeight="1">
-      <c r="A58" s="5" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B58" s="6" t="n">
-        <v>240</v>
-      </c>
-      <c r="C58" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D58" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="E58" s="9" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="inlineStr">
-        <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="10" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B59" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D59" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E59" s="14" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F59" s="14" t="inlineStr">
-        <is>
           <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F59"/>
+  <autoFilter ref="A3:F54"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -2321,14 +2181,14 @@
       <c r="B4" s="6" t="n">
         <v>1005</v>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>EXTREME</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2349,14 +2209,14 @@
       <c r="B5" s="11" t="n">
         <v>215</v>
       </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -2377,12 +2237,12 @@
       <c r="B6" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Raffle</t>
         </is>
@@ -2405,14 +2265,14 @@
       <c r="B7" s="11" t="n">
         <v>120</v>
       </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -2433,14 +2293,14 @@
       <c r="B8" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2461,14 +2321,14 @@
       <c r="B9" s="11" t="n">
         <v>120</v>
       </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
@@ -2489,14 +2349,14 @@
       <c r="B10" s="6" t="n">
         <v>130</v>
       </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2517,14 +2377,14 @@
       <c r="B11" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="C11" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -2545,14 +2405,14 @@
       <c r="B12" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2573,7 +2433,7 @@
       <c r="B13" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2601,14 +2461,14 @@
       <c r="B14" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2629,14 +2489,14 @@
       <c r="B15" s="11" t="n">
         <v>190</v>
       </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D15" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -2657,14 +2517,14 @@
       <c r="B16" s="6" t="n">
         <v>240</v>
       </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -2685,14 +2545,14 @@
       <c r="B17" s="11" t="n">
         <v>240</v>
       </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D17" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -2713,12 +2573,12 @@
       <c r="B18" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -2739,7 +2599,7 @@
         <v>46109</v>
       </c>
       <c r="B19" s="11" t="inlineStr"/>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2767,14 +2627,14 @@
       <c r="B20" s="6" t="n">
         <v>230</v>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>EXTREME</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -2795,14 +2655,14 @@
       <c r="B21" s="11" t="n">
         <v>215</v>
       </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D21" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -2823,14 +2683,14 @@
       <c r="B22" s="6" t="n">
         <v>162</v>
       </c>
-      <c r="C22" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -2851,14 +2711,14 @@
       <c r="B23" s="11" t="n">
         <v>130</v>
       </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D23" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
@@ -2879,14 +2739,14 @@
       <c r="B24" s="6" t="n">
         <v>235</v>
       </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -2907,14 +2767,14 @@
       <c r="B25" s="11" t="n">
         <v>205</v>
       </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D25" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
@@ -2935,14 +2795,14 @@
       <c r="B26" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -2961,7 +2821,7 @@
         <v>46125</v>
       </c>
       <c r="B27" s="11" t="inlineStr"/>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2989,14 +2849,14 @@
       <c r="B28" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3017,14 +2877,14 @@
       <c r="B29" s="11" t="n">
         <v>220</v>
       </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D29" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
@@ -3045,14 +2905,14 @@
       <c r="B30" s="6" t="n">
         <v>240</v>
       </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D30" s="18" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3073,14 +2933,14 @@
       <c r="B31" s="11" t="n">
         <v>240</v>
       </c>
-      <c r="C31" s="15" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D31" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="14" t="inlineStr">
@@ -3127,14 +2987,14 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-20 07:59 UTC</t>
+          <t>Generated: 2026-03-21 04:49 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>Total releases tracked: 56</t>
+          <t>Total releases tracked: 51</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3012,7 @@
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -3219,7 +3079,7 @@
         </is>
       </c>
       <c r="B14" s="24" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -3246,7 +3106,7 @@
         </is>
       </c>
       <c r="B18" s="24" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19">
@@ -3256,7 +3116,7 @@
         </is>
       </c>
       <c r="B19" s="24" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
@@ -3266,7 +3126,7 @@
         </is>
       </c>
       <c r="B20" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-22 04:14 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$3:$F$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Hype Alerts'!$A$3:$F$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$3:$F$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Hype Alerts'!$A$3:$F$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="M/D/YYYY"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,31 +66,25 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00888888"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0000B050"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FF6B35"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00888888"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFC000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FF9800"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0000B050"/>
       <sz val="11"/>
     </font>
     <font>
@@ -160,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -196,45 +190,38 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -600,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -669,38 +656,38 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="5" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>1005</v>
+        <v>120</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>EXTREME</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Swarovski x Air Jordan 1 High OG</t>
+          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="10" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B5" s="11" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
@@ -714,58 +701,58 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Black University Blue” 2026</t>
+          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>300</v>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
+        <v>120</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Pharrell adidas Adistar Jellyfish “Triple Black”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="10" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B7" s="11" t="n">
-        <v>250</v>
+        <v>130</v>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -775,44 +762,44 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
+          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="5" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Avirex x adidas Superstar 82</t>
+          <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="10" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>120</v>
+        <v>210</v>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
@@ -831,48 +818,48 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
+          <t>Nike LeBron 23 “Masked Menace”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="5" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>200</v>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
+        <v>80</v>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
+          <t>Thug Club x adidas Adifom IIInfinity Mule</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="10" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B11" s="11" t="n">
-        <v>120</v>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -882,46 +869,46 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
+          <t>Thug Club x adidas Superstar Vintage</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="5" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>130</v>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
+          <t>Thug Club x adidas AdiFom Megaride</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="10" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>200</v>
@@ -931,9 +918,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -943,23 +930,23 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
+          <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="5" t="n">
-        <v>46105</v>
+        <v>46107</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -971,20 +958,20 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Masked Menace”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="10" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B15" s="11" t="n">
-        <v>80</v>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
@@ -994,53 +981,53 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Thug Club x adidas Adifom IIInfinity Mule</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="5" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>160</v>
-      </c>
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Thug Club x adidas Superstar Vintage</t>
+          <t>Nike Air Max 95 “Greedy”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="10" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B17" s="11" t="n">
-        <v>170</v>
-      </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>230</v>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -1050,21 +1037,21 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Thug Club x adidas AdiFom Megaride</t>
+          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="5" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
@@ -1073,7 +1060,7 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -1083,20 +1070,20 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Paisley Bandana”</t>
+          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="10" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B19" s="11" t="n">
-        <v>150</v>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
@@ -1111,23 +1098,23 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Nike GT Cut “Dylan Harper”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="5" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1139,25 +1126,25 @@
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="10" t="n">
-        <v>46107</v>
+        <v>46109</v>
       </c>
       <c r="B21" s="11" t="n">
-        <v>230</v>
-      </c>
-      <c r="C21" s="20" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -1167,25 +1154,25 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
+          <t>Nike GT Future “Swooshman”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="5" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -1195,25 +1182,23 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="10" t="n">
-        <v>46108</v>
-      </c>
-      <c r="B23" s="11" t="n">
-        <v>200</v>
-      </c>
-      <c r="C23" s="20" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46109</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr"/>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
@@ -1223,35 +1208,35 @@
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Nike GT Cut “Dylan Harper”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="5" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>240</v>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
+        <v>160</v>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue”</t>
+          <t>adidas BadBo 1.0 “Rise”</t>
         </is>
       </c>
     </row>
@@ -1260,26 +1245,26 @@
         <v>46109</v>
       </c>
       <c r="B25" s="11" t="n">
-        <v>190</v>
+        <v>230</v>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D25" s="21" t="inlineStr">
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1272,9 @@
       <c r="A26" s="5" t="n">
         <v>46109</v>
       </c>
-      <c r="B26" s="6" t="inlineStr"/>
+      <c r="B26" s="6" t="n">
+        <v>215</v>
+      </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -1295,17 +1282,17 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -1314,11 +1301,11 @@
         <v>46109</v>
       </c>
       <c r="B27" s="11" t="n">
-        <v>160</v>
-      </c>
-      <c r="C27" s="19" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>162</v>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
@@ -1328,53 +1315,53 @@
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>adidas BadBo 1.0 “Rise”</t>
+          <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="5" t="n">
-        <v>46109</v>
+        <v>46111</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>230</v>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Nike GT Future “Galaxy Aura”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="10" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B29" s="11" t="n">
-        <v>215</v>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
@@ -1389,25 +1376,25 @@
       </c>
       <c r="F29" s="14" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Jordan Jumpman Pro “Black Concord”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="5" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>190</v>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -1417,20 +1404,20 @@
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Nike GT Future “Swooshman”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="10" t="n">
-        <v>46109</v>
+        <v>46113</v>
       </c>
       <c r="B31" s="11" t="n">
-        <v>162</v>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -1445,25 +1432,25 @@
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 (GS)</t>
+          <t>Nike Sabrina 3 “What The”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="5" t="n">
-        <v>46111</v>
+        <v>46114</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="C32" s="15" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -1473,18 +1460,18 @@
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Nike GT Future “Galaxy Aura”</t>
+          <t>Nike Mind 001 “Sail”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="10" t="n">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B33" s="11" t="n">
-        <v>145</v>
-      </c>
-      <c r="C33" s="20" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1496,51 +1483,51 @@
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>Jordan Jumpman Pro “Black Concord”</t>
+          <t>Nike Mind 001 “Geode Teal”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="5" t="n">
-        <v>46112</v>
+        <v>46115</v>
       </c>
       <c r="B34" s="6" t="n">
         <v>130</v>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Converse SHAI 001 “Camo”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="10" t="n">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B35" s="11" t="n">
-        <v>145</v>
-      </c>
-      <c r="C35" s="20" t="inlineStr">
+        <v>225</v>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1557,23 +1544,23 @@
       </c>
       <c r="F35" s="14" t="inlineStr">
         <is>
-          <t>Nike Sabrina 3 “What The”</t>
+          <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="5" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>95</v>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D36" s="16" t="inlineStr">
+        <v>235</v>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1585,20 +1572,20 @@
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Sail”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="10" t="n">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B37" s="11" t="n">
-        <v>95</v>
-      </c>
-      <c r="C37" s="20" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
@@ -1608,51 +1595,51 @@
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Geode Teal”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="5" t="n">
-        <v>46115</v>
+        <v>46122</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>130</v>
-      </c>
-      <c r="C38" s="18" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C38" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 “Camo”</t>
+          <t>Nike Ja 3 “Jurassic Park”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="10" t="n">
-        <v>46115</v>
+        <v>46122</v>
       </c>
       <c r="B39" s="11" t="n">
-        <v>225</v>
-      </c>
-      <c r="C39" s="20" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C39" s="18" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1669,23 +1656,23 @@
       </c>
       <c r="F39" s="14" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="5" t="n">
-        <v>46115</v>
+        <v>46122</v>
       </c>
       <c r="B40" s="6" t="n">
-        <v>235</v>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C40" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1697,20 +1684,20 @@
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="10" t="n">
-        <v>46116</v>
+        <v>46123</v>
       </c>
       <c r="B41" s="11" t="n">
-        <v>205</v>
-      </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
@@ -1720,53 +1707,53 @@
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="14" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="5" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B42" s="6" t="n">
-        <v>135</v>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr">
+        <v>185</v>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Jurassic Park”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="10" t="n">
-        <v>46122</v>
+        <v>46124</v>
       </c>
       <c r="B43" s="11" t="n">
-        <v>135</v>
-      </c>
-      <c r="C43" s="20" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
@@ -1776,30 +1763,28 @@
       </c>
       <c r="E43" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F43" s="14" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="5" t="n">
-        <v>46122</v>
-      </c>
-      <c r="B44" s="6" t="n">
-        <v>135</v>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr"/>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D44" s="19" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -1809,20 +1794,20 @@
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="10" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B45" s="11" t="n">
-        <v>170</v>
-      </c>
-      <c r="C45" s="20" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
@@ -1837,46 +1822,46 @@
       </c>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="5" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B46" s="6" t="n">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
+      <c r="D46" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="10" t="n">
-        <v>46124</v>
+        <v>46128</v>
       </c>
       <c r="B47" s="11" t="n">
-        <v>130</v>
-      </c>
-      <c r="C47" s="19" t="inlineStr">
+        <v>160</v>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1893,15 +1878,17 @@
       </c>
       <c r="F47" s="14" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="5" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B48" s="6" t="inlineStr"/>
+        <v>46129</v>
+      </c>
+      <c r="B48" s="6" t="n">
+        <v>240</v>
+      </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -1909,7 +1896,7 @@
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -1919,25 +1906,25 @@
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="10" t="n">
-        <v>46125</v>
+        <v>46130</v>
       </c>
       <c r="B49" s="11" t="n">
-        <v>190</v>
-      </c>
-      <c r="C49" s="12" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D49" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E49" s="14" t="inlineStr">
@@ -1947,23 +1934,23 @@
       </c>
       <c r="F49" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="5" t="n">
-        <v>46125</v>
+        <v>46130</v>
       </c>
       <c r="B50" s="6" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D50" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1975,20 +1962,20 @@
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="10" t="n">
-        <v>46128</v>
+        <v>46133</v>
       </c>
       <c r="B51" s="11" t="n">
-        <v>160</v>
-      </c>
-      <c r="C51" s="19" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>145</v>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
@@ -1998,101 +1985,17 @@
       </c>
       <c r="E51" s="14" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="14" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="15" customHeight="1">
-      <c r="A52" s="5" t="n">
-        <v>46129</v>
-      </c>
-      <c r="B52" s="6" t="n">
-        <v>240</v>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D52" s="16" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="15" customHeight="1">
-      <c r="A53" s="10" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B53" s="11" t="n">
-        <v>240</v>
-      </c>
-      <c r="C53" s="12" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D53" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E53" s="14" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F53" s="14" t="inlineStr">
-        <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="15" customHeight="1">
-      <c r="A54" s="5" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B54" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="C54" s="15" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="inlineStr">
-        <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F54"/>
+  <autoFilter ref="A3:F51"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -2107,7 +2010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2176,38 +2079,38 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="5" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>1005</v>
+        <v>120</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>EXTREME</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Swarovski x Air Jordan 1 High OG</t>
+          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="10" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B5" s="11" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
@@ -2221,30 +2124,30 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Black University Blue” 2026</t>
+          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="n">
-        <v>46102</v>
+        <v>46104</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2254,7 +2157,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Division St. x Nike Air Max 95 “Oregon Ducks” Pack</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2166,7 @@
         <v>46104</v>
       </c>
       <c r="B7" s="11" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
@@ -2282,7 +2185,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
+          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2201,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2310,16 +2213,16 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
+          <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="10" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>120</v>
+        <v>210</v>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
@@ -2338,25 +2241,25 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
+          <t>Nike LeBron 23 “Masked Menace”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="5" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2366,16 +2269,16 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
+          <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="10" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B11" s="11" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
@@ -2394,23 +2297,23 @@
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="5" t="n">
-        <v>46105</v>
+        <v>46107</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2422,7 +2325,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Masked Menace”</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
     </row>
@@ -2431,16 +2334,16 @@
         <v>46107</v>
       </c>
       <c r="B13" s="11" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -2450,23 +2353,23 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Paisley Bandana”</t>
+          <t>Nike Air Max 95 “Greedy”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="5" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2478,16 +2381,16 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="10" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B15" s="11" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
@@ -2506,25 +2409,25 @@
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="5" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -2534,25 +2437,23 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="10" t="n">
-        <v>46108</v>
-      </c>
-      <c r="B17" s="11" t="n">
-        <v>240</v>
-      </c>
+        <v>46109</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr"/>
       <c r="C17" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -2562,7 +2463,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
@@ -2571,26 +2472,26 @@
         <v>46109</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>190</v>
+        <v>230</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -2598,25 +2499,27 @@
       <c r="A19" s="10" t="n">
         <v>46109</v>
       </c>
-      <c r="B19" s="11" t="inlineStr"/>
+      <c r="B19" s="11" t="n">
+        <v>215</v>
+      </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -2625,35 +2528,35 @@
         <v>46109</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>230</v>
+        <v>162</v>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>EXTREME</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="10" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B21" s="11" t="n">
-        <v>215</v>
+        <v>130</v>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
@@ -2667,28 +2570,28 @@
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="5" t="n">
-        <v>46109</v>
+        <v>46115</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>162</v>
+        <v>235</v>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2700,16 +2603,16 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 (GS)</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="10" t="n">
-        <v>46112</v>
+        <v>46116</v>
       </c>
       <c r="B23" s="11" t="n">
-        <v>130</v>
+        <v>205</v>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
@@ -2723,96 +2626,94 @@
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="5" t="n">
-        <v>46115</v>
+        <v>46123</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>235</v>
+        <v>185</v>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="10" t="n">
-        <v>46116</v>
-      </c>
-      <c r="B25" s="11" t="n">
-        <v>205</v>
-      </c>
+        <v>46125</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr"/>
       <c r="C25" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="5" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="16" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -2820,15 +2721,17 @@
       <c r="A27" s="10" t="n">
         <v>46125</v>
       </c>
-      <c r="B27" s="11" t="inlineStr"/>
+      <c r="B27" s="11" t="n">
+        <v>220</v>
+      </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
@@ -2838,23 +2741,23 @@
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="5" t="n">
-        <v>46125</v>
+        <v>46129</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2866,16 +2769,16 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="10" t="n">
-        <v>46125</v>
+        <v>46130</v>
       </c>
       <c r="B29" s="11" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
@@ -2894,68 +2797,12 @@
       </c>
       <c r="F29" s="14" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="5" t="n">
-        <v>46129</v>
-      </c>
-      <c r="B30" s="6" t="n">
-        <v>240</v>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="10" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B31" s="11" t="n">
-        <v>240</v>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
           <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F31"/>
+  <autoFilter ref="A3:F29"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -2970,7 +2817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2978,155 +2825,145 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Sneaker Release Report — Summary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
-        <is>
-          <t>Generated: 2026-03-21 06:11 UTC</t>
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Generated: 2026-03-22 04:14 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
-        <is>
-          <t>Total releases tracked: 51</t>
+      <c r="A3" s="22" t="inlineStr">
+        <is>
+          <t>Total releases tracked: 48</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Releases by Brand</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>35</v>
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="22" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Converse</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Releases by Hype Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>Releases by Sale Method</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="n">
         <v>8</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>Jordan</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="24" t="inlineStr">
-        <is>
-          <t>Converse</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="25" t="inlineStr">
-        <is>
-          <t>Releases by Hype Level</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="B12" s="24" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="B13" s="24" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="27" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="B14" s="24" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="28" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="B15" s="24" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>Releases by Sale Method</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="29" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="B18" s="24" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="B19" s="24" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="31" t="inlineStr">
-        <is>
-          <t>Raffle</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-22 04:20 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$3:$F$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Hype Alerts'!$A$3:$F$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$3:$F$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Hype Alerts'!$A$3:$F$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="M/D/YYYY"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,6 +85,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFC000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FF9800"/>
       <sz val="11"/>
     </font>
     <font>
@@ -154,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -214,14 +220,21 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -587,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1994,8 +2007,1174 @@
         </is>
       </c>
     </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B52" s="6" t="n">
+        <v>220</v>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="A53" s="10" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B53" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="A54" s="5" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr"/>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15" customHeight="1">
+      <c r="A55" s="10" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B55" s="11" t="n">
+        <v>215</v>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15" customHeight="1">
+      <c r="A56" s="5" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B56" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="15" customHeight="1">
+      <c r="A57" s="10" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B57" s="11" t="n">
+        <v>180</v>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F57" s="14" t="inlineStr">
+        <is>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="15" customHeight="1">
+      <c r="A58" s="5" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr"/>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 6 “Cap and Gown”</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1">
+      <c r="A59" s="10" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B59" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C59" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D59" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E59" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>Nike Mind 001 “Blackened Blue”</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15" customHeight="1">
+      <c r="A60" s="5" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B60" s="6" t="n">
+        <v>135</v>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>Nike Ja 3 “Uncle Phil”</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15" customHeight="1">
+      <c r="A61" s="10" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B61" s="11" t="n">
+        <v>190</v>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E61" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="inlineStr">
+        <is>
+          <t>Nike Air Zoom Huarache 2K4</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15" customHeight="1">
+      <c r="A62" s="5" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B62" s="6" t="n">
+        <v>220</v>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15" customHeight="1">
+      <c r="A63" s="10" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B63" s="11" t="n">
+        <v>195</v>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F63" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15" customHeight="1">
+      <c r="A64" s="5" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B64" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="C64" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E64" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="inlineStr">
+        <is>
+          <t>Nike A’Two “Pink Beam”</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="15" customHeight="1">
+      <c r="A65" s="10" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B65" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="15" customHeight="1">
+      <c r="A66" s="5" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B66" s="6" t="n">
+        <v>230</v>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E66" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="inlineStr">
+        <is>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1">
+      <c r="A67" s="10" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B67" s="11" t="n">
+        <v>120</v>
+      </c>
+      <c r="C67" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D67" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F67" s="14" t="inlineStr">
+        <is>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="15" customHeight="1">
+      <c r="A68" s="5" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B68" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="inlineStr">
+        <is>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="15" customHeight="1">
+      <c r="A69" s="10" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B69" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="C69" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E69" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F69" s="14" t="inlineStr">
+        <is>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="15" customHeight="1">
+      <c r="A70" s="5" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B70" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 1 Low OG “Banned”</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="15" customHeight="1">
+      <c r="A71" s="10" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B71" s="11" t="n">
+        <v>160</v>
+      </c>
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D71" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E71" s="14" t="inlineStr">
+        <is>
+          <t>Adidas</t>
+        </is>
+      </c>
+      <c r="F71" s="14" t="inlineStr">
+        <is>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="15" customHeight="1">
+      <c r="A72" s="5" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B72" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="inlineStr">
+        <is>
+          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="15" customHeight="1">
+      <c r="A73" s="10" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B73" s="11" t="n">
+        <v>205</v>
+      </c>
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E73" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F73" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 12 “Bloodline”</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="15" customHeight="1">
+      <c r="A74" s="5" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B74" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="inlineStr">
+        <is>
+          <t>Nike KD 19 “Bright Ceramic”</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="15" customHeight="1">
+      <c r="A75" s="10" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B75" s="11" t="n">
+        <v>240</v>
+      </c>
+      <c r="C75" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D75" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E75" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F75" s="14" t="inlineStr">
+        <is>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="15" customHeight="1">
+      <c r="A76" s="5" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr"/>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="15" customHeight="1">
+      <c r="A77" s="10" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B77" s="11" t="inlineStr"/>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>Adidas</t>
+        </is>
+      </c>
+      <c r="F77" s="14" t="inlineStr">
+        <is>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="15" customHeight="1">
+      <c r="A78" s="5" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B78" s="6" t="n">
+        <v>240</v>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="inlineStr">
+        <is>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="15" customHeight="1">
+      <c r="A79" s="10" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B79" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="C79" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E79" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F79" s="14" t="inlineStr">
+        <is>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="15" customHeight="1">
+      <c r="A80" s="5" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B80" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="C80" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="15" customHeight="1">
+      <c r="A81" s="10" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B81" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D81" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E81" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F81" s="14" t="inlineStr">
+        <is>
+          <t>Nike KD 6 “Night Vision” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="15" customHeight="1">
+      <c r="A82" s="5" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B82" s="6" t="inlineStr"/>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" s="10" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B83" s="11" t="n">
+        <v>355</v>
+      </c>
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D83" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E83" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F83" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 3 “BIN 23”</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15" customHeight="1">
+      <c r="A84" s="5" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B84" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="C84" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="inlineStr">
+        <is>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1">
+      <c r="A85" s="10" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B85" s="11" t="n">
+        <v>170</v>
+      </c>
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D85" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E85" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F85" s="14" t="inlineStr">
+        <is>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1">
+      <c r="A86" s="5" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B86" s="6" t="n">
+        <v>210</v>
+      </c>
+      <c r="C86" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D86" s="19" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F86" s="9" t="inlineStr">
+        <is>
+          <t>Patta x Nike Cryoshot Mercurial</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" s="10" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B87" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="C87" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D87" s="22" t="inlineStr">
+        <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="E87" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F87" s="14" t="inlineStr">
+        <is>
+          <t>Patta x Nike Air Max 1 ’87</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15" customHeight="1">
+      <c r="A88" s="5" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B88" s="6" t="n">
+        <v>210</v>
+      </c>
+      <c r="C88" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F88" s="9" t="inlineStr">
+        <is>
+          <t>PJ Tucker x Nike GT Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="15" customHeight="1">
+      <c r="A89" s="10" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B89" s="11" t="n">
+        <v>155</v>
+      </c>
+      <c r="C89" s="18" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D89" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E89" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F89" s="14" t="inlineStr">
+        <is>
+          <t>Nike KD 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="15" customHeight="1">
+      <c r="A90" s="5" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B90" s="6" t="n">
+        <v>135</v>
+      </c>
+      <c r="C90" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F90" s="9" t="inlineStr">
+        <is>
+          <t>Nike KD 6 “Night Vision”</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" s="10" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B91" s="11" t="n">
+        <v>215</v>
+      </c>
+      <c r="C91" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D91" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E91" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F91" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="15" customHeight="1">
+      <c r="A92" s="5" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B92" s="6" t="n">
+        <v>210</v>
+      </c>
+      <c r="C92" s="20" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D92" s="19" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F92" s="9" t="inlineStr">
+        <is>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="15" customHeight="1">
+      <c r="A93" s="10" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B93" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="C93" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D93" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E93" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F93" s="14" t="inlineStr">
+        <is>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F51"/>
+  <autoFilter ref="A3:F93"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -2010,7 +3189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2801,8 +3980,644 @@
         </is>
       </c>
     </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>220</v>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="10" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B31" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="5" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr"/>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="10" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B33" s="11" t="n">
+        <v>215</v>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="5" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="10" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B35" s="11" t="n">
+        <v>180</v>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="5" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr"/>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 6 “Cap and Gown”</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="10" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B37" s="11" t="n">
+        <v>220</v>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="5" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>195</v>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="10" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B39" s="11" t="n">
+        <v>230</v>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="5" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1">
+      <c r="A41" s="10" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B41" s="11" t="n">
+        <v>155</v>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15" customHeight="1">
+      <c r="A42" s="5" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B42" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15" customHeight="1">
+      <c r="A43" s="10" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B43" s="11" t="n">
+        <v>145</v>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 1 Low OG “Banned”</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="5" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B44" s="6" t="n">
+        <v>205</v>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 12 “Bloodline”</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15" customHeight="1">
+      <c r="A45" s="10" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B45" s="11" t="n">
+        <v>240</v>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="1">
+      <c r="A46" s="5" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr"/>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15" customHeight="1">
+      <c r="A47" s="10" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B47" s="11" t="n">
+        <v>240</v>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="A48" s="5" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr"/>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15" customHeight="1">
+      <c r="A49" s="10" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B49" s="11" t="n">
+        <v>355</v>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 3 “BIN 23”</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15" customHeight="1">
+      <c r="A50" s="5" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B50" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D50" s="21" t="inlineStr">
+        <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>Patta x Nike Air Max 1 ’87</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15" customHeight="1">
+      <c r="A51" s="10" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B51" s="11" t="n">
+        <v>215</v>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="5" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B52" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F29"/>
+  <autoFilter ref="A3:F52"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -2817,7 +4632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2825,145 +4640,155 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Sneaker Release Report — Summary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Generated: 2026-03-22 04:14 UTC</t>
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>Generated: 2026-03-22 04:20 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
-        <is>
-          <t>Total releases tracked: 48</t>
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Total releases tracked: 90</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Releases by Brand</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="B6" s="22" t="n">
-        <v>36</v>
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>62</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="22" t="inlineStr">
-        <is>
-          <t>Jordan</t>
-        </is>
-      </c>
-      <c r="B8" s="22" t="n">
-        <v>5</v>
+      <c r="B8" s="24" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Converse</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="24" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>Releases by Hype Level</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>EXTREME</t>
         </is>
       </c>
-      <c r="B12" s="22" t="n">
-        <v>1</v>
+      <c r="B12" s="24" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="B13" s="22" t="n">
-        <v>25</v>
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="B14" s="22" t="n">
-        <v>15</v>
+      <c r="B14" s="24" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n">
-        <v>7</v>
+      <c r="B15" s="24" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>Releases by Sale Method</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="B18" s="22" t="n">
-        <v>40</v>
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="n">
+        <v>77</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
-      <c r="B19" s="22" t="n">
-        <v>8</v>
+      <c r="B19" s="24" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>Raffle</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-22 04:59 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -140,7 +140,7 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1178,7 +1178,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>7</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="4320000"/>
@@ -1198,12 +1198,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>11</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="4320000"/>
+    <ext cx="5760000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1220,9 +1220,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="4320000"/>
@@ -1242,12 +1242,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>11</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="4320000"/>
+    <ext cx="5760000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 22, 2026  ·  04:52 UTC</t>
+          <t>Generated March 22, 2026  ·  04:59 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2670,10 +2670,10 @@
     <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>March 2026 Shoe Releases</t>
+          <t>Sneaker Release Report — All Releases</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2682,10 +2682,10 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Calculated Hype Level</t>
+          <t>Generated March 22, 2026  ·  04:59 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -4347,7 +4347,7 @@
         <v>46144</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="C62" s="40" t="inlineStr">
         <is>
@@ -4366,7 +4366,7 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
         <v>46144</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>195</v>
+        <v>220</v>
       </c>
       <c r="C63" s="42" t="inlineStr">
         <is>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4459,16 +4459,16 @@
         <v>46151</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C66" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D66" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>155</v>
+      </c>
+      <c r="C66" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D66" s="41" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E66" s="30" t="inlineStr">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -4487,7 +4487,7 @@
         <v>46151</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C67" s="42" t="inlineStr">
         <is>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4515,16 +4515,16 @@
         <v>46151</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C68" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D68" s="41" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>230</v>
+      </c>
+      <c r="C68" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D68" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
         <v>46151</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C69" s="42" t="inlineStr">
         <is>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -4819,7 +4819,7 @@
         <v>46173</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="C79" s="56" t="inlineStr">
         <is>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
@@ -4847,7 +4847,7 @@
         <v>46173</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="C80" s="49" t="inlineStr">
         <is>
@@ -4866,7 +4866,7 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
@@ -5153,26 +5153,26 @@
         <v>46193</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C91" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D91" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C91" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D91" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E91" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -5181,16 +5181,16 @@
         <v>46193</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C92" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D92" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C92" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D92" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E92" s="30" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5209,7 +5209,7 @@
         <v>46193</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="C93" s="42" t="inlineStr">
         <is>
@@ -5223,12 +5223,12 @@
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -5259,10 +5259,10 @@
     <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>March 2026 Shoe Releases</t>
+          <t>Sneaker Release Report — High Hype Alerts</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -5271,10 +5271,10 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Calculated Hype Level</t>
+          <t>Generated March 22, 2026  ·  04:59 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -6236,7 +6236,7 @@
         <v>46144</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="C37" s="42" t="inlineStr">
         <is>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
         <v>46144</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>195</v>
+        <v>220</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -6283,7 +6283,7 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -6292,16 +6292,16 @@
         <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C39" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D39" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>155</v>
+      </c>
+      <c r="C39" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
@@ -6311,7 +6311,7 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6320,7 @@
         <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6348,16 +6348,16 @@
         <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C41" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D41" s="39" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>230</v>
+      </c>
+      <c r="C41" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D41" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
         <v>46151</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -6395,7 +6395,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6624,7 @@
         <v>46193</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="C51" s="42" t="inlineStr">
         <is>
@@ -6638,12 +6638,12 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -6652,7 +6652,7 @@
         <v>46193</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
@@ -6666,12 +6666,12 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-22 05:25 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -74,7 +74,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="007030A0"/>
       <sz val="20"/>
     </font>
     <font>
@@ -97,7 +97,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="007030A0"/>
       <sz val="11"/>
     </font>
     <font>
@@ -115,7 +115,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FF0000"/>
+      <color rgb="00E02000"/>
       <sz val="11"/>
     </font>
     <font>
@@ -127,7 +127,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFC000"/>
+      <color rgb="00D4A000"/>
       <sz val="11"/>
     </font>
     <font>
@@ -170,8 +170,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
-        <bgColor rgb="00C00000"/>
+        <fgColor rgb="007030A0"/>
+        <bgColor rgb="007030A0"/>
       </patternFill>
     </fill>
     <fill>
@@ -365,13 +365,13 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </left>
       <right style="thin">
         <color rgb="00CCCCCC"/>
       </right>
       <top style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </top>
       <bottom style="thin">
         <color rgb="00CCCCCC"/>
@@ -382,10 +382,10 @@
         <color rgb="00CCCCCC"/>
       </left>
       <right style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </right>
       <top style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </top>
       <bottom style="thin">
         <color rgb="00CCCCCC"/>
@@ -393,7 +393,7 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </left>
       <right style="thin">
         <color rgb="00CCCCCC"/>
@@ -410,7 +410,7 @@
         <color rgb="00CCCCCC"/>
       </left>
       <right style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </right>
       <top style="thin">
         <color rgb="00CCCCCC"/>
@@ -421,7 +421,7 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </left>
       <right style="thin">
         <color rgb="00CCCCCC"/>
@@ -430,7 +430,7 @@
         <color rgb="00CCCCCC"/>
       </top>
       <bottom style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </bottom>
     </border>
     <border>
@@ -438,13 +438,13 @@
         <color rgb="00CCCCCC"/>
       </left>
       <right style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </right>
       <top style="thin">
         <color rgb="00CCCCCC"/>
       </top>
       <bottom style="medium">
-        <color rgb="00C00000"/>
+        <color rgb="007030A0"/>
       </bottom>
     </border>
     <border>
@@ -907,7 +907,7 @@
             <idx val="0"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="C00000"/>
+                <a:srgbClr val="7030A0"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -918,7 +918,7 @@
             <idx val="1"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="FF0000"/>
+                <a:srgbClr val="E02000"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -929,7 +929,7 @@
             <idx val="2"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="FFC000"/>
+                <a:srgbClr val="D4A000"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -1104,11 +1104,11 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="FFC000"/>
+              <a:srgbClr val="D4A000"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
-                <a:srgbClr val="FFC000"/>
+                <a:srgbClr val="D4A000"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 22, 2026  ·  04:59 UTC</t>
+          <t>Generated March 22, 2026  ·  05:25 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2685,7 +2685,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 22, 2026  ·  04:59 UTC</t>
+          <t>Generated March 22, 2026  ·  05:25 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5274,7 +5274,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 22, 2026  ·  04:59 UTC</t>
+          <t>Generated March 22, 2026  ·  05:25 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-23 09:16 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 22, 2026  ·  05:25 UTC</t>
+          <t>Generated March 23, 2026  ·  09:16 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1740,7 +1740,7 @@
         <v>46109</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         <v>46151</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
         <v>46186</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
         <v>46104</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="42" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
         <v>46104</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1910,7 +1910,7 @@
         <v>46104</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="42" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
         <v>46104</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>3/22 – 3/28</t>
+          <t>3/23 – 3/29</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>3/29 – 4/4</t>
+          <t>3/30 – 4/5</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
@@ -2198,17 +2198,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/5 – 4/11</t>
+          <t>4/6 – 4/12</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D29" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/12 – 4/18</t>
+          <t>4/13 – 4/19</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D30" s="42" t="n">
         <v>5</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>4/19 – 4/25</t>
+          <t>4/20 – 4/26</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>4/26 – 5/2</t>
+          <t>4/27 – 5/3</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/3 – 5/9</t>
+          <t>5/4 – 5/10</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/10 – 5/16</t>
+          <t>5/11 – 5/17</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>5/17 – 5/23</t>
+          <t>5/18 – 5/24</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
@@ -2345,17 +2345,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>5/24 – 5/30</t>
+          <t>5/25 – 5/31</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D36" s="42" t="n">
         <v>3</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>5.8</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2366,17 +2366,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>5/31 – 6/6</t>
+          <t>6/1 – 6/7</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D37" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/7 – 6/13</t>
+          <t>6/8 – 6/14</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>6/14 – 6/20</t>
+          <t>6/15 – 6/21</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2685,7 +2685,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 22, 2026  ·  05:25 UTC</t>
+          <t>Generated March 23, 2026  ·  09:16 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3207,26 +3207,26 @@
         <v>46109</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C21" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D21" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>215</v>
+      </c>
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D21" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Future “Swooshman”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -3237,9 +3237,9 @@
       <c r="B22" s="33" t="n">
         <v>190</v>
       </c>
-      <c r="C22" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C22" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D22" s="34" t="inlineStr">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>Nike GT Future “Swooshman”</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,9 @@
       <c r="A23" s="36" t="n">
         <v>46109</v>
       </c>
-      <c r="B23" s="38" t="inlineStr"/>
+      <c r="B23" s="38" t="n">
+        <v>190</v>
+      </c>
       <c r="C23" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3280,7 +3282,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
@@ -3288,27 +3290,25 @@
       <c r="A24" s="31" t="n">
         <v>46109</v>
       </c>
-      <c r="B24" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C24" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D24" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B24" s="33" t="inlineStr"/>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>adidas BadBo 1.0 “Rise”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
@@ -3317,26 +3317,26 @@
         <v>46109</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C25" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D25" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C25" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D25" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>adidas BadBo 1.0 “Rise”</t>
         </is>
       </c>
     </row>
@@ -3345,16 +3345,16 @@
         <v>46109</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C26" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D26" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D26" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -3765,11 +3765,11 @@
         <v>46123</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C41" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>185</v>
+      </c>
+      <c r="C41" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D41" s="43" t="inlineStr">
@@ -3779,12 +3779,12 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -3793,11 +3793,11 @@
         <v>46123</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>185</v>
-      </c>
-      <c r="C42" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C42" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D42" s="44" t="inlineStr">
@@ -3807,12 +3807,12 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,9 @@
       <c r="A54" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B54" s="33" t="inlineStr"/>
+      <c r="B54" s="33" t="n">
+        <v>180</v>
+      </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4144,7 +4146,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -4152,9 +4154,7 @@
       <c r="A55" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B55" s="38" t="n">
-        <v>215</v>
-      </c>
+      <c r="B55" s="38" t="inlineStr"/>
       <c r="C55" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4167,12 +4167,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
         <v>46137</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
         <v>46137</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C57" s="42" t="inlineStr">
         <is>
@@ -4223,12 +4223,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -4459,16 +4459,16 @@
         <v>46151</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C66" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D66" s="41" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>230</v>
+      </c>
+      <c r="C66" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D66" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E66" s="30" t="inlineStr">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -4487,7 +4487,7 @@
         <v>46151</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C67" s="42" t="inlineStr">
         <is>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -4515,16 +4515,16 @@
         <v>46151</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C68" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D68" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>155</v>
+      </c>
+      <c r="C68" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D68" s="41" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
         <v>46151</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C69" s="42" t="inlineStr">
         <is>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -5020,9 +5020,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D86" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D86" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E86" s="30" t="inlineStr">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -5041,16 +5041,16 @@
         <v>46186</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C87" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D87" s="39" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>210</v>
+      </c>
+      <c r="C87" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D87" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -5069,16 +5069,16 @@
         <v>46186</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C88" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D88" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C88" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D88" s="41" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -5153,16 +5153,16 @@
         <v>46193</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C91" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D91" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C91" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D91" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E91" s="35" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
         <v>46193</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="C92" s="40" t="inlineStr">
         <is>
@@ -5195,12 +5195,12 @@
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -5209,26 +5209,26 @@
         <v>46193</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C93" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D93" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C93" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D93" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 22, 2026  ·  05:25 UTC</t>
+          <t>Generated March 23, 2026  ·  09:16 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5656,26 +5656,26 @@
         <v>46109</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D16" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,9 @@
       <c r="A17" s="36" t="n">
         <v>46109</v>
       </c>
-      <c r="B17" s="38" t="inlineStr"/>
+      <c r="B17" s="38" t="n">
+        <v>190</v>
+      </c>
       <c r="C17" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5701,7 +5703,7 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
@@ -5709,12 +5711,10 @@
       <c r="A18" s="31" t="n">
         <v>46109</v>
       </c>
-      <c r="B18" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C18" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
+      <c r="B18" s="33" t="inlineStr"/>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D18" s="34" t="inlineStr">
@@ -5724,12 +5724,12 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
@@ -5738,16 +5738,16 @@
         <v>46109</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C19" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D19" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D19" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,9 @@
       <c r="A32" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B32" s="33" t="inlineStr"/>
+      <c r="B32" s="33" t="n">
+        <v>180</v>
+      </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6117,7 +6119,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -6125,9 +6127,7 @@
       <c r="A33" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B33" s="38" t="n">
-        <v>215</v>
-      </c>
+      <c r="B33" s="38" t="inlineStr"/>
       <c r="C33" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6140,12 +6140,12 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -6154,7 +6154,7 @@
         <v>46137</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -6182,7 +6182,7 @@
         <v>46137</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C35" s="42" t="inlineStr">
         <is>
@@ -6196,12 +6196,12 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -6292,16 +6292,16 @@
         <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C39" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D39" s="39" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>230</v>
+      </c>
+      <c r="C39" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D39" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
@@ -6311,7 +6311,7 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6320,7 @@
         <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -6348,16 +6348,16 @@
         <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C41" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D41" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>155</v>
+      </c>
+      <c r="C41" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
         <v>46151</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -6395,7 +6395,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-25 04:34 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -811,12 +811,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Charts'!$A$2:$A$5</f>
+              <f>'Charts'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$B$2:$B$5</f>
+              <f>'Charts'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1554,7 +1554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 23, 2026  ·  09:16 UTC</t>
+          <t>Generated March 25, 2026  ·  04:34 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1624,11 +1624,11 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1637,7 +1637,7 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$180</t>
+          <t>$184</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1737,10 +1737,10 @@
         </is>
       </c>
       <c r="C10" s="31" t="n">
-        <v>46109</v>
+        <v>46115</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         <v>46151</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1796,7 +1796,7 @@
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Patta x Nike Air Max 1</t>
         </is>
       </c>
       <c r="B12" s="30" t="inlineStr">
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="C12" s="31" t="n">
-        <v>46186</v>
+        <v>46107</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
       <c r="B13" s="35" t="inlineStr">
@@ -1839,10 +1839,10 @@
         </is>
       </c>
       <c r="C13" s="36" t="n">
-        <v>46104</v>
+        <v>46186</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="E13" s="42" t="inlineStr">
         <is>
@@ -1850,21 +1850,21 @@
         </is>
       </c>
       <c r="F13" s="35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G13" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="H13" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="H13" s="39" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
+          <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -1873,10 +1873,10 @@
         </is>
       </c>
       <c r="C14" s="31" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1889,16 +1889,16 @@
       <c r="G14" s="33" t="n">
         <v>200</v>
       </c>
-      <c r="H14" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1907,10 +1907,10 @@
         </is>
       </c>
       <c r="C15" s="36" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="42" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="H15" s="43" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1941,10 +1941,10 @@
         </is>
       </c>
       <c r="C16" s="31" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1955,7 +1955,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="H16" s="44" t="inlineStr">
         <is>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D21" s="42" t="inlineStr">
         <is>
@@ -2059,7 +2059,7 @@
         </is>
       </c>
       <c r="H21" s="35" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -2085,13 +2085,13 @@
         </is>
       </c>
       <c r="H22" s="30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="47" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="B23" s="35" t="n">
@@ -2103,321 +2103,331 @@
         </is>
       </c>
       <c r="E23" s="35" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>Converse</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" ht="10" customHeight="1"/>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Weekly Outlook (Next 13 Weeks)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>Releases</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="inlineStr">
+        <is>
+          <t>HIGH+EXTREME</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>Avg Hype Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Week 1</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>3/25 – 3/31</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="n">
+        <v>25</v>
+      </c>
+      <c r="D28" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="E28" s="30" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>4/1 – 4/7</t>
+        </is>
+      </c>
+      <c r="C29" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="35" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Week 3</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>4/8 – 4/14</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="n">
         <v>9</v>
       </c>
-    </row>
-    <row r="24" ht="10" customHeight="1"/>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="28" t="inlineStr">
-        <is>
-          <t>Weekly Outlook (Next 13 Weeks)</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="B26" s="29" t="inlineStr">
-        <is>
-          <t>Dates</t>
-        </is>
-      </c>
-      <c r="C26" s="29" t="inlineStr">
-        <is>
-          <t>Releases</t>
-        </is>
-      </c>
-      <c r="D26" s="29" t="inlineStr">
-        <is>
-          <t>HIGH+EXTREME</t>
-        </is>
-      </c>
-      <c r="E26" s="29" t="inlineStr">
-        <is>
-          <t>Avg Hype Score</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>Week 1</t>
-        </is>
-      </c>
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t>3/23 – 3/29</t>
-        </is>
-      </c>
-      <c r="C27" s="30" t="n">
-        <v>24</v>
-      </c>
-      <c r="D27" s="40" t="n">
-        <v>17</v>
-      </c>
-      <c r="E27" s="30" t="n">
+      <c r="D30" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" s="30" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="35" t="inlineStr">
+        <is>
+          <t>Week 4</t>
+        </is>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>4/15 – 4/21</t>
+        </is>
+      </c>
+      <c r="C31" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="D31" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="35" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>4/22 – 4/28</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="35" t="inlineStr">
-        <is>
-          <t>Week 2</t>
-        </is>
-      </c>
-      <c r="B28" s="35" t="inlineStr">
-        <is>
-          <t>3/30 – 4/5</t>
-        </is>
-      </c>
-      <c r="C28" s="35" t="n">
-        <v>10</v>
-      </c>
-      <c r="D28" s="42" t="n">
+      <c r="D32" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="30" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="35" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="B33" s="35" t="inlineStr">
+        <is>
+          <t>4/29 – 5/5</t>
+        </is>
+      </c>
+      <c r="C33" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="D33" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="E28" s="35" t="n">
-        <v>5.1</v>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>Week 3</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>4/6 – 4/12</t>
-        </is>
-      </c>
-      <c r="C29" s="30" t="n">
+      <c r="E33" s="35" t="n">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Week 7</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>5/6 – 5/12</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="n">
         <v>6</v>
       </c>
-      <c r="D29" s="40" t="n">
+      <c r="D34" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" s="30" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="35" t="inlineStr">
+        <is>
+          <t>Week 8</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>5/13 – 5/19</t>
+        </is>
+      </c>
+      <c r="C35" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="E29" s="30" t="n">
-        <v>4.3</v>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="35" t="inlineStr">
-        <is>
-          <t>Week 4</t>
-        </is>
-      </c>
-      <c r="B30" s="35" t="inlineStr">
-        <is>
-          <t>4/13 – 4/19</t>
-        </is>
-      </c>
-      <c r="C30" s="35" t="n">
-        <v>7</v>
-      </c>
-      <c r="D30" s="42" t="n">
+      <c r="E35" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="E30" s="35" t="n">
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>Week 9</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>5/20 – 5/26</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>Week 10</t>
+        </is>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>5/27 – 6/2</t>
+        </is>
+      </c>
+      <c r="C37" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="E37" s="35" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Week 11</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>6/3 – 6/9</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" s="30" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>Week 12</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>6/10 – 6/16</t>
+        </is>
+      </c>
+      <c r="C39" s="35" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Week 5</t>
-        </is>
-      </c>
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>4/20 – 4/26</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="n">
-        <v>7</v>
-      </c>
-      <c r="D31" s="40" t="n">
-        <v>6</v>
-      </c>
-      <c r="E31" s="30" t="n">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="35" t="inlineStr">
-        <is>
-          <t>Week 6</t>
-        </is>
-      </c>
-      <c r="B32" s="35" t="inlineStr">
-        <is>
-          <t>4/27 – 5/3</t>
-        </is>
-      </c>
-      <c r="C32" s="35" t="n">
-        <v>7</v>
-      </c>
-      <c r="D32" s="42" t="n">
-        <v>3</v>
-      </c>
-      <c r="E32" s="35" t="n">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>Week 7</t>
-        </is>
-      </c>
-      <c r="B33" s="30" t="inlineStr">
-        <is>
-          <t>5/4 – 5/10</t>
-        </is>
-      </c>
-      <c r="C33" s="30" t="n">
-        <v>5</v>
-      </c>
-      <c r="D33" s="40" t="n">
+      <c r="D39" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="35" t="n">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Week 13</t>
+        </is>
+      </c>
+      <c r="B40" s="30" t="inlineStr">
+        <is>
+          <t>6/17 – 6/23</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="E33" s="30" t="n">
-        <v>6.8</v>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="35" t="inlineStr">
-        <is>
-          <t>Week 8</t>
-        </is>
-      </c>
-      <c r="B34" s="35" t="inlineStr">
-        <is>
-          <t>5/11 – 5/17</t>
-        </is>
-      </c>
-      <c r="C34" s="35" t="n">
+      <c r="D40" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="D34" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="35" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="30" t="inlineStr">
-        <is>
-          <t>Week 9</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>5/18 – 5/24</t>
-        </is>
-      </c>
-      <c r="C35" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="30" t="n">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="36" ht="15" customHeight="1">
-      <c r="A36" s="35" t="inlineStr">
-        <is>
-          <t>Week 10</t>
-        </is>
-      </c>
-      <c r="B36" s="35" t="inlineStr">
-        <is>
-          <t>5/25 – 5/31</t>
-        </is>
-      </c>
-      <c r="C36" s="35" t="n">
-        <v>7</v>
-      </c>
-      <c r="D36" s="42" t="n">
-        <v>3</v>
-      </c>
-      <c r="E36" s="35" t="n">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="30" t="inlineStr">
-        <is>
-          <t>Week 11</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="inlineStr">
-        <is>
-          <t>6/1 – 6/7</t>
-        </is>
-      </c>
-      <c r="C37" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="30" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="35" t="inlineStr">
-        <is>
-          <t>Week 12</t>
-        </is>
-      </c>
-      <c r="B38" s="35" t="inlineStr">
-        <is>
-          <t>6/8 – 6/14</t>
-        </is>
-      </c>
-      <c r="C38" s="35" t="n">
-        <v>7</v>
-      </c>
-      <c r="D38" s="42" t="n">
-        <v>2</v>
-      </c>
-      <c r="E38" s="35" t="n">
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="30" t="inlineStr">
-        <is>
-          <t>Week 13</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="inlineStr">
-        <is>
-          <t>6/15 – 6/21</t>
-        </is>
-      </c>
-      <c r="C39" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="D39" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="E39" s="30" t="n">
+      <c r="E40" s="30" t="n">
         <v>6.2</v>
       </c>
     </row>
@@ -2429,7 +2439,7 @@
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="A5:B5"/>
@@ -2516,7 +2526,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2532,7 +2542,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2550,7 +2560,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2566,7 +2576,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2574,7 +2584,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -2600,7 +2610,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -2608,13 +2618,13 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2626,7 +2636,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2634,10 +2644,18 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Converse</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>$300+</t>
@@ -2659,7 +2677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2685,7 +2703,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 23, 2026  ·  09:16 UTC</t>
+          <t>Generated March 25, 2026  ·  04:34 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2728,14 +2746,14 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C4" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>80</v>
+      </c>
+      <c r="C4" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D4" s="44" t="inlineStr">
@@ -2745,25 +2763,25 @@
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
+          <t>Thug Club x adidas Adifom IIInfinity Mule</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C5" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C5" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D5" s="43" t="inlineStr">
@@ -2773,25 +2791,25 @@
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
+          <t>Thug Club x adidas Superstar Vintage</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C6" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D6" s="44" t="inlineStr">
@@ -2801,30 +2819,30 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
+          <t>Thug Club x adidas AdiFom Megaride</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="36" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="C7" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D7" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
@@ -2834,25 +2852,25 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
+          <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
@@ -2862,16 +2880,16 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
+          <t>Patta x Nike Air Max 1</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46105</v>
+        <v>46107</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="C9" s="42" t="inlineStr">
         <is>
@@ -2890,20 +2908,20 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Masked Menace”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>80</v>
-      </c>
-      <c r="C10" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D10" s="44" t="inlineStr">
@@ -2913,25 +2931,25 @@
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Thug Club x adidas Adifom IIInfinity Mule</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C11" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C11" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D11" s="43" t="inlineStr">
@@ -2941,25 +2959,25 @@
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Thug Club x adidas Superstar Vintage</t>
+          <t>Nike Air Max 95 “Greedy”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>230</v>
+      </c>
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D12" s="44" t="inlineStr">
@@ -2969,12 +2987,12 @@
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Thug Club x adidas AdiFom Megaride</t>
+          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
         </is>
       </c>
     </row>
@@ -2983,16 +3001,16 @@
         <v>46107</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C13" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D13" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -3002,7 +3020,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Paisley Bandana”</t>
+          <t>Oregon Ducks x Nike Air Max 95 “Lumber Yard”</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3029,7 @@
         <v>46107</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
@@ -3030,16 +3048,16 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Oregon Ducks x Nike Air Max 95 “The Woods”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C15" s="42" t="inlineStr">
         <is>
@@ -3058,20 +3076,20 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C16" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D16" s="44" t="inlineStr">
@@ -3081,21 +3099,21 @@
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Greedy”</t>
+          <t>Reebok Angel Reese 1 “Unapologetically Angel”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C17" s="56" t="inlineStr">
         <is>
@@ -3114,7 +3132,7 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
+          <t>Nike GT Cut “Dylan Harper”</t>
         </is>
       </c>
     </row>
@@ -3142,25 +3160,25 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
+          <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C19" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D19" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D19" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
@@ -3170,35 +3188,35 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut “Dylan Harper”</t>
+          <t>Nike GT Future “Swooshman”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C20" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D20" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>205</v>
+      </c>
+      <c r="C20" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue”</t>
+          <t>Travis Scott x Jordan Jumpman Jack “Green Spark”</t>
         </is>
       </c>
     </row>
@@ -3207,26 +3225,26 @@
         <v>46109</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>215</v>
+        <v>190</v>
       </c>
       <c r="C21" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D21" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
@@ -3234,12 +3252,10 @@
       <c r="A22" s="31" t="n">
         <v>46109</v>
       </c>
-      <c r="B22" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C22" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B22" s="33" t="inlineStr"/>
+      <c r="C22" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D22" s="34" t="inlineStr">
@@ -3254,7 +3270,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Future “Swooshman”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
@@ -3263,26 +3279,26 @@
         <v>46109</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C23" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D23" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C23" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D23" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>adidas BadBo 1.0 “Rise”</t>
         </is>
       </c>
     </row>
@@ -3290,25 +3306,27 @@
       <c r="A24" s="31" t="n">
         <v>46109</v>
       </c>
-      <c r="B24" s="33" t="inlineStr"/>
+      <c r="B24" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D24" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -3317,11 +3335,11 @@
         <v>46109</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C25" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>162</v>
+      </c>
+      <c r="C25" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D25" s="43" t="inlineStr">
@@ -3331,25 +3349,25 @@
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>adidas BadBo 1.0 “Rise”</t>
+          <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46109</v>
+        <v>46111</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C26" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
+        <v>210</v>
+      </c>
+      <c r="C26" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D26" s="34" t="inlineStr">
@@ -3359,25 +3377,25 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Nike GT Future “Galaxy Aura”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>162</v>
-      </c>
-      <c r="C27" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C27" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D27" s="43" t="inlineStr">
@@ -3387,30 +3405,30 @@
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 (GS)</t>
+          <t>Jordan Jumpman Pro “Black Concord”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C28" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D28" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D28" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
@@ -3420,13 +3438,13 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Future “Galaxy Aura”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B29" s="38" t="n">
         <v>145</v>
@@ -3443,25 +3461,25 @@
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Jordan Jumpman Pro “Black Concord”</t>
+          <t>Nike Sabrina 3 “What The”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C30" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>95</v>
+      </c>
+      <c r="C30" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D30" s="44" t="inlineStr">
@@ -3476,16 +3494,16 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Nike Mind 001 “Sail”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>145</v>
+        <v>95</v>
       </c>
       <c r="C31" s="56" t="inlineStr">
         <is>
@@ -3504,20 +3522,20 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Sabrina 3 “What The”</t>
+          <t>Nike Mind 001 “Geode Teal”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C32" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C32" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D32" s="44" t="inlineStr">
@@ -3527,40 +3545,40 @@
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Sail”</t>
+          <t>Converse SHAI 001 “Camo”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C33" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D33" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C33" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D33" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Geode Teal”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -3569,11 +3587,11 @@
         <v>46115</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C34" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>225</v>
+      </c>
+      <c r="C34" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D34" s="44" t="inlineStr">
@@ -3583,12 +3601,12 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 “Camo”</t>
+          <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
     </row>
@@ -3597,11 +3615,11 @@
         <v>46115</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>225</v>
-      </c>
-      <c r="C35" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C35" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D35" s="43" t="inlineStr">
@@ -3616,16 +3634,16 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
@@ -3639,25 +3657,25 @@
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46116</v>
+        <v>46122</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C37" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C37" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D37" s="43" t="inlineStr">
@@ -3667,12 +3685,12 @@
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
@@ -3700,16 +3718,16 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Jurassic Park”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>135</v>
+        <v>170</v>
       </c>
       <c r="C39" s="56" t="inlineStr">
         <is>
@@ -3728,20 +3746,20 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C40" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>185</v>
+      </c>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D40" s="44" t="inlineStr">
@@ -3751,25 +3769,25 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C41" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C41" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D41" s="43" t="inlineStr">
@@ -3779,30 +3797,28 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46123</v>
-      </c>
-      <c r="B42" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C42" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D42" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B42" s="33" t="inlineStr"/>
+      <c r="C42" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D42" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
@@ -3812,20 +3828,20 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C43" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C43" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D43" s="43" t="inlineStr">
@@ -3835,12 +3851,12 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3848,15 +3864,17 @@
       <c r="A44" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B44" s="33" t="inlineStr"/>
+      <c r="B44" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D44" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D44" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E44" s="30" t="inlineStr">
@@ -3866,7 +3884,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3893,7 @@
         <v>46125</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C45" s="42" t="inlineStr">
         <is>
@@ -3894,20 +3912,20 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46125</v>
+        <v>46128</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C46" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C46" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D46" s="44" t="inlineStr">
@@ -3917,25 +3935,25 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C47" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>240</v>
+      </c>
+      <c r="C47" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D47" s="43" t="inlineStr">
@@ -3945,30 +3963,30 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C48" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D48" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C48" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D48" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
@@ -3978,7 +3996,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
@@ -3987,16 +4005,16 @@
         <v>46130</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C49" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D49" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>240</v>
+      </c>
+      <c r="C49" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D49" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E49" s="35" t="inlineStr">
@@ -4006,20 +4024,20 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C50" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C50" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D50" s="44" t="inlineStr">
@@ -4034,20 +4052,20 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C51" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C51" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D51" s="43" t="inlineStr">
@@ -4057,21 +4075,21 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
@@ -4085,22 +4103,20 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B53" s="38" t="n">
-        <v>200</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B53" s="38" t="inlineStr"/>
       <c r="C53" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4118,7 +4134,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4143,7 @@
         <v>46137</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>180</v>
+        <v>215</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
@@ -4141,12 +4157,12 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -4154,7 +4170,9 @@
       <c r="A55" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B55" s="38" t="inlineStr"/>
+      <c r="B55" s="38" t="n">
+        <v>200</v>
+      </c>
       <c r="C55" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4167,12 +4185,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4199,7 @@
         <v>46137</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>215</v>
+        <v>180</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -4195,22 +4213,20 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B57" s="38" t="n">
-        <v>200</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B57" s="38" t="inlineStr"/>
       <c r="C57" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4228,7 +4244,7 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -4236,10 +4252,12 @@
       <c r="A58" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B58" s="33" t="inlineStr"/>
-      <c r="C58" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B58" s="33" t="n">
+        <v>95</v>
+      </c>
+      <c r="C58" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D58" s="44" t="inlineStr">
@@ -4249,21 +4267,21 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
       <c r="C59" s="56" t="inlineStr">
         <is>
@@ -4282,7 +4300,7 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4309,7 @@
         <v>46143</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C60" s="49" t="inlineStr">
         <is>
@@ -4310,20 +4328,20 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C61" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C61" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D61" s="43" t="inlineStr">
@@ -4333,12 +4351,12 @@
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4375,11 +4393,11 @@
         <v>46144</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C63" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C63" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D63" s="43" t="inlineStr">
@@ -4389,25 +4407,25 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C64" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C64" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D64" s="44" t="inlineStr">
@@ -4422,7 +4440,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
@@ -4816,14 +4834,14 @@
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C79" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C79" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D79" s="43" t="inlineStr">
@@ -4838,7 +4856,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
@@ -4847,7 +4865,7 @@
         <v>46173</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="C80" s="49" t="inlineStr">
         <is>
@@ -4866,16 +4884,16 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46177</v>
+        <v>46173</v>
       </c>
       <c r="B81" s="38" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="C81" s="56" t="inlineStr">
         <is>
@@ -4894,18 +4912,20 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B82" s="33" t="inlineStr"/>
-      <c r="C82" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46177</v>
+      </c>
+      <c r="B82" s="33" t="n">
+        <v>140</v>
+      </c>
+      <c r="C82" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D82" s="44" t="inlineStr">
@@ -4915,22 +4935,20 @@
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="36" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B83" s="38" t="n">
-        <v>355</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B83" s="38" t="inlineStr"/>
       <c r="C83" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4948,20 +4966,20 @@
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C84" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>355</v>
+      </c>
+      <c r="C84" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D84" s="44" t="inlineStr">
@@ -4971,12 +4989,12 @@
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -5004,16 +5022,16 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C86" s="49" t="inlineStr">
         <is>
@@ -5032,7 +5050,7 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5115,7 @@
         <v>46186</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>155</v>
+        <v>210</v>
       </c>
       <c r="C89" s="56" t="inlineStr">
         <is>
@@ -5116,16 +5134,16 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="C90" s="49" t="inlineStr">
         <is>
@@ -5144,20 +5162,20 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C91" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C91" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D91" s="43" t="inlineStr">
@@ -5172,7 +5190,7 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5199,7 @@
         <v>46193</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="C92" s="40" t="inlineStr">
         <is>
@@ -5195,12 +5213,12 @@
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5209,31 +5227,59 @@
         <v>46193</v>
       </c>
       <c r="B93" s="38" t="n">
+        <v>215</v>
+      </c>
+      <c r="C93" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D93" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E93" s="35" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F93" s="35" t="inlineStr">
+        <is>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="15" customHeight="1">
+      <c r="A94" s="31" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B94" s="33" t="n">
         <v>210</v>
       </c>
-      <c r="C93" s="56" t="inlineStr">
+      <c r="C94" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D93" s="55" t="inlineStr">
+      <c r="D94" s="34" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
-      <c r="E93" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F93" s="35" t="inlineStr">
+      <c r="E94" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F94" s="30" t="inlineStr">
         <is>
           <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F93"/>
+  <autoFilter ref="A3:F94"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5274,7 +5320,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 23, 2026  ·  09:16 UTC</t>
+          <t>Generated March 25, 2026  ·  04:34 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5317,19 +5363,19 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C4" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D4" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D4" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
@@ -5339,25 +5385,25 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant x Nike Air Force 1 Low “Lower Merion Aces Away”</t>
+          <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C5" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D5" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D5" s="39" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -5367,16 +5413,16 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away” 2026</t>
+          <t>Patta x Nike Air Max 1</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
@@ -5395,16 +5441,16 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Lower Merion Aces”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="36" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="C7" s="42" t="inlineStr">
         <is>
@@ -5423,16 +5469,16 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Dunk Low Protro “Lower Merion Aces”</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46104</v>
+        <v>46107</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -5451,16 +5497,16 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 5 Protro “Lower Merion Aces Away”</t>
+          <t>Nike Air Max 95 “Greedy”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46105</v>
+        <v>46107</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>210</v>
+        <v>250</v>
       </c>
       <c r="C9" s="42" t="inlineStr">
         <is>
@@ -5479,7 +5525,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Masked Menace”</t>
+          <t>Oregon Ducks x Nike Air Max 95 “Lumber Yard”</t>
         </is>
       </c>
     </row>
@@ -5488,16 +5534,16 @@
         <v>46107</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D10" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -5507,16 +5553,16 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Paisley Bandana”</t>
+          <t>Oregon Ducks x Nike Air Max 95 “The Woods”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="C11" s="42" t="inlineStr">
         <is>
@@ -5535,16 +5581,16 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
@@ -5563,13 +5609,13 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46107</v>
+        <v>46109</v>
       </c>
       <c r="B13" s="38" t="n">
         <v>190</v>
@@ -5579,9 +5625,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -5591,25 +5637,23 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Greedy”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46108</v>
-      </c>
-      <c r="B14" s="33" t="n">
-        <v>240</v>
-      </c>
+        <v>46109</v>
+      </c>
+      <c r="B14" s="33" t="inlineStr"/>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -5619,16 +5663,16 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C15" s="42" t="inlineStr">
         <is>
@@ -5642,12 +5686,12 @@
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5700,7 @@
         <v>46109</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>215</v>
+        <v>162</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
@@ -5670,30 +5714,30 @@
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>190</v>
+        <v>130</v>
       </c>
       <c r="C17" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D17" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
@@ -5703,18 +5747,20 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46109</v>
-      </c>
-      <c r="B18" s="33" t="inlineStr"/>
-      <c r="C18" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46115</v>
+      </c>
+      <c r="B18" s="33" t="n">
+        <v>230</v>
+      </c>
+      <c r="C18" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D18" s="34" t="inlineStr">
@@ -5724,49 +5770,49 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46109</v>
+        <v>46115</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C19" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D19" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>235</v>
+      </c>
+      <c r="C19" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46109</v>
+        <v>46116</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>162</v>
+        <v>205</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -5780,21 +5826,21 @@
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 (GS)</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C21" s="42" t="inlineStr">
         <is>
@@ -5808,30 +5854,28 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46115</v>
-      </c>
-      <c r="B22" s="33" t="n">
-        <v>235</v>
-      </c>
+        <v>46125</v>
+      </c>
+      <c r="B22" s="33" t="inlineStr"/>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D22" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -5841,16 +5885,16 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46116</v>
+        <v>46125</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C23" s="42" t="inlineStr">
         <is>
@@ -5864,21 +5908,21 @@
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
@@ -5892,12 +5936,12 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5905,15 +5949,17 @@
       <c r="A25" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B25" s="38" t="inlineStr"/>
+      <c r="B25" s="38" t="n">
+        <v>220</v>
+      </c>
       <c r="C25" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D25" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D25" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E25" s="35" t="inlineStr">
@@ -5923,16 +5969,16 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46125</v>
+        <v>46129</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
@@ -5951,16 +5997,16 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46125</v>
+        <v>46130</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C27" s="42" t="inlineStr">
         <is>
@@ -5979,16 +6025,16 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46129</v>
+        <v>46135</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C28" s="40" t="inlineStr">
         <is>
@@ -6002,21 +6048,21 @@
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46130</v>
+        <v>46136</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="C29" s="42" t="inlineStr">
         <is>
@@ -6035,17 +6081,15 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46135</v>
-      </c>
-      <c r="B30" s="33" t="n">
-        <v>220</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B30" s="33" t="inlineStr"/>
       <c r="C30" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6058,21 +6102,21 @@
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -6086,12 +6130,12 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6144,7 @@
         <v>46137</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -6114,12 +6158,12 @@
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6171,9 @@
       <c r="A33" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B33" s="38" t="inlineStr"/>
+      <c r="B33" s="38" t="n">
+        <v>180</v>
+      </c>
       <c r="C33" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6145,17 +6191,15 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B34" s="33" t="n">
-        <v>215</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B34" s="33" t="inlineStr"/>
       <c r="C34" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6173,16 +6217,16 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46137</v>
+        <v>46144</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="C35" s="42" t="inlineStr">
         <is>
@@ -6201,15 +6245,17 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B36" s="33" t="inlineStr"/>
+        <v>46144</v>
+      </c>
+      <c r="B36" s="33" t="n">
+        <v>195</v>
+      </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6227,16 +6273,16 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C37" s="42" t="inlineStr">
         <is>
@@ -6250,30 +6296,30 @@
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46144</v>
+        <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D38" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D38" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
@@ -6283,7 +6329,7 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -6292,26 +6338,26 @@
         <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>230</v>
+        <v>120</v>
       </c>
       <c r="C39" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D39" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D39" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -6320,26 +6366,26 @@
         <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C40" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D40" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C40" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D40" s="41" t="inlineStr">
+        <is>
+          <t>Raffle</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -6348,35 +6394,35 @@
         <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C41" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D41" s="39" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>200</v>
+      </c>
+      <c r="C41" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D41" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46151</v>
+        <v>46158</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>200</v>
+        <v>145</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -6390,21 +6436,21 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46158</v>
+        <v>46165</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="C43" s="42" t="inlineStr">
         <is>
@@ -6423,16 +6469,16 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46165</v>
+        <v>46171</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
@@ -6446,22 +6492,20 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46171</v>
-      </c>
-      <c r="B45" s="38" t="n">
-        <v>240</v>
-      </c>
+        <v>46172</v>
+      </c>
+      <c r="B45" s="38" t="inlineStr"/>
       <c r="C45" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6474,12 +6518,12 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6531,9 @@
       <c r="A46" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B46" s="33" t="inlineStr"/>
+      <c r="B46" s="33" t="n">
+        <v>240</v>
+      </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6500,12 +6546,12 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6560,7 @@
         <v>46172</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C47" s="42" t="inlineStr">
         <is>
@@ -6533,7 +6579,7 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-25 08:07 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$94</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -654,9 +654,6 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -683,6 +680,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 25, 2026  ·  04:34 UTC</t>
+          <t>Generated March 25, 2026  ·  08:07 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1624,15 +1624,15 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="H11" s="39" t="inlineStr">
         <is>
-          <t>Raffle</t>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="H12" s="41" t="inlineStr">
         <is>
-          <t>Raffle</t>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="H13" s="39" t="inlineStr">
         <is>
-          <t>Raffle</t>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Nike Air Max 90 “Infrared 3M”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1932,7 +1932,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1957,9 +1957,9 @@
       <c r="G16" s="33" t="n">
         <v>190</v>
       </c>
-      <c r="H16" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
@@ -2011,13 +2011,13 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="45" t="inlineStr">
+      <c r="A20" s="44" t="inlineStr">
         <is>
           <t>Nike</t>
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
       <c r="E20" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="46" t="inlineStr">
+      <c r="G20" s="45" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2037,7 +2037,7 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="47" t="inlineStr">
+      <c r="A21" s="46" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
@@ -2051,19 +2051,19 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>47</v>
-      </c>
-      <c r="G21" s="48" t="inlineStr">
+        <v>49</v>
+      </c>
+      <c r="G21" s="47" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
       <c r="H21" s="35" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="45" t="inlineStr">
+      <c r="A22" s="44" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
@@ -2071,7 +2071,7 @@
       <c r="B22" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="D22" s="49" t="inlineStr">
+      <c r="D22" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2079,9 +2079,9 @@
       <c r="E22" s="30" t="n">
         <v>32</v>
       </c>
-      <c r="G22" s="50" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+      <c r="G22" s="49" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="H22" s="30" t="n">
@@ -2089,7 +2089,7 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="47" t="inlineStr">
+      <c r="A23" s="46" t="inlineStr">
         <is>
           <t>Reebok</t>
         </is>
@@ -2097,7 +2097,7 @@
       <c r="B23" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="51" t="inlineStr">
+      <c r="D23" s="50" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2107,7 +2107,7 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="45" t="inlineStr">
+      <c r="A24" s="44" t="inlineStr">
         <is>
           <t>Converse</t>
         </is>
@@ -2170,13 +2170,13 @@
         </is>
       </c>
       <c r="C28" s="30" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D28" s="40" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E28" s="30" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2191,13 +2191,13 @@
         </is>
       </c>
       <c r="C29" s="35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D29" s="42" t="n">
         <v>3</v>
       </c>
       <c r="E29" s="35" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2478,42 +2478,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="51" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="B1" s="52" t="inlineStr">
+      <c r="B1" s="51" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="D1" s="52" t="inlineStr">
+      <c r="D1" s="51" t="inlineStr">
         <is>
           <t>Hype Level</t>
         </is>
       </c>
-      <c r="E1" s="52" t="inlineStr">
+      <c r="E1" s="51" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="G1" s="52" t="inlineStr">
+      <c r="G1" s="51" t="inlineStr">
         <is>
           <t>Sale Method</t>
         </is>
       </c>
-      <c r="H1" s="52" t="inlineStr">
+      <c r="H1" s="51" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="J1" s="52" t="inlineStr">
+      <c r="J1" s="51" t="inlineStr">
         <is>
           <t>Price Range</t>
         </is>
       </c>
-      <c r="K1" s="52" t="inlineStr">
+      <c r="K1" s="51" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
@@ -2526,7 +2526,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Raffle</t>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -2618,7 +2618,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -2644,7 +2644,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -2677,7 +2677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2701,9 +2701,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="53" t="inlineStr">
-        <is>
-          <t>Generated March 25, 2026  ·  04:34 UTC</t>
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>Generated March 25, 2026  ·  08:07 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2751,12 +2751,12 @@
       <c r="B4" s="33" t="n">
         <v>80</v>
       </c>
-      <c r="C4" s="54" t="inlineStr">
+      <c r="C4" s="53" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="D4" s="44" t="inlineStr">
+      <c r="D4" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2779,7 +2779,7 @@
       <c r="B5" s="38" t="n">
         <v>160</v>
       </c>
-      <c r="C5" s="51" t="inlineStr">
+      <c r="C5" s="50" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2807,12 +2807,12 @@
       <c r="B6" s="33" t="n">
         <v>170</v>
       </c>
-      <c r="C6" s="54" t="inlineStr">
+      <c r="C6" s="53" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="D6" s="44" t="inlineStr">
+      <c r="D6" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2861,16 +2861,16 @@
         <v>46107</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C8" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D8" s="41" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>230</v>
+      </c>
+      <c r="C8" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1</t>
+          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Nike Air Max 90 “Infrared 3M”</t>
         </is>
       </c>
     </row>
@@ -2924,9 +2924,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D10" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
         </is>
       </c>
     </row>
@@ -2945,16 +2945,16 @@
         <v>46107</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C11" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D11" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Greedy”</t>
+          <t>Patta x Nike Air Max 1</t>
         </is>
       </c>
     </row>
@@ -2973,14 +2973,14 @@
         <v>46107</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C12" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D12" s="44" t="inlineStr">
+        <v>150</v>
+      </c>
+      <c r="C12" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
         <v>46107</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>250</v>
+        <v>190</v>
       </c>
       <c r="C13" s="42" t="inlineStr">
         <is>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Max 95 “Lumber Yard”</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
     </row>
@@ -3029,14 +3029,14 @@
         <v>46107</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>250</v>
+        <v>190</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="44" t="inlineStr">
+      <c r="D14" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3048,16 +3048,16 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Max 95 “The Woods”</t>
+          <t>Nike Air Max 95 “Greedy”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46108</v>
+        <v>46107</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C15" s="42" t="inlineStr">
         <is>
@@ -3076,35 +3076,35 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
+          <t>Oregon Ducks x Nike Air Max 95 “Lumber Yard”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46108</v>
+        <v>46107</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C16" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D16" s="44" t="inlineStr">
+        <v>250</v>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Reebok Angel Reese 1 “Unapologetically Angel”</t>
+          <t>Oregon Ducks x Nike Air Max 95 “The Woods”</t>
         </is>
       </c>
     </row>
@@ -3113,11 +3113,11 @@
         <v>46108</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C17" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C17" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D17" s="43" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut “Dylan Harper”</t>
+          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -3141,44 +3141,44 @@
         <v>46108</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C18" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D18" s="44" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C18" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D18" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue”</t>
+          <t>Reebok Angel Reese 1 “Unapologetically Angel”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46109</v>
+        <v>46108</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C19" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D19" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D19" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
@@ -3188,35 +3188,35 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Future “Swooshman”</t>
+          <t>Nike GT Cut “Dylan Harper”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46109</v>
+        <v>46108</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C20" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D20" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>240</v>
+      </c>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D20" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Jordan Jumpman Jack “Green Spark”</t>
+          <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
     </row>
@@ -3225,11 +3225,11 @@
         <v>46109</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C21" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>205</v>
+      </c>
+      <c r="C21" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D21" s="55" t="inlineStr">
@@ -3239,12 +3239,12 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>Travis Scott x Jordan Jumpman Jack “Green Spark”</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,9 @@
       <c r="A22" s="31" t="n">
         <v>46109</v>
       </c>
-      <c r="B22" s="33" t="inlineStr"/>
+      <c r="B22" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3270,7 +3272,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3283,7 @@
       <c r="B23" s="38" t="n">
         <v>160</v>
       </c>
-      <c r="C23" s="51" t="inlineStr">
+      <c r="C23" s="50" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -3306,27 +3308,25 @@
       <c r="A24" s="31" t="n">
         <v>46109</v>
       </c>
-      <c r="B24" s="33" t="n">
-        <v>215</v>
-      </c>
+      <c r="B24" s="33" t="inlineStr"/>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
         <v>46109</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>162</v>
+        <v>215</v>
       </c>
       <c r="C25" s="42" t="inlineStr">
         <is>
@@ -3349,30 +3349,30 @@
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 (GS)</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46111</v>
+        <v>46109</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C26" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D26" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>162</v>
+      </c>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D26" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
@@ -3382,35 +3382,35 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Future “Galaxy Aura”</t>
+          <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46112</v>
+        <v>46111</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>145</v>
+        <v>210</v>
       </c>
       <c r="C27" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D27" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D27" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Jordan Jumpman Pro “Black Concord”</t>
+          <t>Nike GT Future “Galaxy Aura”</t>
         </is>
       </c>
     </row>
@@ -3419,39 +3419,39 @@
         <v>46112</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C28" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D28" s="44" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C28" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D28" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Jordan Jumpman Pro “Black Concord”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46113</v>
+        <v>46112</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C29" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C29" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D29" s="43" t="inlineStr">
@@ -3466,23 +3466,23 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Sabrina 3 “What The”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46114</v>
+        <v>46113</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C30" s="49" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C30" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D30" s="44" t="inlineStr">
+      <c r="D30" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3494,7 +3494,7 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Sail”</t>
+          <t>Nike Sabrina 3 “What The”</t>
         </is>
       </c>
     </row>
@@ -3522,35 +3522,35 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Geode Teal”</t>
+          <t>Nike Mind 001 “Sail”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46115</v>
+        <v>46114</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C32" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D32" s="44" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C32" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D32" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 “Camo”</t>
+          <t>Nike Mind 001 “Geode Teal”</t>
         </is>
       </c>
     </row>
@@ -3559,26 +3559,26 @@
         <v>46115</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D33" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C33" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D33" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Converse SHAI 001 “Camo”</t>
         </is>
       </c>
     </row>
@@ -3587,26 +3587,26 @@
         <v>46115</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>225</v>
-      </c>
-      <c r="C34" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D34" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C34" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D34" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -3615,16 +3615,16 @@
         <v>46115</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C35" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D35" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>225</v>
+      </c>
+      <c r="C35" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D35" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
@@ -3634,48 +3634,48 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Fragment x Nike Air Liquid Max “Black”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46116</v>
+        <v>46115</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C36" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D36" s="44" t="inlineStr">
+        <v>225</v>
+      </c>
+      <c r="C36" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D36" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46122</v>
+        <v>46115</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C37" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C37" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D37" s="43" t="inlineStr">
@@ -3690,44 +3690,44 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46122</v>
+        <v>46116</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C38" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D38" s="44" t="inlineStr">
+        <v>205</v>
+      </c>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D38" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46123</v>
+        <v>46122</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="C39" s="56" t="inlineStr">
         <is>
@@ -3746,48 +3746,48 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46123</v>
+        <v>46122</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>185</v>
-      </c>
-      <c r="C40" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D40" s="44" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C40" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D40" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46124</v>
+        <v>46123</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C41" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>170</v>
+      </c>
+      <c r="C41" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D41" s="43" t="inlineStr">
@@ -3797,51 +3797,53 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B42" s="33" t="inlineStr"/>
+        <v>46123</v>
+      </c>
+      <c r="B42" s="33" t="n">
+        <v>185</v>
+      </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D42" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D42" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46125</v>
+        <v>46124</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C43" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C43" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D43" s="43" t="inlineStr">
@@ -3851,12 +3853,12 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
@@ -3872,7 +3874,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D44" s="44" t="inlineStr">
+      <c r="D44" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3884,7 +3886,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3892,17 +3894,15 @@
       <c r="A45" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B45" s="38" t="n">
-        <v>220</v>
-      </c>
+      <c r="B45" s="38" t="inlineStr"/>
       <c r="C45" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D45" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D45" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
@@ -3912,44 +3912,44 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46128</v>
+        <v>46125</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C46" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D46" s="44" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C46" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D46" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46129</v>
+        <v>46125</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C47" s="42" t="inlineStr">
         <is>
@@ -3968,41 +3968,41 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46130</v>
+        <v>46128</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C48" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D48" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C48" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D48" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46130</v>
+        <v>46129</v>
       </c>
       <c r="B49" s="38" t="n">
         <v>240</v>
@@ -4024,25 +4024,25 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46133</v>
+        <v>46130</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C50" s="49" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C50" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D50" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D50" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E50" s="30" t="inlineStr">
@@ -4052,16 +4052,16 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46135</v>
+        <v>46130</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C51" s="42" t="inlineStr">
         <is>
@@ -4075,28 +4075,28 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46136</v>
+        <v>46133</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C52" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D52" s="44" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C52" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D52" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4108,15 +4108,17 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B53" s="38" t="inlineStr"/>
+        <v>46135</v>
+      </c>
+      <c r="B53" s="38" t="n">
+        <v>220</v>
+      </c>
       <c r="C53" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4129,40 +4131,40 @@
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="44" t="inlineStr">
+      <c r="D54" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -4170,9 +4172,7 @@
       <c r="A55" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B55" s="38" t="n">
-        <v>200</v>
-      </c>
+      <c r="B55" s="38" t="inlineStr"/>
       <c r="C55" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4185,12 +4185,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -4199,34 +4199,36 @@
         <v>46137</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>180</v>
+        <v>215</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="44" t="inlineStr">
+      <c r="D56" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B57" s="38" t="inlineStr"/>
+        <v>46137</v>
+      </c>
+      <c r="B57" s="38" t="n">
+        <v>200</v>
+      </c>
       <c r="C57" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4244,23 +4246,23 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C58" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D58" s="44" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D58" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4272,20 +4274,18 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B59" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C59" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46142</v>
+      </c>
+      <c r="B59" s="38" t="inlineStr"/>
+      <c r="C59" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D59" s="43" t="inlineStr">
@@ -4295,28 +4295,28 @@
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C60" s="49" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C60" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D60" s="44" t="inlineStr">
+      <c r="D60" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4328,20 +4328,20 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C61" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C61" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D61" s="43" t="inlineStr">
@@ -4351,40 +4351,40 @@
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>195</v>
-      </c>
-      <c r="C62" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D62" s="44" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C62" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D62" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
@@ -4393,11 +4393,11 @@
         <v>46144</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C63" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C63" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D63" s="43" t="inlineStr">
@@ -4407,49 +4407,49 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C64" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D64" s="44" t="inlineStr">
+      <c r="D64" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46150</v>
+        <v>46144</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>210</v>
+        <v>145</v>
       </c>
       <c r="C65" s="56" t="inlineStr">
         <is>
@@ -4468,48 +4468,48 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46151</v>
+        <v>46149</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>230</v>
+        <v>190</v>
       </c>
       <c r="C66" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D66" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D66" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C67" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C67" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D67" s="43" t="inlineStr">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -4533,16 +4533,16 @@
         <v>46151</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C68" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D68" s="41" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>230</v>
+      </c>
+      <c r="C68" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D68" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
         <v>46151</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C69" s="42" t="inlineStr">
         <is>
@@ -4580,25 +4580,25 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46158</v>
+        <v>46151</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C70" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D70" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C70" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D70" s="41" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E70" s="30" t="inlineStr">
@@ -4608,20 +4608,20 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46158</v>
+        <v>46151</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C71" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C71" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D71" s="43" t="inlineStr">
@@ -4631,53 +4631,53 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46164</v>
+        <v>46158</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C72" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D72" s="44" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C72" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D72" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46165</v>
+        <v>46158</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C73" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C73" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D73" s="43" t="inlineStr">
@@ -4687,28 +4687,28 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46171</v>
+        <v>46164</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C74" s="49" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C74" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D74" s="44" t="inlineStr">
+      <c r="D74" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4720,16 +4720,16 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B75" s="38" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C75" s="42" t="inlineStr">
         <is>
@@ -4743,49 +4743,53 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B76" s="33" t="inlineStr"/>
-      <c r="C76" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D76" s="44" t="inlineStr">
+        <v>46171</v>
+      </c>
+      <c r="B76" s="33" t="n">
+        <v>155</v>
+      </c>
+      <c r="C76" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D76" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B77" s="38" t="inlineStr"/>
-      <c r="C77" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>46171</v>
+      </c>
+      <c r="B77" s="38" t="n">
+        <v>240</v>
+      </c>
+      <c r="C77" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D77" s="43" t="inlineStr">
@@ -4795,12 +4799,12 @@
       </c>
       <c r="E77" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -4808,27 +4812,25 @@
       <c r="A78" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B78" s="33" t="n">
-        <v>240</v>
-      </c>
+      <c r="B78" s="33" t="inlineStr"/>
       <c r="C78" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D78" s="44" t="inlineStr">
+      <c r="D78" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -4836,12 +4838,10 @@
       <c r="A79" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B79" s="38" t="n">
-        <v>250</v>
-      </c>
-      <c r="C79" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B79" s="38" t="inlineStr"/>
+      <c r="C79" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D79" s="43" t="inlineStr">
@@ -4851,28 +4851,28 @@
       </c>
       <c r="E79" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C80" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D80" s="44" t="inlineStr">
+        <v>240</v>
+      </c>
+      <c r="C80" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D80" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4884,20 +4884,20 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B81" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C81" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C81" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D81" s="43" t="inlineStr">
@@ -4912,23 +4912,23 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="31" t="n">
-        <v>46177</v>
+        <v>46173</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C82" s="49" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C82" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D82" s="44" t="inlineStr">
+      <c r="D82" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4940,18 +4940,20 @@
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B83" s="38" t="inlineStr"/>
-      <c r="C83" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46173</v>
+      </c>
+      <c r="B83" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C83" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D83" s="43" t="inlineStr">
@@ -4961,53 +4963,51 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46182</v>
+        <v>46177</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="C84" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D84" s="44" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C84" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D84" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="36" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B85" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C85" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B85" s="38" t="inlineStr"/>
+      <c r="C85" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D85" s="43" t="inlineStr">
@@ -5017,58 +5017,58 @@
       </c>
       <c r="E85" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C86" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D86" s="44" t="inlineStr">
+        <v>355</v>
+      </c>
+      <c r="C86" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D86" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E86" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="36" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C87" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D87" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D87" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
@@ -5078,25 +5078,25 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C88" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D88" s="41" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>170</v>
+      </c>
+      <c r="C88" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D88" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -5122,9 +5122,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D89" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D89" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -5143,16 +5143,16 @@
         <v>46186</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C90" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D90" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C90" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D90" s="41" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5162,16 +5162,16 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="C91" s="56" t="inlineStr">
         <is>
@@ -5190,23 +5190,23 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C92" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D92" s="44" t="inlineStr">
+        <v>155</v>
+      </c>
+      <c r="C92" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D92" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5218,20 +5218,20 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C93" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C93" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D93" s="43" t="inlineStr">
@@ -5241,12 +5241,12 @@
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
@@ -5255,31 +5255,87 @@
         <v>46193</v>
       </c>
       <c r="B94" s="33" t="n">
+        <v>215</v>
+      </c>
+      <c r="C94" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D94" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E94" s="30" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F94" s="30" t="inlineStr">
+        <is>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="15" customHeight="1">
+      <c r="A95" s="36" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B95" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C94" s="49" t="inlineStr">
+      <c r="C95" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D94" s="34" t="inlineStr">
+      <c r="D95" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
-      <c r="E94" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F94" s="30" t="inlineStr">
+      <c r="E95" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F95" s="35" t="inlineStr">
         <is>
           <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
+    <row r="96" ht="15" customHeight="1">
+      <c r="A96" s="31" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B96" s="33" t="n">
+        <v>150</v>
+      </c>
+      <c r="C96" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D96" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E96" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F96" s="30" t="inlineStr">
+        <is>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F94"/>
+  <autoFilter ref="A3:F96"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5294,7 +5350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5318,9 +5374,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="53" t="inlineStr">
-        <is>
-          <t>Generated March 25, 2026  ·  04:34 UTC</t>
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>Generated March 25, 2026  ·  08:07 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5401,9 +5457,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D5" s="39" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+      <c r="D5" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -5413,7 +5469,7 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1</t>
+          <t>Nike Air Max 90 “Infrared 3M”</t>
         </is>
       </c>
     </row>
@@ -5422,16 +5478,16 @@
         <v>46107</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D6" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
@@ -5441,7 +5497,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
         </is>
       </c>
     </row>
@@ -5450,16 +5506,16 @@
         <v>46107</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C7" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D7" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
@@ -5469,7 +5525,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Patta x Nike Air Max 1</t>
         </is>
       </c>
     </row>
@@ -5478,14 +5534,14 @@
         <v>46107</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="44" t="inlineStr">
+      <c r="D8" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5497,7 +5553,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Greedy”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5562,7 @@
         <v>46107</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>250</v>
+        <v>190</v>
       </c>
       <c r="C9" s="42" t="inlineStr">
         <is>
@@ -5525,7 +5581,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Max 95 “Lumber Yard”</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
     </row>
@@ -5534,14 +5590,14 @@
         <v>46107</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>250</v>
+        <v>190</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="44" t="inlineStr">
+      <c r="D10" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5553,16 +5609,16 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Max 95 “The Woods”</t>
+          <t>Nike Air Max 95 “Greedy”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46108</v>
+        <v>46107</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C11" s="42" t="inlineStr">
         <is>
@@ -5581,23 +5637,23 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
+          <t>Oregon Ducks x Nike Air Max 95 “Lumber Yard”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46108</v>
+        <v>46107</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="44" t="inlineStr">
+      <c r="D12" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5609,25 +5665,25 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue”</t>
+          <t>Oregon Ducks x Nike Air Max 95 “The Woods”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46109</v>
+        <v>46108</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C13" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D13" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -5637,23 +5693,25 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46109</v>
-      </c>
-      <c r="B14" s="33" t="inlineStr"/>
+        <v>46108</v>
+      </c>
+      <c r="B14" s="33" t="n">
+        <v>240</v>
+      </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -5663,7 +5721,7 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
     </row>
@@ -5672,26 +5730,26 @@
         <v>46109</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>215</v>
+        <v>190</v>
       </c>
       <c r="C15" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D15" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
@@ -5699,17 +5757,15 @@
       <c r="A16" s="31" t="n">
         <v>46109</v>
       </c>
-      <c r="B16" s="33" t="n">
-        <v>162</v>
-      </c>
+      <c r="B16" s="33" t="inlineStr"/>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -5719,16 +5775,16 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 (GS)</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46112</v>
+        <v>46109</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>130</v>
+        <v>215</v>
       </c>
       <c r="C17" s="42" t="inlineStr">
         <is>
@@ -5742,49 +5798,49 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46115</v>
+        <v>46109</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C18" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D18" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>162</v>
+      </c>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D18" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46115</v>
+        <v>46112</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C19" s="42" t="inlineStr">
         <is>
@@ -5803,25 +5859,25 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46116</v>
+        <v>46115</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C20" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D20" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
@@ -5831,16 +5887,16 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46123</v>
+        <v>46115</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>185</v>
+        <v>235</v>
       </c>
       <c r="C21" s="42" t="inlineStr">
         <is>
@@ -5854,47 +5910,49 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B22" s="33" t="inlineStr"/>
+        <v>46116</v>
+      </c>
+      <c r="B22" s="33" t="n">
+        <v>205</v>
+      </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D22" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46125</v>
+        <v>46123</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C23" s="42" t="inlineStr">
         <is>
@@ -5908,12 +5966,12 @@
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -5929,7 +5987,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="44" t="inlineStr">
+      <c r="D24" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5941,7 +5999,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5949,17 +6007,15 @@
       <c r="A25" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B25" s="38" t="n">
-        <v>220</v>
-      </c>
+      <c r="B25" s="38" t="inlineStr"/>
       <c r="C25" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D25" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D25" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E25" s="35" t="inlineStr">
@@ -5969,23 +6025,23 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46129</v>
+        <v>46125</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="44" t="inlineStr">
+      <c r="D26" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5997,16 +6053,16 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46130</v>
+        <v>46125</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C27" s="42" t="inlineStr">
         <is>
@@ -6025,44 +6081,44 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46135</v>
+        <v>46129</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C28" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D28" s="44" t="inlineStr">
+      <c r="D28" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46136</v>
+        <v>46130</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C29" s="42" t="inlineStr">
         <is>
@@ -6081,42 +6137,44 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B30" s="33" t="inlineStr"/>
+        <v>46135</v>
+      </c>
+      <c r="B30" s="33" t="n">
+        <v>220</v>
+      </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D30" s="44" t="inlineStr">
+      <c r="D30" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -6130,12 +6188,12 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -6143,27 +6201,25 @@
       <c r="A32" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B32" s="33" t="n">
-        <v>200</v>
-      </c>
+      <c r="B32" s="33" t="inlineStr"/>
       <c r="C32" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D32" s="44" t="inlineStr">
+      <c r="D32" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -6172,7 +6228,7 @@
         <v>46137</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>180</v>
+        <v>215</v>
       </c>
       <c r="C33" s="42" t="inlineStr">
         <is>
@@ -6186,26 +6242,28 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B34" s="33" t="inlineStr"/>
+        <v>46137</v>
+      </c>
+      <c r="B34" s="33" t="n">
+        <v>200</v>
+      </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D34" s="44" t="inlineStr">
+      <c r="D34" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6217,16 +6275,16 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46144</v>
+        <v>46137</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="C35" s="42" t="inlineStr">
         <is>
@@ -6240,28 +6298,26 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46144</v>
-      </c>
-      <c r="B36" s="33" t="n">
-        <v>195</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B36" s="33" t="inlineStr"/>
       <c r="C36" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="44" t="inlineStr">
+      <c r="D36" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6273,16 +6329,16 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C37" s="42" t="inlineStr">
         <is>
@@ -6296,30 +6352,30 @@
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46151</v>
+        <v>46144</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D38" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D38" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
@@ -6329,16 +6385,16 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46151</v>
+        <v>46149</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="C39" s="42" t="inlineStr">
         <is>
@@ -6357,7 +6413,7 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
@@ -6366,16 +6422,16 @@
         <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C40" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D40" s="41" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+        <v>230</v>
+      </c>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
@@ -6385,7 +6441,7 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -6394,7 +6450,7 @@
         <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C41" s="42" t="inlineStr">
         <is>
@@ -6413,25 +6469,25 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46158</v>
+        <v>46151</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C42" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D42" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C42" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D42" s="41" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
@@ -6441,16 +6497,16 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46165</v>
+        <v>46151</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C43" s="42" t="inlineStr">
         <is>
@@ -6464,48 +6520,50 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46171</v>
+        <v>46158</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>240</v>
+        <v>145</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D44" s="44" t="inlineStr">
+      <c r="D44" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B45" s="38" t="inlineStr"/>
+        <v>46165</v>
+      </c>
+      <c r="B45" s="38" t="n">
+        <v>205</v>
+      </c>
       <c r="C45" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6523,13 +6581,13 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="B46" s="33" t="n">
         <v>240</v>
@@ -6539,7 +6597,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D46" s="44" t="inlineStr">
+      <c r="D46" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6551,7 +6609,7 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -6559,9 +6617,7 @@
       <c r="A47" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B47" s="38" t="n">
-        <v>250</v>
-      </c>
+      <c r="B47" s="38" t="inlineStr"/>
       <c r="C47" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6574,47 +6630,49 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B48" s="33" t="inlineStr"/>
+        <v>46172</v>
+      </c>
+      <c r="B48" s="33" t="n">
+        <v>240</v>
+      </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D48" s="44" t="inlineStr">
+      <c r="D48" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46182</v>
+        <v>46172</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>355</v>
+        <v>250</v>
       </c>
       <c r="C49" s="42" t="inlineStr">
         <is>
@@ -6628,49 +6686,47 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B50" s="33" t="n">
-        <v>150</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B50" s="33" t="inlineStr"/>
       <c r="C50" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D50" s="41" t="inlineStr">
-        <is>
-          <t>Raffle</t>
+      <c r="D50" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46193</v>
+        <v>46182</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>150</v>
+        <v>355</v>
       </c>
       <c r="C51" s="42" t="inlineStr">
         <is>
@@ -6684,45 +6740,101 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B52" s="33" t="n">
+        <v>150</v>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D52" s="41" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
+        </is>
+      </c>
+      <c r="E52" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F52" s="30" t="inlineStr">
+        <is>
+          <t>Patta x Nike Air Max 1 ’87</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="A53" s="36" t="n">
         <v>46193</v>
       </c>
-      <c r="B52" s="33" t="n">
+      <c r="B53" s="38" t="n">
         <v>215</v>
       </c>
-      <c r="C52" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D52" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E52" s="30" t="inlineStr">
+      <c r="C53" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D53" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E53" s="35" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="F52" s="30" t="inlineStr">
+      <c r="F53" s="35" t="inlineStr">
         <is>
           <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="A54" s="31" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B54" s="33" t="n">
+        <v>150</v>
+      </c>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D54" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E54" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F54" s="30" t="inlineStr">
+        <is>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F52"/>
+  <autoFilter ref="A3:F54"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-26 05:26 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$96</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -651,7 +651,10 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -679,13 +682,10 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 25, 2026  ·  08:07 UTC</t>
+          <t>Generated March 26, 2026  ·  05:26 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1628,16 +1628,16 @@
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$184</t>
+          <t>$186</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1740,7 +1740,7 @@
         <v>46115</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         <v>46151</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
         <v>46107</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
         <v>46186</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E13" s="42" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Paisley Bandana”</t>
+          <t>Nike Air Max 90 “Infrared 3M”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -1876,7 +1876,7 @@
         <v>46107</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1887,18 +1887,18 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="H14" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared 3M”</t>
+          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1910,7 +1910,7 @@
         <v>46107</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="42" t="inlineStr">
         <is>
@@ -1921,18 +1921,18 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="H15" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>190</v>
+      </c>
+      <c r="H15" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
+          <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1944,7 +1944,7 @@
         <v>46107</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1955,7 +1955,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="H16" s="34" t="inlineStr">
         <is>
@@ -2011,13 +2011,13 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="44" t="inlineStr">
+      <c r="A20" s="45" t="inlineStr">
         <is>
           <t>Nike</t>
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
       <c r="E20" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="45" t="inlineStr">
+      <c r="G20" s="46" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2037,7 +2037,7 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="46" t="inlineStr">
+      <c r="A21" s="47" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
@@ -2051,9 +2051,9 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>49</v>
-      </c>
-      <c r="G21" s="47" t="inlineStr">
+        <v>50</v>
+      </c>
+      <c r="G21" s="48" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -2063,23 +2063,23 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="45" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>8</v>
-      </c>
-      <c r="D22" s="48" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="D22" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>32</v>
-      </c>
-      <c r="G22" s="49" t="inlineStr">
+        <v>34</v>
+      </c>
+      <c r="G22" s="50" t="inlineStr">
         <is>
           <t>Raffle/Dropship</t>
         </is>
@@ -2089,7 +2089,7 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="46" t="inlineStr">
+      <c r="A23" s="47" t="inlineStr">
         <is>
           <t>Reebok</t>
         </is>
@@ -2097,17 +2097,17 @@
       <c r="B23" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="50" t="inlineStr">
+      <c r="D23" s="51" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
       <c r="E23" s="35" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="44" t="inlineStr">
+      <c r="A24" s="45" t="inlineStr">
         <is>
           <t>Converse</t>
         </is>
@@ -2166,17 +2166,17 @@
       </c>
       <c r="B28" s="30" t="inlineStr">
         <is>
-          <t>3/25 – 3/31</t>
+          <t>3/26 – 4/1</t>
         </is>
       </c>
       <c r="C28" s="30" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D28" s="40" t="n">
         <v>16</v>
       </c>
       <c r="E28" s="30" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2187,17 +2187,17 @@
       </c>
       <c r="B29" s="35" t="inlineStr">
         <is>
-          <t>4/1 – 4/7</t>
+          <t>4/2 – 4/8</t>
         </is>
       </c>
       <c r="C29" s="35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D29" s="42" t="n">
         <v>3</v>
       </c>
       <c r="E29" s="35" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="B30" s="30" t="inlineStr">
         <is>
-          <t>4/8 – 4/14</t>
+          <t>4/9 – 4/15</t>
         </is>
       </c>
       <c r="C30" s="30" t="n">
@@ -2229,17 +2229,17 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>4/15 – 4/21</t>
+          <t>4/16 – 4/22</t>
         </is>
       </c>
       <c r="C31" s="35" t="n">
         <v>5</v>
       </c>
       <c r="D31" s="42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" s="35" t="n">
-        <v>5</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="B32" s="30" t="inlineStr">
         <is>
-          <t>4/22 – 4/28</t>
+          <t>4/23 – 4/29</t>
         </is>
       </c>
       <c r="C32" s="30" t="n">
@@ -2271,17 +2271,17 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>4/29 – 5/5</t>
+          <t>4/30 – 5/6</t>
         </is>
       </c>
       <c r="C33" s="35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D33" s="42" t="n">
         <v>3</v>
       </c>
       <c r="E33" s="35" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2292,17 +2292,17 @@
       </c>
       <c r="B34" s="30" t="inlineStr">
         <is>
-          <t>5/6 – 5/12</t>
+          <t>5/7 – 5/13</t>
         </is>
       </c>
       <c r="C34" s="30" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D34" s="40" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E34" s="30" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2313,17 +2313,17 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>5/13 – 5/19</t>
+          <t>5/14 – 5/20</t>
         </is>
       </c>
       <c r="C35" s="35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D35" s="42" t="n">
         <v>1</v>
       </c>
       <c r="E35" s="35" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="B36" s="30" t="inlineStr">
         <is>
-          <t>5/20 – 5/26</t>
+          <t>5/21 – 5/27</t>
         </is>
       </c>
       <c r="C36" s="30" t="n">
@@ -2355,17 +2355,17 @@
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>5/27 – 6/2</t>
+          <t>5/28 – 6/3</t>
         </is>
       </c>
       <c r="C37" s="35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D37" s="42" t="n">
         <v>4</v>
       </c>
       <c r="E37" s="35" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="B38" s="30" t="inlineStr">
         <is>
-          <t>6/3 – 6/9</t>
+          <t>6/4 – 6/10</t>
         </is>
       </c>
       <c r="C38" s="30" t="n">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>6/10 – 6/16</t>
+          <t>6/11 – 6/17</t>
         </is>
       </c>
       <c r="C39" s="35" t="n">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="B40" s="30" t="inlineStr">
         <is>
-          <t>6/17 – 6/23</t>
+          <t>6/18 – 6/24</t>
         </is>
       </c>
       <c r="C40" s="30" t="n">
@@ -2478,42 +2478,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="51" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="B1" s="51" t="inlineStr">
+      <c r="B1" s="52" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="D1" s="51" t="inlineStr">
+      <c r="D1" s="52" t="inlineStr">
         <is>
           <t>Hype Level</t>
         </is>
       </c>
-      <c r="E1" s="51" t="inlineStr">
+      <c r="E1" s="52" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="G1" s="51" t="inlineStr">
+      <c r="G1" s="52" t="inlineStr">
         <is>
           <t>Sale Method</t>
         </is>
       </c>
-      <c r="H1" s="51" t="inlineStr">
+      <c r="H1" s="52" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="J1" s="51" t="inlineStr">
+      <c r="J1" s="52" t="inlineStr">
         <is>
           <t>Price Range</t>
         </is>
       </c>
-      <c r="K1" s="51" t="inlineStr">
+      <c r="K1" s="52" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
@@ -2526,7 +2526,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -2568,7 +2568,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2618,7 +2618,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -2636,7 +2636,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2644,7 +2644,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -2701,9 +2701,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="52" t="inlineStr">
-        <is>
-          <t>Generated March 25, 2026  ·  08:07 UTC</t>
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>Generated March 26, 2026  ·  05:26 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2746,85 +2746,85 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>80</v>
-      </c>
-      <c r="C4" s="53" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D4" s="54" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D4" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Thug Club x adidas Adifom IIInfinity Mule</t>
+          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C5" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D5" s="43" t="inlineStr">
+        <v>150</v>
+      </c>
+      <c r="C5" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D5" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Thug Club x adidas Superstar Vintage</t>
+          <t>Nike Air Max 90 “Infrared 3M”</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C6" s="53" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D6" s="54" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>190</v>
+      </c>
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Thug Club x adidas AdiFom Megaride</t>
+          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2840,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="55" t="inlineStr">
+      <c r="D7" s="44" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -2861,16 +2861,16 @@
         <v>46107</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C8" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D8" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C8" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Liquid Max “Poison Dart Frog”</t>
+          <t>Patta x Nike Air Max 1</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="43" t="inlineStr">
+      <c r="D9" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared 3M”</t>
+          <t>Nike Air Max 90 “Infrared Reflective”</t>
         </is>
       </c>
     </row>
@@ -2924,9 +2924,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
+          <t>Nike Air Max 95 “Pink Foam” (W)</t>
         </is>
       </c>
     </row>
@@ -2945,16 +2945,16 @@
         <v>46107</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C11" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D11" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1</t>
+          <t>Nike Air Max 95 “Greedy”</t>
         </is>
       </c>
     </row>
@@ -2973,14 +2973,14 @@
         <v>46107</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="54" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared Reflective”</t>
+          <t>Oregon Ducks x Nike Air Max 95 “Lumber Yard”</t>
         </is>
       </c>
     </row>
@@ -3001,14 +3001,14 @@
         <v>46107</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>190</v>
+        <v>250</v>
       </c>
       <c r="C13" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
+      <c r="D13" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3020,23 +3020,23 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” (W)</t>
+          <t>Oregon Ducks x Nike Air Max 95 “The Woods”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="54" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3048,51 +3048,51 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Greedy”</t>
+          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>250</v>
-      </c>
-      <c r="C15" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D15" s="43" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C15" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Max 95 “Lumber Yard”</t>
+          <t>Reebok Angel Reese 1 “Unapologetically Angel”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="C16" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D16" s="54" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C16" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D16" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Max 95 “The Woods”</t>
+          <t>Nike GT Cut “Dylan Harper”</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3120,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
+      <c r="D17" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3132,53 +3132,51 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue” 2026</t>
+          <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C18" s="53" t="inlineStr">
+        <v>160</v>
+      </c>
+      <c r="C18" s="55" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="D18" s="54" t="inlineStr">
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Reebok Angel Reese 1 “Unapologetically Angel”</t>
+          <t>adidas BadBo 1.0 “Rise”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46108</v>
-      </c>
-      <c r="B19" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C19" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D19" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46109</v>
+      </c>
+      <c r="B19" s="38" t="inlineStr"/>
+      <c r="C19" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D19" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
@@ -3188,35 +3186,35 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut “Dylan Harper”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D20" s="54" t="inlineStr">
+      <c r="D20" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “University Blue”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3230,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D21" s="55" t="inlineStr">
+      <c r="D21" s="44" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3281,37 +3279,39 @@
         <v>46109</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C23" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D23" s="43" t="inlineStr">
+        <v>162</v>
+      </c>
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D23" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>adidas BadBo 1.0 “Rise”</t>
+          <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46109</v>
-      </c>
-      <c r="B24" s="33" t="inlineStr"/>
-      <c r="C24" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46111</v>
+      </c>
+      <c r="B24" s="33" t="n">
+        <v>210</v>
+      </c>
+      <c r="C24" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D24" s="34" t="inlineStr">
@@ -3326,23 +3326,23 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Nike GT Future “Galaxy Aura”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C25" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D25" s="43" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C25" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D25" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3354,23 +3354,23 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Jordan Jumpman Pro “Black Concord”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="54" t="inlineStr">
+      <c r="D26" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3382,25 +3382,25 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 (GS)</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>210</v>
+        <v>145</v>
       </c>
       <c r="C27" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D27" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D27" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
@@ -3410,51 +3410,51 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Future “Galaxy Aura”</t>
+          <t>Nike Sabrina 3 “What The”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C28" s="48" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C28" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D28" s="54" t="inlineStr">
+      <c r="D28" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Jordan Jumpman Pro “Black Concord”</t>
+          <t>Nike Mind 001 “Sail”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C29" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D29" s="43" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C29" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D29" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3466,53 +3466,53 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Nike Mind 001 “Geode Teal”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C30" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D30" s="54" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C30" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D30" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Sabrina 3 “What The”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>95</v>
+        <v>225</v>
       </c>
       <c r="C31" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D31" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D31" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
@@ -3522,35 +3522,35 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Sail”</t>
+          <t>Fragment x Nike Air Liquid Max “Black”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C32" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D32" s="54" t="inlineStr">
+        <v>130</v>
+      </c>
+      <c r="C32" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D32" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Geode Teal”</t>
+          <t>Converse SHAI 001 “Camo”</t>
         </is>
       </c>
     </row>
@@ -3559,26 +3559,26 @@
         <v>46115</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C33" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D33" s="43" t="inlineStr">
+        <v>225</v>
+      </c>
+      <c r="C33" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D33" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 “Camo”</t>
+          <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
     </row>
@@ -3587,70 +3587,70 @@
         <v>46115</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C34" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D34" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>235</v>
+      </c>
+      <c r="C34" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D34" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>225</v>
-      </c>
-      <c r="C35" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D35" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>205</v>
+      </c>
+      <c r="C35" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D35" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max “Black”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46115</v>
+        <v>46122</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>225</v>
-      </c>
-      <c r="C36" s="48" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C36" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D36" s="54" t="inlineStr">
+      <c r="D36" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3662,23 +3662,23 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46115</v>
+        <v>46122</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C37" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D37" s="43" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C37" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D37" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3690,109 +3690,107 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46116</v>
+        <v>46123</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C38" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D38" s="54" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C38" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D38" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C39" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D39" s="43" t="inlineStr">
+        <v>185</v>
+      </c>
+      <c r="C39" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D39" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46122</v>
+        <v>46124</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C40" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D40" s="54" t="inlineStr">
+        <v>130</v>
+      </c>
+      <c r="C40" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D40" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46123</v>
-      </c>
-      <c r="B41" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C41" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D41" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B41" s="38" t="inlineStr"/>
+      <c r="C41" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D41" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
@@ -3802,63 +3800,63 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D42" s="54" t="inlineStr">
+      <c r="D42" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C43" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D43" s="43" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C43" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D43" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3867,14 +3865,14 @@
         <v>46125</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D44" s="54" t="inlineStr">
+      <c r="D44" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3886,49 +3884,51 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B45" s="38" t="inlineStr"/>
-      <c r="C45" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D45" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>46128</v>
+      </c>
+      <c r="B45" s="38" t="n">
+        <v>160</v>
+      </c>
+      <c r="C45" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D45" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46125</v>
+        <v>46129</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C46" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D46" s="54" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C46" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3940,25 +3940,25 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46125</v>
+        <v>46130</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C47" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D47" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C47" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D47" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E47" s="35" t="inlineStr">
@@ -3968,51 +3968,51 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46128</v>
+        <v>46130</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C48" s="53" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D48" s="54" t="inlineStr">
+        <v>240</v>
+      </c>
+      <c r="C48" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46129</v>
+        <v>46133</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C49" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D49" s="43" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C49" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D49" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4024,51 +4024,51 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46130</v>
+        <v>46135</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C50" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D50" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>220</v>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D50" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46130</v>
+        <v>46136</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="C51" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="43" t="inlineStr">
+      <c r="D51" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4080,51 +4080,51 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46133</v>
+        <v>46137</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C52" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D52" s="54" t="inlineStr">
+        <v>215</v>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D52" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46135</v>
+        <v>46137</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="C53" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D53" s="43" t="inlineStr">
+      <c r="D53" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4136,23 +4136,23 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="54" t="inlineStr">
+      <c r="D54" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4164,7 +4164,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4178,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D55" s="43" t="inlineStr">
+      <c r="D55" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4196,17 +4196,15 @@
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B56" s="33" t="n">
-        <v>215</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B56" s="33" t="inlineStr"/>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="54" t="inlineStr">
+      <c r="D56" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4218,51 +4216,51 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C57" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D57" s="43" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C57" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D57" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C58" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D58" s="54" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C58" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D58" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4274,49 +4272,51 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B59" s="38" t="inlineStr"/>
-      <c r="C59" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D59" s="43" t="inlineStr">
+        <v>46143</v>
+      </c>
+      <c r="B59" s="38" t="n">
+        <v>135</v>
+      </c>
+      <c r="C59" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D59" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C60" s="48" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C60" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D60" s="54" t="inlineStr">
+      <c r="D60" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4328,63 +4328,63 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C61" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D61" s="43" t="inlineStr">
+        <v>195</v>
+      </c>
+      <c r="C61" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D61" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C62" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D62" s="54" t="inlineStr">
+        <v>220</v>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D62" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4393,70 +4393,70 @@
         <v>46144</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C63" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D63" s="43" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C63" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D63" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C64" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D64" s="54" t="inlineStr">
+      <c r="D64" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46144</v>
+        <v>46150</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C65" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D65" s="43" t="inlineStr">
+        <v>240</v>
+      </c>
+      <c r="C65" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D65" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4468,23 +4468,23 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="C66" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D66" s="54" t="inlineStr">
+      <c r="D66" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4512,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D67" s="43" t="inlineStr">
+      <c r="D67" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4533,26 +4533,26 @@
         <v>46151</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C68" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D68" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D68" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4561,26 +4561,26 @@
         <v>46151</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>120</v>
+        <v>230</v>
       </c>
       <c r="C69" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D69" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D69" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E69" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -4589,26 +4589,26 @@
         <v>46151</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C70" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D70" s="41" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>120</v>
+      </c>
+      <c r="C70" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D70" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E70" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -4617,54 +4617,54 @@
         <v>46151</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C71" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D71" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C71" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D71" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C72" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D72" s="54" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C72" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D72" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
@@ -4673,110 +4673,110 @@
         <v>46158</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C73" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D73" s="43" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C73" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D73" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46164</v>
+        <v>46158</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C74" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D74" s="54" t="inlineStr">
+        <v>160</v>
+      </c>
+      <c r="C74" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D74" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46165</v>
+        <v>46164</v>
       </c>
       <c r="B75" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C75" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D75" s="43" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C75" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D75" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C76" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D76" s="54" t="inlineStr">
+        <v>205</v>
+      </c>
+      <c r="C76" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D76" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4792,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D77" s="43" t="inlineStr">
+      <c r="D77" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4804,59 +4804,63 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B78" s="33" t="inlineStr"/>
-      <c r="C78" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D78" s="54" t="inlineStr">
+        <v>46171</v>
+      </c>
+      <c r="B78" s="33" t="n">
+        <v>155</v>
+      </c>
+      <c r="C78" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D78" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B79" s="38" t="inlineStr"/>
-      <c r="C79" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D79" s="43" t="inlineStr">
+        <v>46171</v>
+      </c>
+      <c r="B79" s="38" t="n">
+        <v>240</v>
+      </c>
+      <c r="C79" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D79" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E79" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -4864,27 +4868,25 @@
       <c r="A80" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B80" s="33" t="n">
-        <v>240</v>
-      </c>
+      <c r="B80" s="33" t="inlineStr"/>
       <c r="C80" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D80" s="54" t="inlineStr">
+      <c r="D80" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E80" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -4892,43 +4894,41 @@
       <c r="A81" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B81" s="38" t="n">
-        <v>250</v>
-      </c>
-      <c r="C81" s="42" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D81" s="43" t="inlineStr">
+      <c r="B81" s="38" t="inlineStr"/>
+      <c r="C81" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D81" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="31" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C82" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D82" s="54" t="inlineStr">
+        <v>250</v>
+      </c>
+      <c r="C82" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D82" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D83" s="43" t="inlineStr">
+      <c r="D83" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4979,12 +4979,12 @@
       <c r="B84" s="33" t="n">
         <v>140</v>
       </c>
-      <c r="C84" s="48" t="inlineStr">
+      <c r="C84" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D84" s="54" t="inlineStr">
+      <c r="D84" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5010,7 +5010,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D85" s="43" t="inlineStr">
+      <c r="D85" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5038,7 +5038,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D86" s="54" t="inlineStr">
+      <c r="D86" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5066,7 +5066,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D87" s="43" t="inlineStr">
+      <c r="D87" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5089,12 +5089,12 @@
       <c r="B88" s="33" t="n">
         <v>170</v>
       </c>
-      <c r="C88" s="48" t="inlineStr">
+      <c r="C88" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D88" s="54" t="inlineStr">
+      <c r="D88" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5122,9 +5122,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D89" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D89" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -5143,16 +5143,16 @@
         <v>46186</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C90" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D90" s="41" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>210</v>
+      </c>
+      <c r="C90" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D90" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -5171,16 +5171,16 @@
         <v>46186</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C91" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D91" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C91" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D91" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E91" s="35" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -5201,12 +5201,12 @@
       <c r="B92" s="33" t="n">
         <v>155</v>
       </c>
-      <c r="C92" s="48" t="inlineStr">
+      <c r="C92" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D92" s="54" t="inlineStr">
+      <c r="D92" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5234,7 +5234,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D93" s="43" t="inlineStr">
+      <c r="D93" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5255,26 +5255,26 @@
         <v>46193</v>
       </c>
       <c r="B94" s="33" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="C94" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D94" s="54" t="inlineStr">
+      <c r="D94" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5283,26 +5283,26 @@
         <v>46193</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C95" s="56" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D95" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>215</v>
+      </c>
+      <c r="C95" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D95" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -5311,16 +5311,16 @@
         <v>46193</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C96" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D96" s="54" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C96" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D96" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -5350,7 +5350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5374,9 +5374,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="52" t="inlineStr">
-        <is>
-          <t>Generated March 25, 2026  ·  08:07 UTC</t>
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>Generated March 26, 2026  ·  05:26 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5422,16 +5422,16 @@
         <v>46107</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C4" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D4" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D4" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Paisley Bandana”</t>
+          <t>Nike Air Max 90 “Infrared 3M”</t>
         </is>
       </c>
     </row>
@@ -5450,16 +5450,16 @@
         <v>46107</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C5" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D5" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D5" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Infrared 3M”</t>
+          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
         </is>
       </c>
     </row>
@@ -5478,7 +5478,7 @@
         <v>46107</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Greedy”</t>
+          <t>Nike Air Max 95 “Paisley Bandana”</t>
         </is>
       </c>
     </row>
@@ -5541,7 +5541,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="54" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5569,7 +5569,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="43" t="inlineStr">
+      <c r="D9" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5597,7 +5597,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="54" t="inlineStr">
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5625,7 +5625,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5653,7 +5653,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="54" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5681,7 +5681,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
+      <c r="D13" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5709,7 +5709,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="54" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5729,15 +5729,13 @@
       <c r="A15" s="36" t="n">
         <v>46109</v>
       </c>
-      <c r="B15" s="38" t="n">
-        <v>190</v>
-      </c>
+      <c r="B15" s="38" t="inlineStr"/>
       <c r="C15" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="55" t="inlineStr">
+      <c r="D15" s="44" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5749,7 +5747,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Pink Foam” 2026</t>
+          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
     </row>
@@ -5757,25 +5755,27 @@
       <c r="A16" s="31" t="n">
         <v>46109</v>
       </c>
-      <c r="B16" s="33" t="inlineStr"/>
+      <c r="B16" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
+          <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
     </row>
@@ -5784,26 +5784,26 @@
         <v>46109</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>215</v>
+        <v>190</v>
       </c>
       <c r="C17" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring is in the Air”</t>
+          <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D18" s="54" t="inlineStr">
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5847,7 +5847,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D19" s="43" t="inlineStr">
+      <c r="D19" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5903,7 +5903,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="43" t="inlineStr">
+      <c r="D21" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5931,7 +5931,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="54" t="inlineStr">
+      <c r="D22" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5959,7 +5959,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="43" t="inlineStr">
+      <c r="D23" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5979,17 +5979,15 @@
       <c r="A24" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B24" s="33" t="n">
-        <v>190</v>
-      </c>
+      <c r="B24" s="33" t="inlineStr"/>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="54" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
@@ -5999,7 +5997,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
@@ -6007,15 +6005,17 @@
       <c r="A25" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B25" s="38" t="inlineStr"/>
+      <c r="B25" s="38" t="n">
+        <v>190</v>
+      </c>
       <c r="C25" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D25" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D25" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E25" s="35" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6041,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="54" t="inlineStr">
+      <c r="D26" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6069,7 +6069,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D27" s="43" t="inlineStr">
+      <c r="D27" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6087,7 +6087,7 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B28" s="33" t="n">
         <v>240</v>
@@ -6097,7 +6097,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D28" s="54" t="inlineStr">
+      <c r="D28" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6109,91 +6109,91 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46130</v>
+        <v>46135</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C29" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D29" s="43" t="inlineStr">
+      <c r="D29" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D30" s="54" t="inlineStr">
+      <c r="D30" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D31" s="43" t="inlineStr">
+      <c r="D31" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -6201,25 +6201,27 @@
       <c r="A32" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B32" s="33" t="inlineStr"/>
+      <c r="B32" s="33" t="n">
+        <v>200</v>
+      </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D32" s="54" t="inlineStr">
+      <c r="D32" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -6228,26 +6230,26 @@
         <v>46137</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>215</v>
+        <v>180</v>
       </c>
       <c r="C33" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D33" s="43" t="inlineStr">
+      <c r="D33" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -6255,69 +6257,67 @@
       <c r="A34" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B34" s="33" t="n">
-        <v>200</v>
-      </c>
+      <c r="B34" s="33" t="inlineStr"/>
       <c r="C34" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D34" s="54" t="inlineStr">
+      <c r="D34" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B35" s="38" t="n">
-        <v>180</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B35" s="38" t="inlineStr"/>
       <c r="C35" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D35" s="43" t="inlineStr">
+      <c r="D35" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B36" s="33" t="inlineStr"/>
+        <v>46144</v>
+      </c>
+      <c r="B36" s="33" t="n">
+        <v>195</v>
+      </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="54" t="inlineStr">
+      <c r="D36" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -6345,7 +6345,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="43" t="inlineStr">
+      <c r="D37" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6363,45 +6363,45 @@
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D38" s="54" t="inlineStr">
+      <c r="D38" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C39" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D39" s="43" t="inlineStr">
+      <c r="D39" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6413,35 +6413,35 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D40" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -6450,14 +6450,14 @@
         <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C41" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D41" s="43" t="inlineStr">
+      <c r="D41" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6469,7 +6469,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6478,16 +6478,16 @@
         <v>46151</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C42" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D42" s="41" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>230</v>
+      </c>
+      <c r="C42" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D42" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -6506,14 +6506,14 @@
         <v>46151</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C43" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D43" s="43" t="inlineStr">
+      <c r="D43" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6525,25 +6525,25 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46158</v>
+        <v>46151</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C44" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D44" s="54" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C44" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D44" s="41" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E44" s="30" t="inlineStr">
@@ -6553,23 +6553,23 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46165</v>
+        <v>46158</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>205</v>
+        <v>145</v>
       </c>
       <c r="C45" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D45" s="43" t="inlineStr">
+      <c r="D45" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6581,67 +6581,69 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D46" s="54" t="inlineStr">
+      <c r="D46" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B47" s="38" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="B47" s="38" t="n">
+        <v>240</v>
+      </c>
       <c r="C47" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D47" s="43" t="inlineStr">
+      <c r="D47" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="B48" s="33" t="n">
         <v>240</v>
@@ -6651,7 +6653,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D48" s="54" t="inlineStr">
+      <c r="D48" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6663,7 +6665,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -6671,69 +6673,67 @@
       <c r="A49" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B49" s="38" t="n">
-        <v>250</v>
-      </c>
+      <c r="B49" s="38" t="inlineStr"/>
       <c r="C49" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D49" s="43" t="inlineStr">
+      <c r="D49" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B50" s="33" t="inlineStr"/>
+        <v>46172</v>
+      </c>
+      <c r="B50" s="33" t="n">
+        <v>250</v>
+      </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D50" s="54" t="inlineStr">
+      <c r="D50" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B51" s="38" t="n">
-        <v>355</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B51" s="38" t="inlineStr"/>
       <c r="C51" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="43" t="inlineStr">
+      <c r="D51" s="54" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6745,63 +6745,63 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46186</v>
+        <v>46182</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>150</v>
+        <v>355</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D52" s="41" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D52" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="C53" s="42" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D53" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D53" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -6817,7 +6817,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="54" t="inlineStr">
+      <c r="D54" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6833,8 +6833,36 @@
         </is>
       </c>
     </row>
+    <row r="55" ht="15" customHeight="1">
+      <c r="A55" s="36" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B55" s="38" t="n">
+        <v>215</v>
+      </c>
+      <c r="C55" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D55" s="54" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E55" s="35" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F55" s="35" t="inlineStr">
+        <is>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F54"/>
+  <autoFilter ref="A3:F55"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-28 07:59 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 28, 2026  ·  04:50 UTC</t>
+          <t>Generated March 28, 2026  ·  07:59 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2683,7 +2683,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="54" t="inlineStr">
         <is>
-          <t>Generated March 28, 2026  ·  04:50 UTC</t>
+          <t>Generated March 28, 2026  ·  07:59 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -4038,10 +4038,12 @@
       <c r="A51" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B51" s="38" t="inlineStr"/>
-      <c r="C51" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B51" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C51" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="44" t="inlineStr">
@@ -4051,12 +4053,12 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
@@ -4064,9 +4066,7 @@
       <c r="A52" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B52" s="33" t="n">
-        <v>215</v>
-      </c>
+      <c r="B52" s="33" t="inlineStr"/>
       <c r="C52" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -4093,11 +4093,11 @@
         <v>46142</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C53" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C53" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D53" s="44" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -5039,16 +5039,16 @@
         <v>46186</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C87" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D87" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>210</v>
+      </c>
+      <c r="C87" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D87" s="42" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -5067,16 +5067,16 @@
         <v>46186</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C88" s="50" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D88" s="45" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C88" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D88" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -5102,9 +5102,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D89" s="42" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D89" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="54" t="inlineStr">
         <is>
-          <t>Generated March 28, 2026  ·  04:50 UTC</t>
+          <t>Generated March 28, 2026  ·  07:59 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-30 10:45 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$96</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -654,7 +654,7 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -682,10 +682,10 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 29, 2026  ·  08:04 UTC</t>
+          <t>Generated March 30, 2026  ·  10:45 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1624,20 +1624,20 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$181</t>
+          <t>$179</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1740,7 +1740,7 @@
         <v>46115</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         <v>46151</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
         <v>46186</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
         <v>46112</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="41" t="inlineStr">
         <is>
@@ -1864,19 +1864,19 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Shoe Bag”</t>
+          <t>Air Jordan 3 “Spring Flowers”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
-        <v>46115</v>
+        <v>46113</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1887,7 +1887,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="H14" s="43" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Good Intentions”</t>
+          <t>Nike LeBron 23 “Shoe Bag”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1910,7 +1910,7 @@
         <v>46115</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" s="41" t="inlineStr">
         <is>
@@ -1921,18 +1921,18 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="H15" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="H15" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Nike LeBron 23 Elite “Good Intentions”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1944,7 +1944,7 @@
         <v>46115</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1955,11 +1955,11 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>235</v>
-      </c>
-      <c r="H16" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="H16" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D21" s="41" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G21" s="48" t="inlineStr">
         <is>
@@ -2059,7 +2059,7 @@
         </is>
       </c>
       <c r="H21" s="35" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G22" s="50" t="inlineStr">
         <is>
@@ -2156,17 +2156,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>3/29 – 4/4</t>
+          <t>3/30 – 4/5</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D27" s="40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2177,17 +2177,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/5 – 4/11</t>
+          <t>4/6 – 4/12</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D28" s="41" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2198,17 +2198,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/12 – 4/18</t>
+          <t>4/13 – 4/19</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D29" s="40" t="n">
         <v>5</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/19 – 4/25</t>
+          <t>4/20 – 4/26</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>4/26 – 5/2</t>
+          <t>4/27 – 5/3</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/3 – 5/9</t>
+          <t>5/4 – 5/10</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/10 – 5/16</t>
+          <t>5/11 – 5/17</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/17 – 5/23</t>
+          <t>5/18 – 5/24</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
@@ -2324,17 +2324,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>5/24 – 5/30</t>
+          <t>5/25 – 5/31</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D35" s="40" t="n">
         <v>4</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2345,17 +2345,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>5/31 – 6/6</t>
+          <t>6/1 – 6/7</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/7 – 6/13</t>
+          <t>6/8 – 6/14</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/14 – 6/20</t>
+          <t>6/15 – 6/21</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>6/21 – 6/27</t>
+          <t>6/22 – 6/28</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2574,7 +2574,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2608,7 +2608,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -2659,7 +2659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2685,7 +2685,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 29, 2026  ·  08:04 UTC</t>
+          <t>Generated March 30, 2026  ·  10:45 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2738,7 +2738,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D4" s="54" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -2787,11 +2787,11 @@
         <v>46113</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>115</v>
-      </c>
-      <c r="C6" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>155</v>
+      </c>
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D6" s="43" t="inlineStr">
@@ -2801,12 +2801,12 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Giannis Freak 7 “Light Aqua”</t>
+          <t>Air Jordan 3 “Spring Flowers”</t>
         </is>
       </c>
     </row>
@@ -2815,9 +2815,9 @@
         <v>46113</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C7" s="55" t="inlineStr">
+        <v>115</v>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2834,16 +2834,16 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Sabrina 3 “What The”</t>
+          <t>Nike Giannis Freak 7 “Light Aqua”</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46114</v>
+        <v>46113</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="C8" s="49" t="inlineStr">
         <is>
@@ -2862,18 +2862,18 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Sail”</t>
+          <t>Nike Sabrina 3 “What The”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46114</v>
+        <v>46113</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C9" s="55" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2885,21 +2885,21 @@
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Team Red”</t>
+          <t>Jordan Luka 5 “Black White”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46114</v>
+        <v>46113</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>95</v>
+        <v>130</v>
       </c>
       <c r="C10" s="49" t="inlineStr">
         <is>
@@ -2913,30 +2913,30 @@
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Geode Teal”</t>
+          <t>Jordan Tatum 4 “Offseason”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46115</v>
+        <v>46114</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>225</v>
-      </c>
-      <c r="C11" s="55" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D11" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -2946,20 +2946,20 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max “Black”</t>
+          <t>Nike Mind 001 “Sail”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46115</v>
+        <v>46114</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C12" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>95</v>
+      </c>
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D12" s="43" t="inlineStr">
@@ -2974,25 +2974,25 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Shoe Bag”</t>
+          <t>Nike Mind 001 “Team Red”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46115</v>
+        <v>46114</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C13" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D13" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>95</v>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Good Intentions”</t>
+          <t>Nike Mind 001 “Geode Teal”</t>
         </is>
       </c>
     </row>
@@ -3011,26 +3011,26 @@
         <v>46115</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C14" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D14" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 “Camo”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -3039,26 +3039,26 @@
         <v>46115</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C15" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D15" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>225</v>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D15" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Fragment x Nike Air Liquid Max “Black”</t>
         </is>
       </c>
     </row>
@@ -3067,11 +3067,11 @@
         <v>46115</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>225</v>
-      </c>
-      <c r="C16" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>200</v>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D16" s="43" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max</t>
+          <t>Nike LeBron 23 “Shoe Bag”</t>
         </is>
       </c>
     </row>
@@ -3095,16 +3095,16 @@
         <v>46115</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>235</v>
+        <v>210</v>
       </c>
       <c r="C17" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D17" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
@@ -3114,20 +3114,20 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Nike LeBron 23 Elite “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46116</v>
+        <v>46115</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C18" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C18" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D18" s="43" t="inlineStr">
@@ -3137,25 +3137,25 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Converse SHAI 001 “Camo”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46116</v>
+        <v>46115</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C19" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>225</v>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
@@ -3165,25 +3165,25 @@
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46120</v>
+        <v>46115</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C20" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D20" s="43" t="inlineStr">
@@ -3198,18 +3198,18 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Pegasus Premium</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46120</v>
+        <v>46116</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>260</v>
-      </c>
-      <c r="C21" s="55" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3226,16 +3226,16 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Vomero Premium</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46121</v>
+        <v>46116</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
@@ -3249,25 +3249,25 @@
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46121</v>
+        <v>46120</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C23" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>220</v>
+      </c>
+      <c r="C23" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D23" s="42" t="inlineStr">
@@ -3282,20 +3282,20 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Melitta Baumeister x Nike Pegasus Premium</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46121</v>
+        <v>46120</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C24" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>260</v>
+      </c>
+      <c r="C24" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D24" s="43" t="inlineStr">
@@ -3310,20 +3310,20 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Melitta Baumeister x Nike Vomero Premium</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46122</v>
+        <v>46121</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C25" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D25" s="42" t="inlineStr">
@@ -3338,16 +3338,16 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46122</v>
+        <v>46121</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>235</v>
+        <v>120</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
@@ -3366,16 +3366,16 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46122</v>
+        <v>46121</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C27" s="41" t="inlineStr">
         <is>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
         </is>
       </c>
     </row>
@@ -3403,11 +3403,11 @@
         <v>46122</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C28" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D28" s="43" t="inlineStr">
@@ -3422,20 +3422,20 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46123</v>
+        <v>46122</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C29" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C29" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D29" s="42" t="inlineStr">
@@ -3445,25 +3445,25 @@
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46123</v>
+        <v>46122</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C30" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C30" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D30" s="43" t="inlineStr">
@@ -3478,20 +3478,20 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46124</v>
+        <v>46122</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C31" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>135</v>
+      </c>
+      <c r="C31" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D31" s="42" t="inlineStr">
@@ -3501,28 +3501,30 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B32" s="33" t="inlineStr"/>
-      <c r="C32" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D32" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>46123</v>
+      </c>
+      <c r="B32" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C32" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D32" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
@@ -3532,16 +3534,16 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46125</v>
+        <v>46123</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C33" s="41" t="inlineStr">
         <is>
@@ -3555,25 +3557,25 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46125</v>
+        <v>46124</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C34" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C34" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D34" s="43" t="inlineStr">
@@ -3583,12 +3585,12 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3599,7 @@
         <v>46125</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="C35" s="41" t="inlineStr">
         <is>
@@ -3616,48 +3618,46 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B36" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C36" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D36" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B36" s="33" t="inlineStr"/>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D36" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46129</v>
+        <v>46125</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C37" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C37" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D37" s="42" t="inlineStr">
@@ -3672,25 +3672,25 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46130</v>
+        <v>46125</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C38" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D38" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>220</v>
+      </c>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D38" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
@@ -3700,20 +3700,20 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46130</v>
+        <v>46128</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C39" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C39" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D39" s="42" t="inlineStr">
@@ -3723,21 +3723,21 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46133</v>
+        <v>46129</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>145</v>
+        <v>200</v>
       </c>
       <c r="C40" s="49" t="inlineStr">
         <is>
@@ -3756,44 +3756,44 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46135</v>
+        <v>46130</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C41" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D41" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C41" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D41" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46136</v>
+        <v>46130</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -3812,20 +3812,20 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46137</v>
+        <v>46133</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C43" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C43" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D43" s="42" t="inlineStr">
@@ -3840,15 +3840,17 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B44" s="33" t="inlineStr"/>
+        <v>46135</v>
+      </c>
+      <c r="B44" s="33" t="n">
+        <v>220</v>
+      </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3861,40 +3863,40 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C45" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D45" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D45" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -3902,9 +3904,7 @@
       <c r="A46" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B46" s="33" t="n">
-        <v>200</v>
-      </c>
+      <c r="B46" s="33" t="inlineStr"/>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3917,18 +3917,18 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B47" s="38" t="n">
         <v>215</v>
@@ -3950,15 +3950,17 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B48" s="33" t="inlineStr"/>
+        <v>46137</v>
+      </c>
+      <c r="B48" s="33" t="n">
+        <v>200</v>
+      </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3976,20 +3978,20 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C49" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>180</v>
+      </c>
+      <c r="C49" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D49" s="42" t="inlineStr">
@@ -4004,7 +4006,7 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -4012,12 +4014,10 @@
       <c r="A50" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B50" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C50" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B50" s="33" t="inlineStr"/>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D50" s="43" t="inlineStr">
@@ -4027,25 +4027,25 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C51" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C51" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4055,21 +4055,21 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>190</v>
+        <v>95</v>
       </c>
       <c r="C52" s="49" t="inlineStr">
         <is>
@@ -4088,20 +4088,20 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46144</v>
+        <v>46142</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>195</v>
-      </c>
-      <c r="C53" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C53" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D53" s="42" t="inlineStr">
@@ -4111,25 +4111,25 @@
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C54" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C54" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D54" s="43" t="inlineStr">
@@ -4139,23 +4139,23 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C55" s="55" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C55" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4172,16 +4172,16 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -4195,21 +4195,21 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46150</v>
+        <v>46144</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C57" s="41" t="inlineStr">
         <is>
@@ -4223,25 +4223,25 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46150</v>
+        <v>46144</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C58" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C58" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D58" s="43" t="inlineStr">
@@ -4256,20 +4256,20 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46150</v>
+        <v>46149</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C59" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C59" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D59" s="42" t="inlineStr">
@@ -4284,44 +4284,44 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D60" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D60" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>120</v>
+        <v>210</v>
       </c>
       <c r="C61" s="41" t="inlineStr">
         <is>
@@ -4340,35 +4340,35 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C62" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D62" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>210</v>
+      </c>
+      <c r="C62" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D62" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -4377,39 +4377,39 @@
         <v>46151</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C63" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D63" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C63" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D63" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C64" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>200</v>
+      </c>
+      <c r="C64" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D64" s="43" t="inlineStr">
@@ -4424,44 +4424,44 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>150</v>
+        <v>230</v>
       </c>
       <c r="C65" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D65" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D65" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46158</v>
+        <v>46151</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="C66" s="40" t="inlineStr">
         <is>
@@ -4475,25 +4475,25 @@
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C67" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>170</v>
+      </c>
+      <c r="C67" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D67" s="42" t="inlineStr">
@@ -4503,25 +4503,25 @@
       </c>
       <c r="E67" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46164</v>
+        <v>46157</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C68" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C68" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D68" s="43" t="inlineStr">
@@ -4536,16 +4536,16 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="36" t="n">
-        <v>46165</v>
+        <v>46158</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>205</v>
+        <v>145</v>
       </c>
       <c r="C69" s="41" t="inlineStr">
         <is>
@@ -4564,20 +4564,20 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46171</v>
+        <v>46158</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C70" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C70" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D70" s="43" t="inlineStr">
@@ -4587,23 +4587,23 @@
       </c>
       <c r="E70" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46171</v>
+        <v>46164</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C71" s="55" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C71" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4620,16 +4620,16 @@
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C72" s="40" t="inlineStr">
         <is>
@@ -4643,20 +4643,22 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B73" s="38" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="B73" s="38" t="n">
+        <v>240</v>
+      </c>
       <c r="C73" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4669,25 +4671,25 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="C74" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C74" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D74" s="43" t="inlineStr">
@@ -4702,18 +4704,20 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B75" s="38" t="inlineStr"/>
-      <c r="C75" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>46171</v>
+      </c>
+      <c r="B75" s="38" t="n">
+        <v>240</v>
+      </c>
+      <c r="C75" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D75" s="42" t="inlineStr">
@@ -4723,25 +4727,23 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B76" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C76" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46172</v>
+      </c>
+      <c r="B76" s="33" t="inlineStr"/>
+      <c r="C76" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D76" s="43" t="inlineStr">
@@ -4751,25 +4753,25 @@
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46177</v>
+        <v>46172</v>
       </c>
       <c r="B77" s="38" t="n">
-        <v>140</v>
-      </c>
-      <c r="C77" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C77" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D77" s="42" t="inlineStr">
@@ -4784,18 +4786,18 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46179</v>
+        <v>46172</v>
       </c>
       <c r="B78" s="33" t="inlineStr"/>
-      <c r="C78" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C78" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D78" s="43" t="inlineStr">
@@ -4805,25 +4807,25 @@
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46182</v>
+        <v>46173</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>355</v>
-      </c>
-      <c r="C79" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C79" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4833,21 +4835,21 @@
       </c>
       <c r="E79" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46185</v>
+        <v>46177</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="C80" s="49" t="inlineStr">
         <is>
@@ -4866,20 +4868,18 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B81" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C81" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B81" s="38" t="inlineStr"/>
+      <c r="C81" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D81" s="42" t="inlineStr">
@@ -4889,25 +4889,25 @@
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="31" t="n">
-        <v>46186</v>
+        <v>46182</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C82" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>355</v>
+      </c>
+      <c r="C82" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D82" s="43" t="inlineStr">
@@ -4917,30 +4917,30 @@
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="36" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B83" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C83" s="55" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C83" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D83" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D83" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E83" s="35" t="inlineStr">
@@ -4950,25 +4950,25 @@
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C84" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D84" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>170</v>
+      </c>
+      <c r="C84" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D84" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E84" s="30" t="inlineStr">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -4987,16 +4987,16 @@
         <v>46186</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C85" s="55" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C85" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D85" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D85" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E85" s="35" t="inlineStr">
@@ -5006,25 +5006,25 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C86" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D86" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C86" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D86" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E86" s="30" t="inlineStr">
@@ -5034,20 +5034,20 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="36" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C87" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C87" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D87" s="42" t="inlineStr">
@@ -5062,20 +5062,20 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C88" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C88" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D88" s="43" t="inlineStr">
@@ -5085,30 +5085,30 @@
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C89" s="55" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C89" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D89" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D89" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5118,25 +5118,25 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C90" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D90" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D90" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5146,20 +5146,20 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C91" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C91" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D91" s="42" t="inlineStr">
@@ -5174,16 +5174,16 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46200</v>
+        <v>46193</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>170</v>
+        <v>215</v>
       </c>
       <c r="C92" s="40" t="inlineStr">
         <is>
@@ -5197,25 +5197,25 @@
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C93" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C93" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D93" s="42" t="inlineStr">
@@ -5225,30 +5225,30 @@
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="31" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B94" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C94" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D94" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>180</v>
+      </c>
+      <c r="C94" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D94" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
@@ -5258,7 +5258,7 @@
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
@@ -5267,7 +5267,7 @@
         <v>46200</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C95" s="41" t="inlineStr">
         <is>
@@ -5281,12 +5281,12 @@
       </c>
       <c r="E95" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -5294,30 +5294,114 @@
       <c r="A96" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B96" s="33" t="inlineStr"/>
-      <c r="C96" s="49" t="inlineStr">
+      <c r="B96" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="C96" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D96" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E96" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F96" s="30" t="inlineStr">
+        <is>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="15" customHeight="1">
+      <c r="A97" s="36" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B97" s="38" t="n">
+        <v>190</v>
+      </c>
+      <c r="C97" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D97" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E97" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F97" s="35" t="inlineStr">
+        <is>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="15" customHeight="1">
+      <c r="A98" s="31" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B98" s="33" t="inlineStr"/>
+      <c r="C98" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D96" s="54" t="inlineStr">
+      <c r="D98" s="44" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
-      <c r="E96" s="30" t="inlineStr">
+      <c r="E98" s="30" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="F96" s="30" t="inlineStr">
+      <c r="F98" s="30" t="inlineStr">
         <is>
           <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
+    <row r="99" ht="15" customHeight="1">
+      <c r="A99" s="36" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B99" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C99" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D99" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E99" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F99" s="35" t="inlineStr">
+        <is>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F96"/>
+  <autoFilter ref="A3:F99"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5332,7 +5416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5358,7 +5442,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 29, 2026  ·  08:04 UTC</t>
+          <t>Generated March 30, 2026  ·  10:45 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5429,10 +5513,10 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46115</v>
+        <v>46113</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="C5" s="41" t="inlineStr">
         <is>
@@ -5446,12 +5530,12 @@
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Shoe Bag”</t>
+          <t>Air Jordan 3 “Spring Flowers”</t>
         </is>
       </c>
     </row>
@@ -5460,26 +5544,26 @@
         <v>46115</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C6" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D6" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>230</v>
+      </c>
+      <c r="C6" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Good Intentions”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -5488,26 +5572,26 @@
         <v>46115</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C7" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D7" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>200</v>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Nike LeBron 23 “Shoe Bag”</t>
         </is>
       </c>
     </row>
@@ -5516,16 +5600,16 @@
         <v>46115</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>235</v>
+        <v>210</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D8" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
@@ -5535,16 +5619,16 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Nike LeBron 23 Elite “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46116</v>
+        <v>46115</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C9" s="41" t="inlineStr">
         <is>
@@ -5558,21 +5642,21 @@
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46121</v>
+        <v>46116</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
@@ -5586,12 +5670,12 @@
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -5619,7 +5703,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
         </is>
       </c>
     </row>
@@ -5647,16 +5731,16 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46122</v>
+        <v>46121</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>235</v>
+        <v>120</v>
       </c>
       <c r="C13" s="41" t="inlineStr">
         <is>
@@ -5675,7 +5759,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
         </is>
       </c>
     </row>
@@ -5709,10 +5793,10 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46123</v>
+        <v>46122</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>185</v>
+        <v>235</v>
       </c>
       <c r="C15" s="41" t="inlineStr">
         <is>
@@ -5726,38 +5810,40 @@
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B16" s="33" t="inlineStr"/>
+        <v>46123</v>
+      </c>
+      <c r="B16" s="33" t="n">
+        <v>185</v>
+      </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -5793,17 +5879,15 @@
       <c r="A18" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B18" s="33" t="n">
-        <v>190</v>
-      </c>
+      <c r="B18" s="33" t="inlineStr"/>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D18" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D18" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
@@ -5813,7 +5897,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
@@ -5822,7 +5906,7 @@
         <v>46125</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="C19" s="41" t="inlineStr">
         <is>
@@ -5841,16 +5925,16 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46130</v>
+        <v>46125</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -5869,16 +5953,16 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46135</v>
+        <v>46130</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C21" s="41" t="inlineStr">
         <is>
@@ -5892,21 +5976,21 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46136</v>
+        <v>46135</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
@@ -5920,30 +6004,30 @@
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C23" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D23" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
@@ -5953,7 +6037,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -6041,10 +6125,10 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>215</v>
+        <v>180</v>
       </c>
       <c r="C27" s="41" t="inlineStr">
         <is>
@@ -6058,12 +6142,12 @@
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -6095,10 +6179,10 @@
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46144</v>
+        <v>46142</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>195</v>
+        <v>215</v>
       </c>
       <c r="C29" s="41" t="inlineStr">
         <is>
@@ -6117,7 +6201,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -6126,7 +6210,7 @@
         <v>46144</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
@@ -6145,16 +6229,16 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C31" s="41" t="inlineStr">
         <is>
@@ -6168,21 +6252,21 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46150</v>
+        <v>46149</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -6201,7 +6285,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6294,7 @@
         <v>46150</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="C33" s="41" t="inlineStr">
         <is>
@@ -6229,35 +6313,35 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D34" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D34" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -6266,26 +6350,26 @@
         <v>46151</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C35" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D35" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D35" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -6294,26 +6378,26 @@
         <v>46151</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C36" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D36" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>200</v>
+      </c>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D36" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6322,35 +6406,35 @@
         <v>46151</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="C37" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D37" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -6369,16 +6453,16 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C39" s="41" t="inlineStr">
         <is>
@@ -6392,21 +6476,21 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46165</v>
+        <v>46158</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>205</v>
+        <v>145</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -6425,16 +6509,16 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C41" s="41" t="inlineStr">
         <is>
@@ -6448,12 +6532,12 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
@@ -6481,15 +6565,17 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B43" s="38" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="B43" s="38" t="n">
+        <v>240</v>
+      </c>
       <c r="C43" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6502,12 +6588,12 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -6515,9 +6601,7 @@
       <c r="A44" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B44" s="33" t="n">
-        <v>250</v>
-      </c>
+      <c r="B44" s="33" t="inlineStr"/>
       <c r="C44" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6530,20 +6614,22 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B45" s="38" t="inlineStr"/>
+        <v>46172</v>
+      </c>
+      <c r="B45" s="38" t="n">
+        <v>250</v>
+      </c>
       <c r="C45" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6556,22 +6642,20 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B46" s="33" t="n">
-        <v>355</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B46" s="33" t="inlineStr"/>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6589,41 +6673,41 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46186</v>
+        <v>46182</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>150</v>
+        <v>355</v>
       </c>
       <c r="C47" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D47" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D47" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B48" s="33" t="n">
         <v>150</v>
@@ -6633,9 +6717,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D48" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D48" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
@@ -6645,7 +6729,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -6654,7 +6738,7 @@
         <v>46193</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="C49" s="41" t="inlineStr">
         <is>
@@ -6668,21 +6752,21 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46200</v>
+        <v>46193</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>170</v>
+        <v>215</v>
       </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
@@ -6696,12 +6780,12 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -6745,7 +6829,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D52" s="54" t="inlineStr">
+      <c r="D52" s="44" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -6789,8 +6873,36 @@
         </is>
       </c>
     </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="A54" s="31" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B54" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D54" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E54" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F54" s="30" t="inlineStr">
+        <is>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F53"/>
+  <autoFilter ref="A3:F54"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-31 09:47 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -654,7 +654,7 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -685,7 +685,7 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated March 30, 2026  ·  10:45 UTC</t>
+          <t>Generated March 31, 2026  ·  09:47 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1624,11 +1624,11 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1740,7 +1740,7 @@
         <v>46115</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         <v>46151</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
         <v>46186</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
         <v>46112</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="41" t="inlineStr">
         <is>
@@ -1864,19 +1864,19 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring Flowers”</t>
+          <t>Nike LeBron 23 “Shoe Bag”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1887,7 +1887,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>155</v>
+        <v>200</v>
       </c>
       <c r="H14" s="43" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Shoe Bag”</t>
+          <t>Nike LeBron 23 Elite “Good Intentions”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1910,7 +1910,7 @@
         <v>46115</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E15" s="41" t="inlineStr">
         <is>
@@ -1921,18 +1921,18 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="H15" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="H15" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Good Intentions”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1944,7 +1944,7 @@
         <v>46115</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1955,11 +1955,11 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="H16" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>235</v>
+      </c>
+      <c r="H16" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D21" s="41" t="inlineStr">
         <is>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D22" s="49" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="E23" s="35" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" ht="10" customHeight="1"/>
@@ -2156,17 +2156,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>3/30 – 4/5</t>
+          <t>3/31 – 4/6</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D27" s="40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2177,17 +2177,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/6 – 4/12</t>
+          <t>4/7 – 4/13</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D28" s="41" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2198,17 +2198,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/13 – 4/19</t>
+          <t>4/14 – 4/20</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D29" s="40" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>5.8</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/20 – 4/26</t>
+          <t>4/21 – 4/27</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>4/27 – 5/3</t>
+          <t>4/28 – 5/4</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/4 – 5/10</t>
+          <t>5/5 – 5/11</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/11 – 5/17</t>
+          <t>5/12 – 5/18</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/18 – 5/24</t>
+          <t>5/19 – 5/25</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>5/25 – 5/31</t>
+          <t>5/26 – 6/1</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/1 – 6/7</t>
+          <t>6/2 – 6/8</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/8 – 6/14</t>
+          <t>6/9 – 6/15</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/15 – 6/21</t>
+          <t>6/16 – 6/22</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>6/22 – 6/28</t>
+          <t>6/23 – 6/29</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2516,7 +2516,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2574,7 +2574,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2626,7 +2626,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2634,7 +2634,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -2659,7 +2659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2685,7 +2685,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 30, 2026  ·  10:45 UTC</t>
+          <t>Generated March 31, 2026  ·  09:47 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2728,19 +2728,19 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C4" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D4" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C4" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D4" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
@@ -2750,20 +2750,20 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Future “Galaxy Aura”</t>
+          <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C5" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>115</v>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D5" s="42" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>NOTE Manchester x Nike SB Dunk Low</t>
+          <t>Nike Giannis Freak 7 “Light Aqua”</t>
         </is>
       </c>
     </row>
@@ -2787,11 +2787,11 @@
         <v>46113</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C6" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C6" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D6" s="43" t="inlineStr">
@@ -2801,12 +2801,12 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring Flowers”</t>
+          <t>Nike Sabrina 3 “What The”</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
         <v>46113</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -2829,12 +2829,12 @@
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Giannis Freak 7 “Light Aqua”</t>
+          <t>Jordan Luka 5 “Black White”</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2843,7 @@
         <v>46113</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="C8" s="49" t="inlineStr">
         <is>
@@ -2857,12 +2857,12 @@
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Sabrina 3 “What The”</t>
+          <t>Jordan Tatum 4 “Offseason”</t>
         </is>
       </c>
     </row>
@@ -2871,35 +2871,35 @@
         <v>46113</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="C9" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Jordan Luka 5 “Black White”</t>
+          <t>Nike V5 RNR “Jackie Robinson Day”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="C10" s="49" t="inlineStr">
         <is>
@@ -2913,12 +2913,12 @@
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Jordan Tatum 4 “Offseason”</t>
+          <t>Nike Mind 001 “Sail”</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Sail”</t>
+          <t>Nike Mind 001 “Team Red”</t>
         </is>
       </c>
     </row>
@@ -2974,35 +2974,35 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Team Red”</t>
+          <t>Nike Mind 001 “Geode Teal”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C13" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D13" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Geode Teal”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -3011,26 +3011,26 @@
         <v>46115</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C14" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D14" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>225</v>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D14" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Fragment x Nike Air Liquid Max “Black”</t>
         </is>
       </c>
     </row>
@@ -3039,16 +3039,16 @@
         <v>46115</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>225</v>
-      </c>
-      <c r="C15" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D15" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max “Black”</t>
+          <t>Nike LeBron 23 “Shoe Bag”</t>
         </is>
       </c>
     </row>
@@ -3067,16 +3067,16 @@
         <v>46115</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D16" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Shoe Bag”</t>
+          <t>Nike LeBron 23 Elite “Good Intentions”</t>
         </is>
       </c>
     </row>
@@ -3095,26 +3095,26 @@
         <v>46115</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C17" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D17" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C17" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D17" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Good Intentions”</t>
+          <t>Converse SHAI 001 “Camo”</t>
         </is>
       </c>
     </row>
@@ -3123,11 +3123,11 @@
         <v>46115</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C18" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>225</v>
+      </c>
+      <c r="C18" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D18" s="43" t="inlineStr">
@@ -3137,12 +3137,12 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 “Camo”</t>
+          <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
     </row>
@@ -3151,11 +3151,11 @@
         <v>46115</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>225</v>
-      </c>
-      <c r="C19" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C19" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
@@ -3170,20 +3170,20 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>235</v>
-      </c>
-      <c r="C20" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C20" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D20" s="43" t="inlineStr">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
@@ -3207,11 +3207,11 @@
         <v>46116</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C21" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C21" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D21" s="42" t="inlineStr">
@@ -3221,25 +3221,25 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46116</v>
+        <v>46120</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C22" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>220</v>
+      </c>
+      <c r="C22" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D22" s="43" t="inlineStr">
@@ -3249,12 +3249,12 @@
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Melitta Baumeister x Nike Pegasus Premium</t>
         </is>
       </c>
     </row>
@@ -3263,7 +3263,7 @@
         <v>46120</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>220</v>
+        <v>260</v>
       </c>
       <c r="C23" s="54" t="inlineStr">
         <is>
@@ -3282,20 +3282,20 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Pegasus Premium</t>
+          <t>Melitta Baumeister x Nike Vomero Premium</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>260</v>
-      </c>
-      <c r="C24" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D24" s="43" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Vomero Premium</t>
+          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
         </is>
       </c>
     </row>
@@ -3366,16 +3366,16 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C27" s="41" t="inlineStr">
         <is>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -3403,11 +3403,11 @@
         <v>46122</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C28" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C28" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D28" s="43" t="inlineStr">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
@@ -3431,11 +3431,11 @@
         <v>46122</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C29" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C29" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D29" s="42" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -3459,11 +3459,11 @@
         <v>46122</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>235</v>
-      </c>
-      <c r="C30" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C30" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D30" s="43" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
@@ -3487,11 +3487,11 @@
         <v>46122</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C31" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>200</v>
+      </c>
+      <c r="C31" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D31" s="42" t="inlineStr">
@@ -3501,12 +3501,12 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
         </is>
       </c>
     </row>
@@ -3596,14 +3596,14 @@
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46125</v>
+        <v>46124</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C35" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C35" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D35" s="42" t="inlineStr">
@@ -3613,12 +3613,12 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>adidas Harden Vol. 10 “Marathon”</t>
         </is>
       </c>
     </row>
@@ -3626,15 +3626,17 @@
       <c r="A36" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B36" s="33" t="inlineStr"/>
+      <c r="B36" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D36" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
@@ -3644,7 +3646,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3652,17 +3654,15 @@
       <c r="A37" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B37" s="38" t="n">
-        <v>190</v>
-      </c>
+      <c r="B37" s="38" t="inlineStr"/>
       <c r="C37" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D37" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
         <v>46125</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -3700,20 +3700,20 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46128</v>
+        <v>46125</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C39" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C39" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D39" s="42" t="inlineStr">
@@ -3723,25 +3723,25 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46129</v>
+        <v>46125</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C40" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D40" s="43" t="inlineStr">
@@ -3756,48 +3756,48 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46130</v>
+        <v>46128</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C41" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D41" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C41" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D41" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46130</v>
+        <v>46129</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C42" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C42" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D42" s="43" t="inlineStr">
@@ -3812,25 +3812,25 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46133</v>
+        <v>46130</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>145</v>
+        <v>210</v>
       </c>
       <c r="C43" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D43" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D43" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E43" s="35" t="inlineStr">
@@ -3840,16 +3840,16 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46135</v>
+        <v>46130</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
@@ -3863,30 +3863,30 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46136</v>
+        <v>46133</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C45" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D45" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>145</v>
+      </c>
+      <c r="C45" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D45" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
@@ -3896,15 +3896,17 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B46" s="33" t="inlineStr"/>
+        <v>46135</v>
+      </c>
+      <c r="B46" s="33" t="n">
+        <v>220</v>
+      </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3917,40 +3919,40 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C47" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D47" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D47" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3961,7 @@
         <v>46137</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
@@ -3978,7 +3980,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -3987,7 +3989,7 @@
         <v>46137</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C49" s="41" t="inlineStr">
         <is>
@@ -4001,20 +4003,22 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B50" s="33" t="inlineStr"/>
+        <v>46137</v>
+      </c>
+      <c r="B50" s="33" t="n">
+        <v>180</v>
+      </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4027,22 +4031,20 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B51" s="38" t="n">
-        <v>215</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B51" s="38" t="inlineStr"/>
       <c r="C51" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4055,12 +4057,12 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -4068,12 +4070,10 @@
       <c r="A52" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B52" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C52" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B52" s="33" t="inlineStr"/>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D52" s="43" t="inlineStr">
@@ -4083,12 +4083,12 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -4097,11 +4097,11 @@
         <v>46142</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C53" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C53" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D53" s="42" t="inlineStr">
@@ -4111,21 +4111,21 @@
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>135</v>
+        <v>95</v>
       </c>
       <c r="C54" s="49" t="inlineStr">
         <is>
@@ -4144,16 +4144,16 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C55" s="54" t="inlineStr">
         <is>
@@ -4172,20 +4172,20 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>195</v>
-      </c>
-      <c r="C56" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C56" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D56" s="43" t="inlineStr">
@@ -4195,25 +4195,25 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C57" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C57" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D57" s="42" t="inlineStr">
@@ -4223,12 +4223,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
@@ -4237,11 +4237,11 @@
         <v>46144</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C58" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>195</v>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D58" s="43" t="inlineStr">
@@ -4251,21 +4251,21 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C59" s="41" t="inlineStr">
         <is>
@@ -4279,25 +4279,25 @@
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46150</v>
+        <v>46144</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C60" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C60" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
@@ -4312,16 +4312,16 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46150</v>
+        <v>46149</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="C61" s="41" t="inlineStr">
         <is>
@@ -4340,7 +4340,7 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
@@ -4349,11 +4349,11 @@
         <v>46150</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C62" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D62" s="43" t="inlineStr">
@@ -4368,48 +4368,48 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C63" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D63" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>210</v>
+      </c>
+      <c r="C63" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D63" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C64" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C64" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D64" s="43" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -4433,16 +4433,16 @@
         <v>46151</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C65" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D65" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>155</v>
+      </c>
+      <c r="C65" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D65" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E65" s="35" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
         <v>46151</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C66" s="40" t="inlineStr">
         <is>
@@ -4480,44 +4480,44 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C67" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D67" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C67" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D67" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E67" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="C68" s="40" t="inlineStr">
         <is>
@@ -4536,20 +4536,20 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="36" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C69" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C69" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D69" s="42" t="inlineStr">
@@ -4559,25 +4559,25 @@
       </c>
       <c r="E69" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C70" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>150</v>
+      </c>
+      <c r="C70" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D70" s="43" t="inlineStr">
@@ -4587,25 +4587,25 @@
       </c>
       <c r="E70" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46164</v>
+        <v>46158</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C71" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>145</v>
+      </c>
+      <c r="C71" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D71" s="42" t="inlineStr">
@@ -4615,25 +4615,25 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46165</v>
+        <v>46158</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C72" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C72" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D72" s="43" t="inlineStr">
@@ -4643,25 +4643,25 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46171</v>
+        <v>46164</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C73" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C73" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
@@ -4676,20 +4676,20 @@
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C74" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C74" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D74" s="43" t="inlineStr">
@@ -4699,12 +4699,12 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
@@ -4732,18 +4732,20 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B76" s="33" t="inlineStr"/>
-      <c r="C76" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46171</v>
+      </c>
+      <c r="B76" s="33" t="n">
+        <v>155</v>
+      </c>
+      <c r="C76" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D76" s="43" t="inlineStr">
@@ -4753,21 +4755,21 @@
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="B77" s="38" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C77" s="41" t="inlineStr">
         <is>
@@ -4786,7 +4788,7 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -4795,9 +4797,9 @@
         <v>46172</v>
       </c>
       <c r="B78" s="33" t="inlineStr"/>
-      <c r="C78" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="C78" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D78" s="43" t="inlineStr">
@@ -4807,25 +4809,25 @@
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C79" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C79" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4840,20 +4842,18 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B80" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C80" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46172</v>
+      </c>
+      <c r="B80" s="33" t="inlineStr"/>
+      <c r="C80" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D80" s="43" t="inlineStr">
@@ -4863,23 +4863,25 @@
       </c>
       <c r="E80" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B81" s="38" t="inlineStr"/>
-      <c r="C81" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46173</v>
+      </c>
+      <c r="B81" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C81" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D81" s="42" t="inlineStr">
@@ -4889,25 +4891,25 @@
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="31" t="n">
-        <v>46182</v>
+        <v>46177</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="C82" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C82" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D82" s="43" t="inlineStr">
@@ -4917,25 +4919,23 @@
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="36" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B83" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C83" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B83" s="38" t="inlineStr"/>
+      <c r="C83" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D83" s="42" t="inlineStr">
@@ -4945,25 +4945,25 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C84" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>355</v>
+      </c>
+      <c r="C84" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D84" s="43" t="inlineStr">
@@ -4973,30 +4973,30 @@
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="36" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C85" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D85" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D85" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E85" s="35" t="inlineStr">
@@ -5006,25 +5006,25 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C86" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D86" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>170</v>
+      </c>
+      <c r="C86" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D86" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E86" s="30" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -5050,9 +5050,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D87" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D87" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -5071,16 +5071,16 @@
         <v>46186</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C88" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D88" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C88" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D88" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
@@ -5090,16 +5090,16 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="C89" s="54" t="inlineStr">
         <is>
@@ -5118,25 +5118,25 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="C90" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D90" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D90" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5146,20 +5146,20 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C91" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C91" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D91" s="42" t="inlineStr">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
@@ -5183,7 +5183,7 @@
         <v>46193</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="C92" s="40" t="inlineStr">
         <is>
@@ -5197,25 +5197,25 @@
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C93" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C93" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D93" s="42" t="inlineStr">
@@ -5225,30 +5225,30 @@
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="31" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B94" s="33" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C94" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D94" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D94" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
@@ -5258,20 +5258,20 @@
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="36" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C95" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C95" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D95" s="42" t="inlineStr">
@@ -5281,30 +5281,30 @@
       </c>
       <c r="E95" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="A96" s="31" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C96" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D96" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>180</v>
+      </c>
+      <c r="C96" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D96" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
@@ -5323,7 +5323,7 @@
         <v>46200</v>
       </c>
       <c r="B97" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C97" s="41" t="inlineStr">
         <is>
@@ -5337,12 +5337,12 @@
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -5350,25 +5350,27 @@
       <c r="A98" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B98" s="33" t="inlineStr"/>
-      <c r="C98" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D98" s="44" t="inlineStr">
+      <c r="B98" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="C98" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D98" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
       <c r="E98" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -5377,31 +5379,85 @@
         <v>46200</v>
       </c>
       <c r="B99" s="38" t="n">
+        <v>190</v>
+      </c>
+      <c r="C99" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D99" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E99" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F99" s="35" t="inlineStr">
+        <is>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15" customHeight="1">
+      <c r="A100" s="31" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B100" s="33" t="inlineStr"/>
+      <c r="C100" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D100" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E100" s="30" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F100" s="30" t="inlineStr">
+        <is>
+          <t>Air Jordan 7 “Miro” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1">
+      <c r="A101" s="36" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B101" s="38" t="n">
         <v>170</v>
       </c>
-      <c r="C99" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D99" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E99" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F99" s="35" t="inlineStr">
+      <c r="C101" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D101" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E101" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F101" s="35" t="inlineStr">
         <is>
           <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F99"/>
+  <autoFilter ref="A3:F101"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5442,7 +5498,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
-          <t>Generated March 30, 2026  ·  10:45 UTC</t>
+          <t>Generated March 31, 2026  ·  09:47 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5513,19 +5569,19 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C5" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D5" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D5" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -5535,7 +5591,7 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring Flowers”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
@@ -5544,26 +5600,26 @@
         <v>46115</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C6" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D6" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>200</v>
+      </c>
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D6" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Nike LeBron 23 “Shoe Bag”</t>
         </is>
       </c>
     </row>
@@ -5572,16 +5628,16 @@
         <v>46115</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C7" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D7" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
@@ -5591,7 +5647,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Shoe Bag”</t>
+          <t>Nike LeBron 23 Elite “Good Intentions”</t>
         </is>
       </c>
     </row>
@@ -5600,16 +5656,16 @@
         <v>46115</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>210</v>
+        <v>235</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
@@ -5619,16 +5675,16 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Good Intentions”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="C9" s="41" t="inlineStr">
         <is>
@@ -5642,21 +5698,21 @@
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46116</v>
+        <v>46121</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>205</v>
+        <v>120</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
@@ -5670,12 +5726,12 @@
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5759,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
         </is>
       </c>
     </row>
@@ -5731,16 +5787,16 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C13" s="41" t="inlineStr">
         <is>
@@ -5759,7 +5815,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -5768,7 +5824,7 @@
         <v>46122</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
@@ -5787,16 +5843,16 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>235</v>
+        <v>185</v>
       </c>
       <c r="C15" s="41" t="inlineStr">
         <is>
@@ -5810,21 +5866,21 @@
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
@@ -5838,12 +5894,12 @@
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5851,17 +5907,15 @@
       <c r="A17" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B17" s="38" t="n">
-        <v>190</v>
-      </c>
+      <c r="B17" s="38" t="inlineStr"/>
       <c r="C17" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
@@ -5871,7 +5925,7 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
     </row>
@@ -5879,15 +5933,17 @@
       <c r="A18" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B18" s="33" t="inlineStr"/>
+      <c r="B18" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D18" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D18" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
@@ -5897,7 +5953,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5962,7 @@
         <v>46125</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C19" s="41" t="inlineStr">
         <is>
@@ -5925,7 +5981,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6081,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="55" t="inlineStr">
+      <c r="D23" s="44" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -6045,7 +6101,9 @@
       <c r="A24" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B24" s="33" t="inlineStr"/>
+      <c r="B24" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6058,12 +6116,12 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6130,7 @@
         <v>46137</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C25" s="41" t="inlineStr">
         <is>
@@ -6091,7 +6149,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6158,7 @@
         <v>46137</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
@@ -6114,12 +6172,12 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -6127,9 +6185,7 @@
       <c r="A27" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B27" s="38" t="n">
-        <v>180</v>
-      </c>
+      <c r="B27" s="38" t="inlineStr"/>
       <c r="C27" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6147,7 +6203,7 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6469,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="55" t="inlineStr">
+      <c r="D37" s="44" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -6829,7 +6885,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D52" s="44" t="inlineStr">
+      <c r="D52" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-03 08:37 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -691,16 +691,16 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -823,12 +823,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Charts'!$A$2:$A$5</f>
+              <f>'Charts'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$B$2:$B$5</f>
+              <f>'Charts'!$B$2:$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1596,7 +1596,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 02, 2026  ·  09:42 UTC</t>
+          <t>Generated April 03, 2026  ·  08:37 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1636,11 +1636,11 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1649,7 +1649,7 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$179</t>
+          <t>$183</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1752,7 +1752,7 @@
         <v>46115</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
         <v>46151</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         <v>46186</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1854,7 +1854,7 @@
         <v>46115</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="41" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         <v>46115</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
         <v>46115</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="41" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
         <v>46121</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G22" s="50" t="inlineStr">
         <is>
@@ -2101,21 +2101,13 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="47" t="inlineStr">
-        <is>
-          <t>Converse</t>
-        </is>
-      </c>
-      <c r="B23" s="35" t="n">
-        <v>1</v>
-      </c>
       <c r="D23" s="51" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
       <c r="E23" s="35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G23" s="52" t="inlineStr">
         <is>
@@ -2176,17 +2168,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/2 – 4/8</t>
+          <t>4/3 – 4/9</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D27" s="40" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2197,17 +2189,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/9 – 4/15</t>
+          <t>4/10 – 4/16</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D28" s="41" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2218,17 +2210,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/16 – 4/22</t>
+          <t>4/17 – 4/23</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
         <v>5</v>
       </c>
       <c r="D29" s="40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2239,17 +2231,17 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/23 – 4/29</t>
+          <t>4/24 – 4/30</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D30" s="41" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2260,14 +2252,14 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>4/30 – 5/6</t>
+          <t>5/1 – 5/7</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D31" s="40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>5.5</v>
@@ -2281,14 +2273,14 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/7 – 5/13</t>
+          <t>5/8 – 5/14</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D32" s="41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E32" s="35" t="n">
         <v>6.9</v>
@@ -2302,7 +2294,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/14 – 5/20</t>
+          <t>5/15 – 5/21</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2323,17 +2315,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/21 – 5/27</t>
+          <t>5/22 – 5/28</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D34" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2344,17 +2336,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>5/28 – 6/3</t>
+          <t>5/29 – 6/4</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D35" s="40" t="n">
         <v>4</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2365,17 +2357,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/4 – 6/10</t>
+          <t>6/5 – 6/11</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" s="41" t="n">
         <v>2</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2386,7 +2378,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/11 – 6/17</t>
+          <t>6/12 – 6/18</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2407,7 +2399,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/18 – 6/24</t>
+          <t>6/19 – 6/25</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2428,7 +2420,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>6/25 – 7/1</t>
+          <t>6/26 – 7/2</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2536,7 +2528,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2552,7 +2544,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2560,7 +2552,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -2594,7 +2586,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -2612,7 +2604,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2628,25 +2620,17 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Converse</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2687,7 +2671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2713,7 +2697,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="54" t="inlineStr">
         <is>
-          <t>Generated April 02, 2026  ·  09:42 UTC</t>
+          <t>Generated April 03, 2026  ·  08:37 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2756,47 +2740,47 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C4" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D4" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C4" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D4" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Sail”</t>
+          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C5" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D5" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D5" s="42" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -2806,25 +2790,25 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Team Red”</t>
+          <t>Nike LeBron 23 Elite “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C6" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D6" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D6" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
@@ -2834,35 +2818,35 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Geode Teal”</t>
+          <t>Nike Moon Shoe “Soft Pearl”</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="36" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C7" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D7" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>225</v>
+      </c>
+      <c r="C7" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 “Camo”</t>
+          <t>Fragment x Nike Air Liquid Max “Black”</t>
         </is>
       </c>
     </row>
@@ -2871,26 +2855,26 @@
         <v>46115</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C8" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D8" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>200</v>
+      </c>
+      <c r="C8" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
+          <t>Nike LeBron 23 “Shoe Bag”</t>
         </is>
       </c>
     </row>
@@ -2899,16 +2883,16 @@
         <v>46115</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C9" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>225</v>
+      </c>
+      <c r="C9" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
@@ -2918,7 +2902,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Good Intentions”</t>
+          <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
     </row>
@@ -2927,16 +2911,16 @@
         <v>46115</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>105</v>
-      </c>
-      <c r="C10" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D10" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>235</v>
+      </c>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -2946,25 +2930,25 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Moon Shoe “Soft Pearl”</t>
+          <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>225</v>
-      </c>
-      <c r="C11" s="55" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C11" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D11" s="42" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -2974,20 +2958,20 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max “Black”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C12" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>230</v>
+      </c>
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D12" s="43" t="inlineStr">
@@ -3002,18 +2986,18 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Shoe Bag”</t>
+          <t>Melitta Baumeister x Nike Pegasus Premium</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>225</v>
-      </c>
-      <c r="C13" s="55" t="inlineStr">
+        <v>240</v>
+      </c>
+      <c r="C13" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3030,16 +3014,16 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Fragment x Nike Air Liquid Max</t>
+          <t>Melitta Baumeister x Nike Vomero Premium</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46115</v>
+        <v>46121</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>235</v>
+        <v>120</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
@@ -3058,20 +3042,20 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Good Intentions”</t>
+          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46116</v>
+        <v>46121</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C15" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D15" s="44" t="inlineStr">
@@ -3086,20 +3070,20 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C16" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D16" s="43" t="inlineStr">
@@ -3114,20 +3098,20 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Pegasus Premium</t>
+          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46120</v>
+        <v>46122</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C17" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C17" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D17" s="44" t="inlineStr">
@@ -3142,48 +3126,48 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Vomero Premium</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C18" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D18" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C18" s="57" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D18" s="58" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C19" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C19" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D19" s="44" t="inlineStr">
@@ -3198,16 +3182,16 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>120</v>
+        <v>235</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -3226,7 +3210,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -3235,11 +3219,11 @@
         <v>46122</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C21" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C21" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D21" s="44" t="inlineStr">
@@ -3254,25 +3238,25 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D22" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -3282,44 +3266,44 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C23" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D23" s="57" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+        <v>130</v>
+      </c>
+      <c r="C23" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>135</v>
+        <v>170</v>
       </c>
       <c r="C24" s="49" t="inlineStr">
         <is>
@@ -3338,20 +3322,20 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C25" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>185</v>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D25" s="44" t="inlineStr">
@@ -3361,12 +3345,12 @@
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -3375,11 +3359,11 @@
         <v>46123</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>185</v>
-      </c>
-      <c r="C26" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C26" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D26" s="43" t="inlineStr">
@@ -3389,86 +3373,84 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C27" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D27" s="42" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C27" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D27" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C28" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D28" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C28" s="57" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D28" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>adidas Harden Vol. 10 “Marathon”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46123</v>
-      </c>
-      <c r="B29" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C29" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D29" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B29" s="38" t="inlineStr"/>
+      <c r="C29" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
@@ -3478,20 +3460,20 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C30" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C30" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D30" s="43" t="inlineStr">
@@ -3501,25 +3483,25 @@
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C31" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C31" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D31" s="44" t="inlineStr">
@@ -3529,25 +3511,25 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C32" s="58" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>220</v>
+      </c>
+      <c r="C32" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D32" s="43" t="inlineStr">
@@ -3557,28 +3539,30 @@
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Marathon”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B33" s="38" t="inlineStr"/>
-      <c r="C33" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D33" s="42" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>46126</v>
+      </c>
+      <c r="B33" s="38" t="n">
+        <v>120</v>
+      </c>
+      <c r="C33" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D33" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
@@ -3588,16 +3572,16 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -3616,25 +3600,25 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46125</v>
+        <v>46127</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C35" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D35" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>100</v>
+      </c>
+      <c r="C35" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D35" s="42" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
@@ -3644,20 +3628,20 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike V5 RNR “Jackie Robinson Day”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46125</v>
+        <v>46128</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C36" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C36" s="57" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D36" s="43" t="inlineStr">
@@ -3667,23 +3651,23 @@
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46126</v>
+        <v>46129</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C37" s="55" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C37" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3700,25 +3684,25 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46126</v>
+        <v>46130</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C38" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D38" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C38" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D38" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
@@ -3728,25 +3712,25 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46127</v>
+        <v>46130</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>100</v>
-      </c>
-      <c r="C39" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D39" s="42" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>240</v>
+      </c>
+      <c r="C39" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D39" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
@@ -3756,20 +3740,20 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike V5 RNR “Jackie Robinson Day”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46128</v>
+        <v>46133</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C40" s="58" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>145</v>
+      </c>
+      <c r="C40" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D40" s="43" t="inlineStr">
@@ -3779,25 +3763,25 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46129</v>
+        <v>46135</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C41" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C41" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D41" s="44" t="inlineStr">
@@ -3807,28 +3791,28 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46130</v>
+        <v>46136</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C42" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D42" s="56" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C42" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D42" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3840,16 +3824,16 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46130</v>
+        <v>46136</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C43" s="41" t="inlineStr">
         <is>
@@ -3868,20 +3852,20 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46133</v>
+        <v>46137</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C44" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>180</v>
+      </c>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D44" s="43" t="inlineStr">
@@ -3896,17 +3880,15 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46135</v>
-      </c>
-      <c r="B45" s="38" t="n">
-        <v>220</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B45" s="38" t="inlineStr"/>
       <c r="C45" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3919,49 +3901,49 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D46" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C47" s="41" t="inlineStr">
         <is>
@@ -3975,22 +3957,20 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B48" s="33" t="n">
-        <v>180</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B48" s="33" t="inlineStr"/>
       <c r="C48" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4003,20 +3983,22 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B49" s="38" t="inlineStr"/>
+        <v>46142</v>
+      </c>
+      <c r="B49" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C49" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4029,21 +4011,21 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
@@ -4062,20 +4044,20 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C51" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>95</v>
+      </c>
+      <c r="C51" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="44" t="inlineStr">
@@ -4085,12 +4067,12 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -4099,11 +4081,11 @@
         <v>46142</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C52" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C52" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D52" s="43" t="inlineStr">
@@ -4113,23 +4095,25 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B53" s="38" t="inlineStr"/>
-      <c r="C53" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46143</v>
+      </c>
+      <c r="B53" s="38" t="n">
+        <v>135</v>
+      </c>
+      <c r="C53" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D53" s="44" t="inlineStr">
@@ -4139,25 +4123,25 @@
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C54" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C54" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D54" s="43" t="inlineStr">
@@ -4167,25 +4151,25 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46142</v>
+        <v>46144</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C55" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>195</v>
+      </c>
+      <c r="C55" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D55" s="44" t="inlineStr">
@@ -4195,25 +4179,25 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46142</v>
+        <v>46144</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C56" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D56" s="43" t="inlineStr">
@@ -4223,23 +4207,23 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C57" s="55" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C57" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4256,20 +4240,20 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46143</v>
+        <v>46149</v>
       </c>
       <c r="B58" s="33" t="n">
         <v>190</v>
       </c>
-      <c r="C58" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D58" s="43" t="inlineStr">
@@ -4284,16 +4268,16 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46144</v>
+        <v>46150</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C59" s="41" t="inlineStr">
         <is>
@@ -4307,21 +4291,21 @@
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46144</v>
+        <v>46150</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
@@ -4335,23 +4319,23 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46144</v>
+        <v>46150</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C61" s="55" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C61" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4368,44 +4352,44 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46149</v>
+        <v>46151</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>190</v>
+        <v>230</v>
       </c>
       <c r="C62" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D62" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D62" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C63" s="41" t="inlineStr">
         <is>
@@ -4424,48 +4408,48 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C64" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D64" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C64" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D64" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C65" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>200</v>
+      </c>
+      <c r="C65" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D65" s="44" t="inlineStr">
@@ -4480,44 +4464,44 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C66" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D66" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>170</v>
+      </c>
+      <c r="C66" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D66" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="C67" s="41" t="inlineStr">
         <is>
@@ -4536,25 +4520,25 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46151</v>
+        <v>46158</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C68" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D68" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>145</v>
+      </c>
+      <c r="C68" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D68" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -4564,20 +4548,20 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="36" t="n">
-        <v>46151</v>
+        <v>46158</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C69" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C69" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D69" s="44" t="inlineStr">
@@ -4587,18 +4571,18 @@
       </c>
       <c r="E69" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46157</v>
+        <v>46164</v>
       </c>
       <c r="B70" s="33" t="n">
         <v>170</v>
@@ -4620,16 +4604,16 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46157</v>
+        <v>46165</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C71" s="41" t="inlineStr">
         <is>
@@ -4643,21 +4627,21 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46158</v>
+        <v>46165</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="C72" s="40" t="inlineStr">
         <is>
@@ -4676,20 +4660,20 @@
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46158</v>
+        <v>46168</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C73" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>235</v>
+      </c>
+      <c r="C73" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D73" s="44" t="inlineStr">
@@ -4699,25 +4683,25 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46164</v>
+        <v>46171</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C74" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C74" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D74" s="43" t="inlineStr">
@@ -4732,18 +4716,18 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Hyper Pink”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46164</v>
+        <v>46171</v>
       </c>
       <c r="B75" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C75" s="55" t="inlineStr">
+        <v>155</v>
+      </c>
+      <c r="C75" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4760,16 +4744,16 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46165</v>
+        <v>46171</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="C76" s="40" t="inlineStr">
         <is>
@@ -4783,25 +4767,23 @@
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46165</v>
-      </c>
-      <c r="B77" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C77" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46172</v>
+      </c>
+      <c r="B77" s="38" t="inlineStr"/>
+      <c r="C77" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D77" s="44" t="inlineStr">
@@ -4811,21 +4793,21 @@
       </c>
       <c r="E77" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46168</v>
+        <v>46172</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="C78" s="40" t="inlineStr">
         <is>
@@ -4844,17 +4826,15 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46171</v>
-      </c>
-      <c r="B79" s="38" t="n">
-        <v>240</v>
-      </c>
+        <v>46172</v>
+      </c>
+      <c r="B79" s="38" t="inlineStr"/>
       <c r="C79" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4867,21 +4847,21 @@
       </c>
       <c r="E79" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46171</v>
+        <v>46173</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="C80" s="49" t="inlineStr">
         <is>
@@ -4900,20 +4880,20 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46171</v>
+        <v>46177</v>
       </c>
       <c r="B81" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C81" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C81" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D81" s="44" t="inlineStr">
@@ -4928,18 +4908,18 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="31" t="n">
-        <v>46172</v>
+        <v>46179</v>
       </c>
       <c r="B82" s="33" t="inlineStr"/>
-      <c r="C82" s="58" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="C82" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D82" s="43" t="inlineStr">
@@ -4949,21 +4929,21 @@
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="36" t="n">
-        <v>46172</v>
+        <v>46182</v>
       </c>
       <c r="B83" s="38" t="n">
-        <v>250</v>
+        <v>355</v>
       </c>
       <c r="C83" s="41" t="inlineStr">
         <is>
@@ -4977,23 +4957,25 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B84" s="33" t="inlineStr"/>
-      <c r="C84" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46185</v>
+      </c>
+      <c r="B84" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C84" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D84" s="43" t="inlineStr">
@@ -5003,23 +4985,23 @@
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="36" t="n">
-        <v>46173</v>
+        <v>46185</v>
       </c>
       <c r="B85" s="38" t="n">
         <v>170</v>
       </c>
-      <c r="C85" s="55" t="inlineStr">
+      <c r="C85" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5036,25 +5018,25 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46177</v>
+        <v>46186</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="C86" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D86" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D86" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E86" s="30" t="inlineStr">
@@ -5064,42 +5046,44 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B87" s="38" t="inlineStr"/>
+        <v>46186</v>
+      </c>
+      <c r="B87" s="38" t="n">
+        <v>150</v>
+      </c>
       <c r="C87" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D87" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D87" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46182</v>
+        <v>46186</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>355</v>
+        <v>205</v>
       </c>
       <c r="C88" s="40" t="inlineStr">
         <is>
@@ -5118,18 +5102,18 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C89" s="55" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C89" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5146,16 +5130,16 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="C90" s="49" t="inlineStr">
         <is>
@@ -5174,18 +5158,18 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C91" s="55" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C91" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5202,25 +5186,25 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C92" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D92" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C92" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D92" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E92" s="30" t="inlineStr">
@@ -5230,74 +5214,74 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="C93" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D93" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D93" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="31" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B94" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C94" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D94" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C94" s="49" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D94" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="36" t="n">
-        <v>46186</v>
+        <v>46199</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C95" s="55" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="C95" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5314,16 +5298,16 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="A96" s="31" t="n">
-        <v>46192</v>
+        <v>46199</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="C96" s="49" t="inlineStr">
         <is>
@@ -5342,16 +5326,16 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="36" t="n">
-        <v>46193</v>
+        <v>46200</v>
       </c>
       <c r="B97" s="38" t="n">
-        <v>150</v>
+        <v>185</v>
       </c>
       <c r="C97" s="41" t="inlineStr">
         <is>
@@ -5365,22 +5349,20 @@
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" s="31" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B98" s="33" t="n">
-        <v>215</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B98" s="33" t="inlineStr"/>
       <c r="C98" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5398,20 +5380,20 @@
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="A99" s="36" t="n">
-        <v>46193</v>
+        <v>46200</v>
       </c>
       <c r="B99" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C99" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C99" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D99" s="42" t="inlineStr">
@@ -5426,48 +5408,46 @@
       </c>
       <c r="F99" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="31" t="n">
-        <v>46199</v>
-      </c>
-      <c r="B100" s="33" t="n">
-        <v>180</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B100" s="33" t="inlineStr"/>
       <c r="C100" s="49" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D100" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D100" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E100" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="36" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="B101" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C101" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C101" s="41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D101" s="44" t="inlineStr">
@@ -5482,7 +5462,7 @@
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -5491,7 +5471,7 @@
         <v>46200</v>
       </c>
       <c r="B102" s="33" t="n">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="C102" s="40" t="inlineStr">
         <is>
@@ -5505,181 +5485,45 @@
       </c>
       <c r="E102" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1">
       <c r="A103" s="36" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B103" s="38" t="inlineStr"/>
+        <v>46203</v>
+      </c>
+      <c r="B103" s="38" t="n">
+        <v>135</v>
+      </c>
       <c r="C103" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D103" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D103" s="42" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E103" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F103" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="15" customHeight="1">
-      <c r="A104" s="31" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B104" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C104" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D104" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="E104" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F104" s="30" t="inlineStr">
-        <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="15" customHeight="1">
-      <c r="A105" s="36" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B105" s="38" t="inlineStr"/>
-      <c r="C105" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D105" s="42" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="E105" s="35" t="inlineStr">
-        <is>
-          <t>Jordan</t>
-        </is>
-      </c>
-      <c r="F105" s="35" t="inlineStr">
-        <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="15" customHeight="1">
-      <c r="A106" s="31" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B106" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C106" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D106" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E106" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F106" s="30" t="inlineStr">
-        <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="15" customHeight="1">
-      <c r="A107" s="36" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B107" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C107" s="41" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D107" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E107" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F107" s="35" t="inlineStr">
-        <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="15" customHeight="1">
-      <c r="A108" s="31" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B108" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C108" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D108" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="E108" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F108" s="30" t="inlineStr">
-        <is>
           <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F108"/>
+  <autoFilter ref="A3:F103"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5720,7 +5564,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="54" t="inlineStr">
         <is>
-          <t>Generated April 02, 2026  ·  09:42 UTC</t>
+          <t>Generated April 03, 2026  ·  08:37 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5962,7 +5806,7 @@
         <v>46122</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C11" s="41" t="inlineStr">
         <is>
@@ -5981,7 +5825,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5834,7 @@
         <v>46122</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
@@ -6009,7 +5853,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -6018,26 +5862,26 @@
         <v>46123</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="C13" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="44" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -6046,14 +5890,14 @@
         <v>46123</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="56" t="inlineStr">
+      <c r="D14" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -6065,7 +5909,7 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
@@ -6074,26 +5918,26 @@
         <v>46123</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C15" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="42" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D15" s="44" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -6107,7 +5951,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="56" t="inlineStr">
+      <c r="D16" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -6461,9 +6305,7 @@
       <c r="A29" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B29" s="38" t="n">
-        <v>205</v>
-      </c>
+      <c r="B29" s="38" t="inlineStr"/>
       <c r="C29" s="41" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6481,7 +6323,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -6489,7 +6331,9 @@
       <c r="A30" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B30" s="33" t="inlineStr"/>
+      <c r="B30" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6507,7 +6351,7 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -6516,7 +6360,7 @@
         <v>46142</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C31" s="41" t="inlineStr">
         <is>
@@ -6535,7 +6379,7 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -6871,7 +6715,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -6899,7 +6743,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
@@ -7273,7 +7117,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D58" s="56" t="inlineStr">
+      <c r="D58" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-05 08:05 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -685,19 +685,19 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1596,7 +1596,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 04, 2026  ·  08:02 UTC</t>
+          <t>Generated April 05, 2026  ·  08:05 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1752,7 +1752,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         <v>46121</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1854,7 +1854,7 @@
         <v>46121</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         <v>46121</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1910,7 +1910,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1922,7 +1922,7 @@
         <v>46122</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="H15" s="42" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1956,7 +1956,7 @@
         <v>46122</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1967,7 +1967,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="H16" s="41" t="inlineStr">
         <is>
@@ -2168,17 +2168,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/4 – 4/10</t>
+          <t>4/5 – 4/11</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D27" s="40" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.1</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2189,17 +2189,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/11 – 4/17</t>
+          <t>4/12 – 4/18</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D28" s="37" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2210,17 +2210,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/18 – 4/24</t>
+          <t>4/19 – 4/25</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="D29" s="40" t="n">
         <v>7</v>
       </c>
-      <c r="D29" s="40" t="n">
-        <v>4</v>
-      </c>
       <c r="E29" s="30" t="n">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2231,17 +2231,17 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/25 – 5/1</t>
+          <t>4/26 – 5/2</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D30" s="37" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2252,17 +2252,17 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/2 – 5/8</t>
+          <t>5/3 – 5/9</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="40" t="n">
         <v>7</v>
       </c>
-      <c r="D31" s="40" t="n">
-        <v>5</v>
-      </c>
       <c r="E31" s="30" t="n">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/9 – 5/15</t>
+          <t>5/10 – 5/16</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D32" s="37" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E32" s="35" t="n">
-        <v>6.8</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2294,17 +2294,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/16 – 5/22</t>
+          <t>5/17 – 5/23</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
         <v>3</v>
       </c>
       <c r="D33" s="40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" s="30" t="n">
-        <v>4.7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2315,17 +2315,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/23 – 5/29</t>
+          <t>5/24 – 5/30</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D34" s="37" t="n">
         <v>5</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>6.7</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2336,17 +2336,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>5/30 – 6/5</t>
+          <t>5/31 – 6/6</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D35" s="40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2357,17 +2357,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/6 – 6/12</t>
+          <t>6/7 – 6/13</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D36" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2378,17 +2378,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/13 – 6/19</t>
+          <t>6/14 – 6/20</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D37" s="40" t="n">
         <v>2</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2399,17 +2399,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/20 – 6/26</t>
+          <t>6/21 – 6/27</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D38" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="D38" s="37" t="n">
-        <v>2</v>
-      </c>
       <c r="E38" s="35" t="n">
-        <v>5.6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2420,17 +2420,17 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>6/27 – 7/3</t>
+          <t>6/28 – 7/4</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D39" s="40" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E39" s="30" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
   </sheetData>
@@ -2697,7 +2697,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 04, 2026  ·  08:02 UTC</t>
+          <t>Generated April 05, 2026  ·  08:05 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2740,14 +2740,14 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C4" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C4" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D4" s="41" t="inlineStr">
@@ -2757,25 +2757,25 @@
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>adidas Anthony Edwards 2 “Easter”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46116</v>
+        <v>46120</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C5" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>230</v>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D5" s="42" t="inlineStr">
@@ -2785,12 +2785,12 @@
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Antlanta”</t>
+          <t>Melitta Baumeister x Nike Pegasus Premium</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
         <v>46120</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C6" s="47" t="inlineStr">
         <is>
@@ -2818,20 +2818,20 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Pegasus Premium</t>
+          <t>Melitta Baumeister x Nike Vomero Premium</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="36" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C7" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D7" s="42" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Vomero Premium</t>
+          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
         </is>
       </c>
     </row>
@@ -2902,16 +2902,16 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="D11" s="54" t="inlineStr">
+      <c r="D11" s="55" t="inlineStr">
         <is>
           <t>Confirmed App</t>
         </is>
@@ -3023,11 +3023,11 @@
         <v>46122</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C14" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C14" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D14" s="41" t="inlineStr">
@@ -3042,25 +3042,25 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C15" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D15" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D15" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
@@ -3070,7 +3070,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -3079,16 +3079,16 @@
         <v>46123</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C16" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D16" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>130</v>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D16" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
@@ -3107,11 +3107,11 @@
         <v>46123</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C17" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -3121,12 +3121,12 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
@@ -3135,26 +3135,26 @@
         <v>46123</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D18" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D18" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -3163,39 +3163,39 @@
         <v>46123</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C19" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D19" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>140</v>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C20" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C20" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D20" s="41" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
         <v>46124</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="C21" s="49" t="inlineStr">
         <is>
@@ -3238,35 +3238,33 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>adidas Harden Vol. 10 “Marathon”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46124</v>
-      </c>
-      <c r="B22" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C22" s="57" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D22" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B22" s="33" t="inlineStr"/>
+      <c r="C22" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D22" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Marathon”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
@@ -3274,15 +3272,17 @@
       <c r="A23" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B23" s="38" t="inlineStr"/>
+      <c r="B23" s="38" t="n">
+        <v>190</v>
+      </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3320,7 +3320,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3329,7 @@
         <v>46125</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
@@ -3348,20 +3348,20 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C26" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>120</v>
+      </c>
+      <c r="C26" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D26" s="41" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
         </is>
       </c>
     </row>
@@ -3385,11 +3385,11 @@
         <v>46126</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C27" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C27" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D27" s="42" t="inlineStr">
@@ -3404,25 +3404,25 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C28" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D28" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>100</v>
+      </c>
+      <c r="C28" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D28" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
@@ -3432,48 +3432,48 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Nike V5 RNR “Jackie Robinson Day”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>100</v>
-      </c>
-      <c r="C29" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D29" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C29" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike V5 RNR “Jackie Robinson Day”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C30" s="57" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C30" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D30" s="41" t="inlineStr">
@@ -3483,30 +3483,30 @@
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C31" s="53" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C31" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D31" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D31" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
@@ -3550,19 +3550,19 @@
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C33" s="53" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C33" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D33" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D33" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
@@ -3572,20 +3572,20 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C34" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C34" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D34" s="41" t="inlineStr">
@@ -3595,12 +3595,12 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -3609,11 +3609,11 @@
         <v>46135</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C35" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D35" s="42" t="inlineStr">
@@ -3623,30 +3623,30 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Homecoming x Nike Air Max Plus</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C36" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D36" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D36" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Homecoming x Nike Air Max Plus</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -3665,16 +3665,16 @@
         <v>46136</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D37" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
@@ -3684,17 +3684,15 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B38" s="33" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B38" s="33" t="inlineStr"/>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3712,7 +3710,7 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3800,7 @@
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B42" s="33" t="inlineStr"/>
       <c r="C42" s="40" t="inlineStr">
@@ -3817,12 +3815,12 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3828,9 @@
       <c r="A43" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B43" s="38" t="inlineStr"/>
+      <c r="B43" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3857,7 +3857,7 @@
         <v>46142</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3885,11 +3885,11 @@
         <v>46142</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C45" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>95</v>
+      </c>
+      <c r="C45" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D45" s="42" t="inlineStr">
@@ -3899,12 +3899,12 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
         <v>46142</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>95</v>
+        <v>200</v>
       </c>
       <c r="C46" s="47" t="inlineStr">
         <is>
@@ -3932,18 +3932,18 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C47" s="53" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C47" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
@@ -3969,7 +3969,7 @@
         <v>46143</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C48" s="47" t="inlineStr">
         <is>
@@ -3988,20 +3988,20 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C49" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C49" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D49" s="42" t="inlineStr">
@@ -4011,12 +4011,12 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4053,11 +4053,11 @@
         <v>46144</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C51" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C51" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4067,25 +4067,25 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C52" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D52" s="41" t="inlineStr">
@@ -4100,16 +4100,16 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -4137,7 +4137,7 @@
         <v>46150</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
@@ -4156,7 +4156,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -4167,9 +4167,9 @@
       <c r="B55" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C55" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C55" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D55" s="42" t="inlineStr">
@@ -4184,35 +4184,35 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C56" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D56" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D56" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -4221,26 +4221,26 @@
         <v>46151</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C57" s="58" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D57" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>120</v>
+      </c>
+      <c r="C57" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D57" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -4249,26 +4249,26 @@
         <v>46151</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C58" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D58" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C58" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D58" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -4277,39 +4277,39 @@
         <v>46151</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C59" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D59" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D59" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C60" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C60" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D60" s="41" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
@@ -4333,11 +4333,11 @@
         <v>46157</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C61" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C61" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D61" s="42" t="inlineStr">
@@ -4352,16 +4352,16 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C62" s="40" t="inlineStr">
         <is>
@@ -4375,12 +4375,12 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
@@ -4389,11 +4389,11 @@
         <v>46158</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C63" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C63" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D63" s="42" t="inlineStr">
@@ -4403,25 +4403,25 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46158</v>
+        <v>46164</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C64" s="57" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>170</v>
+      </c>
+      <c r="C64" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D64" s="41" t="inlineStr">
@@ -4431,25 +4431,25 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C65" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C65" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D65" s="42" t="inlineStr">
@@ -4459,12 +4459,12 @@
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -4492,16 +4492,16 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C67" s="37" t="inlineStr">
         <is>
@@ -4515,21 +4515,21 @@
       </c>
       <c r="E67" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C68" s="40" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4557,11 +4557,11 @@
         <v>46171</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C69" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C69" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D69" s="42" t="inlineStr">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
@@ -4585,11 +4585,11 @@
         <v>46171</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C70" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C70" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D70" s="41" t="inlineStr">
@@ -4604,20 +4604,18 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46171</v>
-      </c>
-      <c r="B71" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C71" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46172</v>
+      </c>
+      <c r="B71" s="38" t="inlineStr"/>
+      <c r="C71" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D71" s="42" t="inlineStr">
@@ -4627,12 +4625,12 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
@@ -4640,10 +4638,12 @@
       <c r="A72" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B72" s="33" t="inlineStr"/>
-      <c r="C72" s="57" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B72" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="C72" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D72" s="41" t="inlineStr">
@@ -4653,12 +4653,12 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
@@ -4666,9 +4666,7 @@
       <c r="A73" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B73" s="38" t="n">
-        <v>250</v>
-      </c>
+      <c r="B73" s="38" t="inlineStr"/>
       <c r="C73" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4681,23 +4679,25 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B74" s="33" t="inlineStr"/>
-      <c r="C74" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46173</v>
+      </c>
+      <c r="B74" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C74" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D74" s="41" t="inlineStr">
@@ -4707,23 +4707,23 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B75" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C75" s="53" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C75" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4740,20 +4740,18 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B76" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C76" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B76" s="33" t="inlineStr"/>
+      <c r="C76" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D76" s="41" t="inlineStr">
@@ -4763,20 +4761,22 @@
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B77" s="38" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B77" s="38" t="n">
+        <v>355</v>
+      </c>
       <c r="C77" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4794,20 +4794,20 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46182</v>
+        <v>46185</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="C78" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C78" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D78" s="41" t="inlineStr">
@@ -4817,12 +4817,12 @@
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4833,7 @@
       <c r="B79" s="38" t="n">
         <v>170</v>
       </c>
-      <c r="C79" s="53" t="inlineStr">
+      <c r="C79" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4850,7 +4850,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -4878,7 +4878,7 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4889,7 @@
       <c r="B81" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C81" s="53" t="inlineStr">
+      <c r="C81" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5001,7 +5001,7 @@
       <c r="B85" s="38" t="n">
         <v>155</v>
       </c>
-      <c r="C85" s="53" t="inlineStr">
+      <c r="C85" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5055,7 +5055,7 @@
         <v>46193</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="C87" s="37" t="inlineStr">
         <is>
@@ -5069,12 +5069,12 @@
       </c>
       <c r="E87" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -5083,26 +5083,26 @@
         <v>46193</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C88" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D88" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C88" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D88" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -5111,16 +5111,16 @@
         <v>46193</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C89" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D89" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C89" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D89" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5169,7 +5169,7 @@
       <c r="B91" s="38" t="n">
         <v>180</v>
       </c>
-      <c r="C91" s="53" t="inlineStr">
+      <c r="C91" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5195,7 +5195,7 @@
         <v>46200</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C92" s="40" t="inlineStr">
         <is>
@@ -5209,12 +5209,12 @@
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -5222,9 +5222,7 @@
       <c r="A93" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B93" s="38" t="n">
-        <v>170</v>
-      </c>
+      <c r="B93" s="38" t="inlineStr"/>
       <c r="C93" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5237,12 +5235,12 @@
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -5251,26 +5249,26 @@
         <v>46200</v>
       </c>
       <c r="B94" s="33" t="n">
-        <v>185</v>
+        <v>120</v>
       </c>
       <c r="C94" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D94" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D94" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -5279,14 +5277,14 @@
         <v>46200</v>
       </c>
       <c r="B95" s="38" t="inlineStr"/>
-      <c r="C95" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D95" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C95" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D95" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
@@ -5296,7 +5294,7 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
@@ -5305,16 +5303,16 @@
         <v>46200</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="C96" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D96" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D96" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
@@ -5324,7 +5322,7 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -5332,25 +5330,27 @@
       <c r="A97" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B97" s="38" t="inlineStr"/>
-      <c r="C97" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D97" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B97" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C97" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D97" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D98" s="55" t="inlineStr">
+      <c r="D98" s="57" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5389,7 +5389,7 @@
       <c r="B99" s="38" t="n">
         <v>130</v>
       </c>
-      <c r="C99" s="53" t="inlineStr">
+      <c r="C99" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5452,7 +5452,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 04, 2026  ·  08:02 UTC</t>
+          <t>Generated April 05, 2026  ·  08:05 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5582,7 +5582,7 @@
         <v>46122</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5610,7 @@
         <v>46122</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -5638,26 +5638,26 @@
         <v>46123</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D9" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -5666,14 +5666,14 @@
         <v>46123</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="55" t="inlineStr">
+      <c r="D10" s="57" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
@@ -5694,26 +5694,26 @@
         <v>46123</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -5727,7 +5727,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="55" t="inlineStr">
+      <c r="D12" s="57" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5971,9 +5971,7 @@
       <c r="A21" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B21" s="38" t="n">
-        <v>215</v>
-      </c>
+      <c r="B21" s="38" t="inlineStr"/>
       <c r="C21" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5986,12 +5984,12 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -6000,7 +5998,7 @@
         <v>46137</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
@@ -6019,7 +6017,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6026,7 @@
         <v>46137</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
@@ -6042,12 +6040,12 @@
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6053,9 @@
       <c r="A24" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B24" s="33" t="inlineStr"/>
+      <c r="B24" s="33" t="n">
+        <v>180</v>
+      </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -6164,7 +6164,7 @@
         <v>46144</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>195</v>
+        <v>220</v>
       </c>
       <c r="C28" s="40" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6192,7 @@
         <v>46144</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
@@ -6211,7 +6211,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -6304,16 +6304,16 @@
         <v>46151</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C33" s="58" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D33" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>230</v>
+      </c>
+      <c r="C33" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D33" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6332,7 @@
         <v>46151</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -6360,16 +6360,16 @@
         <v>46151</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D35" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>155</v>
+      </c>
+      <c r="C35" s="58" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D35" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -6388,7 +6388,7 @@
         <v>46151</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6776,7 +6776,7 @@
         <v>46193</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
@@ -6790,12 +6790,12 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -6804,7 +6804,7 @@
         <v>46193</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
@@ -6818,12 +6818,12 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -6832,7 +6832,7 @@
         <v>46200</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
@@ -6846,12 +6846,12 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -6859,9 +6859,7 @@
       <c r="A53" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B53" s="38" t="n">
-        <v>170</v>
-      </c>
+      <c r="B53" s="38" t="inlineStr"/>
       <c r="C53" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6874,12 +6872,12 @@
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -6888,26 +6886,26 @@
         <v>46200</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>185</v>
+        <v>120</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D54" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6913,9 @@
       <c r="A55" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B55" s="38" t="inlineStr"/>
+      <c r="B55" s="38" t="n">
+        <v>190</v>
+      </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6928,12 +6928,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -6942,16 +6942,16 @@
         <v>46200</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D56" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-06 07:48 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -685,19 +685,19 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1596,7 +1596,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 05, 2026  ·  08:05 UTC</t>
+          <t>Generated April 06, 2026  ·  07:48 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1636,11 +1636,11 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1649,7 +1649,7 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$180</t>
+          <t>$181</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1752,7 +1752,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         <v>46121</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1854,7 +1854,7 @@
         <v>46121</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         <v>46121</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1910,7 +1910,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1922,7 +1922,7 @@
         <v>46122</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="H15" s="42" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1956,7 +1956,7 @@
         <v>46122</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1967,7 +1967,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="H16" s="41" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D22" s="47" t="inlineStr">
         <is>
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="E23" s="35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G23" s="50" t="inlineStr">
         <is>
@@ -2168,17 +2168,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/5 – 4/11</t>
+          <t>4/6 – 4/12</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D27" s="40" t="n">
         <v>8</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2189,17 +2189,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/12 – 4/18</t>
+          <t>4/13 – 4/19</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D28" s="37" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/19 – 4/25</t>
+          <t>4/20 – 4/26</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/26 – 5/2</t>
+          <t>4/27 – 5/3</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/3 – 5/9</t>
+          <t>5/4 – 5/10</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/10 – 5/16</t>
+          <t>5/11 – 5/17</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/17 – 5/23</t>
+          <t>5/18 – 5/24</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2315,17 +2315,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/24 – 5/30</t>
+          <t>5/25 – 5/31</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D34" s="37" t="n">
         <v>5</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2336,17 +2336,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>5/31 – 6/6</t>
+          <t>6/1 – 6/7</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D35" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/7 – 6/13</t>
+          <t>6/8 – 6/14</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/14 – 6/20</t>
+          <t>6/15 – 6/21</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/21 – 6/27</t>
+          <t>6/22 – 6/28</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>6/28 – 7/4</t>
+          <t>6/29 – 7/5</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -2596,7 +2596,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2630,7 +2630,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2671,7 +2671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2697,7 +2697,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 05, 2026  ·  08:05 UTC</t>
+          <t>Generated April 06, 2026  ·  07:48 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2740,14 +2740,14 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46117</v>
+        <v>46120</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C4" s="53" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>230</v>
+      </c>
+      <c r="C4" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D4" s="41" t="inlineStr">
@@ -2757,12 +2757,12 @@
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Easter”</t>
+          <t>Melitta Baumeister x Nike Pegasus Premium</t>
         </is>
       </c>
     </row>
@@ -2771,9 +2771,9 @@
         <v>46120</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C5" s="54" t="inlineStr">
+        <v>240</v>
+      </c>
+      <c r="C5" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2790,20 +2790,20 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Pegasus Premium</t>
+          <t>Melitta Baumeister x Nike Vomero Premium</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C6" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D6" s="41" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Vomero Premium</t>
+          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
         </is>
       </c>
     </row>
@@ -2874,35 +2874,35 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C9" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C9" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
         </is>
       </c>
     </row>
@@ -2911,11 +2911,11 @@
         <v>46122</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C10" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D10" s="41" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
@@ -2939,26 +2939,26 @@
         <v>46122</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C11" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D11" s="55" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+        <v>235</v>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -2967,11 +2967,11 @@
         <v>46122</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C12" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C12" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D12" s="41" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -2995,11 +2995,11 @@
         <v>46122</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C13" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C13" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D13" s="42" t="inlineStr">
@@ -3014,25 +3014,25 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C14" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D14" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C14" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D14" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
         <v>46123</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C15" s="37" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
@@ -3079,16 +3079,16 @@
         <v>46123</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C16" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D16" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>170</v>
+      </c>
+      <c r="C16" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
     </row>
@@ -3107,11 +3107,11 @@
         <v>46123</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C17" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>185</v>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -3121,12 +3121,12 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -3135,11 +3135,11 @@
         <v>46123</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>185</v>
-      </c>
-      <c r="C18" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C18" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D18" s="41" t="inlineStr">
@@ -3149,25 +3149,25 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>140</v>
-      </c>
-      <c r="C19" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C19" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
@@ -3191,9 +3191,9 @@
         <v>46124</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C20" s="53" t="inlineStr">
+        <v>160</v>
+      </c>
+      <c r="C20" s="57" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -3210,20 +3210,20 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>adidas Harden Vol. 10 “Marathon”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C21" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C21" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D21" s="42" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Marathon”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="57" t="inlineStr">
+      <c r="D22" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
         <v>46125</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
@@ -3320,20 +3320,20 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C25" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>120</v>
+      </c>
+      <c r="C25" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D25" s="42" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
         </is>
       </c>
     </row>
@@ -3357,11 +3357,11 @@
         <v>46126</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C26" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D26" s="41" t="inlineStr">
@@ -3376,25 +3376,25 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C27" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D27" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>100</v>
+      </c>
+      <c r="C27" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D27" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
@@ -3404,48 +3404,48 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Nike V5 RNR “Jackie Robinson Day”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>100</v>
-      </c>
-      <c r="C28" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D28" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C28" s="57" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D28" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike V5 RNR “Jackie Robinson Day”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C29" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C29" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D29" s="42" t="inlineStr">
@@ -3455,30 +3455,30 @@
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D30" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D30" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
@@ -3488,7 +3488,7 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
@@ -3497,16 +3497,16 @@
         <v>46130</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C31" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D31" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>240</v>
+      </c>
+      <c r="C31" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D31" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
@@ -3516,20 +3516,20 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C32" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C32" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D32" s="41" t="inlineStr">
@@ -3544,20 +3544,20 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C33" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C33" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D33" s="42" t="inlineStr">
@@ -3567,12 +3567,12 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -3581,11 +3581,11 @@
         <v>46135</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C34" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D34" s="41" t="inlineStr">
@@ -3595,30 +3595,30 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Homecoming x Nike Air Max Plus</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C35" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D35" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D35" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Homecoming x Nike Air Max Plus</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -3637,16 +3637,16 @@
         <v>46136</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D36" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
@@ -3656,17 +3656,15 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B37" s="38" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B37" s="38" t="inlineStr"/>
       <c r="C37" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3684,7 +3682,7 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3692,7 +3690,9 @@
       <c r="A38" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B38" s="33" t="inlineStr"/>
+      <c r="B38" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3705,12 +3705,12 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3719,7 @@
         <v>46137</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3747,7 @@
         <v>46137</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -3761,22 +3761,20 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B41" s="38" t="n">
-        <v>180</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B41" s="38" t="inlineStr"/>
       <c r="C41" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3789,12 +3787,12 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3800,9 @@
       <c r="A42" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B42" s="33" t="inlineStr"/>
+      <c r="B42" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
         <v>46142</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3857,11 +3857,11 @@
         <v>46142</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C44" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>95</v>
+      </c>
+      <c r="C44" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D44" s="41" t="inlineStr">
@@ -3871,12 +3871,12 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -3885,9 +3885,9 @@
         <v>46142</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C45" s="54" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C45" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3904,16 +3904,16 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>200</v>
+        <v>135</v>
       </c>
       <c r="C46" s="47" t="inlineStr">
         <is>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
@@ -3941,9 +3941,9 @@
         <v>46143</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C47" s="54" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C47" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3960,20 +3960,20 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C48" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C48" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D48" s="41" t="inlineStr">
@@ -3983,12 +3983,12 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
         <v>46144</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -4025,11 +4025,11 @@
         <v>46144</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>195</v>
-      </c>
-      <c r="C50" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C50" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D50" s="41" t="inlineStr">
@@ -4039,25 +4039,25 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C51" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C51" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4072,16 +4072,16 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4109,7 @@
         <v>46150</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -4139,9 +4139,9 @@
       <c r="B54" s="33" t="n">
         <v>210</v>
       </c>
-      <c r="C54" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C54" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D54" s="41" t="inlineStr">
@@ -4156,35 +4156,35 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C55" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D55" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C55" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D55" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -4193,26 +4193,26 @@
         <v>46151</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>230</v>
+        <v>120</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D56" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -4221,26 +4221,26 @@
         <v>46151</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C57" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D57" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C57" s="58" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D57" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -4249,39 +4249,39 @@
         <v>46151</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C58" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D58" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>200</v>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C59" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C59" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D59" s="42" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
@@ -4305,11 +4305,11 @@
         <v>46157</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C60" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D60" s="41" t="inlineStr">
@@ -4324,16 +4324,16 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C61" s="37" t="inlineStr">
         <is>
@@ -4347,12 +4347,12 @@
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
@@ -4361,11 +4361,11 @@
         <v>46158</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C62" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C62" s="57" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D62" s="41" t="inlineStr">
@@ -4375,25 +4375,25 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46158</v>
+        <v>46164</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C63" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>170</v>
+      </c>
+      <c r="C63" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D63" s="42" t="inlineStr">
@@ -4403,25 +4403,25 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C64" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C64" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D64" s="41" t="inlineStr">
@@ -4431,12 +4431,12 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -4464,16 +4464,16 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C66" s="40" t="inlineStr">
         <is>
@@ -4487,21 +4487,21 @@
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C67" s="37" t="inlineStr">
         <is>
@@ -4520,7 +4520,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4529,11 +4529,11 @@
         <v>46171</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C68" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C68" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D68" s="41" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
@@ -4557,11 +4557,11 @@
         <v>46171</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C69" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C69" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D69" s="42" t="inlineStr">
@@ -4576,16 +4576,16 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C70" s="40" t="inlineStr">
         <is>
@@ -4604,7 +4604,7 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
@@ -4613,9 +4613,9 @@
         <v>46172</v>
       </c>
       <c r="B71" s="38" t="inlineStr"/>
-      <c r="C71" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="C71" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D71" s="42" t="inlineStr">
@@ -4625,12 +4625,12 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -4638,12 +4638,10 @@
       <c r="A72" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B72" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="C72" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B72" s="33" t="inlineStr"/>
+      <c r="C72" s="57" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D72" s="41" t="inlineStr">
@@ -4653,23 +4651,25 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B73" s="38" t="inlineStr"/>
-      <c r="C73" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46173</v>
+      </c>
+      <c r="B73" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C73" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
@@ -4679,21 +4679,21 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="C74" s="47" t="inlineStr">
         <is>
@@ -4712,20 +4712,18 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B75" s="38" t="n">
-        <v>140</v>
-      </c>
-      <c r="C75" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B75" s="38" t="inlineStr"/>
+      <c r="C75" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D75" s="42" t="inlineStr">
@@ -4735,20 +4733,22 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B76" s="33" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B76" s="33" t="n">
+        <v>355</v>
+      </c>
       <c r="C76" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4766,20 +4766,20 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46182</v>
+        <v>46185</v>
       </c>
       <c r="B77" s="38" t="n">
-        <v>355</v>
-      </c>
-      <c r="C77" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C77" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D77" s="42" t="inlineStr">
@@ -4789,12 +4789,12 @@
       </c>
       <c r="E77" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
@@ -4822,7 +4822,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4833,7 @@
       <c r="B79" s="38" t="n">
         <v>170</v>
       </c>
-      <c r="C79" s="54" t="inlineStr">
+      <c r="C79" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4850,25 +4850,25 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="C80" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D80" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D80" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E80" s="30" t="inlineStr">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -4887,16 +4887,16 @@
         <v>46186</v>
       </c>
       <c r="B81" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C81" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D81" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C81" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D81" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E81" s="35" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -4915,26 +4915,26 @@
         <v>46186</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C82" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D82" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D82" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -4943,11 +4943,11 @@
         <v>46186</v>
       </c>
       <c r="B83" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C83" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C83" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D83" s="42" t="inlineStr">
@@ -4957,12 +4957,12 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
         <v>46186</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="C84" s="47" t="inlineStr">
         <is>
@@ -4990,18 +4990,18 @@
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="36" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C85" s="54" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C85" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5018,20 +5018,20 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C86" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C86" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D86" s="41" t="inlineStr">
@@ -5041,12 +5041,12 @@
       </c>
       <c r="E86" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -5055,26 +5055,26 @@
         <v>46193</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C87" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D87" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C87" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D87" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -5083,16 +5083,16 @@
         <v>46193</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C88" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D88" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C88" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D88" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
@@ -5102,20 +5102,20 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C89" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C89" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D89" s="42" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
@@ -5158,20 +5158,20 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C91" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>185</v>
+      </c>
+      <c r="C91" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D91" s="42" t="inlineStr">
@@ -5181,12 +5181,12 @@
       </c>
       <c r="E91" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -5194,9 +5194,7 @@
       <c r="A92" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B92" s="33" t="n">
-        <v>185</v>
-      </c>
+      <c r="B92" s="33" t="inlineStr"/>
       <c r="C92" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5214,7 +5212,7 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -5222,25 +5220,27 @@
       <c r="A93" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B93" s="38" t="inlineStr"/>
+      <c r="B93" s="38" t="n">
+        <v>120</v>
+      </c>
       <c r="C93" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D93" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D93" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -5248,27 +5248,25 @@
       <c r="A94" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B94" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C94" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D94" s="57" t="inlineStr">
+      <c r="B94" s="33" t="inlineStr"/>
+      <c r="C94" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D94" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
@@ -5276,25 +5274,27 @@
       <c r="A95" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B95" s="38" t="inlineStr"/>
-      <c r="C95" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D95" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B95" s="38" t="n">
+        <v>190</v>
+      </c>
+      <c r="C95" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D95" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -5303,7 +5303,7 @@
         <v>46200</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="C96" s="40" t="inlineStr">
         <is>
@@ -5322,25 +5322,25 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="36" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="B97" s="38" t="n">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="C97" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D97" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D97" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E97" s="35" t="inlineStr">
@@ -5350,25 +5350,25 @@
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" s="31" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="B98" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C98" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D98" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C98" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D98" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E98" s="30" t="inlineStr">
@@ -5378,40 +5378,12 @@
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="15" customHeight="1">
-      <c r="A99" s="36" t="n">
-        <v>46206</v>
-      </c>
-      <c r="B99" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C99" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D99" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E99" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F99" s="35" t="inlineStr">
-        <is>
           <t>Nike Ja 3 “Animal Instinct”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F99"/>
+  <autoFilter ref="A3:F98"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5452,7 +5424,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 05, 2026  ·  08:05 UTC</t>
+          <t>Generated April 06, 2026  ·  07:48 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5582,7 +5554,7 @@
         <v>46122</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -5601,7 +5573,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5582,7 @@
         <v>46122</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -5629,7 +5601,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5645,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="57" t="inlineStr">
+      <c r="D10" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5721,15 +5693,17 @@
       <c r="A12" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B12" s="33" t="inlineStr"/>
+      <c r="B12" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
@@ -5739,7 +5713,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5747,17 +5721,15 @@
       <c r="A13" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B13" s="38" t="n">
-        <v>190</v>
-      </c>
+      <c r="B13" s="38" t="inlineStr"/>
       <c r="C13" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D13" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -5767,7 +5739,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6865,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="57" t="inlineStr">
+      <c r="D54" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-07 07:22 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$98</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -688,16 +688,16 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1596,7 +1596,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 06, 2026  ·  07:48 UTC</t>
+          <t>Generated April 07, 2026  ·  07:22 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1636,15 +1636,15 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
@@ -1752,7 +1752,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         <v>46121</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1854,7 +1854,7 @@
         <v>46121</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         <v>46121</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1910,7 +1910,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1922,7 +1922,7 @@
         <v>46122</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="H15" s="42" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1956,7 +1956,7 @@
         <v>46122</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1967,7 +1967,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="H16" s="41" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G21" s="46" t="inlineStr">
         <is>
@@ -2168,17 +2168,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/6 – 4/12</t>
+          <t>4/7 – 4/13</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D27" s="40" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2189,17 +2189,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/13 – 4/19</t>
+          <t>4/14 – 4/20</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D28" s="37" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/20 – 4/26</t>
+          <t>4/21 – 4/27</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
@@ -2231,17 +2231,17 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/27 – 5/3</t>
+          <t>4/28 – 5/4</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
         <v>10</v>
       </c>
       <c r="D30" s="37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2252,14 +2252,14 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/4 – 5/10</t>
+          <t>5/5 – 5/11</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="D31" s="40" t="n">
         <v>8</v>
-      </c>
-      <c r="D31" s="40" t="n">
-        <v>7</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>6.9</v>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/11 – 5/17</t>
+          <t>5/12 – 5/18</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/18 – 5/24</t>
+          <t>5/19 – 5/25</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/25 – 5/31</t>
+          <t>5/26 – 6/1</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>6/1 – 6/7</t>
+          <t>6/2 – 6/8</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/8 – 6/14</t>
+          <t>6/9 – 6/15</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/15 – 6/21</t>
+          <t>6/16 – 6/22</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/22 – 6/28</t>
+          <t>6/23 – 6/29</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>6/29 – 7/5</t>
+          <t>6/30 – 7/6</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2528,7 +2528,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2570,7 +2570,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -2646,7 +2646,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -2671,7 +2671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2697,7 +2697,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 06, 2026  ·  07:48 UTC</t>
+          <t>Generated April 07, 2026  ·  07:22 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2883,26 +2883,26 @@
         <v>46122</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C9" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D9" s="54" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+        <v>130</v>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -2911,26 +2911,26 @@
         <v>46122</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C10" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D10" s="55" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
         </is>
       </c>
     </row>
@@ -2939,11 +2939,11 @@
         <v>46122</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C11" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C11" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D11" s="42" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
         <v>46122</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -2995,11 +2995,11 @@
         <v>46122</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C13" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D13" s="42" t="inlineStr">
@@ -3014,25 +3014,25 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46123</v>
+        <v>46122</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C14" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D14" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>135</v>
+      </c>
+      <c r="C14" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
@@ -3051,26 +3051,26 @@
         <v>46123</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C15" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -3079,16 +3079,16 @@
         <v>46123</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C16" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D16" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D16" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -3107,11 +3107,11 @@
         <v>46123</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C17" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C17" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -3121,25 +3121,25 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C18" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C18" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D18" s="41" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
+          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3163,7 @@
         <v>46124</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="C19" s="49" t="inlineStr">
         <is>
@@ -3182,35 +3182,33 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>adidas Harden Vol. 10 “Marathon”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46124</v>
-      </c>
-      <c r="B20" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C20" s="57" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D20" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B20" s="33" t="inlineStr"/>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D20" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Marathon”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
@@ -3246,15 +3244,17 @@
       <c r="A22" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B22" s="33" t="inlineStr"/>
+      <c r="B22" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D22" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3273,7 @@
         <v>46125</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
@@ -3292,25 +3292,25 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D24" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D27" s="56" t="inlineStr">
+      <c r="D27" s="57" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3415,7 +3415,7 @@
       <c r="B28" s="33" t="n">
         <v>160</v>
       </c>
-      <c r="C28" s="57" t="inlineStr">
+      <c r="C28" s="54" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -3466,19 +3466,19 @@
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46130</v>
+        <v>46129</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C30" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D30" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>235</v>
+      </c>
+      <c r="C30" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D30" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
@@ -3488,7 +3488,7 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
@@ -3497,16 +3497,16 @@
         <v>46130</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C31" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D31" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C31" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D31" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
@@ -3516,20 +3516,20 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46133</v>
+        <v>46130</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C32" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C32" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D32" s="41" t="inlineStr">
@@ -3544,20 +3544,20 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46135</v>
+        <v>46133</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C33" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D33" s="42" t="inlineStr">
@@ -3567,12 +3567,12 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
@@ -3581,11 +3581,11 @@
         <v>46135</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C34" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C34" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D34" s="41" t="inlineStr">
@@ -3595,30 +3595,30 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Homecoming x Nike Air Max Plus</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46136</v>
+        <v>46135</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D35" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>190</v>
+      </c>
+      <c r="C35" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D35" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Homecoming x Nike Air Max Plus</t>
         </is>
       </c>
     </row>
@@ -3637,16 +3637,16 @@
         <v>46136</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D36" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
@@ -3656,15 +3656,17 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B37" s="38" t="inlineStr"/>
+        <v>46136</v>
+      </c>
+      <c r="B37" s="38" t="n">
+        <v>210</v>
+      </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3682,7 +3684,7 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3693,7 @@
         <v>46137</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>215</v>
+        <v>180</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -3705,12 +3707,12 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -3718,9 +3720,7 @@
       <c r="A39" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B39" s="38" t="n">
-        <v>200</v>
-      </c>
+      <c r="B39" s="38" t="inlineStr"/>
       <c r="C39" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3733,12 +3733,12 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3747,7 @@
         <v>46137</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>180</v>
+        <v>215</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -3761,20 +3761,22 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B41" s="38" t="inlineStr"/>
+        <v>46137</v>
+      </c>
+      <c r="B41" s="38" t="n">
+        <v>200</v>
+      </c>
       <c r="C41" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3792,7 +3794,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -3800,9 +3802,7 @@
       <c r="A42" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B42" s="33" t="n">
-        <v>215</v>
-      </c>
+      <c r="B42" s="33" t="inlineStr"/>
       <c r="C42" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
         <v>46142</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3857,11 +3857,11 @@
         <v>46142</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C44" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D44" s="41" t="inlineStr">
@@ -3871,12 +3871,12 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
         <v>46142</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>200</v>
+        <v>95</v>
       </c>
       <c r="C45" s="53" t="inlineStr">
         <is>
@@ -3904,16 +3904,16 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>135</v>
+        <v>200</v>
       </c>
       <c r="C46" s="47" t="inlineStr">
         <is>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
@@ -3960,20 +3960,20 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike Air Zoom Huarache 2K4 “White Varsity Red”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C48" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C48" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D48" s="41" t="inlineStr">
@@ -3983,25 +3983,25 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>195</v>
-      </c>
-      <c r="C49" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C49" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D49" s="42" t="inlineStr">
@@ -4011,12 +4011,12 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
@@ -4025,11 +4025,11 @@
         <v>46144</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C50" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D50" s="41" t="inlineStr">
@@ -4039,25 +4039,25 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C51" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C51" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4072,16 +4072,16 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46150</v>
+        <v>46149</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4109,7 @@
         <v>46150</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -4139,9 +4139,9 @@
       <c r="B54" s="33" t="n">
         <v>210</v>
       </c>
-      <c r="C54" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D54" s="41" t="inlineStr">
@@ -4156,35 +4156,35 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C55" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D55" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>210</v>
+      </c>
+      <c r="C55" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D55" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4193,7 @@
         <v>46151</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>120</v>
+        <v>195</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -4207,12 +4207,12 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -4221,26 +4221,26 @@
         <v>46151</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C57" s="58" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D57" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>120</v>
+      </c>
+      <c r="C57" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D57" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -4249,63 +4249,63 @@
         <v>46151</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D58" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D58" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C59" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D59" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C59" s="58" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D59" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
@@ -4324,20 +4324,20 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C61" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C61" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D61" s="42" t="inlineStr">
@@ -4347,25 +4347,25 @@
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C62" s="57" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>150</v>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D62" s="41" t="inlineStr">
@@ -4375,25 +4375,25 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46164</v>
+        <v>46158</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C63" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>145</v>
+      </c>
+      <c r="C63" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D63" s="42" t="inlineStr">
@@ -4403,25 +4403,25 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46165</v>
+        <v>46158</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C64" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C64" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D64" s="41" t="inlineStr">
@@ -4431,25 +4431,25 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46165</v>
+        <v>46164</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C65" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C65" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D65" s="42" t="inlineStr">
@@ -4459,21 +4459,21 @@
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46168</v>
+        <v>46165</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="C66" s="40" t="inlineStr">
         <is>
@@ -4487,21 +4487,21 @@
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C67" s="37" t="inlineStr">
         <is>
@@ -4515,25 +4515,25 @@
       </c>
       <c r="E67" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46171</v>
+        <v>46168</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C68" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C68" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D68" s="41" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
@@ -4576,20 +4576,20 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="C70" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C70" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D70" s="41" t="inlineStr">
@@ -4604,15 +4604,17 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B71" s="38" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="B71" s="38" t="n">
+        <v>240</v>
+      </c>
       <c r="C71" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4625,12 +4627,12 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -4639,7 +4641,7 @@
         <v>46172</v>
       </c>
       <c r="B72" s="33" t="inlineStr"/>
-      <c r="C72" s="57" t="inlineStr">
+      <c r="C72" s="54" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -4662,14 +4664,14 @@
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C73" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C73" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
@@ -4684,20 +4686,18 @@
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B74" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C74" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46172</v>
+      </c>
+      <c r="B74" s="33" t="inlineStr"/>
+      <c r="C74" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D74" s="41" t="inlineStr">
@@ -4707,23 +4707,25 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B75" s="38" t="inlineStr"/>
-      <c r="C75" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46173</v>
+      </c>
+      <c r="B75" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C75" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D75" s="42" t="inlineStr">
@@ -4733,25 +4735,25 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46182</v>
+        <v>46177</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="C76" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C76" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D76" s="41" t="inlineStr">
@@ -4761,25 +4763,23 @@
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B77" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C77" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B77" s="38" t="inlineStr"/>
+      <c r="C77" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D77" s="42" t="inlineStr">
@@ -4789,25 +4789,25 @@
       </c>
       <c r="E77" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C78" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>355</v>
+      </c>
+      <c r="C78" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D78" s="41" t="inlineStr">
@@ -4817,12 +4817,12 @@
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -4856,19 +4856,19 @@
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C80" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D80" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D80" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E80" s="30" t="inlineStr">
@@ -4878,25 +4878,25 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B81" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C81" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D81" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>170</v>
+      </c>
+      <c r="C81" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D81" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E81" s="35" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -4915,11 +4915,11 @@
         <v>46186</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C82" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C82" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D82" s="41" t="inlineStr">
@@ -4929,12 +4929,12 @@
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4950,9 +4950,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D83" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D83" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E83" s="35" t="inlineStr">
@@ -4962,7 +4962,7 @@
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -4971,11 +4971,11 @@
         <v>46186</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C84" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C84" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D84" s="41" t="inlineStr">
@@ -4985,30 +4985,30 @@
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="36" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C85" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D85" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C85" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D85" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E85" s="35" t="inlineStr">
@@ -5018,20 +5018,20 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C86" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C86" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D86" s="41" t="inlineStr">
@@ -5041,30 +5041,30 @@
       </c>
       <c r="E86" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="36" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>210</v>
+        <v>135</v>
       </c>
       <c r="C87" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D87" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D87" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
@@ -5108,14 +5108,14 @@
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C89" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C89" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D89" s="42" t="inlineStr">
@@ -5125,30 +5125,30 @@
       </c>
       <c r="E89" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C90" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D90" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D90" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5158,20 +5158,20 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C91" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C91" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D91" s="42" t="inlineStr">
@@ -5181,23 +5181,25 @@
       </c>
       <c r="E91" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B92" s="33" t="inlineStr"/>
-      <c r="C92" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46199</v>
+      </c>
+      <c r="B92" s="33" t="n">
+        <v>180</v>
+      </c>
+      <c r="C92" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D92" s="41" t="inlineStr">
@@ -5207,12 +5209,12 @@
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
@@ -5220,27 +5222,25 @@
       <c r="A93" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B93" s="38" t="n">
-        <v>120</v>
-      </c>
+      <c r="B93" s="38" t="inlineStr"/>
       <c r="C93" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D93" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D93" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -5248,25 +5248,27 @@
       <c r="A94" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B94" s="33" t="inlineStr"/>
-      <c r="C94" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D94" s="55" t="inlineStr">
+      <c r="B94" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="C94" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D94" s="56" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -5275,7 +5277,7 @@
         <v>46200</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C95" s="37" t="inlineStr">
         <is>
@@ -5289,12 +5291,12 @@
       </c>
       <c r="E95" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -5302,45 +5304,43 @@
       <c r="A96" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B96" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C96" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D96" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B96" s="33" t="inlineStr"/>
+      <c r="C96" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D96" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="36" t="n">
-        <v>46203</v>
+        <v>46200</v>
       </c>
       <c r="B97" s="38" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C97" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D97" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D97" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E97" s="35" t="inlineStr">
@@ -5350,40 +5350,96 @@
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" s="31" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B98" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C98" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D98" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E98" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F98" s="30" t="inlineStr">
+        <is>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="15" customHeight="1">
+      <c r="A99" s="36" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B99" s="38" t="n">
+        <v>135</v>
+      </c>
+      <c r="C99" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D99" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E99" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F99" s="35" t="inlineStr">
+        <is>
+          <t>Bluetile x Nike SB Dunk Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15" customHeight="1">
+      <c r="A100" s="31" t="n">
         <v>46206</v>
       </c>
-      <c r="B98" s="33" t="n">
+      <c r="B100" s="33" t="n">
         <v>130</v>
       </c>
-      <c r="C98" s="47" t="inlineStr">
+      <c r="C100" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D98" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E98" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F98" s="30" t="inlineStr">
+      <c r="D100" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E100" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F100" s="30" t="inlineStr">
         <is>
           <t>Nike Ja 3 “Animal Instinct”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F98"/>
+  <autoFilter ref="A3:F100"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5398,7 +5454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5424,7 +5480,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 06, 2026  ·  07:48 UTC</t>
+          <t>Generated April 07, 2026  ·  07:22 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5554,7 +5610,7 @@
         <v>46122</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -5573,7 +5629,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -5582,7 +5638,7 @@
         <v>46122</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -5601,25 +5657,25 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46123</v>
+        <v>46122</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
@@ -5629,7 +5685,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
         </is>
       </c>
     </row>
@@ -5638,26 +5694,26 @@
         <v>46123</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
@@ -5666,26 +5722,26 @@
         <v>46123</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D11" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -5693,17 +5749,15 @@
       <c r="A12" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B12" s="33" t="n">
-        <v>190</v>
-      </c>
+      <c r="B12" s="33" t="inlineStr"/>
       <c r="C12" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D12" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
@@ -5713,7 +5767,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
@@ -5721,15 +5775,17 @@
       <c r="A13" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B13" s="38" t="inlineStr"/>
+      <c r="B13" s="38" t="n">
+        <v>190</v>
+      </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -5739,7 +5795,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5804,16 +5860,16 @@
         <v>46126</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D16" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -5823,16 +5879,16 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46130</v>
+        <v>46126</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>240</v>
+        <v>150</v>
       </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
@@ -5851,16 +5907,16 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46135</v>
+        <v>46129</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
@@ -5874,30 +5930,30 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46136</v>
+        <v>46130</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D19" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
@@ -5907,16 +5963,16 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46136</v>
+        <v>46135</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -5930,28 +5986,30 @@
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B21" s="38" t="inlineStr"/>
+        <v>46136</v>
+      </c>
+      <c r="B21" s="38" t="n">
+        <v>200</v>
+      </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D21" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
@@ -5961,16 +6019,16 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
@@ -5984,12 +6042,12 @@
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
@@ -5998,7 +6056,7 @@
         <v>46137</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
@@ -6012,12 +6070,12 @@
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -6025,9 +6083,7 @@
       <c r="A24" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B24" s="33" t="n">
-        <v>180</v>
-      </c>
+      <c r="B24" s="33" t="inlineStr"/>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6045,15 +6101,17 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B25" s="38" t="inlineStr"/>
+        <v>46137</v>
+      </c>
+      <c r="B25" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6071,16 +6129,16 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
@@ -6099,7 +6157,7 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -6107,9 +6165,7 @@
       <c r="A27" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B27" s="38" t="n">
-        <v>205</v>
-      </c>
+      <c r="B27" s="38" t="inlineStr"/>
       <c r="C27" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6127,16 +6183,16 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46144</v>
+        <v>46142</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C28" s="40" t="inlineStr">
         <is>
@@ -6155,16 +6211,16 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46144</v>
+        <v>46142</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
@@ -6183,16 +6239,16 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
@@ -6206,21 +6262,21 @@
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46150</v>
+        <v>46149</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
@@ -6239,7 +6295,7 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6304,7 @@
         <v>46150</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -6267,35 +6323,35 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D33" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D33" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6360,7 @@
         <v>46151</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>120</v>
+        <v>195</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -6318,12 +6374,12 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -6332,26 +6388,26 @@
         <v>46151</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C35" s="58" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D35" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>120</v>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D35" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -6360,63 +6416,63 @@
         <v>46151</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D36" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C37" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D37" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C37" s="58" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D37" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46158</v>
+        <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>145</v>
+        <v>200</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -6430,21 +6486,21 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46165</v>
+        <v>46157</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
@@ -6458,21 +6514,21 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46165</v>
+        <v>46158</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>205</v>
+        <v>145</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -6491,16 +6547,16 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46168</v>
+        <v>46165</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="C41" s="37" t="inlineStr">
         <is>
@@ -6514,21 +6570,21 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -6542,21 +6598,21 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46171</v>
+        <v>46168</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
@@ -6575,16 +6631,16 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
@@ -6603,15 +6659,17 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B45" s="38" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="B45" s="38" t="n">
+        <v>240</v>
+      </c>
       <c r="C45" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6624,20 +6682,22 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B46" s="33" t="inlineStr"/>
+        <v>46172</v>
+      </c>
+      <c r="B46" s="33" t="n">
+        <v>250</v>
+      </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6650,22 +6710,20 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B47" s="38" t="n">
-        <v>355</v>
-      </c>
+        <v>46172</v>
+      </c>
+      <c r="B47" s="38" t="inlineStr"/>
       <c r="C47" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6683,44 +6741,42 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B48" s="33" t="n">
-        <v>150</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B48" s="33" t="inlineStr"/>
       <c r="C48" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D48" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D48" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46186</v>
+        <v>46182</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>205</v>
+        <v>355</v>
       </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
@@ -6739,16 +6795,16 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
@@ -6767,13 +6823,13 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B51" s="38" t="n">
         <v>150</v>
@@ -6783,9 +6839,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D51" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E51" s="35" t="inlineStr">
@@ -6795,16 +6851,16 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46200</v>
+        <v>46193</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>185</v>
+        <v>150</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
@@ -6818,20 +6874,22 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B53" s="38" t="inlineStr"/>
+        <v>46193</v>
+      </c>
+      <c r="B53" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6849,7 +6907,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -6857,27 +6915,25 @@
       <c r="A54" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B54" s="33" t="n">
-        <v>120</v>
-      </c>
+      <c r="B54" s="33" t="inlineStr"/>
       <c r="C54" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D54" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -6886,16 +6942,16 @@
         <v>46200</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>190</v>
+        <v>120</v>
       </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D55" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D55" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E55" s="35" t="inlineStr">
@@ -6905,7 +6961,7 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6970,7 @@
         <v>46200</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -6928,45 +6984,101 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B57" s="38" t="n">
+        <v>190</v>
+      </c>
+      <c r="C57" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D57" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E57" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F57" s="35" t="inlineStr">
+        <is>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="15" customHeight="1">
+      <c r="A58" s="31" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B58" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E58" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F58" s="30" t="inlineStr">
+        <is>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1">
+      <c r="A59" s="36" t="n">
         <v>46203</v>
       </c>
-      <c r="B57" s="38" t="n">
+      <c r="B59" s="38" t="n">
         <v>135</v>
       </c>
-      <c r="C57" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D57" s="56" t="inlineStr">
+      <c r="C59" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D59" s="57" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
-      <c r="E57" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F57" s="35" t="inlineStr">
+      <c r="E59" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F59" s="35" t="inlineStr">
         <is>
           <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F57"/>
+  <autoFilter ref="A3:F59"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-08 07:25 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$100</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -698,9 +698,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1596,7 +1593,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 07, 2026  ·  07:22 UTC</t>
+          <t>Generated April 08, 2026  ·  07:25 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1636,15 +1633,15 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
@@ -1752,7 +1749,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1786,7 +1783,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1820,7 +1817,7 @@
         <v>46121</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1854,7 +1851,7 @@
         <v>46121</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1888,7 +1885,7 @@
         <v>46121</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1910,7 +1907,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1922,7 +1919,7 @@
         <v>46122</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1933,7 +1930,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="H15" s="42" t="inlineStr">
         <is>
@@ -1944,7 +1941,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1956,7 +1953,7 @@
         <v>46122</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1967,7 +1964,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="H16" s="41" t="inlineStr">
         <is>
@@ -2029,7 +2026,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2045,7 +2042,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2063,7 +2060,7 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G21" s="46" t="inlineStr">
         <is>
@@ -2168,14 +2165,14 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/7 – 4/13</t>
+          <t>4/8 – 4/14</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D27" s="40" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>5.7</v>
@@ -2189,17 +2186,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/14 – 4/20</t>
+          <t>4/15 – 4/21</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D28" s="37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.2</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2210,17 +2207,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/21 – 4/27</t>
+          <t>4/22 – 4/28</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D29" s="40" t="n">
         <v>7</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>6.4</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2231,7 +2228,7 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/28 – 5/4</t>
+          <t>4/29 – 5/5</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
@@ -2252,7 +2249,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/5 – 5/11</t>
+          <t>5/6 – 5/12</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2273,7 +2270,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/12 – 5/18</t>
+          <t>5/13 – 5/19</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2294,17 +2291,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/19 – 5/25</t>
+          <t>5/20 – 5/26</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="40" t="n">
         <v>3</v>
       </c>
-      <c r="D33" s="40" t="n">
-        <v>2</v>
-      </c>
       <c r="E33" s="30" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2315,17 +2312,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/26 – 6/1</t>
+          <t>5/27 – 6/2</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D34" s="37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2336,17 +2333,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>6/2 – 6/8</t>
+          <t>6/3 – 6/9</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="40" t="n">
-        <v>1</v>
-      </c>
       <c r="E35" s="30" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2357,17 +2354,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/9 – 6/15</t>
+          <t>6/10 – 6/16</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D36" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2378,7 +2375,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/16 – 6/22</t>
+          <t>6/17 – 6/23</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2399,17 +2396,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/23 – 6/29</t>
+          <t>6/24 – 6/30</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D38" s="37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E38" s="35" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2420,7 +2417,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>6/30 – 7/6</t>
+          <t>7/1 – 7/7</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2528,7 +2525,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2544,7 +2541,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2570,7 +2567,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2646,7 +2643,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -2671,7 +2668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2697,7 +2694,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 07, 2026  ·  07:22 UTC</t>
+          <t>Generated April 08, 2026  ·  07:25 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2883,11 +2880,11 @@
         <v>46122</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C9" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C9" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D9" s="42" t="inlineStr">
@@ -2902,7 +2899,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
@@ -2911,26 +2908,26 @@
         <v>46122</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C10" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D10" s="55" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+        <v>235</v>
+      </c>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -2939,11 +2936,11 @@
         <v>46122</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C11" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D11" s="42" t="inlineStr">
@@ -2958,7 +2955,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -2967,26 +2964,26 @@
         <v>46122</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>235</v>
-      </c>
-      <c r="C12" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D12" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D12" s="55" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3326,7 @@
         <v>46126</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C25" s="53" t="inlineStr">
         <is>
@@ -3693,7 +3690,7 @@
         <v>46137</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>180</v>
+        <v>215</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -3707,12 +3704,12 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3717,9 @@
       <c r="A39" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B39" s="38" t="inlineStr"/>
+      <c r="B39" s="38" t="n">
+        <v>200</v>
+      </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3733,12 +3732,12 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3746,7 @@
         <v>46137</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>215</v>
+        <v>180</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -3761,12 +3760,12 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -3774,9 +3773,7 @@
       <c r="A41" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B41" s="38" t="n">
-        <v>200</v>
-      </c>
+      <c r="B41" s="38" t="inlineStr"/>
       <c r="C41" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3789,12 +3786,12 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3799,9 @@
       <c r="A42" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B42" s="33" t="inlineStr"/>
+      <c r="B42" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3820,7 +3819,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3828,7 @@
         <v>46142</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
@@ -3848,7 +3847,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3856,9 +3855,7 @@
       <c r="A44" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B44" s="33" t="n">
-        <v>205</v>
-      </c>
+      <c r="B44" s="33" t="inlineStr"/>
       <c r="C44" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3876,7 +3873,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4190,7 @@
         <v>46151</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -4207,12 +4204,12 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4218,7 @@
         <v>46151</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>120</v>
+        <v>195</v>
       </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
@@ -4235,12 +4232,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -4249,26 +4246,26 @@
         <v>46151</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>230</v>
+        <v>120</v>
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D58" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -4277,16 +4274,16 @@
         <v>46151</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C59" s="58" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D59" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>230</v>
+      </c>
+      <c r="C59" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D59" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
@@ -4296,7 +4293,7 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -4305,26 +4302,26 @@
         <v>46151</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C60" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D60" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C60" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D60" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4489,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -4520,7 +4517,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
@@ -4915,16 +4912,16 @@
         <v>46186</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C82" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D82" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C82" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D82" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E82" s="30" t="inlineStr">
@@ -4934,7 +4931,7 @@
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -4950,9 +4947,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D83" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D83" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E83" s="35" t="inlineStr">
@@ -4962,7 +4959,7 @@
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4971,26 +4968,26 @@
         <v>46186</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C84" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D84" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C84" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D84" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -4999,26 +4996,26 @@
         <v>46186</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C85" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D85" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D85" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E85" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5219,9 @@
       <c r="A93" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B93" s="38" t="inlineStr"/>
+      <c r="B93" s="38" t="n">
+        <v>170</v>
+      </c>
       <c r="C93" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5235,12 +5234,12 @@
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -5248,27 +5247,25 @@
       <c r="A94" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B94" s="33" t="n">
-        <v>120</v>
-      </c>
+      <c r="B94" s="33" t="inlineStr"/>
       <c r="C94" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D94" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D94" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -5277,26 +5274,26 @@
         <v>46200</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>185</v>
+        <v>120</v>
       </c>
       <c r="C95" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D95" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D95" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -5304,15 +5301,17 @@
       <c r="A96" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B96" s="33" t="inlineStr"/>
-      <c r="C96" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D96" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B96" s="33" t="n">
+        <v>185</v>
+      </c>
+      <c r="C96" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D96" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
@@ -5322,7 +5321,7 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -5330,27 +5329,25 @@
       <c r="A97" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B97" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C97" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D97" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B97" s="38" t="inlineStr"/>
+      <c r="C97" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D97" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
@@ -5359,7 +5356,7 @@
         <v>46200</v>
       </c>
       <c r="B98" s="33" t="n">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="C98" s="40" t="inlineStr">
         <is>
@@ -5378,7 +5375,7 @@
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -5438,8 +5435,36 @@
         </is>
       </c>
     </row>
+    <row r="101" ht="15" customHeight="1">
+      <c r="A101" s="36" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B101" s="38" t="n">
+        <v>210</v>
+      </c>
+      <c r="C101" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D101" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E101" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F101" s="35" t="inlineStr">
+        <is>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F100"/>
+  <autoFilter ref="A3:F101"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5454,7 +5479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5480,7 +5505,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 07, 2026  ·  07:22 UTC</t>
+          <t>Generated April 08, 2026  ·  07:25 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5610,7 +5635,7 @@
         <v>46122</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -5629,7 +5654,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5663,7 @@
         <v>46122</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -5657,7 +5682,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -6056,7 +6081,7 @@
         <v>46137</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>180</v>
+        <v>215</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
@@ -6070,12 +6095,12 @@
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6108,9 @@
       <c r="A24" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B24" s="33" t="inlineStr"/>
+      <c r="B24" s="33" t="n">
+        <v>200</v>
+      </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6096,12 +6123,12 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -6110,7 +6137,7 @@
         <v>46137</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>215</v>
+        <v>180</v>
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
@@ -6124,12 +6151,12 @@
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
@@ -6137,9 +6164,7 @@
       <c r="A26" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B26" s="33" t="n">
-        <v>200</v>
-      </c>
+      <c r="B26" s="33" t="inlineStr"/>
       <c r="C26" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6152,12 +6177,12 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -6165,7 +6190,9 @@
       <c r="A27" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B27" s="38" t="inlineStr"/>
+      <c r="B27" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C27" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6183,7 +6210,7 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6219,7 @@
         <v>46142</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C28" s="40" t="inlineStr">
         <is>
@@ -6211,7 +6238,7 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -6219,9 +6246,7 @@
       <c r="A29" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B29" s="38" t="n">
-        <v>205</v>
-      </c>
+      <c r="B29" s="38" t="inlineStr"/>
       <c r="C29" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6239,7 +6264,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -6360,7 +6385,7 @@
         <v>46151</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -6374,12 +6399,12 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6388,7 +6413,7 @@
         <v>46151</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>120</v>
+        <v>195</v>
       </c>
       <c r="C35" s="37" t="inlineStr">
         <is>
@@ -6402,12 +6427,12 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -6416,26 +6441,26 @@
         <v>46151</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>230</v>
+        <v>120</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D36" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -6444,16 +6469,16 @@
         <v>46151</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C37" s="58" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D37" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>230</v>
+      </c>
+      <c r="C37" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D37" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
@@ -6463,7 +6488,7 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -6472,26 +6497,26 @@
         <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C38" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D38" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C38" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D38" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -6575,7 +6600,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6628,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
@@ -6804,26 +6829,26 @@
         <v>46186</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D50" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D50" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -6832,26 +6857,26 @@
         <v>46186</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D51" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6940,9 @@
       <c r="A54" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B54" s="33" t="inlineStr"/>
+      <c r="B54" s="33" t="n">
+        <v>170</v>
+      </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6928,12 +6955,12 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -6941,27 +6968,25 @@
       <c r="A55" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B55" s="38" t="n">
-        <v>120</v>
-      </c>
+      <c r="B55" s="38" t="inlineStr"/>
       <c r="C55" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D55" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D55" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -6970,26 +6995,26 @@
         <v>46200</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>185</v>
+        <v>120</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D56" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -6998,7 +7023,7 @@
         <v>46200</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
@@ -7012,12 +7037,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7051,7 @@
         <v>46200</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
@@ -7045,7 +7070,7 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -7077,8 +7102,36 @@
         </is>
       </c>
     </row>
+    <row r="60" ht="15" customHeight="1">
+      <c r="A60" s="31" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B60" s="33" t="n">
+        <v>210</v>
+      </c>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D60" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E60" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F60" s="30" t="inlineStr">
+        <is>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F59"/>
+  <autoFilter ref="A3:F60"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-09 07:27 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$101</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -698,6 +698,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1593,7 +1596,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 08, 2026  ·  07:25 UTC</t>
+          <t>Generated April 09, 2026  ·  07:27 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1633,20 +1636,20 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$181</t>
+          <t>$180</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1749,7 +1752,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1783,7 +1786,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1817,7 +1820,7 @@
         <v>46121</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1851,7 +1854,7 @@
         <v>46121</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1885,7 +1888,7 @@
         <v>46121</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1919,7 +1922,7 @@
         <v>46122</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1953,7 +1956,7 @@
         <v>46122</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -2026,7 +2029,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2042,7 +2045,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2060,7 +2063,7 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G21" s="46" t="inlineStr">
         <is>
@@ -2068,7 +2071,7 @@
         </is>
       </c>
       <c r="H21" s="35" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -2086,7 +2089,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G22" s="48" t="inlineStr">
         <is>
@@ -2165,17 +2168,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/8 – 4/14</t>
+          <t>4/9 – 4/15</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D27" s="40" t="n">
         <v>14</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2186,17 +2189,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/15 – 4/21</t>
+          <t>4/16 – 4/22</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
         <v>7</v>
       </c>
       <c r="D28" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2207,14 +2210,14 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/22 – 4/28</t>
+          <t>4/23 – 4/29</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D29" s="40" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>6.8</v>
@@ -2228,7 +2231,7 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/29 – 5/5</t>
+          <t>4/30 – 5/6</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
@@ -2249,7 +2252,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/6 – 5/12</t>
+          <t>5/7 – 5/13</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2270,7 +2273,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/13 – 5/19</t>
+          <t>5/14 – 5/20</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2291,7 +2294,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/20 – 5/26</t>
+          <t>5/21 – 5/27</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2312,7 +2315,7 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/27 – 6/2</t>
+          <t>5/28 – 6/3</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
@@ -2333,7 +2336,7 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>6/3 – 6/9</t>
+          <t>6/4 – 6/10</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
@@ -2354,7 +2357,7 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/10 – 6/16</t>
+          <t>6/11 – 6/17</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
@@ -2375,7 +2378,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/17 – 6/23</t>
+          <t>6/18 – 6/24</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2396,7 +2399,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/24 – 6/30</t>
+          <t>6/25 – 7/1</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2417,7 +2420,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>7/1 – 7/7</t>
+          <t>7/2 – 7/8</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2525,7 +2528,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2541,7 +2544,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2567,7 +2570,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2575,7 +2578,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2601,7 +2604,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2617,7 +2620,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -2668,7 +2671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2694,7 +2697,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 08, 2026  ·  07:25 UTC</t>
+          <t>Generated April 09, 2026  ·  07:27 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2737,14 +2740,14 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C4" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C4" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D4" s="41" t="inlineStr">
@@ -2759,20 +2762,20 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Pegasus Premium</t>
+          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C5" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D5" s="42" t="inlineStr">
@@ -2787,7 +2790,7 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Melitta Baumeister x Nike Vomero Premium</t>
+          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
         </is>
       </c>
     </row>
@@ -2815,20 +2818,20 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="36" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C7" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C7" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D7" s="42" t="inlineStr">
@@ -2843,16 +2846,16 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>120</v>
+        <v>235</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -2871,7 +2874,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -2880,11 +2883,11 @@
         <v>46122</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C9" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D9" s="42" t="inlineStr">
@@ -2899,7 +2902,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -2908,26 +2911,26 @@
         <v>46122</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>235</v>
-      </c>
-      <c r="C10" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D10" s="55" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2958,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
         </is>
       </c>
     </row>
@@ -2964,35 +2967,35 @@
         <v>46122</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D12" s="55" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+        <v>135</v>
+      </c>
+      <c r="C12" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
@@ -3006,30 +3009,30 @@
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C14" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D14" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C14" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D14" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -3039,7 +3042,7 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -3048,11 +3051,11 @@
         <v>46123</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C15" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C15" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D15" s="42" t="inlineStr">
@@ -3062,53 +3065,53 @@
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C16" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D16" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>adidas Anthony Edwards 2 “Glow”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>140</v>
-      </c>
-      <c r="C17" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>160</v>
+      </c>
+      <c r="C17" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -3123,48 +3126,46 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
+          <t>adidas Harden Vol. 10 “Marathon”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46124</v>
-      </c>
-      <c r="B18" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C18" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D18" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B18" s="33" t="inlineStr"/>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D18" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Lime Burst”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C19" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
@@ -3174,12 +3175,12 @@
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Marathon”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3187,15 +3188,17 @@
       <c r="A20" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B20" s="33" t="inlineStr"/>
+      <c r="B20" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D20" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D20" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
@@ -3205,7 +3208,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3217,7 @@
         <v>46125</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
@@ -3233,25 +3236,25 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D22" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -3261,25 +3264,25 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D23" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
@@ -3289,7 +3292,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
@@ -3298,16 +3301,16 @@
         <v>46126</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C24" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D24" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>110</v>
+      </c>
+      <c r="C24" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D24" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
@@ -3317,25 +3320,25 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C25" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D25" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D25" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E25" s="35" t="inlineStr">
@@ -3345,25 +3348,25 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
+          <t>Nike V5 RNR “Jackie Robinson Day”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D26" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
@@ -3373,48 +3376,48 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Palace x Nike Air Max 95</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>100</v>
-      </c>
-      <c r="C27" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D27" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C27" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike V5 RNR “Jackie Robinson Day”</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C28" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C28" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D28" s="41" t="inlineStr">
@@ -3424,12 +3427,12 @@
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
@@ -3438,11 +3441,11 @@
         <v>46129</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C29" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C29" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D29" s="42" t="inlineStr">
@@ -3457,16 +3460,16 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
@@ -3485,7 +3488,7 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
@@ -3519,14 +3522,14 @@
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C32" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C32" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D32" s="41" t="inlineStr">
@@ -3541,20 +3544,20 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C33" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C33" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D33" s="42" t="inlineStr">
@@ -3564,12 +3567,12 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -3578,11 +3581,11 @@
         <v>46135</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C34" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D34" s="41" t="inlineStr">
@@ -3592,25 +3595,25 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Homecoming x Nike Air Max Plus</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C35" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D35" s="42" t="inlineStr">
@@ -3625,7 +3628,7 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Homecoming x Nike Air Max Plus</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3665,7 @@
         <v>46136</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
@@ -3681,16 +3684,16 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -3704,12 +3707,12 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3721,7 @@
         <v>46137</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
@@ -3737,7 +3740,7 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3749,7 @@
         <v>46137</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -3760,12 +3763,12 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3776,9 @@
       <c r="A41" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B41" s="38" t="inlineStr"/>
+      <c r="B41" s="38" t="n">
+        <v>180</v>
+      </c>
       <c r="C41" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3791,17 +3796,15 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B42" s="33" t="n">
-        <v>215</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B42" s="33" t="inlineStr"/>
       <c r="C42" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3814,12 +3817,12 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3827,9 +3830,7 @@
       <c r="A43" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B43" s="38" t="n">
-        <v>205</v>
-      </c>
+      <c r="B43" s="38" t="inlineStr"/>
       <c r="C43" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3847,7 +3848,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3855,7 +3856,9 @@
       <c r="A44" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B44" s="33" t="inlineStr"/>
+      <c r="B44" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3873,7 +3876,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3882,11 +3885,11 @@
         <v>46142</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C45" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C45" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D45" s="42" t="inlineStr">
@@ -3896,12 +3899,12 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3910,7 +3913,7 @@
         <v>46142</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>200</v>
+        <v>95</v>
       </c>
       <c r="C46" s="47" t="inlineStr">
         <is>
@@ -3929,16 +3932,16 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C47" s="53" t="inlineStr">
         <is>
@@ -3957,7 +3960,7 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4 “White Varsity Red”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3969,7 @@
         <v>46143</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C48" s="47" t="inlineStr">
         <is>
@@ -3985,7 +3988,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Air Zoom Huarache 2K4 “White Varsity Red”</t>
         </is>
       </c>
     </row>
@@ -3994,7 +3997,7 @@
         <v>46143</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>190</v>
+        <v>135</v>
       </c>
       <c r="C49" s="53" t="inlineStr">
         <is>
@@ -4013,20 +4016,20 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C50" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C50" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D50" s="41" t="inlineStr">
@@ -4036,12 +4039,12 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
@@ -4050,11 +4053,11 @@
         <v>46144</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C51" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C51" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4064,25 +4067,25 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C52" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C52" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D52" s="41" t="inlineStr">
@@ -4097,16 +4100,16 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46150</v>
+        <v>46149</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -4125,7 +4128,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4137,7 @@
         <v>46150</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
@@ -4153,7 +4156,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -4164,9 +4167,9 @@
       <c r="B55" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C55" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="C55" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D55" s="42" t="inlineStr">
@@ -4181,20 +4184,20 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C56" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C56" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D56" s="41" t="inlineStr">
@@ -4209,7 +4212,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4221,7 @@
         <v>46151</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
@@ -4232,12 +4235,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4249,7 @@
         <v>46151</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>120</v>
+        <v>195</v>
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
@@ -4260,12 +4263,12 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -4274,26 +4277,26 @@
         <v>46151</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>230</v>
+        <v>120</v>
       </c>
       <c r="C59" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D59" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D59" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -4302,16 +4305,16 @@
         <v>46151</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C60" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D60" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>230</v>
+      </c>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D60" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E60" s="30" t="inlineStr">
@@ -4321,35 +4324,35 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C61" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D61" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C61" s="58" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D61" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -4358,11 +4361,11 @@
         <v>46157</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C62" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C62" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D62" s="41" t="inlineStr">
@@ -4377,16 +4380,16 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C63" s="37" t="inlineStr">
         <is>
@@ -4400,12 +4403,12 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
@@ -4414,11 +4417,11 @@
         <v>46158</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C64" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>145</v>
+      </c>
+      <c r="C64" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D64" s="41" t="inlineStr">
@@ -4428,25 +4431,25 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46164</v>
+        <v>46158</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C65" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>160</v>
+      </c>
+      <c r="C65" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D65" s="42" t="inlineStr">
@@ -4456,25 +4459,25 @@
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46165</v>
+        <v>46164</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C66" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C66" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D66" s="41" t="inlineStr">
@@ -4484,12 +4487,12 @@
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
@@ -4517,16 +4520,16 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46168</v>
+        <v>46165</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="C68" s="40" t="inlineStr">
         <is>
@@ -4540,21 +4543,21 @@
       </c>
       <c r="E68" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="36" t="n">
-        <v>46171</v>
+        <v>46168</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C69" s="37" t="inlineStr">
         <is>
@@ -4573,7 +4576,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
@@ -4582,11 +4585,11 @@
         <v>46171</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C70" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C70" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D70" s="41" t="inlineStr">
@@ -4601,7 +4604,7 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4610,11 +4613,11 @@
         <v>46171</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C71" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C71" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D71" s="42" t="inlineStr">
@@ -4629,18 +4632,20 @@
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B72" s="33" t="inlineStr"/>
-      <c r="C72" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>46171</v>
+      </c>
+      <c r="B72" s="33" t="n">
+        <v>240</v>
+      </c>
+      <c r="C72" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D72" s="41" t="inlineStr">
@@ -4650,12 +4655,12 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -4663,12 +4668,10 @@
       <c r="A73" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B73" s="38" t="n">
-        <v>250</v>
-      </c>
-      <c r="C73" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B73" s="38" t="inlineStr"/>
+      <c r="C73" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
@@ -4678,12 +4681,12 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4694,9 @@
       <c r="A74" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B74" s="33" t="inlineStr"/>
+      <c r="B74" s="33" t="n">
+        <v>250</v>
+      </c>
       <c r="C74" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4704,25 +4709,23 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B75" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C75" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46172</v>
+      </c>
+      <c r="B75" s="38" t="inlineStr"/>
+      <c r="C75" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D75" s="42" t="inlineStr">
@@ -4732,21 +4735,21 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46177</v>
+        <v>46173</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="C76" s="47" t="inlineStr">
         <is>
@@ -4765,18 +4768,20 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B77" s="38" t="inlineStr"/>
-      <c r="C77" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46177</v>
+      </c>
+      <c r="B77" s="38" t="n">
+        <v>140</v>
+      </c>
+      <c r="C77" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D77" s="42" t="inlineStr">
@@ -4786,22 +4791,20 @@
       </c>
       <c r="E77" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B78" s="33" t="n">
-        <v>355</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B78" s="33" t="inlineStr"/>
       <c r="C78" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4819,20 +4822,20 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C79" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>355</v>
+      </c>
+      <c r="C79" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4842,12 +4845,12 @@
       </c>
       <c r="E79" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -4903,25 +4906,25 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="31" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C82" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D82" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>170</v>
+      </c>
+      <c r="C82" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D82" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E82" s="30" t="inlineStr">
@@ -4931,7 +4934,7 @@
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -4940,11 +4943,11 @@
         <v>46186</v>
       </c>
       <c r="B83" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C83" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C83" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D83" s="42" t="inlineStr">
@@ -4954,12 +4957,12 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -4968,16 +4971,16 @@
         <v>46186</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C84" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D84" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C84" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D84" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E84" s="30" t="inlineStr">
@@ -4987,7 +4990,7 @@
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -4996,11 +4999,11 @@
         <v>46186</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C85" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C85" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D85" s="42" t="inlineStr">
@@ -5010,12 +5013,12 @@
       </c>
       <c r="E85" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -5024,16 +5027,16 @@
         <v>46186</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>155</v>
+        <v>210</v>
       </c>
       <c r="C86" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D86" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D86" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E86" s="30" t="inlineStr">
@@ -5043,16 +5046,16 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="36" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="C87" s="53" t="inlineStr">
         <is>
@@ -5071,20 +5074,20 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C88" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C88" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D88" s="41" t="inlineStr">
@@ -5099,7 +5102,7 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
@@ -5161,14 +5164,14 @@
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C91" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>162</v>
+      </c>
+      <c r="C91" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D91" s="42" t="inlineStr">
@@ -5183,7 +5186,7 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
@@ -5211,20 +5214,20 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C93" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C93" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D93" s="42" t="inlineStr">
@@ -5239,7 +5242,7 @@
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5250,9 @@
       <c r="A94" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B94" s="33" t="inlineStr"/>
+      <c r="B94" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C94" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5260,12 +5265,12 @@
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -5274,16 +5279,16 @@
         <v>46200</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="C95" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D95" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D95" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
@@ -5293,7 +5298,7 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -5301,9 +5306,7 @@
       <c r="A96" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B96" s="33" t="n">
-        <v>185</v>
-      </c>
+      <c r="B96" s="33" t="inlineStr"/>
       <c r="C96" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5321,7 +5324,7 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -5329,10 +5332,12 @@
       <c r="A97" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B97" s="38" t="inlineStr"/>
-      <c r="C97" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B97" s="38" t="n">
+        <v>120</v>
+      </c>
+      <c r="C97" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D97" s="57" t="inlineStr">
@@ -5342,12 +5347,12 @@
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5361,7 @@
         <v>46200</v>
       </c>
       <c r="B98" s="33" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C98" s="40" t="inlineStr">
         <is>
@@ -5370,25 +5375,23 @@
       </c>
       <c r="E98" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="A99" s="36" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B99" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C99" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46200</v>
+      </c>
+      <c r="B99" s="38" t="inlineStr"/>
+      <c r="C99" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D99" s="57" t="inlineStr">
@@ -5398,30 +5401,30 @@
       </c>
       <c r="E99" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F99" s="35" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="31" t="n">
-        <v>46206</v>
+        <v>46203</v>
       </c>
       <c r="B100" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C100" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D100" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>135</v>
+      </c>
+      <c r="C100" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D100" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E100" s="30" t="inlineStr">
@@ -5431,40 +5434,68 @@
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Animal Instinct”</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="36" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B101" s="38" t="n">
+        <v>130</v>
+      </c>
+      <c r="C101" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D101" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E101" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F101" s="35" t="inlineStr">
+        <is>
+          <t>Nike Ja 3 “Animal Instinct”</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15" customHeight="1">
+      <c r="A102" s="31" t="n">
         <v>46210</v>
       </c>
-      <c r="B101" s="38" t="n">
+      <c r="B102" s="33" t="n">
         <v>210</v>
       </c>
-      <c r="C101" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D101" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E101" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F101" s="35" t="inlineStr">
+      <c r="C102" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D102" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E102" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F102" s="30" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F101"/>
+  <autoFilter ref="A3:F102"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5479,7 +5510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5505,7 +5536,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 08, 2026  ·  07:25 UTC</t>
+          <t>Generated April 09, 2026  ·  07:27 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5885,7 +5916,7 @@
         <v>46126</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
@@ -5904,7 +5935,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
@@ -5913,16 +5944,16 @@
         <v>46126</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D17" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
@@ -5932,25 +5963,25 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46129</v>
+        <v>46128</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>235</v>
+        <v>200</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D18" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D18" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
@@ -5960,16 +5991,16 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Palace x Nike Air Max 95</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46130</v>
+        <v>46129</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
@@ -5988,16 +6019,16 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46135</v>
+        <v>46130</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -6011,40 +6042,40 @@
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46136</v>
+        <v>46135</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6084,7 @@
         <v>46136</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
@@ -6072,41 +6103,41 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D23" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B24" s="33" t="n">
         <v>200</v>
@@ -6123,21 +6154,21 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
@@ -6156,7 +6187,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
@@ -6164,7 +6195,9 @@
       <c r="A26" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B26" s="33" t="inlineStr"/>
+      <c r="B26" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6177,21 +6210,21 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C27" s="37" t="inlineStr">
         <is>
@@ -6210,16 +6243,16 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>The Whitaker Group x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>205</v>
+        <v>180</v>
       </c>
       <c r="C28" s="40" t="inlineStr">
         <is>
@@ -6233,18 +6266,18 @@
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B29" s="38" t="inlineStr"/>
       <c r="C29" s="37" t="inlineStr">
@@ -6259,22 +6292,20 @@
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46144</v>
-      </c>
-      <c r="B30" s="33" t="n">
-        <v>220</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B30" s="33" t="inlineStr"/>
       <c r="C30" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6292,16 +6323,16 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46149</v>
+        <v>46142</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
@@ -6315,21 +6346,21 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46150</v>
+        <v>46142</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -6343,21 +6374,21 @@
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46150</v>
+        <v>46144</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
@@ -6371,21 +6402,21 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46151</v>
+        <v>46149</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -6404,16 +6435,16 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C35" s="37" t="inlineStr">
         <is>
@@ -6427,21 +6458,21 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>120</v>
+        <v>210</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
@@ -6460,7 +6491,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -6469,26 +6500,26 @@
         <v>46151</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D37" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6497,16 +6528,16 @@
         <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C38" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D38" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>195</v>
+      </c>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D38" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
@@ -6516,16 +6547,16 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
@@ -6544,25 +6575,25 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46158</v>
+        <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>145</v>
+        <v>230</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D40" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D40" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
@@ -6572,25 +6603,25 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46165</v>
+        <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C41" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D41" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C41" s="58" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
@@ -6600,16 +6631,16 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46165</v>
+        <v>46157</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -6623,21 +6654,21 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46168</v>
+        <v>46158</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>235</v>
+        <v>145</v>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
@@ -6651,21 +6682,21 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
@@ -6679,21 +6710,21 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46171</v>
+        <v>46165</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C45" s="37" t="inlineStr">
         <is>
@@ -6707,21 +6738,21 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46172</v>
+        <v>46168</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>250</v>
+        <v>235</v>
       </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
@@ -6740,15 +6771,17 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B47" s="38" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="B47" s="38" t="n">
+        <v>240</v>
+      </c>
       <c r="C47" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6761,20 +6794,22 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B48" s="33" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="B48" s="33" t="n">
+        <v>240</v>
+      </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6787,21 +6822,21 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46182</v>
+        <v>46172</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>355</v>
+        <v>250</v>
       </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
@@ -6815,50 +6850,46 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B50" s="33" t="n">
-        <v>150</v>
-      </c>
+        <v>46172</v>
+      </c>
+      <c r="B50" s="33" t="inlineStr"/>
       <c r="C50" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D50" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D50" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B51" s="38" t="n">
-        <v>205</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B51" s="38" t="inlineStr"/>
       <c r="C51" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6876,16 +6907,16 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46193</v>
+        <v>46182</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>150</v>
+        <v>355</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
@@ -6899,21 +6930,21 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -6932,25 +6963,25 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46200</v>
+        <v>46186</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D54" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E54" s="30" t="inlineStr">
@@ -6960,15 +6991,17 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B55" s="38" t="inlineStr"/>
+        <v>46193</v>
+      </c>
+      <c r="B55" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6986,25 +7019,25 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46200</v>
+        <v>46193</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>120</v>
+        <v>162</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D56" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
@@ -7014,7 +7047,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7056,7 @@
         <v>46200</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
@@ -7037,12 +7070,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -7051,7 +7084,7 @@
         <v>46200</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
@@ -7070,68 +7103,150 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B59" s="38" t="n">
-        <v>135</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B59" s="38" t="inlineStr"/>
       <c r="C59" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D59" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D59" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B60" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D60" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E60" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F60" s="30" t="inlineStr">
+        <is>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15" customHeight="1">
+      <c r="A61" s="36" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B61" s="38" t="n">
+        <v>185</v>
+      </c>
+      <c r="C61" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D61" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E61" s="35" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F61" s="35" t="inlineStr">
+        <is>
+          <t>Air Jordan 1 High OG “Workwear”</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15" customHeight="1">
+      <c r="A62" s="31" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B62" s="33" t="n">
+        <v>135</v>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D62" s="56" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E62" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F62" s="30" t="inlineStr">
+        <is>
+          <t>Bluetile x Nike SB Dunk Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15" customHeight="1">
+      <c r="A63" s="36" t="n">
         <v>46210</v>
       </c>
-      <c r="B60" s="33" t="n">
+      <c r="B63" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C60" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D60" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E60" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F60" s="30" t="inlineStr">
+      <c r="C63" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D63" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E63" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F63" s="35" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F60"/>
+  <autoFilter ref="A3:F63"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-10 07:46 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -657,6 +657,9 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -685,19 +688,16 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1596,7 +1596,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 09, 2026  ·  07:27 UTC</t>
+          <t>Generated April 10, 2026  ·  07:46 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1636,15 +1636,15 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
@@ -1752,7 +1752,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
         </is>
       </c>
       <c r="B12" s="30" t="inlineStr">
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="C12" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="D12" s="30" t="n">
         <v>0</v>
@@ -1831,7 +1831,7 @@
         <v>7</v>
       </c>
       <c r="G12" s="33" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="H12" s="41" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
       <c r="B13" s="35" t="inlineStr">
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="C13" s="36" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="D13" s="35" t="n">
         <v>0</v>
@@ -1865,7 +1865,7 @@
         <v>7</v>
       </c>
       <c r="G13" s="38" t="n">
-        <v>120</v>
+        <v>235</v>
       </c>
       <c r="H13" s="42" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="C14" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="D14" s="30" t="n">
         <v>0</v>
@@ -1899,7 +1899,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="H14" s="41" t="inlineStr">
         <is>
@@ -1910,7 +1910,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="C15" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="D15" s="35" t="n">
         <v>1</v>
@@ -1933,27 +1933,27 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="H15" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="H15" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C16" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="D16" s="30" t="n">
         <v>1</v>
@@ -1967,7 +1967,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="H16" s="41" t="inlineStr">
         <is>
@@ -2023,13 +2023,13 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="43" t="inlineStr">
+      <c r="A20" s="44" t="inlineStr">
         <is>
           <t>Nike</t>
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2039,23 +2039,23 @@
       <c r="E20" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="44" t="inlineStr">
+      <c r="G20" s="45" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="45" t="inlineStr">
+      <c r="A21" s="46" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D21" s="37" t="inlineStr">
         <is>
@@ -2063,19 +2063,19 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>59</v>
-      </c>
-      <c r="G21" s="46" t="inlineStr">
+        <v>61</v>
+      </c>
+      <c r="G21" s="47" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
       <c r="H21" s="35" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="43" t="inlineStr">
+      <c r="A22" s="44" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
@@ -2083,15 +2083,15 @@
       <c r="B22" s="30" t="n">
         <v>7</v>
       </c>
-      <c r="D22" s="47" t="inlineStr">
+      <c r="D22" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>33</v>
-      </c>
-      <c r="G22" s="48" t="inlineStr">
+        <v>36</v>
+      </c>
+      <c r="G22" s="49" t="inlineStr">
         <is>
           <t>Raffle/Dropship</t>
         </is>
@@ -2101,7 +2101,7 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="D23" s="49" t="inlineStr">
+      <c r="D23" s="50" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2109,7 +2109,7 @@
       <c r="E23" s="35" t="n">
         <v>6</v>
       </c>
-      <c r="G23" s="50" t="inlineStr">
+      <c r="G23" s="51" t="inlineStr">
         <is>
           <t>Confirmed App</t>
         </is>
@@ -2168,17 +2168,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/9 – 4/15</t>
+          <t>4/10 – 4/16</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D27" s="40" t="n">
         <v>14</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/16 – 4/22</t>
+          <t>4/17 – 4/23</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
@@ -2199,7 +2199,7 @@
         <v>3</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.1</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2210,17 +2210,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/23 – 4/29</t>
+          <t>4/24 – 4/30</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D29" s="40" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2231,17 +2231,17 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>4/30 – 5/6</t>
+          <t>5/1 – 5/7</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D30" s="37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2252,14 +2252,14 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/7 – 5/13</t>
+          <t>5/8 – 5/14</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D31" s="40" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>6.9</v>
@@ -2273,17 +2273,17 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/14 – 5/20</t>
+          <t>5/15 – 5/21</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D32" s="37" t="n">
         <v>2</v>
       </c>
       <c r="E32" s="35" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2294,17 +2294,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/21 – 5/27</t>
+          <t>5/22 – 5/28</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D33" s="40" t="n">
         <v>3</v>
       </c>
       <c r="E33" s="30" t="n">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2315,17 +2315,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/28 – 6/3</t>
+          <t>5/29 – 6/4</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D34" s="37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2336,17 +2336,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>6/4 – 6/10</t>
+          <t>6/5 – 6/11</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D35" s="40" t="n">
         <v>2</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2357,17 +2357,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/11 – 6/17</t>
+          <t>6/12 – 6/18</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D36" s="37" t="n">
         <v>2</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2378,17 +2378,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/18 – 6/24</t>
+          <t>6/19 – 6/25</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D37" s="40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/25 – 7/1</t>
+          <t>6/26 – 7/2</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>7/2 – 7/8</t>
+          <t>7/3 – 7/9</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2480,42 +2480,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="51" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="B1" s="51" t="inlineStr">
+      <c r="B1" s="52" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="D1" s="51" t="inlineStr">
+      <c r="D1" s="52" t="inlineStr">
         <is>
           <t>Hype Level</t>
         </is>
       </c>
-      <c r="E1" s="51" t="inlineStr">
+      <c r="E1" s="52" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="G1" s="51" t="inlineStr">
+      <c r="G1" s="52" t="inlineStr">
         <is>
           <t>Sale Method</t>
         </is>
       </c>
-      <c r="H1" s="51" t="inlineStr">
+      <c r="H1" s="52" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="J1" s="51" t="inlineStr">
+      <c r="J1" s="52" t="inlineStr">
         <is>
           <t>Price Range</t>
         </is>
       </c>
-      <c r="K1" s="51" t="inlineStr">
+      <c r="K1" s="52" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
@@ -2528,7 +2528,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2570,7 +2570,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2578,7 +2578,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -2646,7 +2646,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -2671,7 +2671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2695,9 +2695,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="52" t="inlineStr">
-        <is>
-          <t>Generated April 09, 2026  ·  07:27 UTC</t>
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>Generated April 10, 2026  ·  07:46 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2740,38 +2740,38 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C4" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D4" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C4" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D4" s="55" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C5" s="37" t="inlineStr">
         <is>
@@ -2790,20 +2790,20 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C6" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C6" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D6" s="41" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
     </row>
@@ -2827,11 +2827,11 @@
         <v>46122</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C7" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D7" s="42" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
         <v>46122</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -2883,11 +2883,11 @@
         <v>46122</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C9" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C9" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D9" s="42" t="inlineStr">
@@ -2902,44 +2902,44 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B10" s="33" t="n">
         <v>200</v>
       </c>
-      <c r="C10" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D10" s="55" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D10" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Hellstar x adidas Superstar “Hazy Orange”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
@@ -2953,23 +2953,23 @@
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C12" s="47" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C12" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2981,25 +2981,25 @@
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
+          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C13" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C13" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D13" s="42" t="inlineStr">
@@ -3009,53 +3009,53 @@
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>adidas Anthony Edwards 2 “Glow”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C14" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D14" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>adidas Harden Vol. 10 “Marathon”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>140</v>
-      </c>
-      <c r="C15" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D15" s="42" t="inlineStr">
@@ -3065,53 +3065,51 @@
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46124</v>
-      </c>
-      <c r="B16" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C16" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D16" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B16" s="33" t="inlineStr"/>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D16" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Glow”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C17" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -3121,12 +3119,12 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Marathon”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -3134,15 +3132,17 @@
       <c r="A18" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B18" s="33" t="inlineStr"/>
+      <c r="B18" s="33" t="n">
+        <v>220</v>
+      </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D18" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D18" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
@@ -3152,25 +3152,25 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>190</v>
+        <v>130</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D19" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D19" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
@@ -3180,25 +3180,25 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D20" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D20" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
@@ -3208,20 +3208,20 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C21" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>110</v>
+      </c>
+      <c r="C21" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D21" s="42" t="inlineStr">
@@ -3236,23 +3236,23 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C22" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D22" s="56" t="inlineStr">
+        <v>100</v>
+      </c>
+      <c r="C22" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D22" s="57" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3264,25 +3264,25 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Nike V5 RNR “Jackie Robinson Day”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
@@ -3292,20 +3292,20 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Caitlin Clark Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>110</v>
-      </c>
-      <c r="C24" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D24" s="41" t="inlineStr">
@@ -3320,23 +3320,23 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>100</v>
-      </c>
-      <c r="C25" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D25" s="57" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C25" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D25" s="43" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike V5 RNR “Jackie Robinson Day”</t>
+          <t>Palace x Nike Air Max 95</t>
         </is>
       </c>
     </row>
@@ -3357,39 +3357,39 @@
         <v>46128</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C26" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D26" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C26" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D26" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Palace x Nike Air Max 95</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C27" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C27" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D27" s="42" t="inlineStr">
@@ -3399,12 +3399,12 @@
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
@@ -3413,11 +3413,11 @@
         <v>46129</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C28" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D28" s="41" t="inlineStr">
@@ -3432,25 +3432,25 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C29" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D29" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C29" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D29" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
@@ -3494,19 +3494,19 @@
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C31" s="53" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C31" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D31" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D31" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
@@ -3516,20 +3516,20 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C32" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C32" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D32" s="41" t="inlineStr">
@@ -3539,12 +3539,12 @@
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -3553,11 +3553,11 @@
         <v>46135</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C33" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D33" s="42" t="inlineStr">
@@ -3567,25 +3567,25 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Homecoming x Nike Air Max Plus</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C34" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C34" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D34" s="41" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Homecoming x Nike Air Max Plus</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3609,16 +3609,16 @@
         <v>46136</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C35" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D35" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D35" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -3644,9 +3644,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D36" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
         <v>46136</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
@@ -3684,17 +3684,15 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B38" s="33" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B38" s="33" t="inlineStr"/>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3712,7 +3710,7 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3800,7 @@
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B42" s="33" t="inlineStr"/>
       <c r="C42" s="40" t="inlineStr">
@@ -3817,12 +3815,12 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3828,9 @@
       <c r="A43" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B43" s="38" t="inlineStr"/>
+      <c r="B43" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3857,7 +3857,7 @@
         <v>46142</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3885,11 +3885,11 @@
         <v>46142</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C45" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>95</v>
+      </c>
+      <c r="C45" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D45" s="42" t="inlineStr">
@@ -3899,12 +3899,12 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -3913,9 +3913,9 @@
         <v>46142</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>95</v>
-      </c>
-      <c r="C46" s="47" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C46" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3932,20 +3932,20 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C47" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>165</v>
+      </c>
+      <c r="C47" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D47" s="42" t="inlineStr">
@@ -3955,12 +3955,12 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Air Jordan 4 GS “Black Infrared 23”</t>
         </is>
       </c>
     </row>
@@ -3969,9 +3969,9 @@
         <v>46143</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C48" s="47" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C48" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4 “White Varsity Red”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
@@ -3997,9 +3997,9 @@
         <v>46143</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C49" s="53" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C49" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4016,20 +4016,20 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C50" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D50" s="41" t="inlineStr">
@@ -4039,12 +4039,12 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4053,11 +4053,11 @@
         <v>46144</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="C51" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C51" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4067,25 +4067,25 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C52" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D52" s="41" t="inlineStr">
@@ -4100,16 +4100,16 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -4137,7 +4137,7 @@
         <v>46150</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
@@ -4156,7 +4156,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -4167,9 +4167,9 @@
       <c r="B55" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C55" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C55" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D55" s="42" t="inlineStr">
@@ -4184,35 +4184,35 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C56" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D56" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C56" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D56" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -4277,26 +4277,26 @@
         <v>46151</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>120</v>
+        <v>230</v>
       </c>
       <c r="C59" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D59" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D59" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
         </is>
       </c>
     </row>
@@ -4305,54 +4305,54 @@
         <v>46151</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>230</v>
+        <v>120</v>
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D60" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D60" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C61" s="58" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D61" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>170</v>
+      </c>
+      <c r="C61" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D61" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
@@ -4361,11 +4361,11 @@
         <v>46157</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C62" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D62" s="41" t="inlineStr">
@@ -4380,16 +4380,16 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C63" s="37" t="inlineStr">
         <is>
@@ -4403,12 +4403,12 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
@@ -4417,11 +4417,11 @@
         <v>46158</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C64" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C64" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D64" s="41" t="inlineStr">
@@ -4431,40 +4431,40 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46158</v>
+        <v>46163</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C65" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D65" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C65" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D65" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Air Max Mad 90 Pack</t>
         </is>
       </c>
     </row>
@@ -4475,7 +4475,7 @@
       <c r="B66" s="33" t="n">
         <v>170</v>
       </c>
-      <c r="C66" s="47" t="inlineStr">
+      <c r="C66" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4582,14 +4582,14 @@
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46171</v>
+        <v>46170</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C70" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>150</v>
+      </c>
+      <c r="C70" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D70" s="41" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Book 2 “Haven and Hector”</t>
         </is>
       </c>
     </row>
@@ -4613,11 +4613,11 @@
         <v>46171</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C71" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C71" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D71" s="42" t="inlineStr">
@@ -4632,7 +4632,7 @@
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4641,11 +4641,11 @@
         <v>46171</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C72" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C72" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D72" s="41" t="inlineStr">
@@ -4660,18 +4660,20 @@
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B73" s="38" t="inlineStr"/>
-      <c r="C73" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>46171</v>
+      </c>
+      <c r="B73" s="38" t="n">
+        <v>240</v>
+      </c>
+      <c r="C73" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
@@ -4681,12 +4683,12 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -4746,14 +4748,14 @@
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C76" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C76" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D76" s="41" t="inlineStr">
@@ -4768,20 +4770,18 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B77" s="38" t="n">
-        <v>140</v>
-      </c>
-      <c r="C77" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46172</v>
+      </c>
+      <c r="B77" s="38" t="inlineStr"/>
+      <c r="C77" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D77" s="42" t="inlineStr">
@@ -4791,23 +4791,25 @@
       </c>
       <c r="E77" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B78" s="33" t="inlineStr"/>
-      <c r="C78" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46173</v>
+      </c>
+      <c r="B78" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C78" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D78" s="41" t="inlineStr">
@@ -4817,25 +4819,25 @@
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46182</v>
+        <v>46177</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>355</v>
-      </c>
-      <c r="C79" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C79" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4845,25 +4847,23 @@
       </c>
       <c r="E79" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B80" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C80" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B80" s="33" t="inlineStr"/>
+      <c r="C80" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D80" s="41" t="inlineStr">
@@ -4873,25 +4873,25 @@
       </c>
       <c r="E80" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="B81" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C81" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>355</v>
+      </c>
+      <c r="C81" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D81" s="42" t="inlineStr">
@@ -4901,12 +4901,12 @@
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
       <c r="B82" s="33" t="n">
         <v>170</v>
       </c>
-      <c r="C82" s="47" t="inlineStr">
+      <c r="C82" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4934,20 +4934,20 @@
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="36" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B83" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C83" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C83" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D83" s="42" t="inlineStr">
@@ -4957,30 +4957,30 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C84" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D84" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>170</v>
+      </c>
+      <c r="C84" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D84" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E84" s="30" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -5001,14 +5001,14 @@
       <c r="B85" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C85" s="53" t="inlineStr">
+      <c r="C85" s="56" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D85" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D85" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E85" s="35" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -5027,16 +5027,16 @@
         <v>46186</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C86" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D86" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C86" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D86" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E86" s="30" t="inlineStr">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -5055,11 +5055,11 @@
         <v>46186</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C87" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C87" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D87" s="42" t="inlineStr">
@@ -5069,23 +5069,23 @@
       </c>
       <c r="E87" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C88" s="47" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C88" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5102,20 +5102,20 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C89" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C89" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D89" s="42" t="inlineStr">
@@ -5125,30 +5125,30 @@
       </c>
       <c r="E89" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Air More Uptempo “Legacy”</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C90" s="47" t="inlineStr">
+        <v>155</v>
+      </c>
+      <c r="C90" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D90" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D90" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5158,20 +5158,20 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>162</v>
-      </c>
-      <c r="C91" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C91" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D91" s="42" t="inlineStr">
@@ -5186,25 +5186,25 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C92" s="47" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C92" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D92" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D92" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E92" s="30" t="inlineStr">
@@ -5214,20 +5214,20 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C93" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>162</v>
+      </c>
+      <c r="C93" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D93" s="42" t="inlineStr">
@@ -5242,25 +5242,25 @@
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="31" t="n">
-        <v>46200</v>
+        <v>46193</v>
       </c>
       <c r="B94" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C94" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D94" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C94" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D94" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
@@ -5270,16 +5270,16 @@
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Nike SB P-Rod 1 Black Gum</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="36" t="n">
-        <v>46200</v>
+        <v>46193</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="C95" s="37" t="inlineStr">
         <is>
@@ -5298,15 +5298,17 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="A96" s="31" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B96" s="33" t="inlineStr"/>
+        <v>46193</v>
+      </c>
+      <c r="B96" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C96" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5324,25 +5326,25 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="36" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B97" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C97" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D97" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>180</v>
+      </c>
+      <c r="C97" s="56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D97" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E97" s="35" t="inlineStr">
@@ -5352,20 +5354,20 @@
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" s="31" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B98" s="33" t="n">
-        <v>185</v>
-      </c>
-      <c r="C98" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C98" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D98" s="41" t="inlineStr">
@@ -5375,12 +5377,12 @@
       </c>
       <c r="E98" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
@@ -5388,15 +5390,17 @@
       <c r="A99" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B99" s="38" t="inlineStr"/>
-      <c r="C99" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D99" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B99" s="38" t="n">
+        <v>185</v>
+      </c>
+      <c r="C99" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D99" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E99" s="35" t="inlineStr">
@@ -5406,53 +5410,51 @@
       </c>
       <c r="F99" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="31" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B100" s="33" t="n">
-        <v>135</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B100" s="33" t="inlineStr"/>
       <c r="C100" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D100" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D100" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E100" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="36" t="n">
-        <v>46206</v>
+        <v>46200</v>
       </c>
       <c r="B101" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C101" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D101" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>120</v>
+      </c>
+      <c r="C101" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D101" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E101" s="35" t="inlineStr">
@@ -5462,40 +5464,178 @@
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Animal Instinct”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="31" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B102" s="33" t="inlineStr"/>
+      <c r="C102" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D102" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E102" s="30" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F102" s="30" t="inlineStr">
+        <is>
+          <t>Air Jordan 7 “Miro” 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="15" customHeight="1">
+      <c r="A103" s="36" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B103" s="38" t="n">
+        <v>190</v>
+      </c>
+      <c r="C103" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D103" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E103" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F103" s="35" t="inlineStr">
+        <is>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="15" customHeight="1">
+      <c r="A104" s="31" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B104" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C104" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D104" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E104" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F104" s="30" t="inlineStr">
+        <is>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="15" customHeight="1">
+      <c r="A105" s="36" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B105" s="38" t="n">
+        <v>135</v>
+      </c>
+      <c r="C105" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D105" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E105" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F105" s="35" t="inlineStr">
+        <is>
+          <t>Bluetile x Nike SB Dunk Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="15" customHeight="1">
+      <c r="A106" s="31" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B106" s="33" t="n">
+        <v>130</v>
+      </c>
+      <c r="C106" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D106" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E106" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F106" s="30" t="inlineStr">
+        <is>
+          <t>Nike Ja 3 “Animal Instinct”</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15" customHeight="1">
+      <c r="A107" s="36" t="n">
         <v>46210</v>
       </c>
-      <c r="B102" s="33" t="n">
+      <c r="B107" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C102" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D102" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E102" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F102" s="30" t="inlineStr">
+      <c r="C107" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D107" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E107" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F107" s="35" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F102"/>
+  <autoFilter ref="A3:F107"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5510,7 +5650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5534,9 +5674,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="52" t="inlineStr">
-        <is>
-          <t>Generated April 09, 2026  ·  07:27 UTC</t>
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>Generated April 10, 2026  ·  07:46 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5579,10 +5719,10 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C4" s="40" t="inlineStr">
         <is>
@@ -5601,16 +5741,16 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Topaz Gold”</t>
+          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>120</v>
+        <v>235</v>
       </c>
       <c r="C5" s="37" t="inlineStr">
         <is>
@@ -5629,16 +5769,16 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Dark Team Red”</t>
+          <t>Nike LeBron 23 “For The Record”</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
@@ -5657,25 +5797,25 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Patent “Mystic Navy”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="36" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>235</v>
+        <v>200</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D7" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
@@ -5685,16 +5825,16 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “For The Record”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -5708,21 +5848,21 @@
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
@@ -5741,53 +5881,51 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Ja Morant x Nike Air Force 1 Low “Denim”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46123</v>
-      </c>
-      <c r="B10" s="33" t="n">
-        <v>185</v>
-      </c>
+        <v>46125</v>
+      </c>
+      <c r="B10" s="33" t="inlineStr"/>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D10" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -5797,7 +5935,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5805,15 +5943,17 @@
       <c r="A12" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B12" s="33" t="inlineStr"/>
+      <c r="B12" s="33" t="n">
+        <v>220</v>
+      </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
@@ -5823,25 +5963,25 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>190</v>
+        <v>130</v>
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D13" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -5851,25 +5991,25 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D14" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -5879,16 +6019,16 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46125</v>
+        <v>46127</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="C15" s="37" t="inlineStr">
         <is>
@@ -5907,25 +6047,25 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Caitlin Clark Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -5935,23 +6075,23 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="57" t="inlineStr">
+      <c r="D17" s="43" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5963,25 +6103,25 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Palace x Nike Air Max 95</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D18" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D18" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
@@ -5991,16 +6131,16 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Palace x Nike Air Max 95</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
@@ -6019,16 +6159,16 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46130</v>
+        <v>46135</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -6042,21 +6182,21 @@
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
@@ -6070,12 +6210,12 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -6084,16 +6224,16 @@
         <v>46136</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D22" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -6103,7 +6243,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
         </is>
       </c>
     </row>
@@ -6119,9 +6259,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="57" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
@@ -6131,7 +6271,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -6140,7 +6280,7 @@
         <v>46136</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
@@ -6159,17 +6299,15 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B25" s="38" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B25" s="38" t="inlineStr"/>
       <c r="C25" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6187,7 +6325,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -6277,7 +6415,7 @@
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B29" s="38" t="inlineStr"/>
       <c r="C29" s="37" t="inlineStr">
@@ -6292,12 +6430,12 @@
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -6305,7 +6443,9 @@
       <c r="A30" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B30" s="33" t="inlineStr"/>
+      <c r="B30" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6323,7 +6463,7 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6472,7 @@
         <v>46142</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
@@ -6351,16 +6491,16 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>205</v>
+        <v>165</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -6379,7 +6519,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 4 GS “Black Infrared 23”</t>
         </is>
       </c>
     </row>
@@ -6500,26 +6640,26 @@
         <v>46151</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C37" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D37" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C37" s="58" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D37" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -6528,7 +6668,7 @@
         <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -6542,12 +6682,12 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6696,7 @@
         <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>120</v>
+        <v>195</v>
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
@@ -6570,12 +6710,12 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6731,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D40" s="56" t="inlineStr">
+      <c r="D40" s="57" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -6612,26 +6752,26 @@
         <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C41" s="58" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D41" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>120</v>
+      </c>
+      <c r="C41" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D41" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -6887,9 +7027,11 @@
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B51" s="38" t="inlineStr"/>
+        <v>46172</v>
+      </c>
+      <c r="B51" s="38" t="n">
+        <v>120</v>
+      </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6902,22 +7044,20 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B52" s="33" t="n">
-        <v>355</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B52" s="33" t="inlineStr"/>
       <c r="C52" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6935,16 +7075,16 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46186</v>
+        <v>46182</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>205</v>
+        <v>355</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -6963,7 +7103,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -6997,10 +7137,10 @@
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
@@ -7019,7 +7159,7 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -7053,10 +7193,10 @@
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46200</v>
+        <v>46193</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
@@ -7075,16 +7215,16 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46200</v>
+        <v>46193</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>170</v>
+        <v>215</v>
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
@@ -7098,12 +7238,12 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -7111,7 +7251,9 @@
       <c r="A59" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B59" s="38" t="inlineStr"/>
+      <c r="B59" s="38" t="n">
+        <v>185</v>
+      </c>
       <c r="C59" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -7129,7 +7271,7 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -7137,27 +7279,25 @@
       <c r="A60" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B60" s="33" t="n">
-        <v>120</v>
-      </c>
+      <c r="B60" s="33" t="inlineStr"/>
       <c r="C60" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D60" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D60" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -7166,44 +7306,44 @@
         <v>46200</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>185</v>
+        <v>120</v>
       </c>
       <c r="C61" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D61" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D61" s="43" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46203</v>
+        <v>46200</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C62" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D62" s="56" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D62" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
@@ -7213,40 +7353,96 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B63" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C63" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D63" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E63" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F63" s="35" t="inlineStr">
+        <is>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15" customHeight="1">
+      <c r="A64" s="31" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B64" s="33" t="n">
+        <v>135</v>
+      </c>
+      <c r="C64" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D64" s="57" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E64" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F64" s="30" t="inlineStr">
+        <is>
+          <t>Bluetile x Nike SB Dunk Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="15" customHeight="1">
+      <c r="A65" s="36" t="n">
         <v>46210</v>
       </c>
-      <c r="B63" s="38" t="n">
+      <c r="B65" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C63" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D63" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E63" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F63" s="35" t="inlineStr">
+      <c r="C65" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D65" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E65" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F65" s="35" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F63"/>
+  <autoFilter ref="A3:F65"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-12 07:19 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -654,9 +654,6 @@
     <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -683,6 +680,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1581,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 11, 2026  ·  07:04 UTC</t>
+          <t>Generated April 12, 2026  ·  07:19 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1634,7 +1634,7 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$181</t>
+          <t>$179</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1737,7 +1737,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
       <c r="B12" s="30" t="inlineStr">
@@ -1802,10 +1802,10 @@
         </is>
       </c>
       <c r="C12" s="31" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1815,9 +1815,7 @@
       <c r="F12" s="30" t="n">
         <v>7</v>
       </c>
-      <c r="G12" s="33" t="n">
-        <v>200</v>
-      </c>
+      <c r="G12" s="30" t="inlineStr"/>
       <c r="H12" s="41" t="inlineStr">
         <is>
           <t>SNKRS App</t>
@@ -1827,19 +1825,19 @@
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C13" s="36" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1850,7 +1848,7 @@
         <v>7</v>
       </c>
       <c r="G13" s="38" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="H13" s="42" t="inlineStr">
         <is>
@@ -1861,7 +1859,7 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -1873,7 +1871,7 @@
         <v>46125</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1895,7 +1893,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1907,7 +1905,7 @@
         <v>46125</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1917,17 +1915,19 @@
       <c r="F15" s="35" t="n">
         <v>7</v>
       </c>
-      <c r="G15" s="35" t="inlineStr"/>
-      <c r="H15" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="G15" s="38" t="n">
+        <v>200</v>
+      </c>
+      <c r="H15" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1939,7 +1939,7 @@
         <v>46125</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="H16" s="43" t="inlineStr">
         <is>
@@ -2006,13 +2006,13 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="45" t="inlineStr">
+      <c r="A20" s="44" t="inlineStr">
         <is>
           <t>Nike</t>
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
       <c r="E20" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="46" t="inlineStr">
+      <c r="G20" s="45" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2032,13 +2032,13 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="47" t="inlineStr">
+      <c r="A21" s="46" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D21" s="37" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
       <c r="E21" s="35" t="n">
         <v>61</v>
       </c>
-      <c r="G21" s="48" t="inlineStr">
+      <c r="G21" s="47" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -2058,15 +2058,15 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="45" t="inlineStr">
+      <c r="A22" s="44" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>6</v>
-      </c>
-      <c r="D22" s="49" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="D22" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2074,7 +2074,7 @@
       <c r="E22" s="30" t="n">
         <v>34</v>
       </c>
-      <c r="G22" s="50" t="inlineStr">
+      <c r="G22" s="49" t="inlineStr">
         <is>
           <t>Raffle/Dropship</t>
         </is>
@@ -2084,7 +2084,7 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="D23" s="51" t="inlineStr">
+      <c r="D23" s="50" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2143,17 +2143,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/11 – 4/17</t>
+          <t>4/12 – 4/18</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D27" s="40" t="n">
         <v>13</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2164,17 +2164,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/18 – 4/24</t>
+          <t>4/19 – 4/25</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" s="37" t="n">
         <v>10</v>
       </c>
-      <c r="D28" s="37" t="n">
-        <v>7</v>
-      </c>
       <c r="E28" s="35" t="n">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2185,17 +2185,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/25 – 5/1</t>
+          <t>4/26 – 5/2</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D29" s="40" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2206,17 +2206,17 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>5/2 – 5/8</t>
+          <t>5/3 – 5/9</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D30" s="37" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>6</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2227,17 +2227,17 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/9 – 5/15</t>
+          <t>5/10 – 5/16</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D31" s="40" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E31" s="30" t="n">
-        <v>6.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -2248,17 +2248,17 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/16 – 5/22</t>
+          <t>5/17 – 5/23</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
         <v>4</v>
       </c>
       <c r="D32" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" s="35" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/23 – 5/29</t>
+          <t>5/24 – 5/30</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="D33" s="40" t="n">
         <v>7</v>
       </c>
-      <c r="D33" s="40" t="n">
-        <v>5</v>
-      </c>
       <c r="E33" s="30" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2290,17 +2290,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/30 – 6/5</t>
+          <t>5/31 – 6/6</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D34" s="37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2311,17 +2311,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>6/6 – 6/12</t>
+          <t>6/7 – 6/13</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D35" s="40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2332,17 +2332,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/13 – 6/19</t>
+          <t>6/14 – 6/20</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D36" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2353,17 +2353,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/20 – 6/26</t>
+          <t>6/21 – 6/27</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D37" s="40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>5.6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2374,17 +2374,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/27 – 7/3</t>
+          <t>6/28 – 7/4</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D38" s="37" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E38" s="35" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2395,14 +2395,14 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>7/4 – 7/10</t>
+          <t>7/5 – 7/11</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D39" s="40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>7</v>
@@ -2455,42 +2455,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="51" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="B1" s="52" t="inlineStr">
+      <c r="B1" s="51" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="D1" s="52" t="inlineStr">
+      <c r="D1" s="51" t="inlineStr">
         <is>
           <t>Hype Level</t>
         </is>
       </c>
-      <c r="E1" s="52" t="inlineStr">
+      <c r="E1" s="51" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="G1" s="52" t="inlineStr">
+      <c r="G1" s="51" t="inlineStr">
         <is>
           <t>Sale Method</t>
         </is>
       </c>
-      <c r="H1" s="52" t="inlineStr">
+      <c r="H1" s="51" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
-      <c r="J1" s="52" t="inlineStr">
+      <c r="J1" s="51" t="inlineStr">
         <is>
           <t>Price Range</t>
         </is>
       </c>
-      <c r="K1" s="52" t="inlineStr">
+      <c r="K1" s="51" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
@@ -2503,7 +2503,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -2613,7 +2613,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -2662,9 +2662,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="53" t="inlineStr">
-        <is>
-          <t>Generated April 11, 2026  ·  07:04 UTC</t>
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>Generated April 12, 2026  ·  07:19 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2707,42 +2707,42 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C4" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D4" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C4" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D4" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>adidas Anthony Edwards 2 “Glow”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C5" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C5" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D5" s="42" t="inlineStr">
@@ -2752,53 +2752,51 @@
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>adidas Harden Vol. 10 “Marathon”</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46123</v>
-      </c>
-      <c r="B6" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C6" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D6" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B6" s="33" t="inlineStr"/>
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Pharrell x adidas VIRGINIA Vario Flat Earther</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="36" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C7" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D7" s="42" t="inlineStr">
@@ -2808,25 +2806,25 @@
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Glow”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C8" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C8" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D8" s="43" t="inlineStr">
@@ -2836,12 +2834,12 @@
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Marathon”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2848,7 @@
         <v>46125</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
@@ -2869,7 +2867,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -2877,15 +2875,17 @@
       <c r="A10" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B10" s="33" t="inlineStr"/>
+      <c r="B10" s="33" t="n">
+        <v>220</v>
+      </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -2895,25 +2895,25 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>190</v>
+        <v>130</v>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D11" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -2923,25 +2923,25 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
@@ -2960,16 +2960,16 @@
         <v>46126</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C13" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D13" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>110</v>
+      </c>
+      <c r="C13" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -2979,25 +2979,25 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D14" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -3007,25 +3007,25 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Caitlin Clark Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C15" s="55" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D15" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
+          <t>Nike V5 RNR “Jackie Robinson Day”</t>
         </is>
       </c>
     </row>
@@ -3063,23 +3063,23 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark Nike Kobe 5 Protro “Rookie of the Year”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>100</v>
-      </c>
-      <c r="C17" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D17" s="44" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D17" s="54" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3091,16 +3091,16 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike V5 RNR “Jackie Robinson Day”</t>
+          <t>Palace x Nike Air Max 95</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>190</v>
+        <v>130</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Rookie of the Year”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -3128,35 +3128,35 @@
         <v>46128</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C19" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D19" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C19" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Palace x Nike Air Max 95</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -3175,48 +3175,48 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46128</v>
+        <v>46130</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C21" s="51" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D21" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C21" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D21" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C22" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C22" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D22" s="43" t="inlineStr">
@@ -3231,20 +3231,20 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46129</v>
+        <v>46133</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C23" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C23" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D23" s="42" t="inlineStr">
@@ -3259,20 +3259,20 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C24" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D24" s="41" t="inlineStr">
@@ -3287,16 +3287,16 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
@@ -3315,20 +3315,20 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C26" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D26" s="43" t="inlineStr">
@@ -3338,12 +3338,12 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
         <v>46135</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C27" s="37" t="inlineStr">
         <is>
@@ -3366,12 +3366,12 @@
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       <c r="B28" s="33" t="n">
         <v>190</v>
       </c>
-      <c r="C28" s="49" t="inlineStr">
+      <c r="C28" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3405,19 +3405,19 @@
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D29" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D29" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3436,16 +3436,16 @@
         <v>46136</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D30" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D30" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3464,7 @@
         <v>46136</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
         <v>46136</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -3511,17 +3511,15 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B33" s="38" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B33" s="38" t="inlineStr"/>
       <c r="C33" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3539,7 +3537,7 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3545,9 @@
       <c r="A34" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B34" s="33" t="inlineStr"/>
+      <c r="B34" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3560,25 +3560,25 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C35" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D35" s="42" t="inlineStr">
@@ -3588,21 +3588,21 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
@@ -3621,17 +3621,15 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B37" s="38" t="n">
-        <v>180</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B37" s="38" t="inlineStr"/>
       <c r="C37" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3644,12 +3642,12 @@
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3655,9 @@
       <c r="A38" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B38" s="33" t="inlineStr"/>
+      <c r="B38" s="33" t="n">
+        <v>205</v>
+      </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3684,11 +3684,11 @@
         <v>46142</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C39" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>95</v>
+      </c>
+      <c r="C39" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D39" s="42" t="inlineStr">
@@ -3698,12 +3698,12 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -3712,11 +3712,11 @@
         <v>46142</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C40" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C40" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D40" s="43" t="inlineStr">
@@ -3726,25 +3726,25 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C41" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>165</v>
+      </c>
+      <c r="C41" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D41" s="42" t="inlineStr">
@@ -3754,23 +3754,23 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Air Jordan 4 GS “Black Infrared 23”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C42" s="49" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C42" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
@@ -3796,11 +3796,11 @@
         <v>46143</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>165</v>
-      </c>
-      <c r="C43" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C43" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D43" s="42" t="inlineStr">
@@ -3810,25 +3810,25 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 GS “Black Infrared 23”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C44" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>145</v>
+      </c>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D44" s="43" t="inlineStr">
@@ -3838,21 +3838,21 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>190</v>
+        <v>145</v>
       </c>
       <c r="C45" s="55" t="inlineStr">
         <is>
@@ -3871,16 +3871,16 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
@@ -3894,18 +3894,18 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46144</v>
+        <v>46150</v>
       </c>
       <c r="B47" s="38" t="n">
         <v>145</v>
@@ -3927,16 +3927,16 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Book 2 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
@@ -3955,7 +3955,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
         <v>46150</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -3994,9 +3994,9 @@
       <c r="B50" s="33" t="n">
         <v>210</v>
       </c>
-      <c r="C50" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C50" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D50" s="43" t="inlineStr">
@@ -4011,20 +4011,20 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C51" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>195</v>
+      </c>
+      <c r="C51" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4034,12 +4034,12 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -4157,14 +4157,14 @@
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>195</v>
-      </c>
-      <c r="C56" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C56" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D56" s="43" t="inlineStr">
@@ -4174,12 +4174,12 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
@@ -4188,11 +4188,11 @@
         <v>46157</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C57" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C57" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D57" s="42" t="inlineStr">
@@ -4207,20 +4207,20 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C58" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C58" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D58" s="43" t="inlineStr">
@@ -4230,53 +4230,53 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46158</v>
+        <v>46163</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C59" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D59" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C59" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D59" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Max Mad 90 Pack</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46158</v>
+        <v>46164</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C60" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>170</v>
+      </c>
+      <c r="C60" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
@@ -4286,53 +4286,53 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46163</v>
+        <v>46165</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C61" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D61" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>205</v>
+      </c>
+      <c r="C61" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D61" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Mad 90 Pack</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C62" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D62" s="43" t="inlineStr">
@@ -4342,21 +4342,21 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C63" s="37" t="inlineStr">
         <is>
@@ -4370,25 +4370,25 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46165</v>
+        <v>46170</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C64" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>150</v>
+      </c>
+      <c r="C64" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D64" s="43" t="inlineStr">
@@ -4398,21 +4398,21 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Book 2 “Haven and Hector”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C65" s="37" t="inlineStr">
         <is>
@@ -4431,18 +4431,18 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C66" s="49" t="inlineStr">
+        <v>155</v>
+      </c>
+      <c r="C66" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Haven and Hector”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
@@ -4487,20 +4487,18 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46171</v>
-      </c>
-      <c r="B68" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C68" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46172</v>
+      </c>
+      <c r="B68" s="33" t="inlineStr"/>
+      <c r="C68" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D68" s="43" t="inlineStr">
@@ -4510,21 +4508,21 @@
       </c>
       <c r="E68" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="36" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C69" s="37" t="inlineStr">
         <is>
@@ -4543,7 +4541,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
@@ -4551,10 +4549,12 @@
       <c r="A70" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B70" s="33" t="inlineStr"/>
-      <c r="C70" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B70" s="33" t="n">
+        <v>220</v>
+      </c>
+      <c r="C70" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D70" s="43" t="inlineStr">
@@ -4564,12 +4564,12 @@
       </c>
       <c r="E70" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4577,9 +4577,7 @@
       <c r="A71" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B71" s="38" t="n">
-        <v>250</v>
-      </c>
+      <c r="B71" s="38" t="inlineStr"/>
       <c r="C71" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4592,12 +4590,12 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4603,9 @@
       <c r="A72" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B72" s="33" t="inlineStr"/>
+      <c r="B72" s="33" t="n">
+        <v>120</v>
+      </c>
       <c r="C72" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4618,25 +4618,25 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C73" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C73" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
@@ -4651,18 +4651,18 @@
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C74" s="49" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C74" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4679,20 +4679,18 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B75" s="38" t="n">
-        <v>140</v>
-      </c>
-      <c r="C75" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B75" s="38" t="inlineStr"/>
+      <c r="C75" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D75" s="42" t="inlineStr">
@@ -4702,20 +4700,22 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B76" s="33" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B76" s="33" t="n">
+        <v>355</v>
+      </c>
       <c r="C76" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4733,20 +4733,20 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46182</v>
+        <v>46185</v>
       </c>
       <c r="B77" s="38" t="n">
-        <v>355</v>
-      </c>
-      <c r="C77" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C77" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D77" s="42" t="inlineStr">
@@ -4756,12 +4756,12 @@
       </c>
       <c r="E77" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
@@ -4772,7 +4772,7 @@
       <c r="B78" s="33" t="n">
         <v>170</v>
       </c>
-      <c r="C78" s="49" t="inlineStr">
+      <c r="C78" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4789,7 +4789,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
@@ -4817,18 +4817,18 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C80" s="49" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="C80" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike Air More Uptempo “Legacy”</t>
         </is>
       </c>
     </row>
@@ -4854,16 +4854,16 @@
         <v>46186</v>
       </c>
       <c r="B81" s="38" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C81" s="55" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D81" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D81" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E81" s="35" t="inlineStr">
@@ -4873,7 +4873,7 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Air More Uptempo “Legacy”</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -4882,26 +4882,26 @@
         <v>46186</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C82" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D82" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>205</v>
+      </c>
+      <c r="C82" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D82" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -4938,11 +4938,11 @@
         <v>46186</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C84" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C84" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D84" s="43" t="inlineStr">
@@ -4952,12 +4952,12 @@
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4966,7 +4966,7 @@
         <v>46186</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="C85" s="55" t="inlineStr">
         <is>
@@ -4985,18 +4985,18 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C86" s="49" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C86" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5013,20 +5013,20 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="36" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C87" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C87" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D87" s="42" t="inlineStr">
@@ -5036,12 +5036,12 @@
       </c>
       <c r="E87" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -5050,26 +5050,26 @@
         <v>46193</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C88" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D88" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C88" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D88" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -5078,16 +5078,16 @@
         <v>46193</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C89" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D89" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>162</v>
+      </c>
+      <c r="C89" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D89" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
@@ -5106,16 +5106,16 @@
         <v>46193</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>162</v>
-      </c>
-      <c r="C90" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D90" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C90" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D90" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5125,7 +5125,7 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Nike SB P-Rod 1 Black Gum</t>
         </is>
       </c>
     </row>
@@ -5134,16 +5134,16 @@
         <v>46193</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>125</v>
-      </c>
-      <c r="C91" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D91" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="C91" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D91" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E91" s="35" t="inlineStr">
@@ -5153,20 +5153,20 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 Black Gum</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C92" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C92" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D92" s="43" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Total 90 “University Red”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
@@ -5209,20 +5209,18 @@
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="31" t="n">
-        <v>46199</v>
-      </c>
-      <c r="B94" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C94" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46200</v>
+      </c>
+      <c r="B94" s="33" t="inlineStr"/>
+      <c r="C94" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D94" s="43" t="inlineStr">
@@ -5232,12 +5230,12 @@
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -5245,17 +5243,15 @@
       <c r="A95" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B95" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C95" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D95" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B95" s="38" t="inlineStr"/>
+      <c r="C95" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D95" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
@@ -5265,7 +5261,7 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
@@ -5273,7 +5269,9 @@
       <c r="A96" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B96" s="33" t="inlineStr"/>
+      <c r="B96" s="33" t="n">
+        <v>185</v>
+      </c>
       <c r="C96" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5291,7 +5289,7 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -5300,16 +5298,16 @@
         <v>46200</v>
       </c>
       <c r="B97" s="38" t="n">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="C97" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D97" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D97" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E97" s="35" t="inlineStr">
@@ -5319,7 +5317,7 @@
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -5327,25 +5325,27 @@
       <c r="A98" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B98" s="33" t="inlineStr"/>
-      <c r="C98" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D98" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B98" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C98" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D98" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E98" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
         <v>46200</v>
       </c>
       <c r="B99" s="38" t="n">
-        <v>190</v>
+        <v>135</v>
       </c>
       <c r="C99" s="37" t="inlineStr">
         <is>
@@ -5373,25 +5373,25 @@
       </c>
       <c r="F99" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="31" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="B100" s="33" t="n">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="C100" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D100" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D100" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E100" s="30" t="inlineStr">
@@ -5401,25 +5401,25 @@
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="36" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="B101" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C101" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D101" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C101" s="55" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D101" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E101" s="35" t="inlineStr">
@@ -5429,20 +5429,20 @@
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Nike Ja 3 “Animal Instinct”</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="31" t="n">
-        <v>46206</v>
+        <v>46210</v>
       </c>
       <c r="B102" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C102" s="49" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>210</v>
+      </c>
+      <c r="C102" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D102" s="43" t="inlineStr">
@@ -5457,16 +5457,16 @@
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Animal Instinct”</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1">
       <c r="A103" s="36" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="B103" s="38" t="n">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C103" s="37" t="inlineStr">
         <is>
@@ -5480,30 +5480,28 @@
       </c>
       <c r="E103" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F103" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Air Jordan 4 “Birds of Paradise”</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
       <c r="A104" s="31" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B104" s="33" t="n">
-        <v>215</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="B104" s="33" t="inlineStr"/>
       <c r="C104" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D104" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D104" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E104" s="30" t="inlineStr">
@@ -5513,7 +5511,7 @@
       </c>
       <c r="F104" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Birds of Paradise”</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
@@ -5557,9 +5555,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="53" t="inlineStr">
-        <is>
-          <t>Generated April 11, 2026  ·  07:04 UTC</t>
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>Generated April 12, 2026  ·  07:19 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5602,11 +5600,9 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46123</v>
-      </c>
-      <c r="B4" s="33" t="n">
-        <v>200</v>
-      </c>
+        <v>46125</v>
+      </c>
+      <c r="B4" s="33" t="inlineStr"/>
       <c r="C4" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5624,16 +5620,16 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C5" s="37" t="inlineStr">
         <is>
@@ -5647,12 +5643,12 @@
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Flight Club”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5680,7 +5676,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -5688,15 +5684,17 @@
       <c r="A7" s="36" t="n">
         <v>46125</v>
       </c>
-      <c r="B7" s="38" t="inlineStr"/>
+      <c r="B7" s="38" t="n">
+        <v>200</v>
+      </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
@@ -5706,7 +5704,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5713,7 @@
         <v>46125</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -5734,25 +5732,25 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
@@ -5762,7 +5760,7 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
@@ -5771,7 +5769,7 @@
         <v>46126</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
@@ -5790,25 +5788,25 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -5818,7 +5816,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Caitlin Clark Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
@@ -5846,25 +5844,25 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark Nike Kobe 5 Protro “Rookie of the Year”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D13" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -5874,7 +5872,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Rookie of the Year”</t>
+          <t>Palace x Nike Air Max 95</t>
         </is>
       </c>
     </row>
@@ -5883,16 +5881,16 @@
         <v>46128</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D14" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -5902,16 +5900,16 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Palace x Nike Air Max 95</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C15" s="37" t="inlineStr">
         <is>
@@ -5930,16 +5928,16 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
@@ -5958,25 +5956,25 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D17" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
@@ -5986,16 +5984,16 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46135</v>
+        <v>46133</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
@@ -6009,12 +6007,12 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
@@ -6023,7 +6021,7 @@
         <v>46135</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
@@ -6037,30 +6035,30 @@
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46136</v>
+        <v>46135</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D20" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D20" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
@@ -6070,7 +6068,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Year of the Horse”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
@@ -6079,16 +6077,16 @@
         <v>46136</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D21" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
@@ -6098,7 +6096,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6105,7 @@
         <v>46136</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
@@ -6126,7 +6124,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6133,7 @@
         <v>46136</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
@@ -6154,15 +6152,17 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B24" s="33" t="inlineStr"/>
+        <v>46136</v>
+      </c>
+      <c r="B24" s="33" t="n">
+        <v>210</v>
+      </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6180,7 +6180,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
@@ -6188,9 +6188,7 @@
       <c r="A25" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B25" s="38" t="n">
-        <v>215</v>
-      </c>
+      <c r="B25" s="38" t="inlineStr"/>
       <c r="C25" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6203,12 +6201,12 @@
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6215,7 @@
         <v>46137</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
@@ -6236,16 +6234,16 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>The Whitaker Group x Air Jordan 11 Low</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>180</v>
+        <v>215</v>
       </c>
       <c r="C27" s="37" t="inlineStr">
         <is>
@@ -6259,12 +6257,12 @@
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Metallic Pack” 2026</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -6299,7 +6297,7 @@
         <v>46142</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
@@ -6318,16 +6316,16 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>205</v>
+        <v>165</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
@@ -6346,16 +6344,16 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 4 GS “Black Infrared 23”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
@@ -6374,16 +6372,16 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 GS “Black Infrared 23”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -6397,21 +6395,21 @@
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
@@ -6430,7 +6428,7 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -6439,7 +6437,7 @@
         <v>46150</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -6458,16 +6456,16 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="C35" s="37" t="inlineStr">
         <is>
@@ -6481,12 +6479,12 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -6604,10 +6602,10 @@
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>195</v>
+        <v>150</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -6621,21 +6619,21 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46157</v>
+        <v>46165</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C41" s="37" t="inlineStr">
         <is>
@@ -6649,21 +6647,21 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46158</v>
+        <v>46165</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -6682,16 +6680,16 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
@@ -6705,21 +6703,21 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46165</v>
+        <v>46171</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
@@ -6733,21 +6731,21 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C45" s="37" t="inlineStr">
         <is>
@@ -6766,16 +6764,16 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
@@ -6794,16 +6792,16 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C47" s="37" t="inlineStr">
         <is>
@@ -6817,12 +6815,12 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -6830,9 +6828,7 @@
       <c r="A48" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B48" s="33" t="n">
-        <v>250</v>
-      </c>
+      <c r="B48" s="33" t="inlineStr"/>
       <c r="C48" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6845,12 +6841,12 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -6858,7 +6854,9 @@
       <c r="A49" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B49" s="38" t="inlineStr"/>
+      <c r="B49" s="38" t="n">
+        <v>120</v>
+      </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6871,22 +6869,20 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B50" s="33" t="n">
-        <v>120</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B50" s="33" t="inlineStr"/>
       <c r="C50" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6899,20 +6895,22 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B51" s="38" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B51" s="38" t="n">
+        <v>355</v>
+      </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6930,16 +6928,16 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46182</v>
+        <v>46186</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>355</v>
+        <v>205</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
@@ -6958,7 +6956,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -6992,10 +6990,10 @@
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
@@ -7014,7 +7012,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7021,7 @@
         <v>46193</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>215</v>
+        <v>162</v>
       </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
@@ -7037,12 +7035,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
@@ -7051,7 +7049,7 @@
         <v>46193</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>162</v>
+        <v>200</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -7070,17 +7068,15 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B57" s="38" t="n">
-        <v>200</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B57" s="38" t="inlineStr"/>
       <c r="C57" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -7093,12 +7089,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Total 90 “University Red”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -7134,7 +7130,9 @@
       <c r="A59" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B59" s="38" t="inlineStr"/>
+      <c r="B59" s="38" t="n">
+        <v>190</v>
+      </c>
       <c r="C59" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -7147,12 +7145,12 @@
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -7161,16 +7159,16 @@
         <v>46200</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D60" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D60" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E60" s="30" t="inlineStr">
@@ -7180,7 +7178,7 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -7189,7 +7187,7 @@
         <v>46200</v>
       </c>
       <c r="B61" s="38" t="n">
-        <v>190</v>
+        <v>135</v>
       </c>
       <c r="C61" s="37" t="inlineStr">
         <is>
@@ -7208,25 +7206,25 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="C62" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D62" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D62" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
@@ -7236,25 +7234,25 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46203</v>
+        <v>46210</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="C63" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D63" s="44" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D63" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E63" s="35" t="inlineStr">
@@ -7264,16 +7262,16 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C64" s="40" t="inlineStr">
         <is>
@@ -7287,30 +7285,28 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Air Jordan 4 “Birds of Paradise”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B65" s="38" t="n">
-        <v>215</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="B65" s="38" t="inlineStr"/>
       <c r="C65" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D65" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D65" s="54" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E65" s="35" t="inlineStr">
@@ -7320,7 +7316,7 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Birds of Paradise”</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-13 08:08 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,13 +679,13 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1581,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 12, 2026  ·  07:19 UTC</t>
+          <t>Generated April 13, 2026  ·  08:08 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1625,16 +1625,16 @@
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$179</t>
+          <t>$182</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1737,7 +1737,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1805,7 +1805,7 @@
         <v>46125</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         <v>46125</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
         <v>46125</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
@@ -1905,7 +1905,7 @@
         <v>46125</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1939,7 +1939,7 @@
         <v>46125</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G21" s="47" t="inlineStr">
         <is>
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="H21" s="35" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D22" s="48" t="inlineStr">
         <is>
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G22" s="49" t="inlineStr">
         <is>
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="E23" s="35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" ht="10" customHeight="1"/>
@@ -2143,17 +2143,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/12 – 4/18</t>
+          <t>4/13 – 4/19</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D27" s="40" t="n">
         <v>13</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.9</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/19 – 4/25</t>
+          <t>4/20 – 4/26</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
@@ -2185,17 +2185,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>4/26 – 5/2</t>
+          <t>4/27 – 5/3</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D29" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" s="30" t="n">
         <v>5</v>
-      </c>
-      <c r="E29" s="30" t="n">
-        <v>5.4</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>5/3 – 5/9</t>
+          <t>5/4 – 5/10</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/10 – 5/16</t>
+          <t>5/11 – 5/17</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/17 – 5/23</t>
+          <t>5/18 – 5/24</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/24 – 5/30</t>
+          <t>5/25 – 5/31</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D33" s="40" t="n">
         <v>7</v>
       </c>
       <c r="E33" s="30" t="n">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2290,17 +2290,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>5/31 – 6/6</t>
+          <t>6/1 – 6/7</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D34" s="37" t="n">
         <v>1</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>6/7 – 6/13</t>
+          <t>6/8 – 6/14</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/14 – 6/20</t>
+          <t>6/15 – 6/21</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/21 – 6/27</t>
+          <t>6/22 – 6/28</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>6/28 – 7/4</t>
+          <t>6/29 – 7/5</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
@@ -2395,17 +2395,17 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>7/5 – 7/11</t>
+          <t>7/6 – 7/12</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" s="40" t="n">
         <v>3</v>
       </c>
       <c r="E39" s="30" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2503,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2545,7 +2545,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2553,7 +2553,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2579,7 +2579,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -2605,7 +2605,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2664,7 +2664,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 12, 2026  ·  07:19 UTC</t>
+          <t>Generated April 13, 2026  ·  08:08 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2707,42 +2707,40 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46124</v>
-      </c>
-      <c r="B4" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C4" s="53" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D4" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46125</v>
+      </c>
+      <c r="B4" s="33" t="inlineStr"/>
+      <c r="C4" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 2 “Glow”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C5" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D5" s="42" t="inlineStr">
@@ -2752,12 +2750,12 @@
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Marathon”</t>
+          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -2765,15 +2763,17 @@
       <c r="A6" s="31" t="n">
         <v>46125</v>
       </c>
-      <c r="B6" s="33" t="inlineStr"/>
+      <c r="B6" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D6" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D6" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Out” (Mamba Day)</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
         <v>46125</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Steam”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
@@ -2820,7 +2820,7 @@
         <v>46125</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -2839,25 +2839,25 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “Steam”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="36" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D9" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
@@ -2867,25 +2867,25 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike SB Dunk Low “Som Tum”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Nike Air Max 90 “Ultramarine”</t>
         </is>
       </c>
     </row>
@@ -2904,16 +2904,16 @@
         <v>46126</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C11" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D11" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>110</v>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -2923,20 +2923,20 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Som Tum”</t>
+          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C12" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>100</v>
+      </c>
+      <c r="C12" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D12" s="41" t="inlineStr">
@@ -2951,20 +2951,20 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 90 “Ultramarine”</t>
+          <t>Nike V5 RNR “Jackie Robinson Day”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>110</v>
-      </c>
-      <c r="C13" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D13" s="42" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Tom Sachs x NikeCraft General Purpose Shoe “Bricolage”</t>
+          <t>Caitlin Clark Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
@@ -3007,25 +3007,25 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark Nike Kobe 5 Protro “Rookie of the Year”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Rookie of the Year”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>100</v>
-      </c>
-      <c r="C15" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D15" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
@@ -3035,25 +3035,25 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike V5 RNR “Jackie Robinson Day”</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Rookie of the Year”</t>
+          <t>Palace x Nike Air Max 95</t>
         </is>
       </c>
     </row>
@@ -3072,35 +3072,35 @@
         <v>46128</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C17" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D17" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C17" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D17" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Palace x Nike Air Max 95</t>
+          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>130</v>
+        <v>235</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
@@ -3119,20 +3119,20 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46128</v>
+        <v>46130</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C19" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>240</v>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
@@ -3142,30 +3142,30 @@
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>235</v>
-      </c>
-      <c r="C20" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D20" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C20" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D20" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
@@ -3175,25 +3175,25 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C21" s="55" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D21" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
@@ -3203,25 +3203,25 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D22" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -3240,11 +3240,11 @@
         <v>46133</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C23" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C23" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D23" s="42" t="inlineStr">
@@ -3259,41 +3259,41 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D24" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="36" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B25" s="38" t="n">
         <v>120</v>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 Low</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
@@ -3324,11 +3324,11 @@
         <v>46135</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C26" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C26" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D26" s="43" t="inlineStr">
@@ -3338,21 +3338,21 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Homecoming x Nike Air Max Plus</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="C27" s="37" t="inlineStr">
         <is>
@@ -3371,25 +3371,25 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C28" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D28" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D28" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Homecoming x Nike Air Max Plus</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3415,9 +3415,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D29" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
         <v>46136</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>150</v>
+        <v>210</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
@@ -3455,16 +3455,16 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
@@ -3478,22 +3478,20 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B32" s="33" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B32" s="33" t="inlineStr"/>
       <c r="C32" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3511,15 +3509,17 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B33" s="38" t="inlineStr"/>
+        <v>46142</v>
+      </c>
+      <c r="B33" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3532,22 +3532,20 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B34" s="33" t="n">
-        <v>215</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B34" s="33" t="inlineStr"/>
       <c r="C34" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3565,7 +3563,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3574,11 +3572,11 @@
         <v>46142</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C35" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D35" s="42" t="inlineStr">
@@ -3588,12 +3586,12 @@
       </c>
       <c r="E35" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3602,11 +3600,11 @@
         <v>46142</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C36" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C36" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D36" s="43" t="inlineStr">
@@ -3616,12 +3614,12 @@
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
@@ -3629,10 +3627,12 @@
       <c r="A37" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B37" s="38" t="inlineStr"/>
-      <c r="C37" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B37" s="38" t="n">
+        <v>95</v>
+      </c>
+      <c r="C37" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D37" s="42" t="inlineStr">
@@ -3642,12 +3642,12 @@
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -3656,11 +3656,11 @@
         <v>46142</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C38" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C38" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D38" s="43" t="inlineStr">
@@ -3670,23 +3670,23 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>95</v>
-      </c>
-      <c r="C39" s="55" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C39" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3703,16 +3703,16 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Air Zoom Huarache 2K4 “White Varsity Red”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>200</v>
+        <v>135</v>
       </c>
       <c r="C40" s="48" t="inlineStr">
         <is>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
@@ -3740,11 +3740,11 @@
         <v>46143</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>165</v>
-      </c>
-      <c r="C41" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C41" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D41" s="42" t="inlineStr">
@@ -3754,25 +3754,25 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 GS “Black Infrared 23”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C42" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>145</v>
+      </c>
+      <c r="C42" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D42" s="43" t="inlineStr">
@@ -3782,23 +3782,23 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C43" s="55" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C43" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike A’Two “A’Pink Shoe”</t>
         </is>
       </c>
     </row>
@@ -3826,9 +3826,9 @@
       <c r="B44" s="33" t="n">
         <v>145</v>
       </c>
-      <c r="C44" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C44" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D44" s="43" t="inlineStr">
@@ -3838,25 +3838,25 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C45" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C45" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D45" s="42" t="inlineStr">
@@ -3871,20 +3871,20 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C46" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C46" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D46" s="43" t="inlineStr">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Book 2 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -3908,11 +3908,11 @@
         <v>46150</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C47" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C47" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D47" s="42" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Book 2 “WNBA 30th Anniversary”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
         <v>46150</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
@@ -3955,7 +3955,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -3966,9 +3966,9 @@
       <c r="B49" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C49" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C49" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D49" s="42" t="inlineStr">
@@ -3983,20 +3983,20 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C50" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>200</v>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D50" s="43" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4129,14 +4129,14 @@
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C55" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C55" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D55" s="42" t="inlineStr">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
@@ -4160,11 +4160,11 @@
         <v>46157</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C56" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D56" s="43" t="inlineStr">
@@ -4179,20 +4179,20 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C57" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C57" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D57" s="42" t="inlineStr">
@@ -4202,58 +4202,58 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46158</v>
+        <v>46163</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C58" s="53" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D58" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C58" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Air Max Mad 90 Pack</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C59" s="55" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C59" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D59" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D59" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
@@ -4263,20 +4263,20 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Mad 90 Pack</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C60" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
@@ -4286,12 +4286,12 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -4319,16 +4319,16 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C62" s="40" t="inlineStr">
         <is>
@@ -4342,25 +4342,25 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46168</v>
+        <v>46170</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C63" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>150</v>
+      </c>
+      <c r="C63" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D63" s="42" t="inlineStr">
@@ -4375,20 +4375,20 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Book 2 “Haven and Hector”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C64" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C64" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D64" s="43" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Haven and Hector”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4412,11 +4412,11 @@
         <v>46171</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C65" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C65" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D65" s="42" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
@@ -4440,11 +4440,11 @@
         <v>46171</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C66" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C66" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D66" s="43" t="inlineStr">
@@ -4459,16 +4459,16 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C67" s="37" t="inlineStr">
         <is>
@@ -4487,7 +4487,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
@@ -4496,7 +4496,7 @@
         <v>46172</v>
       </c>
       <c r="B68" s="33" t="inlineStr"/>
-      <c r="C68" s="53" t="inlineStr">
+      <c r="C68" s="55" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -4601,14 +4601,14 @@
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C72" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C72" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D72" s="43" t="inlineStr">
@@ -4623,18 +4623,18 @@
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C73" s="55" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C73" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4651,20 +4651,18 @@
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B74" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C74" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B74" s="33" t="inlineStr"/>
+      <c r="C74" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D74" s="43" t="inlineStr">
@@ -4674,20 +4672,22 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B75" s="38" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B75" s="38" t="n">
+        <v>355</v>
+      </c>
       <c r="C75" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4705,20 +4705,20 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="31" t="n">
-        <v>46182</v>
+        <v>46185</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="C76" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C76" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D76" s="43" t="inlineStr">
@@ -4728,12 +4728,12 @@
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
       <c r="B77" s="38" t="n">
         <v>170</v>
       </c>
-      <c r="C77" s="55" t="inlineStr">
+      <c r="C77" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4789,25 +4789,25 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C79" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D79" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C79" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D79" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E79" s="35" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
         <v>46186</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C80" s="48" t="inlineStr">
         <is>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air More Uptempo “Legacy”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4854,16 +4854,16 @@
         <v>46186</v>
       </c>
       <c r="B81" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C81" s="55" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="C81" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D81" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D81" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E81" s="35" t="inlineStr">
@@ -4873,7 +4873,7 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Nike Air More Uptempo “Legacy”</t>
         </is>
       </c>
     </row>
@@ -4882,26 +4882,26 @@
         <v>46186</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C82" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D82" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C82" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D82" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -4910,26 +4910,26 @@
         <v>46186</v>
       </c>
       <c r="B83" s="38" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C83" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D83" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D83" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -4938,7 +4938,7 @@
         <v>46186</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="C84" s="48" t="inlineStr">
         <is>
@@ -4957,18 +4957,18 @@
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="36" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C85" s="55" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="C85" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4985,25 +4985,25 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="31" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="C86" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D86" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D86" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E86" s="30" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Nike SB P-Rod 1 Black Gum</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
         <v>46193</v>
       </c>
       <c r="B87" s="38" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C87" s="37" t="inlineStr">
         <is>
@@ -5036,12 +5036,12 @@
       </c>
       <c r="E87" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
@@ -5050,26 +5050,26 @@
         <v>46193</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C88" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D88" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>215</v>
+      </c>
+      <c r="C88" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D88" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -5078,16 +5078,16 @@
         <v>46193</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>162</v>
-      </c>
-      <c r="C89" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D89" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C89" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D89" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -5106,16 +5106,16 @@
         <v>46193</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C90" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D90" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>162</v>
+      </c>
+      <c r="C90" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D90" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5125,20 +5125,20 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 Black Gum</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C91" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C91" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D91" s="42" t="inlineStr">
@@ -5153,7 +5153,7 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Total 90 “University Red”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
@@ -5181,20 +5181,20 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C93" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>170</v>
+      </c>
+      <c r="C93" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D93" s="42" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,9 @@
       <c r="A94" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B94" s="33" t="inlineStr"/>
+      <c r="B94" s="33" t="n">
+        <v>135</v>
+      </c>
       <c r="C94" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5230,12 +5232,12 @@
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
         </is>
       </c>
     </row>
@@ -5244,14 +5246,14 @@
         <v>46200</v>
       </c>
       <c r="B95" s="38" t="inlineStr"/>
-      <c r="C95" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D95" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C95" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D95" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
@@ -5261,7 +5263,7 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -5269,17 +5271,15 @@
       <c r="A96" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B96" s="33" t="n">
-        <v>185</v>
-      </c>
-      <c r="C96" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D96" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B96" s="33" t="inlineStr"/>
+      <c r="C96" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D96" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5298,7 @@
         <v>46200</v>
       </c>
       <c r="B97" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C97" s="37" t="inlineStr">
         <is>
@@ -5312,12 +5312,12 @@
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
         <v>46200</v>
       </c>
       <c r="B98" s="33" t="n">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="C98" s="40" t="inlineStr">
         <is>
@@ -5345,13 +5345,13 @@
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="A99" s="36" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="B99" s="38" t="n">
         <v>135</v>
@@ -5361,9 +5361,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D99" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D99" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E99" s="35" t="inlineStr">
@@ -5373,25 +5373,25 @@
       </c>
       <c r="F99" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="31" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="B100" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C100" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D100" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C100" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D100" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E100" s="30" t="inlineStr">
@@ -5401,20 +5401,20 @@
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Nike Ja 3 “Animal Instinct”</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="36" t="n">
-        <v>46206</v>
+        <v>46210</v>
       </c>
       <c r="B101" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C101" s="55" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>210</v>
+      </c>
+      <c r="C101" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D101" s="42" t="inlineStr">
@@ -5429,35 +5429,35 @@
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Animal Instinct”</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="31" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="B102" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C102" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D102" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>355</v>
+      </c>
+      <c r="C102" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D102" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E102" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Air Jordan 8 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -5531,7 +5531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5557,7 +5557,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 12, 2026  ·  07:19 UTC</t>
+          <t>Generated April 13, 2026  ·  08:08 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
+          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 11 EM Protro “Mamba Day”</t>
+          <t>Nike Kobe 11 Elite Protro “Fade To Black”</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5748,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="54" t="inlineStr">
+      <c r="D9" s="53" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5853,16 +5853,16 @@
         <v>46128</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Palace x Nike Air Max 95</t>
+          <t>Nike Air Force 1 Low “Stadium Green”</t>
         </is>
       </c>
     </row>
@@ -5881,16 +5881,16 @@
         <v>46128</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Stadium Green”</t>
+          <t>Palace x Nike Air Max 95</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5972,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="54" t="inlineStr">
+      <c r="D17" s="53" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -6077,16 +6077,16 @@
         <v>46136</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -6105,16 +6105,16 @@
         <v>46136</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D22" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -6124,7 +6124,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,9 @@
       <c r="A25" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B25" s="38" t="inlineStr"/>
+      <c r="B25" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6201,12 +6203,12 @@
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
@@ -6214,9 +6216,7 @@
       <c r="A26" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B26" s="33" t="n">
-        <v>215</v>
-      </c>
+      <c r="B26" s="33" t="inlineStr"/>
       <c r="C26" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6229,12 +6229,12 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -6322,10 +6322,10 @@
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
@@ -6344,16 +6344,16 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 GS “Black Infrared 23”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>145</v>
+        <v>190</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
@@ -6367,21 +6367,21 @@
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -6400,7 +6400,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -6409,7 +6409,7 @@
         <v>46150</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
@@ -6428,16 +6428,16 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6574,10 +6574,10 @@
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
@@ -6596,16 +6596,16 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46157</v>
+        <v>46165</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -6619,12 +6619,12 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -6652,16 +6652,16 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -6675,21 +6675,21 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6736,16 +6736,16 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C45" s="37" t="inlineStr">
         <is>
@@ -6764,7 +6764,7 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
@@ -6852,11 +6852,9 @@
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B49" s="38" t="n">
-        <v>120</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B49" s="38" t="inlineStr"/>
       <c r="C49" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6869,20 +6867,22 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B50" s="33" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B50" s="33" t="n">
+        <v>355</v>
+      </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6900,35 +6900,35 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46182</v>
+        <v>46186</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>355</v>
+        <v>150</v>
       </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D51" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -6962,19 +6962,19 @@
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D53" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D53" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E53" s="35" t="inlineStr">
@@ -6984,7 +6984,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
@@ -7046,10 +7046,10 @@
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46193</v>
+        <v>46200</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -7068,7 +7068,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Total 90 “University Red”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -7076,7 +7076,9 @@
       <c r="A57" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B57" s="38" t="inlineStr"/>
+      <c r="B57" s="38" t="n">
+        <v>135</v>
+      </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -7089,12 +7091,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
         </is>
       </c>
     </row>
@@ -7102,9 +7104,7 @@
       <c r="A58" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B58" s="33" t="n">
-        <v>185</v>
-      </c>
+      <c r="B58" s="33" t="inlineStr"/>
       <c r="C58" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -7131,7 +7131,7 @@
         <v>46200</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C59" s="37" t="inlineStr">
         <is>
@@ -7145,12 +7145,12 @@
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7159,7 @@
         <v>46200</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
@@ -7178,13 +7178,13 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="B61" s="38" t="n">
         <v>135</v>
@@ -7194,9 +7194,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D61" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D61" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
@@ -7206,25 +7206,25 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46203</v>
+        <v>46210</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="C62" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D62" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D62" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
@@ -7234,16 +7234,16 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="B63" s="38" t="n">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C63" s="37" t="inlineStr">
         <is>
@@ -7257,30 +7257,28 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Air Jordan 4 “Birds of Paradise”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B64" s="33" t="n">
-        <v>215</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="B64" s="33" t="inlineStr"/>
       <c r="C64" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D64" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D64" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E64" s="30" t="inlineStr">
@@ -7290,38 +7288,12 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Birds of Paradise”</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="15" customHeight="1">
-      <c r="A65" s="36" t="n">
-        <v>46214</v>
-      </c>
-      <c r="B65" s="38" t="inlineStr"/>
-      <c r="C65" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D65" s="54" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
-        </is>
-      </c>
-      <c r="E65" s="35" t="inlineStr">
-        <is>
-          <t>Jordan</t>
-        </is>
-      </c>
-      <c r="F65" s="35" t="inlineStr">
-        <is>
           <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F65"/>
+  <autoFilter ref="A3:F64"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-18 07:13 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -115,13 +115,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00888888"/>
+      <color rgb="00FF6B35"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FF6B35"/>
+      <color rgb="00888888"/>
       <sz val="11"/>
     </font>
     <font>
@@ -651,19 +651,19 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -679,16 +679,16 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 17, 2026  ·  07:51 UTC</t>
+          <t>Generated April 18, 2026  ·  07:13 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1624,11 +1624,11 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1637,7 +1637,7 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$183</t>
+          <t>$184</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1740,7 +1740,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1796,7 +1796,7 @@
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
       <c r="B12" s="30" t="inlineStr">
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="C12" s="31" t="n">
-        <v>46129</v>
+        <v>46133</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1819,18 +1819,18 @@
         <v>7</v>
       </c>
       <c r="G12" s="33" t="n">
-        <v>235</v>
+        <v>120</v>
       </c>
       <c r="H12" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Nike SB Air Force 1 Low</t>
         </is>
       </c>
       <c r="B13" s="35" t="inlineStr">
@@ -1842,7 +1842,7 @@
         <v>46133</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1857,26 +1857,26 @@
       </c>
       <c r="H13" s="42" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 Low</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1887,9 +1887,9 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="H14" s="41" t="inlineStr">
+        <v>220</v>
+      </c>
+      <c r="H14" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1898,19 +1898,19 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C15" s="36" t="n">
         <v>46135</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1921,9 +1921,9 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>220</v>
-      </c>
-      <c r="H15" s="43" t="inlineStr">
+        <v>120</v>
+      </c>
+      <c r="H15" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -1932,7 +1932,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="C16" s="31" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="D16" s="30" t="n">
         <v>6</v>
@@ -1955,11 +1955,11 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="H16" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D21" s="37" t="inlineStr">
         <is>
@@ -2059,7 +2059,7 @@
         </is>
       </c>
       <c r="H21" s="35" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G22" s="49" t="inlineStr">
         <is>
@@ -2156,17 +2156,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/17 – 4/23</t>
+          <t>4/18 – 4/24</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D27" s="40" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>5.9</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2177,17 +2177,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/24 – 4/30</t>
+          <t>4/25 – 5/1</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D28" s="37" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>6.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2198,17 +2198,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>5/1 – 5/7</t>
+          <t>5/2 – 5/8</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D29" s="40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>5/8 – 5/14</t>
+          <t>5/9 – 5/15</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D30" s="37" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2240,17 +2240,17 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/15 – 5/21</t>
+          <t>5/16 – 5/22</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
-        <v>5</v>
-      </c>
-      <c r="D31" s="40" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="D31" s="30" t="n">
+        <v>0</v>
       </c>
       <c r="E31" s="30" t="n">
-        <v>4.2</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -2261,17 +2261,17 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/22 – 5/28</t>
+          <t>5/23 – 5/29</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="D32" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="D32" s="37" t="n">
-        <v>2</v>
-      </c>
       <c r="E32" s="35" t="n">
-        <v>5.5</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2282,17 +2282,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/29 – 6/4</t>
+          <t>5/30 – 6/5</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D33" s="40" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E33" s="30" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2303,17 +2303,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>6/5 – 6/11</t>
+          <t>6/6 – 6/12</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D34" s="37" t="n">
         <v>2</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2324,17 +2324,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>6/12 – 6/18</t>
+          <t>6/13 – 6/19</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D35" s="40" t="n">
         <v>2</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2345,17 +2345,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/19 – 6/25</t>
+          <t>6/20 – 6/26</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D36" s="37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2366,17 +2366,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/26 – 7/2</t>
+          <t>6/27 – 7/3</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D37" s="40" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2387,17 +2387,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>7/3 – 7/9</t>
+          <t>7/4 – 7/10</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="D38" s="37" t="n">
-        <v>1</v>
-      </c>
       <c r="E38" s="35" t="n">
-        <v>5.5</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>7/10 – 7/16</t>
+          <t>7/11 – 7/17</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2418,7 +2418,7 @@
         <v>3</v>
       </c>
       <c r="E39" s="30" t="n">
-        <v>6.8</v>
+        <v>6.2</v>
       </c>
     </row>
   </sheetData>
@@ -2516,7 +2516,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2634,7 +2634,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -2659,7 +2659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2685,7 +2685,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 17, 2026  ·  07:51 UTC</t>
+          <t>Generated April 18, 2026  ·  07:13 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2728,57 +2728,57 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>235</v>
-      </c>
-      <c r="C4" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D4" s="41" t="inlineStr">
+        <v>160</v>
+      </c>
+      <c r="C4" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D4" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Willy Chavarria x adidas Superstar</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="36" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C5" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D5" s="43" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D5" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Willy Chavarria x adidas Superstar</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D6" s="53" t="inlineStr">
+      <c r="D6" s="41" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -2815,14 +2815,14 @@
         <v>46133</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C7" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D7" s="43" t="inlineStr">
+        <v>120</v>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2834,35 +2834,35 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="41" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 Low</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -2871,26 +2871,26 @@
         <v>46135</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="43" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
@@ -2899,14 +2899,14 @@
         <v>46135</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C10" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D10" s="41" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C10" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2918,25 +2918,25 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Homecoming x Nike Air Max Plus</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="36" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C11" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D11" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D11" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Homecoming x Nike Air Max Plus</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="41" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -2990,7 +2990,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3018,9 +3018,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D14" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3039,14 +3039,14 @@
         <v>46136</v>
       </c>
       <c r="B15" s="38" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C15" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3058,23 +3058,21 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B16" s="33" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B16" s="33" t="inlineStr"/>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="41" t="inlineStr">
+      <c r="D16" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3086,7 +3084,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3094,53 +3092,55 @@
       <c r="A17" s="36" t="n">
         <v>46137</v>
       </c>
-      <c r="B17" s="38" t="inlineStr"/>
+      <c r="B17" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C18" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D18" s="41" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="C18" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
@@ -3148,27 +3148,25 @@
       <c r="A19" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B19" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C19" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D19" s="43" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr"/>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3182,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D20" s="41" t="inlineStr">
+      <c r="D20" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3204,13 +3202,15 @@
       <c r="A21" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B21" s="38" t="inlineStr"/>
+      <c r="B21" s="38" t="n">
+        <v>205</v>
+      </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="43" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3231,26 +3231,26 @@
         <v>46142</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C22" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D22" s="41" t="inlineStr">
+        <v>95</v>
+      </c>
+      <c r="C22" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D22" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -3259,14 +3259,14 @@
         <v>46142</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>95</v>
+        <v>200</v>
       </c>
       <c r="C23" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D23" s="43" t="inlineStr">
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3278,7 +3278,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
@@ -3287,14 +3287,14 @@
         <v>46142</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="C24" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D24" s="41" t="inlineStr">
+      <c r="D24" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Air Liquid Max “Triple Black”</t>
         </is>
       </c>
     </row>
@@ -3322,7 +3322,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D25" s="43" t="inlineStr">
+      <c r="D25" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3350,7 +3350,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D26" s="41" t="inlineStr">
+      <c r="D26" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3378,7 +3378,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D27" s="43" t="inlineStr">
+      <c r="D27" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3406,7 +3406,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D28" s="41" t="inlineStr">
+      <c r="D28" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3434,7 +3434,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D29" s="43" t="inlineStr">
+      <c r="D29" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3462,7 +3462,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D30" s="41" t="inlineStr">
+      <c r="D30" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3490,7 +3490,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D31" s="43" t="inlineStr">
+      <c r="D31" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3518,7 +3518,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D32" s="41" t="inlineStr">
+      <c r="D32" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3546,7 +3546,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D33" s="43" t="inlineStr">
+      <c r="D33" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3574,7 +3574,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D34" s="41" t="inlineStr">
+      <c r="D34" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3602,7 +3602,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D35" s="43" t="inlineStr">
+      <c r="D35" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3630,7 +3630,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D36" s="41" t="inlineStr">
+      <c r="D36" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3651,7 +3651,7 @@
         <v>46151</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="D37" s="42" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
         <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>120</v>
+        <v>230</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -3688,17 +3688,17 @@
       </c>
       <c r="D38" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
         </is>
       </c>
     </row>
@@ -3707,26 +3707,26 @@
         <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C39" s="55" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D39" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>120</v>
+      </c>
+      <c r="C39" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D39" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -3735,26 +3735,26 @@
         <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C40" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D40" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C40" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -3763,26 +3763,26 @@
         <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C41" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D41" s="43" t="inlineStr">
+      <c r="D41" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -3798,7 +3798,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D42" s="41" t="inlineStr">
+      <c r="D42" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3826,7 +3826,7 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="D43" s="43" t="inlineStr">
+      <c r="D43" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3854,7 +3854,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D44" s="41" t="inlineStr">
+      <c r="D44" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3882,7 +3882,7 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="D45" s="43" t="inlineStr">
+      <c r="D45" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3910,7 +3910,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D46" s="53" t="inlineStr">
+      <c r="D46" s="41" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3938,7 +3938,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D47" s="43" t="inlineStr">
+      <c r="D47" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3966,7 +3966,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D48" s="41" t="inlineStr">
+      <c r="D48" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -3994,7 +3994,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D49" s="43" t="inlineStr">
+      <c r="D49" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4022,7 +4022,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D50" s="41" t="inlineStr">
+      <c r="D50" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4050,7 +4050,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="43" t="inlineStr">
+      <c r="D51" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4078,7 +4078,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D52" s="41" t="inlineStr">
+      <c r="D52" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4106,7 +4106,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D53" s="43" t="inlineStr">
+      <c r="D53" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4126,25 +4126,27 @@
       <c r="A54" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B54" s="33" t="inlineStr"/>
-      <c r="C54" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D54" s="41" t="inlineStr">
+      <c r="B54" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D54" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
@@ -4152,27 +4154,25 @@
       <c r="A55" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B55" s="38" t="n">
-        <v>250</v>
-      </c>
-      <c r="C55" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D55" s="43" t="inlineStr">
+      <c r="B55" s="38" t="inlineStr"/>
+      <c r="C55" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D55" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
@@ -4181,26 +4181,26 @@
         <v>46172</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="41" t="inlineStr">
+      <c r="D56" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
@@ -4208,13 +4208,15 @@
       <c r="A57" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B57" s="38" t="inlineStr"/>
+      <c r="B57" s="38" t="n">
+        <v>220</v>
+      </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D57" s="43" t="inlineStr">
+      <c r="D57" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4226,7 +4228,7 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4234,27 +4236,25 @@
       <c r="A58" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B58" s="33" t="n">
-        <v>120</v>
-      </c>
+      <c r="B58" s="33" t="inlineStr"/>
       <c r="C58" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D58" s="41" t="inlineStr">
+      <c r="D58" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4270,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D59" s="43" t="inlineStr">
+      <c r="D59" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4298,7 +4298,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D60" s="41" t="inlineStr">
+      <c r="D60" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4324,7 +4324,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D61" s="43" t="inlineStr">
+      <c r="D61" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4352,7 +4352,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D62" s="41" t="inlineStr">
+      <c r="D62" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4380,7 +4380,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D63" s="43" t="inlineStr">
+      <c r="D63" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
@@ -4408,7 +4408,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D64" s="41" t="inlineStr">
+      <c r="D64" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D65" s="43" t="inlineStr">
+      <c r="D65" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4464,9 +4464,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D66" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D66" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E66" s="30" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4485,26 +4485,26 @@
         <v>46186</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C67" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D67" s="43" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="C67" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D67" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E67" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Nike Air More Uptempo “Legacy”</t>
         </is>
       </c>
     </row>
@@ -4513,16 +4513,16 @@
         <v>46186</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C68" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D68" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>210</v>
+      </c>
+      <c r="C68" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D68" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -4541,26 +4541,26 @@
         <v>46186</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C69" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D69" s="43" t="inlineStr">
+        <v>205</v>
+      </c>
+      <c r="C69" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D69" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E69" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -4569,16 +4569,16 @@
         <v>46186</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C70" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D70" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C70" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D70" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E70" s="30" t="inlineStr">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike Air More Uptempo “Legacy”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4604,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D71" s="43" t="inlineStr">
+      <c r="D71" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4632,7 +4632,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D72" s="41" t="inlineStr">
+      <c r="D72" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4653,26 +4653,26 @@
         <v>46193</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C73" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C73" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -4681,16 +4681,16 @@
         <v>46193</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>162</v>
-      </c>
-      <c r="C74" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C74" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D74" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E74" s="30" t="inlineStr">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -4709,14 +4709,14 @@
         <v>46193</v>
       </c>
       <c r="B75" s="38" t="n">
-        <v>240</v>
+        <v>162</v>
       </c>
       <c r="C75" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D75" s="43" t="inlineStr">
+      <c r="D75" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4728,7 +4728,7 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
@@ -4737,16 +4737,16 @@
         <v>46193</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C76" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D76" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>240</v>
+      </c>
+      <c r="C76" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D76" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 Black Gum</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
@@ -4765,16 +4765,16 @@
         <v>46193</v>
       </c>
       <c r="B77" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C77" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D77" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C77" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D77" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E77" s="35" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Total 90 “University Red”</t>
+          <t>Nike SB P-Rod 1 Black Gum</t>
         </is>
       </c>
     </row>
@@ -4793,26 +4793,26 @@
         <v>46193</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C78" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D78" s="41" t="inlineStr">
+      <c r="D78" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
@@ -4821,14 +4821,14 @@
         <v>46199</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C79" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D79" s="43" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="C79" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D79" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4840,7 +4840,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
@@ -4849,14 +4849,14 @@
         <v>46199</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C80" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D80" s="41" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C80" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D80" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
         </is>
       </c>
     </row>
@@ -4884,7 +4884,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D81" s="43" t="inlineStr">
+      <c r="D81" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4905,14 +4905,14 @@
         <v>46200</v>
       </c>
       <c r="B82" s="33" t="inlineStr"/>
-      <c r="C82" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C82" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D82" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E82" s="30" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
@@ -4931,14 +4931,14 @@
         <v>46200</v>
       </c>
       <c r="B83" s="38" t="inlineStr"/>
-      <c r="C83" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="C83" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D83" s="42" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E83" s="35" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -4964,7 +4964,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D84" s="41" t="inlineStr">
+      <c r="D84" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -4992,7 +4992,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D85" s="43" t="inlineStr">
+      <c r="D85" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5020,7 +5020,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D86" s="41" t="inlineStr">
+      <c r="D86" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5048,7 +5048,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D87" s="43" t="inlineStr">
+      <c r="D87" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5076,7 +5076,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D88" s="53" t="inlineStr">
+      <c r="D88" s="41" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5104,7 +5104,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D89" s="43" t="inlineStr">
+      <c r="D89" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5132,7 +5132,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D90" s="41" t="inlineStr">
+      <c r="D90" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5160,7 +5160,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D91" s="43" t="inlineStr">
+      <c r="D91" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5188,7 +5188,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D92" s="41" t="inlineStr">
+      <c r="D92" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5216,7 +5216,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D93" s="42" t="inlineStr">
+      <c r="D93" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5242,7 +5242,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D94" s="53" t="inlineStr">
+      <c r="D94" s="41" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5270,7 +5270,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D95" s="43" t="inlineStr">
+      <c r="D95" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5286,8 +5286,64 @@
         </is>
       </c>
     </row>
+    <row r="96" ht="15" customHeight="1">
+      <c r="A96" s="31" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B96" s="33" t="n">
+        <v>210</v>
+      </c>
+      <c r="C96" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D96" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E96" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F96" s="30" t="inlineStr">
+        <is>
+          <t>Nike Air Zoom Huarache 2K4 “Sue Bird” PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="15" customHeight="1">
+      <c r="A97" s="36" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B97" s="38" t="n">
+        <v>250</v>
+      </c>
+      <c r="C97" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D97" s="55" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E97" s="35" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F97" s="35" t="inlineStr">
+        <is>
+          <t>Free The Youth x Air Jordan 16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F95"/>
+  <autoFilter ref="A3:F97"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5328,7 +5384,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 17, 2026  ·  07:51 UTC</t>
+          <t>Generated April 18, 2026  ·  07:13 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5371,10 +5427,10 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46129</v>
+        <v>46133</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>235</v>
+        <v>120</v>
       </c>
       <c r="C4" s="40" t="inlineStr">
         <is>
@@ -5383,7 +5439,7 @@
       </c>
       <c r="D4" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
@@ -5393,7 +5449,7 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Elite “Hurt Feelings Write History”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -5411,7 +5467,7 @@
       </c>
       <c r="D5" s="42" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -5421,35 +5477,35 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D6" s="41" t="inlineStr">
+      <c r="D6" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 Low</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -5458,35 +5514,35 @@
         <v>46135</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -5495,7 +5551,7 @@
       </c>
       <c r="D8" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
@@ -5505,7 +5561,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5521,7 +5577,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="43" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5549,7 +5605,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5579,7 +5635,7 @@
       </c>
       <c r="D11" s="42" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -5589,7 +5645,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5598,14 +5654,14 @@
         <v>46136</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="41" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5617,23 +5673,21 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="36" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B13" s="38" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B13" s="38" t="inlineStr"/>
       <c r="C13" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5645,7 +5699,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -5653,41 +5707,41 @@
       <c r="A14" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B14" s="33" t="inlineStr"/>
+      <c r="B14" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="41" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B15" s="38" t="n">
-        <v>215</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B15" s="38" t="inlineStr"/>
       <c r="C15" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5699,7 +5753,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5769,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="41" t="inlineStr">
+      <c r="D16" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5735,13 +5789,15 @@
       <c r="A17" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B17" s="38" t="inlineStr"/>
+      <c r="B17" s="38" t="n">
+        <v>205</v>
+      </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5753,23 +5809,23 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>205</v>
+        <v>165</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D18" s="41" t="inlineStr">
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5781,23 +5837,23 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 4 GS “Black Infrared 23”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D19" s="43" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5809,51 +5865,51 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 GS “Black Infrared 23”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>145</v>
+        <v>190</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D20" s="41" t="inlineStr">
+      <c r="D20" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="36" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="43" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5865,7 +5921,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -5874,14 +5930,14 @@
         <v>46150</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D22" s="41" t="inlineStr">
+      <c r="D22" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5893,7 +5949,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “WNBA”</t>
         </is>
       </c>
     </row>
@@ -5902,14 +5958,14 @@
         <v>46150</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="43" t="inlineStr">
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -5921,35 +5977,35 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “WNBA”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="41" t="inlineStr">
+      <c r="D24" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -5965,7 +6021,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D25" s="42" t="inlineStr">
+      <c r="D25" s="55" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5977,7 +6033,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Cinnabar” (2026)</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
         </is>
       </c>
     </row>
@@ -5993,7 +6049,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="41" t="inlineStr">
+      <c r="D26" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6016,7 +6072,7 @@
       <c r="B27" s="38" t="n">
         <v>155</v>
       </c>
-      <c r="C27" s="55" t="inlineStr">
+      <c r="C27" s="56" t="inlineStr">
         <is>
           <t>EXTREME</t>
         </is>
@@ -6049,7 +6105,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D28" s="41" t="inlineStr">
+      <c r="D28" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6067,101 +6123,101 @@
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>195</v>
+        <v>150</v>
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D29" s="43" t="inlineStr">
+      <c r="D29" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46157</v>
+        <v>46165</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D30" s="41" t="inlineStr">
+      <c r="D30" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D31" s="43" t="inlineStr">
+      <c r="D31" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D32" s="41" t="inlineStr">
+      <c r="D32" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6173,7 +6229,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6245,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D33" s="43" t="inlineStr">
+      <c r="D33" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6201,23 +6257,23 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="31" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D34" s="41" t="inlineStr">
+      <c r="D34" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6229,7 +6285,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
@@ -6245,7 +6301,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D35" s="43" t="inlineStr">
+      <c r="D35" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6273,7 +6329,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="41" t="inlineStr">
+      <c r="D36" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6299,7 +6355,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="43" t="inlineStr">
+      <c r="D37" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6317,43 +6373,43 @@
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B38" s="33" t="n">
-        <v>120</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B38" s="33" t="inlineStr"/>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D38" s="41" t="inlineStr">
+      <c r="D38" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B39" s="38" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B39" s="38" t="n">
+        <v>355</v>
+      </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D39" s="43" t="inlineStr">
+      <c r="D39" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6365,23 +6421,23 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46182</v>
+        <v>46186</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>355</v>
+        <v>205</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D40" s="41" t="inlineStr">
+      <c r="D40" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6393,7 +6449,7 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -6402,54 +6458,54 @@
         <v>46186</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C41" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D41" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D42" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D42" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6521,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D43" s="43" t="inlineStr">
+      <c r="D43" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6493,7 +6549,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D44" s="41" t="inlineStr">
+      <c r="D44" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6521,7 +6577,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D45" s="43" t="inlineStr">
+      <c r="D45" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6539,57 +6595,55 @@
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>215</v>
+        <v>190</v>
       </c>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D46" s="41" t="inlineStr">
+      <c r="D46" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46199</v>
-      </c>
-      <c r="B47" s="38" t="n">
-        <v>190</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B47" s="38" t="inlineStr"/>
       <c r="C47" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D47" s="43" t="inlineStr">
+      <c r="D47" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -6597,13 +6651,15 @@
       <c r="A48" s="31" t="n">
         <v>46200</v>
       </c>
-      <c r="B48" s="33" t="inlineStr"/>
+      <c r="B48" s="33" t="n">
+        <v>185</v>
+      </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D48" s="41" t="inlineStr">
+      <c r="D48" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6615,7 +6671,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -6624,26 +6680,26 @@
         <v>46200</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D49" s="43" t="inlineStr">
+      <c r="D49" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -6652,14 +6708,14 @@
         <v>46200</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D50" s="41" t="inlineStr">
+      <c r="D50" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6671,7 +6727,7 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -6680,14 +6736,14 @@
         <v>46200</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="43" t="inlineStr">
+      <c r="D51" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6699,13 +6755,13 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="B52" s="33" t="n">
         <v>135</v>
@@ -6717,7 +6773,7 @@
       </c>
       <c r="D52" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E52" s="30" t="inlineStr">
@@ -6727,16 +6783,16 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -6745,7 +6801,7 @@
       </c>
       <c r="D53" s="42" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E53" s="35" t="inlineStr">
@@ -6755,23 +6811,23 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46204</v>
+        <v>46210</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="41" t="inlineStr">
+      <c r="D54" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
@@ -6783,45 +6839,43 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="B55" s="38" t="n">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D55" s="43" t="inlineStr">
+      <c r="D55" s="42" t="inlineStr">
         <is>
           <t>Online + Retail</t>
         </is>
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Air Jordan 4 “Birds of Paradise”</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B56" s="33" t="n">
-        <v>215</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="B56" s="33" t="inlineStr"/>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6829,7 +6883,7 @@
       </c>
       <c r="D56" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
@@ -6839,15 +6893,17 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Birds of Paradise”</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46214</v>
-      </c>
-      <c r="B57" s="38" t="inlineStr"/>
+        <v>46218</v>
+      </c>
+      <c r="B57" s="38" t="n">
+        <v>205</v>
+      </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6855,7 +6911,7 @@
       </c>
       <c r="D57" s="42" t="inlineStr">
         <is>
-          <t>SNKRS App</t>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E57" s="35" t="inlineStr">
@@ -6865,16 +6921,16 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>Air Jordan 3 “Sports Renaissance”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
@@ -6883,7 +6939,7 @@
       </c>
       <c r="D58" s="41" t="inlineStr">
         <is>
-          <t>Online + Retail</t>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
@@ -6893,7 +6949,7 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Sports Renaissance”</t>
+          <t>Free The Youth x Air Jordan 16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-19 07:24 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$97</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,16 +679,16 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1584,7 +1584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 18, 2026  ·  07:13 UTC</t>
+          <t>Generated April 19, 2026  ·  07:24 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1632,12 +1632,12 @@
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$184</t>
+          <t>$185</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1740,7 +1740,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
         <v>46133</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
         <v>46133</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
         <v>46135</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1910,7 +1910,7 @@
         <v>46135</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
         <v>46136</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D21" s="37" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G21" s="47" t="inlineStr">
         <is>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D22" s="48" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="E23" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" ht="10" customHeight="1"/>
@@ -2156,17 +2156,17 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>4/18 – 4/24</t>
+          <t>4/19 – 4/25</t>
         </is>
       </c>
       <c r="C27" s="30" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D27" s="40" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -2177,17 +2177,17 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>4/25 – 5/1</t>
+          <t>4/26 – 5/2</t>
         </is>
       </c>
       <c r="C28" s="35" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D28" s="37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2198,17 +2198,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>5/2 – 5/8</t>
+          <t>5/3 – 5/9</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="D29" s="40" t="n">
         <v>9</v>
       </c>
-      <c r="D29" s="40" t="n">
-        <v>5</v>
-      </c>
       <c r="E29" s="30" t="n">
-        <v>5.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>5/9 – 5/15</t>
+          <t>5/10 – 5/16</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D30" s="37" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>6.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2240,17 +2240,17 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>5/16 – 5/22</t>
+          <t>5/17 – 5/23</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="D31" s="30" t="n">
-        <v>0</v>
+      <c r="D31" s="40" t="n">
+        <v>1</v>
       </c>
       <c r="E31" s="30" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -2261,17 +2261,17 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>5/23 – 5/29</t>
+          <t>5/24 – 5/30</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D32" s="37" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E32" s="35" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2282,17 +2282,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>5/30 – 6/5</t>
+          <t>5/31 – 6/6</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D33" s="40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E33" s="30" t="n">
-        <v>5.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2303,17 +2303,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>6/6 – 6/12</t>
+          <t>6/7 – 6/13</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D34" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2324,17 +2324,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>6/13 – 6/19</t>
+          <t>6/14 – 6/20</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
         <v>7</v>
       </c>
       <c r="D35" s="40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2345,17 +2345,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>6/20 – 6/26</t>
+          <t>6/21 – 6/27</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
         <v>9</v>
       </c>
       <c r="D36" s="37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>5.9</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2366,17 +2366,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>6/27 – 7/3</t>
+          <t>6/28 – 7/4</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D37" s="40" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2387,17 +2387,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>7/4 – 7/10</t>
+          <t>7/5 – 7/11</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="D38" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="D38" s="37" t="n">
-        <v>2</v>
-      </c>
       <c r="E38" s="35" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>7/11 – 7/17</t>
+          <t>7/12 – 7/18</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2608,7 +2608,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -2626,7 +2626,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2634,7 +2634,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -2685,7 +2685,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 18, 2026  ·  07:13 UTC</t>
+          <t>Generated April 19, 2026  ·  07:24 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2728,14 +2728,14 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C4" s="53" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>145</v>
+      </c>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D4" s="43" t="inlineStr">
@@ -2745,12 +2745,12 @@
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Willy Chavarria x adidas Superstar</t>
+          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
         </is>
       </c>
     </row>
@@ -2759,16 +2759,16 @@
         <v>46133</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C5" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D5" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>120</v>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D5" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Jurassic Park x Nike Ja 3 “Metallic Silver”</t>
+          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
         </is>
       </c>
     </row>
@@ -2794,9 +2794,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D6" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D6" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
@@ -2806,16 +2806,16 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 “Light Orewood Brown”</t>
+          <t>Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="36" t="n">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -2829,12 +2829,12 @@
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Air Force 1 Low</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2843,7 @@
         <v>46135</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -2857,12 +2857,12 @@
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
@@ -2871,11 +2871,11 @@
         <v>46135</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C9" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D9" s="42" t="inlineStr">
@@ -2890,25 +2890,25 @@
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Homecoming x Nike Air Max Plus</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C10" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D10" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>200</v>
+      </c>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Homecoming x Nike Air Max Plus</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -2927,26 +2927,26 @@
         <v>46136</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
         <v>46136</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
@@ -2969,12 +2969,12 @@
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -2983,7 +2983,7 @@
         <v>46136</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
         <v>46136</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
         <is>
@@ -3030,17 +3030,15 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B15" s="38" t="n">
-        <v>210</v>
-      </c>
+        <v>46137</v>
+      </c>
+      <c r="B15" s="38" t="inlineStr"/>
       <c r="C15" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3058,7 +3056,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3064,9 @@
       <c r="A16" s="31" t="n">
         <v>46137</v>
       </c>
-      <c r="B16" s="33" t="inlineStr"/>
+      <c r="B16" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C16" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3079,25 +3079,25 @@
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Air Jordan 5 “White Metallic” 2026</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="B17" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C17" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -3107,12 +3107,12 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “White Metallic” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
@@ -3120,12 +3120,10 @@
       <c r="A18" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B18" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C18" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B18" s="33" t="inlineStr"/>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D18" s="43" t="inlineStr">
@@ -3135,12 +3133,12 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3146,9 @@
       <c r="A19" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B19" s="38" t="inlineStr"/>
+      <c r="B19" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3166,7 +3166,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3175,7 +3175,7 @@
         <v>46142</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3203,11 +3203,11 @@
         <v>46142</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C21" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>95</v>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D21" s="42" t="inlineStr">
@@ -3217,12 +3217,12 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
         <v>46142</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>95</v>
+        <v>200</v>
       </c>
       <c r="C22" s="48" t="inlineStr">
         <is>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
         <v>46142</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="C23" s="54" t="inlineStr">
         <is>
@@ -3278,20 +3278,20 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Air Liquid Max “Triple Black”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C24" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>165</v>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D24" s="43" t="inlineStr">
@@ -3301,12 +3301,12 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Liquid Max “Triple Black”</t>
+          <t>Air Jordan 4 GS “Black Infrared 23”</t>
         </is>
       </c>
     </row>
@@ -3315,11 +3315,11 @@
         <v>46143</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>165</v>
-      </c>
-      <c r="C25" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C25" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D25" s="42" t="inlineStr">
@@ -3329,12 +3329,12 @@
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 GS “Black Infrared 23”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3343,7 @@
         <v>46143</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C26" s="48" t="inlineStr">
         <is>
@@ -3362,20 +3362,20 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C27" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>145</v>
+      </c>
+      <c r="C27" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D27" s="42" t="inlineStr">
@@ -3385,12 +3385,12 @@
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
@@ -3401,9 +3401,9 @@
       <c r="B28" s="33" t="n">
         <v>145</v>
       </c>
-      <c r="C28" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C28" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D28" s="43" t="inlineStr">
@@ -3413,12 +3413,12 @@
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike A’Two “A’Pink Shoe”</t>
         </is>
       </c>
     </row>
@@ -3446,20 +3446,20 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “A’Pink Shoe”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C30" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C30" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D30" s="43" t="inlineStr">
@@ -3474,20 +3474,20 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C31" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C31" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D31" s="42" t="inlineStr">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Book 2 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -3511,11 +3511,11 @@
         <v>46150</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C32" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C32" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D32" s="43" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “WNBA 30th Anniversary”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -3539,7 +3539,7 @@
         <v>46150</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “WNBA”</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3567,7 @@
         <v>46150</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “WNBA”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
@@ -3597,9 +3597,9 @@
       <c r="B35" s="38" t="n">
         <v>210</v>
       </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C35" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D35" s="42" t="inlineStr">
@@ -3614,20 +3614,20 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C36" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>195</v>
+      </c>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D36" s="43" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -3651,16 +3651,16 @@
         <v>46151</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D37" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
         </is>
       </c>
     </row>
@@ -3679,26 +3679,26 @@
         <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>230</v>
+        <v>120</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D38" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D38" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
@@ -3707,26 +3707,26 @@
         <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C39" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D39" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C39" s="55" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -3735,39 +3735,39 @@
         <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C40" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D40" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>200</v>
+      </c>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C41" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C41" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D41" s="42" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
@@ -3791,11 +3791,11 @@
         <v>46157</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C42" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C42" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D42" s="43" t="inlineStr">
@@ -3805,12 +3805,12 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Puma</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>PUMA MB.05 Lo “Flourish”</t>
         </is>
       </c>
     </row>
@@ -3819,11 +3819,11 @@
         <v>46157</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="C43" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>150</v>
+      </c>
+      <c r="C43" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D43" s="42" t="inlineStr">
@@ -3833,25 +3833,25 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>PUMA MB.05 Lo “Flourish”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C44" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C44" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D44" s="43" t="inlineStr">
@@ -3861,58 +3861,58 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46158</v>
+        <v>46163</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="C45" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D45" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C45" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D45" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Air Max Mad 90 Pack</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="C46" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D46" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="30" t="inlineStr">
@@ -3922,20 +3922,20 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max Mad 90 Pack</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C47" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C47" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D47" s="42" t="inlineStr">
@@ -3945,21 +3945,21 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
@@ -3973,25 +3973,25 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46168</v>
+        <v>46170</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C49" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>150</v>
+      </c>
+      <c r="C49" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D49" s="42" t="inlineStr">
@@ -4006,20 +4006,20 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Book 2 “Haven and Hector”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C50" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D50" s="43" t="inlineStr">
@@ -4034,7 +4034,7 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Haven and Hector”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4043,11 +4043,11 @@
         <v>46171</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C51" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C51" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
@@ -4071,11 +4071,11 @@
         <v>46171</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C52" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D52" s="43" t="inlineStr">
@@ -4090,16 +4090,16 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
@@ -4126,12 +4126,10 @@
       <c r="A54" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B54" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C54" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B54" s="33" t="inlineStr"/>
+      <c r="C54" s="56" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D54" s="43" t="inlineStr">
@@ -4141,12 +4139,12 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
@@ -4154,10 +4152,12 @@
       <c r="A55" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B55" s="38" t="inlineStr"/>
-      <c r="C55" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B55" s="38" t="n">
+        <v>250</v>
+      </c>
+      <c r="C55" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D55" s="42" t="inlineStr">
@@ -4167,12 +4167,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
         <v>46172</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -4195,12 +4195,12 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4208,9 +4208,7 @@
       <c r="A57" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B57" s="38" t="n">
-        <v>220</v>
-      </c>
+      <c r="B57" s="38" t="inlineStr"/>
       <c r="C57" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4228,18 +4226,20 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B58" s="33" t="inlineStr"/>
-      <c r="C58" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46173</v>
+      </c>
+      <c r="B58" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C58" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D58" s="43" t="inlineStr">
@@ -4249,21 +4249,21 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="C59" s="54" t="inlineStr">
         <is>
@@ -4282,20 +4282,18 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B60" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C60" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B60" s="33" t="inlineStr"/>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
@@ -4305,20 +4303,22 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B61" s="38" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B61" s="38" t="n">
+        <v>355</v>
+      </c>
       <c r="C61" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4336,20 +4336,20 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46182</v>
+        <v>46185</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="C62" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C62" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D62" s="43" t="inlineStr">
@@ -4359,12 +4359,12 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
@@ -4420,16 +4420,16 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="C65" s="54" t="inlineStr">
         <is>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4457,7 +4457,7 @@
         <v>46186</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="C66" s="48" t="inlineStr">
         <is>
@@ -4476,7 +4476,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Nike Air More Uptempo “Legacy”</t>
         </is>
       </c>
     </row>
@@ -4485,16 +4485,16 @@
         <v>46186</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C67" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D67" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D67" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E67" s="35" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike Air More Uptempo “Legacy”</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
@@ -4513,26 +4513,26 @@
         <v>46186</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C68" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D68" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>205</v>
+      </c>
+      <c r="C68" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D68" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -4541,26 +4541,26 @@
         <v>46186</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C69" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D69" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D69" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E69" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -4569,16 +4569,16 @@
         <v>46186</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C70" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D70" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>155</v>
+      </c>
+      <c r="C70" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D70" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E70" s="30" t="inlineStr">
@@ -4588,16 +4588,16 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>155</v>
+        <v>135</v>
       </c>
       <c r="C71" s="54" t="inlineStr">
         <is>
@@ -4616,20 +4616,20 @@
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C72" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C72" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D72" s="43" t="inlineStr">
@@ -4639,12 +4639,12 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -4653,26 +4653,26 @@
         <v>46193</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C73" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D73" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>210</v>
+      </c>
+      <c r="C73" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D73" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -4681,16 +4681,16 @@
         <v>46193</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C74" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D74" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>162</v>
+      </c>
+      <c r="C74" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D74" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E74" s="30" t="inlineStr">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
@@ -4709,7 +4709,7 @@
         <v>46193</v>
       </c>
       <c r="B75" s="38" t="n">
-        <v>162</v>
+        <v>240</v>
       </c>
       <c r="C75" s="37" t="inlineStr">
         <is>
@@ -4728,7 +4728,7 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
@@ -4737,16 +4737,16 @@
         <v>46193</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C76" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D76" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C76" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D76" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike SB P-Rod 1 Black Gum</t>
         </is>
       </c>
     </row>
@@ -4765,16 +4765,16 @@
         <v>46193</v>
       </c>
       <c r="B77" s="38" t="n">
-        <v>125</v>
-      </c>
-      <c r="C77" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D77" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="C77" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D77" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E77" s="35" t="inlineStr">
@@ -4784,20 +4784,20 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 Black Gum</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C78" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C78" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D78" s="43" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Total 90 “University Red”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
@@ -4821,11 +4821,11 @@
         <v>46199</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C79" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C79" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4840,7 +4840,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
         </is>
       </c>
     </row>
@@ -4849,11 +4849,11 @@
         <v>46199</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C80" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C80" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D80" s="43" t="inlineStr">
@@ -4868,35 +4868,33 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46199</v>
-      </c>
-      <c r="B81" s="38" t="n">
-        <v>180</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B81" s="38" t="inlineStr"/>
       <c r="C81" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D81" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D81" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
@@ -4905,14 +4903,14 @@
         <v>46200</v>
       </c>
       <c r="B82" s="33" t="inlineStr"/>
-      <c r="C82" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D82" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C82" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D82" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E82" s="30" t="inlineStr">
@@ -4922,7 +4920,7 @@
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -4930,7 +4928,9 @@
       <c r="A83" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B83" s="38" t="inlineStr"/>
+      <c r="B83" s="38" t="n">
+        <v>185</v>
+      </c>
       <c r="C83" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
         <v>46200</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C84" s="40" t="inlineStr">
         <is>
@@ -4971,12 +4971,12 @@
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
         <v>46200</v>
       </c>
       <c r="B85" s="38" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="C85" s="37" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
         <v>46200</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="C86" s="40" t="inlineStr">
         <is>
@@ -5032,13 +5032,13 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="36" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="B87" s="38" t="n">
         <v>135</v>
@@ -5048,9 +5048,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D87" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D87" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
@@ -5060,25 +5060,25 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C88" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D88" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D88" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
@@ -5088,20 +5088,20 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C89" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C89" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D89" s="42" t="inlineStr">
@@ -5116,20 +5116,20 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
+          <t>Nike Ja 3 “Animal Instinct”</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46206</v>
+        <v>46210</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C90" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>210</v>
+      </c>
+      <c r="C90" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D90" s="43" t="inlineStr">
@@ -5144,16 +5144,16 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Animal Instinct”</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C91" s="37" t="inlineStr">
         <is>
@@ -5167,12 +5167,12 @@
       </c>
       <c r="E91" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Air Jordan 4 “Birds of Paradise”</t>
         </is>
       </c>
     </row>
@@ -5181,16 +5181,16 @@
         <v>46213</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C92" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D92" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>355</v>
+      </c>
+      <c r="C92" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D92" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E92" s="30" t="inlineStr">
@@ -5200,23 +5200,21 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Birds of Paradise”</t>
+          <t>Air Jordan 8 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B93" s="38" t="n">
-        <v>355</v>
-      </c>
-      <c r="C93" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D93" s="55" t="inlineStr">
+        <v>46214</v>
+      </c>
+      <c r="B93" s="38" t="inlineStr"/>
+      <c r="C93" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D93" s="53" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5228,23 +5226,25 @@
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 8 “BIN 23”</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="31" t="n">
-        <v>46214</v>
-      </c>
-      <c r="B94" s="33" t="inlineStr"/>
+        <v>46218</v>
+      </c>
+      <c r="B94" s="33" t="n">
+        <v>205</v>
+      </c>
       <c r="C94" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D94" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D94" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
@@ -5254,20 +5254,20 @@
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>Air Jordan 3 “Sports Renaissance”</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="36" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C95" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C95" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D95" s="42" t="inlineStr">
@@ -5277,12 +5277,12 @@
       </c>
       <c r="E95" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Sports Renaissance”</t>
+          <t>Nike Air Zoom Huarache 2K4 “Sue Bird” PE</t>
         </is>
       </c>
     </row>
@@ -5291,44 +5291,44 @@
         <v>46220</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C96" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D96" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>250</v>
+      </c>
+      <c r="C96" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D96" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4 “Sue Bird” PE</t>
+          <t>Free The Youth x Air Jordan 16</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="36" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="B97" s="38" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="C97" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D97" s="55" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D97" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E97" s="35" t="inlineStr">
@@ -5338,7 +5338,7 @@
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 16</t>
+          <t>Air Jordan 3 OG “True Blue” 2026</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5384,7 +5384,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 18, 2026  ·  07:13 UTC</t>
+          <t>Generated April 19, 2026  ·  07:24 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -6021,7 +6021,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D25" s="55" t="inlineStr">
+      <c r="D25" s="53" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -6072,7 +6072,7 @@
       <c r="B27" s="38" t="n">
         <v>155</v>
       </c>
-      <c r="C27" s="56" t="inlineStr">
+      <c r="C27" s="55" t="inlineStr">
         <is>
           <t>EXTREME</t>
         </is>
@@ -6953,8 +6953,36 @@
         </is>
       </c>
     </row>
+    <row r="59" ht="15" customHeight="1">
+      <c r="A59" s="36" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B59" s="38" t="n">
+        <v>230</v>
+      </c>
+      <c r="C59" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D59" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E59" s="35" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F59" s="35" t="inlineStr">
+        <is>
+          <t>Air Jordan 3 OG “True Blue” 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F58"/>
+  <autoFilter ref="A3:F59"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-20 08:12 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$97</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -549,7 +549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -688,9 +688,6 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -811,12 +808,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Charts'!$A$2:$A$5</f>
+              <f>'Charts'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$B$2:$B$5</f>
+              <f>'Charts'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -1554,7 +1551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1584,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 19, 2026  ·  07:24 UTC</t>
+          <t>Generated April 20, 2026  ·  08:12 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1624,7 +1621,7 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
@@ -1632,7 +1629,7 @@
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
@@ -1740,7 +1737,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1774,7 +1771,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1808,7 +1805,7 @@
         <v>46133</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1842,7 +1839,7 @@
         <v>46133</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1864,19 +1861,19 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
         <v>46135</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1887,7 +1884,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="H14" s="43" t="inlineStr">
         <is>
@@ -1898,19 +1895,19 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C15" s="36" t="n">
         <v>46135</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1921,7 +1918,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="H15" s="42" t="inlineStr">
         <is>
@@ -1932,19 +1929,19 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C16" s="31" t="n">
         <v>46136</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -1955,11 +1952,11 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="H16" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>205</v>
+      </c>
+      <c r="H16" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2014,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2033,7 +2030,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2043,7 +2040,7 @@
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D21" s="37" t="inlineStr">
         <is>
@@ -2051,7 +2048,7 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G21" s="47" t="inlineStr">
         <is>
@@ -2077,7 +2074,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G22" s="49" t="inlineStr">
         <is>
@@ -2091,7 +2088,7 @@
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="46" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="B23" s="35" t="n">
@@ -2103,321 +2100,331 @@
         </is>
       </c>
       <c r="E23" s="35" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="44" t="inlineStr">
+        <is>
+          <t>Puma</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" ht="10" customHeight="1"/>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Weekly Outlook (Next 13 Weeks)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>Releases</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="inlineStr">
+        <is>
+          <t>HIGH+EXTREME</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>Avg Hype Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Week 1</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>4/20 – 4/26</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="n">
+        <v>13</v>
+      </c>
+      <c r="D28" s="40" t="n">
+        <v>11</v>
+      </c>
+      <c r="E28" s="30" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>4/27 – 5/3</t>
+        </is>
+      </c>
+      <c r="C29" s="35" t="n">
+        <v>13</v>
+      </c>
+      <c r="D29" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" s="35" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Week 3</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>5/4 – 5/10</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="n">
+        <v>11</v>
+      </c>
+      <c r="D30" s="40" t="n">
+        <v>9</v>
+      </c>
+      <c r="E30" s="30" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="35" t="inlineStr">
+        <is>
+          <t>Week 4</t>
+        </is>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>5/11 – 5/17</t>
+        </is>
+      </c>
+      <c r="C31" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="D31" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="35" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>5/18 – 5/24</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="24" ht="10" customHeight="1"/>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="28" t="inlineStr">
-        <is>
-          <t>Weekly Outlook (Next 13 Weeks)</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="B26" s="29" t="inlineStr">
-        <is>
-          <t>Dates</t>
-        </is>
-      </c>
-      <c r="C26" s="29" t="inlineStr">
-        <is>
-          <t>Releases</t>
-        </is>
-      </c>
-      <c r="D26" s="29" t="inlineStr">
-        <is>
-          <t>HIGH+EXTREME</t>
-        </is>
-      </c>
-      <c r="E26" s="29" t="inlineStr">
-        <is>
-          <t>Avg Hype Score</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>Week 1</t>
-        </is>
-      </c>
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t>4/19 – 4/25</t>
-        </is>
-      </c>
-      <c r="C27" s="30" t="n">
-        <v>13</v>
-      </c>
-      <c r="D27" s="40" t="n">
+      <c r="D32" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="30" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="35" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="B33" s="35" t="inlineStr">
+        <is>
+          <t>5/25 – 5/31</t>
+        </is>
+      </c>
+      <c r="C33" s="35" t="n">
         <v>11</v>
       </c>
-      <c r="E27" s="30" t="n">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="35" t="inlineStr">
-        <is>
-          <t>Week 2</t>
-        </is>
-      </c>
-      <c r="B28" s="35" t="inlineStr">
-        <is>
-          <t>4/26 – 5/2</t>
-        </is>
-      </c>
-      <c r="C28" s="35" t="n">
-        <v>13</v>
-      </c>
-      <c r="D28" s="37" t="n">
-        <v>5</v>
-      </c>
-      <c r="E28" s="35" t="n">
-        <v>5.2</v>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>Week 3</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>5/3 – 5/9</t>
-        </is>
-      </c>
-      <c r="C29" s="30" t="n">
-        <v>11</v>
-      </c>
-      <c r="D29" s="40" t="n">
+      <c r="D33" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="E33" s="35" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Week 7</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>6/1 – 6/7</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="30" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="35" t="inlineStr">
+        <is>
+          <t>Week 8</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>6/8 – 6/14</t>
+        </is>
+      </c>
+      <c r="C35" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" s="35" t="n">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>Week 9</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>6/15 – 6/21</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="E36" s="30" t="n">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>Week 10</t>
+        </is>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>6/22 – 6/28</t>
+        </is>
+      </c>
+      <c r="C37" s="35" t="n">
         <v>9</v>
       </c>
-      <c r="E29" s="30" t="n">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="35" t="inlineStr">
-        <is>
-          <t>Week 4</t>
-        </is>
-      </c>
-      <c r="B30" s="35" t="inlineStr">
-        <is>
-          <t>5/10 – 5/16</t>
-        </is>
-      </c>
-      <c r="C30" s="35" t="n">
+      <c r="D37" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="E37" s="35" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Week 11</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>6/29 – 7/5</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" s="30" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>Week 12</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>7/6 – 7/12</t>
+        </is>
+      </c>
+      <c r="C39" s="35" t="n">
         <v>4</v>
       </c>
-      <c r="D30" s="37" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="35" t="n">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Week 5</t>
-        </is>
-      </c>
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>5/17 – 5/23</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="n">
+      <c r="D39" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="D31" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="30" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="35" t="inlineStr">
-        <is>
-          <t>Week 6</t>
-        </is>
-      </c>
-      <c r="B32" s="35" t="inlineStr">
-        <is>
-          <t>5/24 – 5/30</t>
-        </is>
-      </c>
-      <c r="C32" s="35" t="n">
-        <v>10</v>
-      </c>
-      <c r="D32" s="37" t="n">
-        <v>7</v>
-      </c>
-      <c r="E32" s="35" t="n">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>Week 7</t>
-        </is>
-      </c>
-      <c r="B33" s="30" t="inlineStr">
-        <is>
-          <t>5/31 – 6/6</t>
-        </is>
-      </c>
-      <c r="C33" s="30" t="n">
+      <c r="E39" s="35" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Week 13</t>
+        </is>
+      </c>
+      <c r="B40" s="30" t="inlineStr">
+        <is>
+          <t>7/13 – 7/19</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" s="40" t="n">
         <v>3</v>
       </c>
-      <c r="D33" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="30" t="n">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="35" t="inlineStr">
-        <is>
-          <t>Week 8</t>
-        </is>
-      </c>
-      <c r="B34" s="35" t="inlineStr">
-        <is>
-          <t>6/7 – 6/13</t>
-        </is>
-      </c>
-      <c r="C34" s="35" t="n">
-        <v>10</v>
-      </c>
-      <c r="D34" s="37" t="n">
-        <v>3</v>
-      </c>
-      <c r="E34" s="35" t="n">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="30" t="inlineStr">
-        <is>
-          <t>Week 9</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>6/14 – 6/20</t>
-        </is>
-      </c>
-      <c r="C35" s="30" t="n">
-        <v>7</v>
-      </c>
-      <c r="D35" s="40" t="n">
-        <v>4</v>
-      </c>
-      <c r="E35" s="30" t="n">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="36" ht="15" customHeight="1">
-      <c r="A36" s="35" t="inlineStr">
-        <is>
-          <t>Week 10</t>
-        </is>
-      </c>
-      <c r="B36" s="35" t="inlineStr">
-        <is>
-          <t>6/21 – 6/27</t>
-        </is>
-      </c>
-      <c r="C36" s="35" t="n">
-        <v>9</v>
-      </c>
-      <c r="D36" s="37" t="n">
-        <v>6</v>
-      </c>
-      <c r="E36" s="35" t="n">
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="30" t="inlineStr">
-        <is>
-          <t>Week 11</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="inlineStr">
-        <is>
-          <t>6/28 – 7/4</t>
-        </is>
-      </c>
-      <c r="C37" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="D37" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="E37" s="30" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="35" t="inlineStr">
-        <is>
-          <t>Week 12</t>
-        </is>
-      </c>
-      <c r="B38" s="35" t="inlineStr">
-        <is>
-          <t>7/5 – 7/11</t>
-        </is>
-      </c>
-      <c r="C38" s="35" t="n">
-        <v>4</v>
-      </c>
-      <c r="D38" s="37" t="n">
-        <v>3</v>
-      </c>
-      <c r="E38" s="35" t="n">
-        <v>6.8</v>
-      </c>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="30" t="inlineStr">
-        <is>
-          <t>Week 13</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="inlineStr">
-        <is>
-          <t>7/12 – 7/18</t>
-        </is>
-      </c>
-      <c r="C39" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="D39" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="E39" s="30" t="n">
+      <c r="E40" s="30" t="n">
         <v>6.2</v>
       </c>
     </row>
@@ -2429,7 +2436,7 @@
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="A5:B5"/>
@@ -2516,7 +2523,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2532,7 +2539,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2550,7 +2557,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2558,7 +2565,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2592,7 +2599,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2608,13 +2615,13 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2626,7 +2633,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2638,6 +2645,14 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Puma</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>$300+</t>
@@ -2659,7 +2674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2685,7 +2700,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 19, 2026  ·  07:24 UTC</t>
+          <t>Generated April 20, 2026  ·  08:12 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2815,7 +2830,7 @@
         <v>46135</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -2829,12 +2844,12 @@
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2858,7 @@
         <v>46135</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -2857,12 +2872,12 @@
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -2899,26 +2914,26 @@
         <v>46136</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2942,7 @@
         <v>46136</v>
       </c>
       <c r="B11" s="38" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
@@ -2941,12 +2956,12 @@
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -2955,16 +2970,16 @@
         <v>46136</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
@@ -2974,7 +2989,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3092,12 +3107,10 @@
       <c r="A17" s="36" t="n">
         <v>46142</v>
       </c>
-      <c r="B17" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C17" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B17" s="38" t="inlineStr"/>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -3107,12 +3120,12 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3133,9 @@
       <c r="A18" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B18" s="33" t="inlineStr"/>
+      <c r="B18" s="33" t="n">
+        <v>215</v>
+      </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3138,7 +3153,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3162,7 @@
         <v>46142</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
@@ -3166,7 +3181,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3175,11 +3190,11 @@
         <v>46142</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C20" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C20" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D20" s="43" t="inlineStr">
@@ -3189,12 +3204,12 @@
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
@@ -3287,11 +3302,11 @@
         <v>46143</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>165</v>
-      </c>
-      <c r="C24" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C24" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D24" s="43" t="inlineStr">
@@ -3301,12 +3316,12 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 GS “Black Infrared 23”</t>
+          <t>Nike Air Zoom Huarache 2K4 “White Varsity Red”</t>
         </is>
       </c>
     </row>
@@ -3623,16 +3638,16 @@
         <v>46151</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>195</v>
-      </c>
-      <c r="C36" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D36" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C36" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
@@ -3642,7 +3657,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -3651,26 +3666,26 @@
         <v>46151</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D37" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3694,7 @@
         <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>120</v>
+        <v>195</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -3693,12 +3708,12 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -3707,16 +3722,16 @@
         <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C39" s="55" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D39" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>230</v>
+      </c>
+      <c r="C39" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D39" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
@@ -3726,7 +3741,7 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3750,7 @@
         <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
@@ -3754,20 +3769,20 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46157</v>
+        <v>46156</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C41" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C41" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D41" s="42" t="inlineStr">
@@ -3777,12 +3792,12 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Converse SHAI 001 Premium “Ink”</t>
         </is>
       </c>
     </row>
@@ -3791,11 +3806,11 @@
         <v>46157</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C42" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>170</v>
+      </c>
+      <c r="C42" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D42" s="43" t="inlineStr">
@@ -3805,12 +3820,12 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>PUMA MB.05 Lo “Flourish”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
@@ -3819,11 +3834,11 @@
         <v>46157</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C43" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>120</v>
+      </c>
+      <c r="C43" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D43" s="42" t="inlineStr">
@@ -3833,25 +3848,25 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Puma</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>PUMA MB.05 Lo “Flourish”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C44" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>150</v>
+      </c>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D44" s="43" t="inlineStr">
@@ -3861,58 +3876,58 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46163</v>
+        <v>46158</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C45" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D45" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C45" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D45" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Mad 90 Pack</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46164</v>
+        <v>46163</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="C46" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D46" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D46" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E46" s="30" t="inlineStr">
@@ -3922,20 +3937,20 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>Nike Air Max Mad 90 Pack</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46165</v>
+        <v>46164</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C47" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C47" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D47" s="42" t="inlineStr">
@@ -3945,21 +3960,21 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46168</v>
+        <v>46165</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
@@ -3973,25 +3988,25 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46170</v>
+        <v>46168</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C49" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C49" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D49" s="42" t="inlineStr">
@@ -4006,20 +4021,20 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Haven and Hector”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46171</v>
+        <v>46170</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C50" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>150</v>
+      </c>
+      <c r="C50" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D50" s="43" t="inlineStr">
@@ -4034,7 +4049,7 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Book 2 “Haven and Hector”</t>
         </is>
       </c>
     </row>
@@ -4043,11 +4058,11 @@
         <v>46171</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C51" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C51" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D51" s="42" t="inlineStr">
@@ -4062,7 +4077,7 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -4071,11 +4086,11 @@
         <v>46171</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C52" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C52" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D52" s="43" t="inlineStr">
@@ -4090,16 +4105,16 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -4118,7 +4133,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -4126,10 +4141,12 @@
       <c r="A54" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B54" s="33" t="inlineStr"/>
-      <c r="C54" s="56" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B54" s="33" t="n">
+        <v>220</v>
+      </c>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D54" s="43" t="inlineStr">
@@ -4139,12 +4156,12 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>adidas Crazy 3 “Silver Metallic”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -4152,9 +4169,7 @@
       <c r="A55" s="36" t="n">
         <v>46172</v>
       </c>
-      <c r="B55" s="38" t="n">
-        <v>250</v>
-      </c>
+      <c r="B55" s="38" t="inlineStr"/>
       <c r="C55" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4167,12 +4182,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4196,7 @@
         <v>46172</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
@@ -4195,12 +4210,12 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
@@ -4209,9 +4224,9 @@
         <v>46172</v>
       </c>
       <c r="B57" s="38" t="inlineStr"/>
-      <c r="C57" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C57" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D57" s="42" t="inlineStr">
@@ -4221,25 +4236,25 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>adidas Crazy 3 “Silver Metallic”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C58" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D58" s="43" t="inlineStr">
@@ -4254,16 +4269,16 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46177</v>
+        <v>46173</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="C59" s="54" t="inlineStr">
         <is>
@@ -4282,18 +4297,20 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B60" s="33" t="inlineStr"/>
-      <c r="C60" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46177</v>
+      </c>
+      <c r="B60" s="33" t="n">
+        <v>140</v>
+      </c>
+      <c r="C60" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
@@ -4303,22 +4320,20 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B61" s="38" t="n">
-        <v>355</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B61" s="38" t="inlineStr"/>
       <c r="C61" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4336,20 +4351,20 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C62" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>355</v>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D62" s="43" t="inlineStr">
@@ -4359,12 +4374,12 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -4420,16 +4435,16 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="36" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B65" s="38" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C65" s="54" t="inlineStr">
         <is>
@@ -4448,7 +4463,7 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -4457,11 +4472,11 @@
         <v>46186</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C66" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C66" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D66" s="43" t="inlineStr">
@@ -4471,12 +4486,12 @@
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nike Air More Uptempo “Legacy”</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -4485,16 +4500,16 @@
         <v>46186</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C67" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D67" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C67" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D67" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E67" s="35" t="inlineStr">
@@ -4504,7 +4519,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -4513,11 +4528,11 @@
         <v>46186</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C68" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C68" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D68" s="43" t="inlineStr">
@@ -4527,12 +4542,12 @@
       </c>
       <c r="E68" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4541,16 +4556,16 @@
         <v>46186</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C69" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D69" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>180</v>
+      </c>
+      <c r="C69" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D69" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E69" s="35" t="inlineStr">
@@ -4560,7 +4575,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air More Uptempo “Legacy”</t>
         </is>
       </c>
     </row>
@@ -4569,16 +4584,16 @@
         <v>46186</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>155</v>
+        <v>210</v>
       </c>
       <c r="C70" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D70" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D70" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E70" s="30" t="inlineStr">
@@ -4588,16 +4603,16 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="C71" s="54" t="inlineStr">
         <is>
@@ -4616,20 +4631,20 @@
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C72" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C72" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D72" s="43" t="inlineStr">
@@ -4639,12 +4654,12 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
@@ -4653,16 +4668,16 @@
         <v>46193</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C73" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D73" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>162</v>
+      </c>
+      <c r="C73" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D73" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E73" s="35" t="inlineStr">
@@ -4672,7 +4687,7 @@
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4696,7 @@
         <v>46193</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>162</v>
+        <v>240</v>
       </c>
       <c r="C74" s="40" t="inlineStr">
         <is>
@@ -4700,7 +4715,7 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
@@ -4709,16 +4724,16 @@
         <v>46193</v>
       </c>
       <c r="B75" s="38" t="n">
-        <v>240</v>
-      </c>
-      <c r="C75" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D75" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C75" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D75" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E75" s="35" t="inlineStr">
@@ -4728,7 +4743,7 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike SB P-Rod 1 Black Gum</t>
         </is>
       </c>
     </row>
@@ -4737,16 +4752,16 @@
         <v>46193</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C76" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D76" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="C76" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D76" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
@@ -4756,7 +4771,7 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 Black Gum</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
@@ -4765,7 +4780,7 @@
         <v>46193</v>
       </c>
       <c r="B77" s="38" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C77" s="37" t="inlineStr">
         <is>
@@ -4779,30 +4794,30 @@
       </c>
       <c r="E77" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Total 90 “University Red”</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="31" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C78" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D78" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D78" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E78" s="30" t="inlineStr">
@@ -4812,7 +4827,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>Off-White x Nike Cryoshot “Virgil Abloh Archives”</t>
         </is>
       </c>
     </row>
@@ -4821,11 +4836,11 @@
         <v>46199</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C79" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C79" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4840,7 +4855,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
@@ -4849,11 +4864,11 @@
         <v>46199</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C80" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C80" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D80" s="43" t="inlineStr">
@@ -4868,33 +4883,35 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B81" s="38" t="inlineStr"/>
+        <v>46199</v>
+      </c>
+      <c r="B81" s="38" t="n">
+        <v>180</v>
+      </c>
       <c r="C81" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D81" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D81" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 7 “Miro” 2026</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
@@ -5038,14 +5055,12 @@
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="36" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B87" s="38" t="n">
-        <v>135</v>
-      </c>
-      <c r="C87" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46200</v>
+      </c>
+      <c r="B87" s="38" t="inlineStr"/>
+      <c r="C87" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D87" s="53" t="inlineStr">
@@ -5055,30 +5070,30 @@
       </c>
       <c r="E87" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Air Jordan 7 “Miro” 2026</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46204</v>
+        <v>46203</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>190</v>
+        <v>135</v>
       </c>
       <c r="C88" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D88" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D88" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
@@ -5088,20 +5103,20 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46206</v>
+        <v>46204</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>130</v>
-      </c>
-      <c r="C89" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C89" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D89" s="42" t="inlineStr">
@@ -5116,20 +5131,20 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Animal Instinct”</t>
+          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46210</v>
+        <v>46206</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C90" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C90" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D90" s="43" t="inlineStr">
@@ -5144,16 +5159,16 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Nike Ja 3 “Animal Instinct”</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46213</v>
+        <v>46210</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="C91" s="37" t="inlineStr">
         <is>
@@ -5167,12 +5182,12 @@
       </c>
       <c r="E91" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Birds of Paradise”</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
@@ -5206,17 +5221,19 @@
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46214</v>
-      </c>
-      <c r="B93" s="38" t="inlineStr"/>
+        <v>46213</v>
+      </c>
+      <c r="B93" s="38" t="n">
+        <v>215</v>
+      </c>
       <c r="C93" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D93" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D93" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E93" s="35" t="inlineStr">
@@ -5226,25 +5243,23 @@
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>Air Jordan 4 “Birds of Paradise”</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="31" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B94" s="33" t="n">
-        <v>205</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="B94" s="33" t="inlineStr"/>
       <c r="C94" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D94" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D94" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
@@ -5254,20 +5269,20 @@
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Sports Renaissance”</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="36" t="n">
-        <v>46220</v>
+        <v>46218</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C95" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C95" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D95" s="42" t="inlineStr">
@@ -5277,12 +5292,12 @@
       </c>
       <c r="E95" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4 “Sue Bird” PE</t>
+          <t>Air Jordan 3 “Sports Renaissance”</t>
         </is>
       </c>
     </row>
@@ -5291,59 +5306,87 @@
         <v>46220</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="C96" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D96" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>210</v>
+      </c>
+      <c r="C96" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D96" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 16</t>
+          <t>Nike Air Zoom Huarache 2K4 “Sue Bird” PE</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="36" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B97" s="38" t="n">
+        <v>250</v>
+      </c>
+      <c r="C97" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D97" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E97" s="35" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F97" s="35" t="inlineStr">
+        <is>
+          <t>Free The Youth x Air Jordan 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="15" customHeight="1">
+      <c r="A98" s="31" t="n">
         <v>46221</v>
       </c>
-      <c r="B97" s="38" t="n">
+      <c r="B98" s="33" t="n">
         <v>230</v>
       </c>
-      <c r="C97" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D97" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E97" s="35" t="inlineStr">
+      <c r="C98" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D98" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E98" s="30" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="F97" s="35" t="inlineStr">
+      <c r="F98" s="30" t="inlineStr">
         <is>
           <t>Air Jordan 3 OG “True Blue” 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F97"/>
+  <autoFilter ref="A3:F98"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5358,7 +5401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5384,7 +5427,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 19, 2026  ·  07:24 UTC</t>
+          <t>Generated April 20, 2026  ·  08:12 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5486,7 +5529,7 @@
         <v>46135</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
@@ -5500,12 +5543,12 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
@@ -5514,7 +5557,7 @@
         <v>46135</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -5528,12 +5571,12 @@
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -5542,26 +5585,26 @@
         <v>46136</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
+          <t>Air Jordan 4028 “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5613,7 @@
         <v>46136</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
@@ -5584,12 +5627,12 @@
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Black Metallic Gold”</t>
+          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5598,16 +5641,16 @@
         <v>46136</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -5617,7 +5660,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low Protro “Siempre Hermanos”</t>
+          <t>Nike Kobe 8 Protro EXT “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -5815,10 +5858,10 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
@@ -5837,16 +5880,16 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 GS “Black Infrared 23”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="36" t="n">
-        <v>46144</v>
+        <v>46149</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>145</v>
+        <v>190</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
@@ -5860,21 +5903,21 @@
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
@@ -5893,7 +5936,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5945,7 @@
         <v>46150</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
@@ -5921,7 +5964,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “WNBA”</t>
         </is>
       </c>
     </row>
@@ -5930,7 +5973,7 @@
         <v>46150</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
@@ -5949,35 +5992,35 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “WNBA”</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="36" t="n">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C23" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D23" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C23" s="55" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
@@ -5986,7 +6029,7 @@
         <v>46151</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
@@ -6000,12 +6043,12 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6014,16 +6057,16 @@
         <v>46151</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D25" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D25" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E25" s="35" t="inlineStr">
@@ -6033,7 +6076,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -6042,26 +6085,26 @@
         <v>46151</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>120</v>
+        <v>230</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D26" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
         </is>
       </c>
     </row>
@@ -6070,35 +6113,35 @@
         <v>46151</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="C27" s="55" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D27" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>120</v>
+      </c>
+      <c r="C27" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46151</v>
+        <v>46157</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C28" s="40" t="inlineStr">
         <is>
@@ -6117,16 +6160,16 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="36" t="n">
-        <v>46157</v>
+        <v>46165</v>
       </c>
       <c r="B29" s="38" t="n">
-        <v>150</v>
+        <v>205</v>
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
@@ -6140,21 +6183,21 @@
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
@@ -6168,21 +6211,21 @@
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
@@ -6201,7 +6244,7 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
@@ -6229,16 +6272,16 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="36" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
@@ -6252,12 +6295,12 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
@@ -6265,9 +6308,7 @@
       <c r="A34" s="31" t="n">
         <v>46172</v>
       </c>
-      <c r="B34" s="33" t="n">
-        <v>120</v>
-      </c>
+      <c r="B34" s="33" t="inlineStr"/>
       <c r="C34" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6280,12 +6321,12 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
@@ -6294,7 +6335,7 @@
         <v>46172</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="C35" s="37" t="inlineStr">
         <is>
@@ -6313,7 +6354,7 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
+          <t>Nike Kobe Air Force 1 Low “Daybreak”</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6363,7 @@
         <v>46172</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
         <is>
@@ -6336,18 +6377,18 @@
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike Air Foamposite One “Tianjin 2.0”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46172</v>
+        <v>46179</v>
       </c>
       <c r="B37" s="38" t="inlineStr"/>
       <c r="C37" s="37" t="inlineStr">
@@ -6367,15 +6408,17 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B38" s="33" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="B38" s="33" t="n">
+        <v>355</v>
+      </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6393,16 +6436,16 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46182</v>
+        <v>46186</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>355</v>
+        <v>205</v>
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
@@ -6421,7 +6464,7 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
@@ -6430,44 +6473,44 @@
         <v>46186</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="C41" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D41" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+      <c r="D41" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
@@ -6477,7 +6520,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
@@ -6486,7 +6529,7 @@
         <v>46193</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>215</v>
+        <v>240</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
         <is>
@@ -6500,12 +6543,12 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Black University Blue” 2026</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6557,7 @@
         <v>46193</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>162</v>
+        <v>200</v>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
@@ -6533,7 +6576,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Nike Air Max 95 Total 90 “University Red”</t>
         </is>
       </c>
     </row>
@@ -6542,7 +6585,7 @@
         <v>46193</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C44" s="40" t="inlineStr">
         <is>
@@ -6556,21 +6599,21 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Air Jordan 5 “Black University Blue” 2026</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46193</v>
+        <v>46199</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C45" s="37" t="inlineStr">
         <is>
@@ -6589,17 +6632,15 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Total 90 “University Red”</t>
+          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46199</v>
-      </c>
-      <c r="B46" s="33" t="n">
-        <v>190</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B46" s="33" t="inlineStr"/>
       <c r="C46" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6612,12 +6653,12 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6666,9 @@
       <c r="A47" s="36" t="n">
         <v>46200</v>
       </c>
-      <c r="B47" s="38" t="inlineStr"/>
+      <c r="B47" s="38" t="n">
+        <v>185</v>
+      </c>
       <c r="C47" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6643,7 +6686,7 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
@@ -6652,7 +6695,7 @@
         <v>46200</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
@@ -6666,12 +6709,12 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
@@ -6680,7 +6723,7 @@
         <v>46200</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
@@ -6699,7 +6742,7 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6751,7 @@
         <v>46200</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="C50" s="40" t="inlineStr">
         <is>
@@ -6727,13 +6770,13 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>JuJu Watkins x Nike LeBron NXXT Gen “Silver Lining”</t>
+          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="B51" s="38" t="n">
         <v>135</v>
@@ -6743,9 +6786,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D51" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E51" s="35" t="inlineStr">
@@ -6755,25 +6798,25 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Cow Print” Pack</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C52" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D52" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D52" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E52" s="30" t="inlineStr">
@@ -6783,16 +6826,16 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46204</v>
+        <v>46210</v>
       </c>
       <c r="B53" s="38" t="n">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
@@ -6811,16 +6854,16 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
@@ -6834,30 +6877,28 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Air Jordan 4 “Birds of Paradise”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B55" s="38" t="n">
-        <v>215</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="B55" s="38" t="inlineStr"/>
       <c r="C55" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D55" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D55" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E55" s="35" t="inlineStr">
@@ -6867,23 +6908,25 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Birds of Paradise”</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46214</v>
-      </c>
-      <c r="B56" s="33" t="inlineStr"/>
+        <v>46218</v>
+      </c>
+      <c r="B56" s="33" t="n">
+        <v>205</v>
+      </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D56" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
@@ -6893,25 +6936,25 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>Air Jordan 3 “Sports Renaissance”</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B57" s="38" t="n">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D57" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D57" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E57" s="35" t="inlineStr">
@@ -6921,25 +6964,25 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Sports Renaissance”</t>
+          <t>Free The Youth x Air Jordan 16</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D58" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D58" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
@@ -6949,40 +6992,12 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 16</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="36" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B59" s="38" t="n">
-        <v>230</v>
-      </c>
-      <c r="C59" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D59" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E59" s="35" t="inlineStr">
-        <is>
-          <t>Jordan</t>
-        </is>
-      </c>
-      <c r="F59" s="35" t="inlineStr">
-        <is>
           <t>Air Jordan 3 OG “True Blue” 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F59"/>
+  <autoFilter ref="A3:F58"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-04-21 07:56 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1581,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated April 20, 2026  ·  08:12 UTC</t>
+          <t>Generated April 21, 2026  ·  07:56 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1621,11 +1621,11 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1634,7 +1634,7 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$185</t>
+          <t>$184</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1737,7 +1737,7 @@
         <v>46151</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46186</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1805,7 +1805,7 @@
         <v>46133</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         <v>46133</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -1861,19 +1861,19 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
         <v>46135</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="H14" s="43" t="inlineStr">
         <is>
@@ -1895,19 +1895,19 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C15" s="36" t="n">
         <v>46135</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="H15" s="42" t="inlineStr">
         <is>
@@ -1941,7 +1941,7 @@
         <v>46136</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" s="40" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G22" s="49" t="inlineStr">
         <is>
@@ -2163,17 +2163,17 @@
       </c>
       <c r="B28" s="30" t="inlineStr">
         <is>
-          <t>4/20 – 4/26</t>
+          <t>4/21 – 4/27</t>
         </is>
       </c>
       <c r="C28" s="30" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D28" s="40" t="n">
         <v>11</v>
       </c>
       <c r="E28" s="30" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2184,11 +2184,11 @@
       </c>
       <c r="B29" s="35" t="inlineStr">
         <is>
-          <t>4/27 – 5/3</t>
+          <t>4/28 – 5/4</t>
         </is>
       </c>
       <c r="C29" s="35" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D29" s="37" t="n">
         <v>4</v>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="B30" s="30" t="inlineStr">
         <is>
-          <t>5/4 – 5/10</t>
+          <t>5/5 – 5/11</t>
         </is>
       </c>
       <c r="C30" s="30" t="n">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>5/11 – 5/17</t>
+          <t>5/12 – 5/18</t>
         </is>
       </c>
       <c r="C31" s="35" t="n">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B32" s="30" t="inlineStr">
         <is>
-          <t>5/18 – 5/24</t>
+          <t>5/19 – 5/25</t>
         </is>
       </c>
       <c r="C32" s="30" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>5/25 – 5/31</t>
+          <t>5/26 – 6/1</t>
         </is>
       </c>
       <c r="C33" s="35" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B34" s="30" t="inlineStr">
         <is>
-          <t>6/1 – 6/7</t>
+          <t>6/2 – 6/8</t>
         </is>
       </c>
       <c r="C34" s="30" t="n">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>6/8 – 6/14</t>
+          <t>6/9 – 6/15</t>
         </is>
       </c>
       <c r="C35" s="35" t="n">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="B36" s="30" t="inlineStr">
         <is>
-          <t>6/15 – 6/21</t>
+          <t>6/16 – 6/22</t>
         </is>
       </c>
       <c r="C36" s="30" t="n">
@@ -2352,17 +2352,17 @@
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>6/22 – 6/28</t>
+          <t>6/23 – 6/29</t>
         </is>
       </c>
       <c r="C37" s="35" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D37" s="37" t="n">
         <v>6</v>
       </c>
       <c r="E37" s="35" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="B38" s="30" t="inlineStr">
         <is>
-          <t>6/29 – 7/5</t>
+          <t>6/30 – 7/6</t>
         </is>
       </c>
       <c r="C38" s="30" t="n">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>7/6 – 7/12</t>
+          <t>7/7 – 7/13</t>
         </is>
       </c>
       <c r="C39" s="35" t="n">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B40" s="30" t="inlineStr">
         <is>
-          <t>7/13 – 7/19</t>
+          <t>7/14 – 7/20</t>
         </is>
       </c>
       <c r="C40" s="30" t="n">
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -2674,7 +2674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2700,7 +2700,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated April 20, 2026  ·  08:12 UTC</t>
+          <t>Generated April 21, 2026  ·  07:56 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2830,7 +2830,7 @@
         <v>46135</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
@@ -2844,12 +2844,12 @@
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low “Steam”</t>
+          <t>Air Jordan 4 Denim “Iced Carmine”</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
         <v>46135</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
@@ -2872,12 +2872,12 @@
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Denim “Iced Carmine”</t>
+          <t>Nike Kobe Air Force 1 Low “Steam”</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
         <v>46136</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
+          <t>Nike LeBron 23 “Motor King”</t>
         </is>
       </c>
     </row>
@@ -3026,11 +3026,11 @@
         <v>46136</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C14" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C14" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D14" s="43" t="inlineStr">
@@ -3045,15 +3045,17 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Motor King”</t>
+          <t>Nike Air Max Uptempo “Derek Fisher”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="36" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B15" s="38" t="inlineStr"/>
+        <v>46136</v>
+      </c>
+      <c r="B15" s="38" t="n">
+        <v>200</v>
+      </c>
       <c r="C15" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3071,7 +3073,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
+          <t>Nike Kobe 8 Protro “Siempre Hermanos”</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3107,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="36" t="n">
-        <v>46142</v>
+        <v>46137</v>
       </c>
       <c r="B17" s="38" t="inlineStr"/>
       <c r="C17" s="37" t="inlineStr">
@@ -3120,12 +3122,12 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Cap and Gown”</t>
+          <t>Kobe Bryant Nike Air Force 1 Low Protro “Denim”</t>
         </is>
       </c>
     </row>
@@ -3133,9 +3135,7 @@
       <c r="A18" s="31" t="n">
         <v>46142</v>
       </c>
-      <c r="B18" s="33" t="n">
-        <v>215</v>
-      </c>
+      <c r="B18" s="33" t="inlineStr"/>
       <c r="C18" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3153,7 +3153,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sail Neutral Olive”</t>
+          <t>Air Jordan 6 “Cap and Gown”</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
         <v>46142</v>
       </c>
       <c r="B19" s="38" t="n">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Orange Citrus” 2026</t>
+          <t>Air Jordan 6 “Sail Neutral Olive”</t>
         </is>
       </c>
     </row>
@@ -3190,11 +3190,11 @@
         <v>46142</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C20" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D20" s="43" t="inlineStr">
@@ -3204,12 +3204,12 @@
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
+          <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3218,7 @@
         <v>46142</v>
       </c>
       <c r="B21" s="38" t="n">
-        <v>95</v>
+        <v>200</v>
       </c>
       <c r="C21" s="54" t="inlineStr">
         <is>
@@ -3237,7 +3237,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Mind 001 “Blackened Blue”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black” 2026</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3246,7 @@
         <v>46142</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>200</v>
+        <v>95</v>
       </c>
       <c r="C22" s="48" t="inlineStr">
         <is>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
+          <t>Nike Mind 001 “Blackened Blue”</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3274,7 @@
         <v>46142</v>
       </c>
       <c r="B23" s="38" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C23" s="54" t="inlineStr">
         <is>
@@ -3293,16 +3293,16 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Liquid Max “Triple Black”</t>
+          <t>Nike Zoom Huarache 2K4 OT “Black”</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46143</v>
+        <v>46142</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>190</v>
+        <v>230</v>
       </c>
       <c r="C24" s="48" t="inlineStr">
         <is>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4 “White Varsity Red”</t>
+          <t>Nike Air Liquid Max “Triple Black”</t>
         </is>
       </c>
     </row>
@@ -3330,7 +3330,7 @@
         <v>46143</v>
       </c>
       <c r="B25" s="38" t="n">
-        <v>135</v>
+        <v>190</v>
       </c>
       <c r="C25" s="54" t="inlineStr">
         <is>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Uncle Phil”</t>
+          <t>Nike Air Zoom Huarache 2K4 “White Varsity Red”</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3358,7 @@
         <v>46143</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="C26" s="48" t="inlineStr">
         <is>
@@ -3377,20 +3377,20 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4</t>
+          <t>Nike Air DT Max 96 Low</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="36" t="n">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="B27" s="38" t="n">
-        <v>145</v>
-      </c>
-      <c r="C27" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C27" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D27" s="42" t="inlineStr">
@@ -3400,12 +3400,12 @@
       </c>
       <c r="E27" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Banned”</t>
+          <t>Nike Air Zoom Huarache 2K4</t>
         </is>
       </c>
     </row>
@@ -3416,9 +3416,9 @@
       <c r="B28" s="33" t="n">
         <v>145</v>
       </c>
-      <c r="C28" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D28" s="43" t="inlineStr">
@@ -3428,12 +3428,12 @@
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike A’Two “A’Pink Shoe”</t>
+          <t>Air Jordan 1 Low OG “Banned”</t>
         </is>
       </c>
     </row>
@@ -3461,20 +3461,20 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “Pink Beam”</t>
+          <t>Nike A’Two “A’Pink Shoe”</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46149</v>
+        <v>46144</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C30" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C30" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D30" s="43" t="inlineStr">
@@ -3489,16 +3489,16 @@
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 Big Bubble “Slate”</t>
+          <t>Nike A’Two “Pink Beam”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="36" t="n">
-        <v>46150</v>
+        <v>46146</v>
       </c>
       <c r="B31" s="38" t="n">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C31" s="54" t="inlineStr">
         <is>
@@ -3517,16 +3517,16 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Nike Book 2 “WNBA 30th Anniversary”</t>
+          <t>Nike Ja 3 “Uncle Phil”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46150</v>
+        <v>46149</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Voltage”</t>
+          <t>Nike Air Max 95 Big Bubble “Slate”</t>
         </is>
       </c>
     </row>
@@ -3554,11 +3554,11 @@
         <v>46150</v>
       </c>
       <c r="B33" s="38" t="n">
-        <v>190</v>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C33" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D33" s="42" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low EM Protro “WNBA”</t>
+          <t>Nike Book 2 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3582,7 @@
         <v>46150</v>
       </c>
       <c r="B34" s="33" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
         <is>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Old Glory”</t>
+          <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
     </row>
@@ -3610,11 +3610,11 @@
         <v>46150</v>
       </c>
       <c r="B35" s="38" t="n">
-        <v>210</v>
-      </c>
-      <c r="C35" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D35" s="42" t="inlineStr">
@@ -3629,48 +3629,48 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
+          <t>Nike Kobe 9 Elite Low EM Protro “WNBA”</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="31" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C36" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D36" s="34" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>210</v>
+      </c>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D36" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
+          <t>Nike LeBron 23 “Old Glory”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46151</v>
+        <v>46150</v>
       </c>
       <c r="B37" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="C37" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>210</v>
+      </c>
+      <c r="C37" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D37" s="42" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Comet Red” 2026</t>
+          <t>Nike GT Cut 4 “WNBA 30th Anniversary”</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3694,7 @@
         <v>46151</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
         <is>
@@ -3708,12 +3708,12 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 Low “Mothers Day”</t>
+          <t>Nike Air Max 95 “Comet Red” 2026</t>
         </is>
       </c>
     </row>
@@ -3722,16 +3722,16 @@
         <v>46151</v>
       </c>
       <c r="B39" s="38" t="n">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D39" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D39" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E39" s="35" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
+          <t>Air Jordan 11 Low “Mothers Day”</t>
         </is>
       </c>
     </row>
@@ -3750,39 +3750,39 @@
         <v>46151</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>120</v>
+        <v>230</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D40" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Mineral Slate”</t>
+          <t>Nigel Sylvester x Air Jordan 4 “Brick After Brick” (2026)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46156</v>
+        <v>46151</v>
       </c>
       <c r="B41" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C41" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>120</v>
+      </c>
+      <c r="C41" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D41" s="42" t="inlineStr">
@@ -3792,49 +3792,49 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Converse SHAI 001 Premium “Ink”</t>
+          <t>Nike SB Dunk Low “Mineral Slate”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46157</v>
+        <v>46151</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C42" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D42" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C42" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D42" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Freshwater”</t>
+          <t>Travis Scott x Air Jordan 1 Low OG “Shy Pink” Pack</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="36" t="n">
-        <v>46157</v>
+        <v>46156</v>
       </c>
       <c r="B43" s="38" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="C43" s="50" t="inlineStr">
         <is>
@@ -3848,12 +3848,12 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>PUMA MB.05 Lo “Flourish”</t>
+          <t>Converse SHAI 001 Premium “Ink”</t>
         </is>
       </c>
     </row>
@@ -3862,11 +3862,11 @@
         <v>46157</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C44" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C44" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D44" s="43" t="inlineStr">
@@ -3881,16 +3881,16 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1 “San Diego Padres”</t>
+          <t>Nike Air Griffey Max 1 “Freshwater”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46158</v>
+        <v>46157</v>
       </c>
       <c r="B45" s="38" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="C45" s="50" t="inlineStr">
         <is>
@@ -3904,30 +3904,30 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Puma</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
+          <t>PUMA MB.05 Lo “Flourish”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46163</v>
+        <v>46157</v>
       </c>
       <c r="B46" s="33" t="n">
         <v>150</v>
       </c>
-      <c r="C46" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D46" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C46" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="30" t="inlineStr">
@@ -3937,20 +3937,20 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max Mad 90 Pack</t>
+          <t>Nike Air Max 1 “San Diego Padres”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46164</v>
+        <v>46158</v>
       </c>
       <c r="B47" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C47" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>160</v>
+      </c>
+      <c r="C47" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D47" s="42" t="inlineStr">
@@ -3960,53 +3960,53 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “DMV”</t>
+          <t>adidas Harden Vol. 10 “Hi-Res Yellow”</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46165</v>
+        <v>46163</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C48" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D48" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C48" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D48" s="41" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Bloodline”</t>
+          <t>Nike Air Max Mad 90 Pack</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="36" t="n">
-        <v>46168</v>
+        <v>46164</v>
       </c>
       <c r="B49" s="38" t="n">
-        <v>235</v>
-      </c>
-      <c r="C49" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C49" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D49" s="42" t="inlineStr">
@@ -4021,20 +4021,20 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
+          <t>Nike Zoom Hyperflight “DMV”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46170</v>
+        <v>46165</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C50" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D50" s="43" t="inlineStr">
@@ -4044,21 +4044,21 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Haven and Hector”</t>
+          <t>Air Jordan 12 “Bloodline”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46171</v>
+        <v>46168</v>
       </c>
       <c r="B51" s="38" t="n">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
@@ -4077,16 +4077,16 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
+          <t>Nike LeBron 23 “Dreams And Nightmares”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46171</v>
+        <v>46170</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C52" s="48" t="inlineStr">
         <is>
@@ -4105,7 +4105,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Bright Ceramic”</t>
+          <t>Nike Book 2 “Haven and Hector”</t>
         </is>
       </c>
     </row>
@@ -4133,20 +4133,20 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Gym Red”</t>
+          <t>Nike Air Foamposite Pro “Gym Red” 2026</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C54" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C54" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D54" s="43" t="inlineStr">
@@ -4156,20 +4156,22 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Toro Bravo” 2026</t>
+          <t>Nike KD 19 “Bright Ceramic”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B55" s="38" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="B55" s="38" t="n">
+        <v>240</v>
+      </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4182,12 +4184,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “World’s Best Dad”</t>
+          <t>Nike Air Foamposite Pro “Gym Red”</t>
         </is>
       </c>
     </row>
@@ -4275,14 +4277,14 @@
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B59" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C59" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C59" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D59" s="42" t="inlineStr">
@@ -4292,25 +4294,23 @@
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Air DT Max 96 Low “Black White”</t>
+          <t>Air Jordan 4 “Toro Bravo” 2026</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B60" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C60" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46172</v>
+      </c>
+      <c r="B60" s="33" t="inlineStr"/>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
@@ -4320,23 +4320,25 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision” 2026</t>
+          <t>Air Jordan 3 “World’s Best Dad”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B61" s="38" t="inlineStr"/>
-      <c r="C61" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46173</v>
+      </c>
+      <c r="B61" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="C61" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D61" s="42" t="inlineStr">
@@ -4346,25 +4348,25 @@
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 23RE “Black Muslin”</t>
+          <t>Nike Air DT Max 96 Low “Black White”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46182</v>
+        <v>46177</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="C62" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C62" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D62" s="43" t="inlineStr">
@@ -4374,25 +4376,23 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “BIN 23”</t>
+          <t>Nike KD 6 “Night Vision” 2026</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B63" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="C63" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46179</v>
+      </c>
+      <c r="B63" s="38" t="inlineStr"/>
+      <c r="C63" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D63" s="42" t="inlineStr">
@@ -4402,25 +4402,25 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
+          <t>Air Jordan 15 23RE “Black Muslin”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C64" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>355</v>
+      </c>
+      <c r="C64" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D64" s="43" t="inlineStr">
@@ -4430,12 +4430,12 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “Royals”</t>
+          <t>Air Jordan 3 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -4463,20 +4463,20 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “49ers”</t>
+          <t>Nike Air Diamond Turf 2 “Royals”</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>205</v>
-      </c>
-      <c r="C66" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C66" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D66" s="43" t="inlineStr">
@@ -4486,30 +4486,30 @@
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4028 “Rui Hachimura”</t>
+          <t>Nike Air Diamond Turf 2 “49ers” 2026</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="B67" s="38" t="n">
-        <v>150</v>
-      </c>
-      <c r="C67" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D67" s="39" t="inlineStr">
-        <is>
-          <t>Raffle/Dropship</t>
+        <v>170</v>
+      </c>
+      <c r="C67" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D67" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E67" s="35" t="inlineStr">
@@ -4519,7 +4519,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 ’87</t>
+          <t>Nike Air Diamond Turf 2 “49ers”</t>
         </is>
       </c>
     </row>
@@ -4528,16 +4528,16 @@
         <v>46186</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C68" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D68" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C68" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D68" s="34" t="inlineStr">
+        <is>
+          <t>Raffle/Dropship</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>PJ Tucker x Nike GT Future</t>
+          <t>Patta x Nike Air Max 1 ’87</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
         <v>46186</v>
       </c>
       <c r="B69" s="38" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C69" s="54" t="inlineStr">
         <is>
@@ -4575,7 +4575,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Air More Uptempo “Legacy”</t>
+          <t>PJ Tucker x Nike GT Future</t>
         </is>
       </c>
     </row>
@@ -4584,16 +4584,16 @@
         <v>46186</v>
       </c>
       <c r="B70" s="33" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="C70" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D70" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D70" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E70" s="30" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Patta x Nike Cryoshot Mercurial</t>
+          <t>Nike Air More Uptempo “Legacy”</t>
         </is>
       </c>
     </row>
@@ -4612,16 +4612,16 @@
         <v>46186</v>
       </c>
       <c r="B71" s="38" t="n">
-        <v>155</v>
+        <v>210</v>
       </c>
       <c r="C71" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D71" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D71" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E71" s="35" t="inlineStr">
@@ -4631,20 +4631,20 @@
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 19</t>
+          <t>Patta x Nike Cryoshot Mercurial</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46192</v>
+        <v>46186</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C72" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C72" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D72" s="43" t="inlineStr">
@@ -4654,25 +4654,25 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Night Vision”</t>
+          <t>Air Jordan 4028 “Rui Hachimura”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46193</v>
+        <v>46186</v>
       </c>
       <c r="B73" s="38" t="n">
-        <v>162</v>
-      </c>
-      <c r="C73" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C73" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
@@ -4687,20 +4687,20 @@
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
+          <t>Nike KD 19</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C74" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C74" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D74" s="43" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Nike KD 6 “Night Vision”</t>
         </is>
       </c>
     </row>
@@ -4780,7 +4780,7 @@
         <v>46193</v>
       </c>
       <c r="B77" s="38" t="n">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C77" s="37" t="inlineStr">
         <is>
@@ -4833,14 +4833,14 @@
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="36" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B79" s="38" t="n">
-        <v>180</v>
-      </c>
-      <c r="C79" s="54" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>162</v>
+      </c>
+      <c r="C79" s="37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4855,16 +4855,16 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic” 2026</t>
+          <t>LEGO x Nike Air Max 95 “Brick Pixel”</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46199</v>
+        <v>46193</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C80" s="40" t="inlineStr">
         <is>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
@@ -4911,15 +4911,17 @@
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Shox BB4 “Olympic”</t>
+          <t>Nike Shox BB4 “Olympic” 2026</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="31" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B82" s="33" t="inlineStr"/>
+        <v>46199</v>
+      </c>
+      <c r="B82" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C82" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4932,25 +4934,25 @@
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “Sashiko”</t>
+          <t>Nike Kobe 4 Protro Draft Day “Boston Celtics”</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="36" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B83" s="38" t="n">
-        <v>185</v>
-      </c>
-      <c r="C83" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C83" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D83" s="42" t="inlineStr">
@@ -4960,25 +4962,25 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Workwear”</t>
+          <t>Nike Book 2 “Just Book”</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C84" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C84" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D84" s="43" t="inlineStr">
@@ -4993,7 +4995,7 @@
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
+          <t>Nike Shox BB4 “Olympic”</t>
         </is>
       </c>
     </row>
@@ -5081,38 +5083,36 @@
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B88" s="33" t="n">
-        <v>135</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B88" s="33" t="inlineStr"/>
       <c r="C88" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D88" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D88" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Bluetile x Nike SB Dunk Low</t>
+          <t>Air Jordan 6 “Sashiko”</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46204</v>
+        <v>46200</v>
       </c>
       <c r="B89" s="38" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C89" s="37" t="inlineStr">
         <is>
@@ -5126,25 +5126,25 @@
       </c>
       <c r="E89" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
+          <t>Air Jordan 1 High OG “Workwear”</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="31" t="n">
-        <v>46206</v>
+        <v>46200</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C90" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C90" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D90" s="43" t="inlineStr">
@@ -5159,25 +5159,25 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Animal Instinct”</t>
+          <t>Caitlin Clark x Nike Kobe 5 Protro “Coconut Milk”</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="36" t="n">
-        <v>46210</v>
+        <v>46203</v>
       </c>
       <c r="B91" s="38" t="n">
-        <v>210</v>
+        <v>135</v>
       </c>
       <c r="C91" s="37" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D91" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D91" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E91" s="35" t="inlineStr">
@@ -5187,48 +5187,48 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Hardwood Classic”</t>
+          <t>Bluetile x Nike SB Dunk Low</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46213</v>
+        <v>46204</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="C92" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D92" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>190</v>
+      </c>
+      <c r="C92" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D92" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 8 “BIN 23”</t>
+          <t>Nike Kobe 3 Low Protro “Atomic Pink”</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46213</v>
+        <v>46206</v>
       </c>
       <c r="B93" s="38" t="n">
-        <v>215</v>
-      </c>
-      <c r="C93" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C93" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D93" s="42" t="inlineStr">
@@ -5238,56 +5238,58 @@
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Birds of Paradise”</t>
+          <t>Nike Ja 3 “Animal Instinct”</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="31" t="n">
-        <v>46214</v>
-      </c>
-      <c r="B94" s="33" t="inlineStr"/>
+        <v>46210</v>
+      </c>
+      <c r="B94" s="33" t="n">
+        <v>210</v>
+      </c>
       <c r="C94" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D94" s="41" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D94" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>Nike LeBron 23 “Hardwood Classic”</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="36" t="n">
-        <v>46218</v>
+        <v>46213</v>
       </c>
       <c r="B95" s="38" t="n">
-        <v>205</v>
-      </c>
-      <c r="C95" s="37" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D95" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>355</v>
+      </c>
+      <c r="C95" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D95" s="53" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
@@ -5297,20 +5299,20 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Sports Renaissance”</t>
+          <t>Air Jordan 8 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="A96" s="31" t="n">
-        <v>46220</v>
+        <v>46213</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>210</v>
-      </c>
-      <c r="C96" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C96" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D96" s="43" t="inlineStr">
@@ -5320,22 +5322,20 @@
       </c>
       <c r="E96" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Huarache 2K4 “Sue Bird” PE</t>
+          <t>Air Jordan 4 “Birds of Paradise”</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight=